<commit_message>
Correccion: Ya no se calcula la duracion de la reparacion de un equipo hasta que se inicia la reparacion del mismo
</commit_message>
<xml_diff>
--- a/1er Entrega/Plantilla.xlsx
+++ b/1er Entrega/Plantilla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\UTN\Simulación\TP 4\Tp4-Simulacion-G5\1er Entrega\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68F53BC4-5D29-495B-A12A-33E34083BB49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{146DAC6F-4680-4A94-A8CA-610AED6A1729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="102">
   <si>
     <t>Horario Apertura</t>
   </si>
@@ -509,41 +509,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -584,16 +551,49 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -911,28 +911,28 @@
         <v>3</v>
       </c>
       <c r="C2" s="2"/>
-      <c r="E2" s="40" t="s">
+      <c r="E2" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
       <c r="J2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="11" t="s">
+      <c r="K2" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="Q2" s="14" t="s">
+      <c r="L2" s="38"/>
+      <c r="M2" s="38"/>
+      <c r="N2" s="38"/>
+      <c r="O2" s="38"/>
+      <c r="Q2" s="41" t="s">
         <v>73</v>
       </c>
-      <c r="R2" s="14"/>
-      <c r="S2" s="14"/>
-      <c r="T2" s="14"/>
+      <c r="R2" s="41"/>
+      <c r="S2" s="41"/>
+      <c r="T2" s="41"/>
     </row>
     <row r="3" spans="2:52" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
@@ -947,24 +947,24 @@
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
-      <c r="Q3" s="9" t="s">
+      <c r="Q3" s="28" t="s">
         <v>72</v>
       </c>
-      <c r="R3" s="9"/>
-      <c r="S3" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="T3" s="9"/>
+      <c r="R3" s="28"/>
+      <c r="S3" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="T3" s="28"/>
     </row>
     <row r="4" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="28" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="9"/>
-      <c r="E4" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9"/>
+      <c r="C4" s="28"/>
+      <c r="E4" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" s="28"/>
       <c r="G4" s="2">
         <v>10</v>
       </c>
@@ -983,20 +983,20 @@
       <c r="O4" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="Q4" s="9" t="s">
+      <c r="Q4" s="28" t="s">
         <v>74</v>
       </c>
-      <c r="R4" s="9"/>
-      <c r="S4" s="9" t="s">
+      <c r="R4" s="28"/>
+      <c r="S4" s="28" t="s">
         <v>76</v>
       </c>
-      <c r="T4" s="9"/>
+      <c r="T4" s="28"/>
     </row>
     <row r="5" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="9"/>
+      <c r="F5" s="28"/>
       <c r="G5" s="2">
         <v>18</v>
       </c>
@@ -1017,10 +1017,6 @@
       <c r="O5" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="Q5" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="R5" s="9"/>
     </row>
     <row r="6" spans="2:52" ht="60" x14ac:dyDescent="0.25">
       <c r="J6" s="6" t="s">
@@ -1048,30 +1044,30 @@
       <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9" t="s">
+      <c r="F7" s="28"/>
+      <c r="G7" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="9"/>
-      <c r="S7" s="30" t="s">
+      <c r="H7" s="28"/>
+      <c r="S7" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="T7" s="41">
+      <c r="T7" s="27">
         <f ca="1">RAND()</f>
-        <v>0.95478665230448911</v>
+        <v>0.98911930971154549</v>
       </c>
     </row>
     <row r="8" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="28" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -1080,68 +1076,68 @@
       <c r="F8" s="2">
         <v>10</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="H8" s="13"/>
+      <c r="H8" s="29"/>
     </row>
     <row r="9" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
       <c r="E9" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="2">
         <v>20</v>
       </c>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="J9" s="10" t="s">
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
+      <c r="J9" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="10"/>
-      <c r="O9" s="10"/>
-      <c r="P9" s="10"/>
-      <c r="Q9" s="10"/>
-      <c r="R9" s="10"/>
-      <c r="S9" s="10"/>
-      <c r="T9" s="10"/>
-      <c r="U9" s="10"/>
-      <c r="V9" s="10"/>
-      <c r="W9" s="10"/>
-      <c r="X9" s="10"/>
-      <c r="Y9" s="10"/>
-      <c r="Z9" s="10"/>
-      <c r="AA9" s="10"/>
-      <c r="AB9" s="10"/>
-      <c r="AC9" s="10"/>
-      <c r="AD9" s="10"/>
-      <c r="AE9" s="10"/>
-      <c r="AF9" s="10"/>
-      <c r="AG9" s="10"/>
-      <c r="AH9" s="10"/>
-      <c r="AI9" s="10"/>
-      <c r="AJ9" s="10"/>
-      <c r="AK9" s="10"/>
-      <c r="AL9" s="10"/>
-      <c r="AM9" s="10"/>
-      <c r="AN9" s="10"/>
-      <c r="AO9" s="10"/>
-      <c r="AP9" s="10"/>
-      <c r="AQ9" s="10"/>
-      <c r="AR9" s="10"/>
-      <c r="AS9" s="10"/>
-      <c r="AT9" s="10"/>
-      <c r="AU9" s="10"/>
-      <c r="AV9" s="10"/>
-      <c r="AW9" s="10"/>
-      <c r="AX9" s="10"/>
-      <c r="AY9" s="10"/>
-      <c r="AZ9" s="10"/>
+      <c r="K9" s="37"/>
+      <c r="L9" s="37"/>
+      <c r="M9" s="37"/>
+      <c r="N9" s="37"/>
+      <c r="O9" s="37"/>
+      <c r="P9" s="37"/>
+      <c r="Q9" s="37"/>
+      <c r="R9" s="37"/>
+      <c r="S9" s="37"/>
+      <c r="T9" s="37"/>
+      <c r="U9" s="37"/>
+      <c r="V9" s="37"/>
+      <c r="W9" s="37"/>
+      <c r="X9" s="37"/>
+      <c r="Y9" s="37"/>
+      <c r="Z9" s="37"/>
+      <c r="AA9" s="37"/>
+      <c r="AB9" s="37"/>
+      <c r="AC9" s="37"/>
+      <c r="AD9" s="37"/>
+      <c r="AE9" s="37"/>
+      <c r="AF9" s="37"/>
+      <c r="AG9" s="37"/>
+      <c r="AH9" s="37"/>
+      <c r="AI9" s="37"/>
+      <c r="AJ9" s="37"/>
+      <c r="AK9" s="37"/>
+      <c r="AL9" s="37"/>
+      <c r="AM9" s="37"/>
+      <c r="AN9" s="37"/>
+      <c r="AO9" s="37"/>
+      <c r="AP9" s="37"/>
+      <c r="AQ9" s="37"/>
+      <c r="AR9" s="37"/>
+      <c r="AS9" s="37"/>
+      <c r="AT9" s="37"/>
+      <c r="AU9" s="37"/>
+      <c r="AV9" s="37"/>
+      <c r="AW9" s="37"/>
+      <c r="AX9" s="37"/>
+      <c r="AY9" s="37"/>
+      <c r="AZ9" s="37"/>
     </row>
     <row r="10" spans="2:52" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
@@ -1159,72 +1155,72 @@
       <c r="F10" s="2">
         <v>90</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="28" t="s">
         <v>29</v>
       </c>
-      <c r="H10" s="9"/>
-      <c r="AD10" s="38" t="s">
+      <c r="H10" s="28"/>
+      <c r="AD10" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="AE10" s="38"/>
-      <c r="AF10" s="38"/>
-      <c r="AG10" s="38"/>
-      <c r="AH10" s="38"/>
-      <c r="AI10" s="38"/>
+      <c r="AE10" s="30"/>
+      <c r="AF10" s="30"/>
+      <c r="AG10" s="30"/>
+      <c r="AH10" s="30"/>
+      <c r="AI10" s="30"/>
       <c r="AJ10" s="2"/>
-      <c r="AK10" s="39" t="s">
+      <c r="AK10" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="AL10" s="39"/>
-      <c r="AM10" s="39"/>
-      <c r="AN10" s="39"/>
-      <c r="AO10" s="39"/>
-      <c r="AP10" s="39"/>
-      <c r="AQ10" s="39"/>
-      <c r="AR10" s="39"/>
-      <c r="AS10" s="39"/>
-      <c r="AT10" s="39"/>
-      <c r="AU10" s="39"/>
-      <c r="AV10" s="39"/>
-      <c r="AW10" s="39"/>
-      <c r="AX10" s="39"/>
-      <c r="AY10" s="39"/>
-      <c r="AZ10" s="39"/>
+      <c r="AL10" s="36"/>
+      <c r="AM10" s="36"/>
+      <c r="AN10" s="36"/>
+      <c r="AO10" s="36"/>
+      <c r="AP10" s="36"/>
+      <c r="AQ10" s="36"/>
+      <c r="AR10" s="36"/>
+      <c r="AS10" s="36"/>
+      <c r="AT10" s="36"/>
+      <c r="AU10" s="36"/>
+      <c r="AV10" s="36"/>
+      <c r="AW10" s="36"/>
+      <c r="AX10" s="36"/>
+      <c r="AY10" s="36"/>
+      <c r="AZ10" s="36"/>
     </row>
     <row r="11" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="I11" s="13" t="s">
+      <c r="I11" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="J11" s="15"/>
-      <c r="K11" s="16"/>
-      <c r="L11" s="17" t="s">
+      <c r="J11" s="9"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="39" t="s">
         <v>72</v>
       </c>
-      <c r="M11" s="17"/>
-      <c r="N11" s="17"/>
-      <c r="O11" s="18" t="s">
+      <c r="M11" s="39"/>
+      <c r="N11" s="39"/>
+      <c r="O11" s="31" t="s">
         <v>77</v>
       </c>
-      <c r="P11" s="18"/>
-      <c r="Q11" s="18"/>
-      <c r="R11" s="18"/>
-      <c r="S11" s="18"/>
-      <c r="T11" s="18"/>
-      <c r="U11" s="18"/>
-      <c r="V11" s="18"/>
-      <c r="W11" s="19" t="s">
+      <c r="P11" s="31"/>
+      <c r="Q11" s="31"/>
+      <c r="R11" s="31"/>
+      <c r="S11" s="31"/>
+      <c r="T11" s="31"/>
+      <c r="U11" s="31"/>
+      <c r="V11" s="31"/>
+      <c r="W11" s="40" t="s">
         <v>78</v>
       </c>
-      <c r="X11" s="19"/>
-      <c r="Y11" s="20" t="s">
+      <c r="X11" s="40"/>
+      <c r="Y11" s="33" t="s">
         <v>69</v>
       </c>
-      <c r="Z11" s="20"/>
-      <c r="AA11" s="21" t="s">
+      <c r="Z11" s="33"/>
+      <c r="AA11" s="32" t="s">
         <v>46</v>
       </c>
-      <c r="AB11" s="21"/>
-      <c r="AC11" s="21"/>
+      <c r="AB11" s="32"/>
+      <c r="AC11" s="32"/>
       <c r="AD11" s="2">
         <v>1</v>
       </c>
@@ -1244,91 +1240,91 @@
         <v>79</v>
       </c>
       <c r="AJ11" s="2"/>
-      <c r="AK11" s="9">
+      <c r="AK11" s="28">
         <v>1</v>
       </c>
-      <c r="AL11" s="9"/>
-      <c r="AM11" s="9"/>
-      <c r="AN11" s="9"/>
-      <c r="AO11" s="9">
+      <c r="AL11" s="28"/>
+      <c r="AM11" s="28"/>
+      <c r="AN11" s="28"/>
+      <c r="AO11" s="28">
         <v>2</v>
       </c>
-      <c r="AP11" s="9"/>
-      <c r="AQ11" s="9"/>
-      <c r="AR11" s="9"/>
-      <c r="AS11" s="9">
+      <c r="AP11" s="28"/>
+      <c r="AQ11" s="28"/>
+      <c r="AR11" s="28"/>
+      <c r="AS11" s="28">
         <v>3</v>
       </c>
-      <c r="AT11" s="9"/>
-      <c r="AU11" s="9"/>
-      <c r="AV11" s="9"/>
-      <c r="AW11" s="9" t="s">
+      <c r="AT11" s="28"/>
+      <c r="AU11" s="28"/>
+      <c r="AV11" s="28"/>
+      <c r="AW11" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="AX11" s="9"/>
-      <c r="AY11" s="9"/>
-      <c r="AZ11" s="9"/>
+      <c r="AX11" s="28"/>
+      <c r="AY11" s="28"/>
+      <c r="AZ11" s="28"/>
     </row>
     <row r="12" spans="2:52" ht="60" x14ac:dyDescent="0.25">
-      <c r="I12" s="13"/>
-      <c r="J12" s="22" t="s">
+      <c r="I12" s="29"/>
+      <c r="J12" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="K12" s="23" t="s">
+      <c r="K12" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="L12" s="24" t="s">
+      <c r="L12" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="M12" s="24" t="s">
+      <c r="M12" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="N12" s="25" t="s">
+      <c r="N12" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="O12" s="26" t="s">
+      <c r="O12" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="P12" s="26" t="s">
+      <c r="P12" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="Q12" s="26" t="s">
+      <c r="Q12" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="R12" s="25" t="s">
+      <c r="R12" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="S12" s="26" t="s">
+      <c r="S12" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="T12" s="26" t="s">
+      <c r="T12" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="U12" s="26" t="s">
+      <c r="U12" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="V12" s="26" t="s">
+      <c r="V12" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="W12" s="27" t="s">
+      <c r="W12" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="X12" s="27" t="s">
+      <c r="X12" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="Y12" s="28" t="s">
+      <c r="Y12" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="Z12" s="28" t="s">
+      <c r="Z12" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="AA12" s="29" t="s">
+      <c r="AA12" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="AB12" s="29" t="s">
+      <c r="AB12" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="AC12" s="29" t="s">
+      <c r="AC12" s="18" t="s">
         <v>49</v>
       </c>
       <c r="AD12" s="8" t="s">
@@ -1403,7 +1399,7 @@
       <c r="I13" s="2">
         <v>1</v>
       </c>
-      <c r="J13" s="30">
+      <c r="J13" s="19">
         <v>0.41666666666666669</v>
       </c>
       <c r="K13" s="2" t="s">
@@ -1412,11 +1408,11 @@
       <c r="L13" s="2">
         <v>0.33300000000000002</v>
       </c>
-      <c r="M13" s="30">
+      <c r="M13" s="19">
         <f>-$C$3*(LN(1-L13)) / 1440</f>
         <v>1.265516353332854E-2</v>
       </c>
-      <c r="N13" s="31">
+      <c r="N13" s="20">
         <f>J13+M13</f>
         <v>0.4293218301999952</v>
       </c>
@@ -1424,24 +1420,24 @@
         <v>54</v>
       </c>
       <c r="P13" s="2"/>
-      <c r="Q13" s="30"/>
+      <c r="Q13" s="19"/>
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
-      <c r="X13" s="30"/>
+      <c r="X13" s="19"/>
       <c r="Y13" s="2">
         <v>0</v>
       </c>
       <c r="Z13" s="2">
         <v>0</v>
       </c>
-      <c r="AA13" s="30">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="30">
+      <c r="AA13" s="19">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="19">
         <v>0</v>
       </c>
       <c r="AC13" s="2">
@@ -1472,18 +1468,18 @@
       <c r="AZ13" s="2"/>
     </row>
     <row r="14" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
       <c r="I14" s="2">
         <f>I13+1</f>
         <v>2</v>
       </c>
-      <c r="J14" s="30">
+      <c r="J14" s="19">
         <v>0.42931712962962965</v>
       </c>
       <c r="K14" s="2" t="s">
@@ -1492,11 +1488,11 @@
       <c r="L14" s="2">
         <v>0.55800000000000005</v>
       </c>
-      <c r="M14" s="30">
+      <c r="M14" s="19">
         <f>-$C$3*(LN(1-L14)) / 1440</f>
         <v>2.5513918653263721E-2</v>
       </c>
-      <c r="N14" s="30">
+      <c r="N14" s="19">
         <f>J14+M14</f>
         <v>0.45483104828289339</v>
       </c>
@@ -1506,11 +1502,11 @@
       <c r="P14" s="2">
         <v>5.5E-2</v>
       </c>
-      <c r="Q14" s="30">
+      <c r="Q14" s="19">
         <f>($F$8+P14*($F$9-$F$8)) / 1440</f>
         <v>7.3263888888888892E-3</v>
       </c>
-      <c r="R14" s="31">
+      <c r="R14" s="20">
         <f>J14+Q14</f>
         <v>0.43664351851851851</v>
       </c>
@@ -1526,10 +1522,10 @@
       <c r="Z14" s="2">
         <v>0</v>
       </c>
-      <c r="AA14" s="30">
-        <v>0</v>
-      </c>
-      <c r="AB14" s="30">
+      <c r="AA14" s="19">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="19">
         <v>0</v>
       </c>
       <c r="AC14" s="2">
@@ -1581,7 +1577,7 @@
         <f t="shared" ref="I15:I22" si="0">I14+1</f>
         <v>3</v>
       </c>
-      <c r="J15" s="30">
+      <c r="J15" s="19">
         <f>R14</f>
         <v>0.43664351851851851</v>
       </c>
@@ -1589,17 +1585,17 @@
         <v>93</v>
       </c>
       <c r="L15" s="8"/>
-      <c r="M15" s="32"/>
-      <c r="N15" s="30">
+      <c r="M15" s="21"/>
+      <c r="N15" s="19">
         <f>N14</f>
         <v>0.45483104828289339</v>
       </c>
-      <c r="O15" s="30" t="s">
+      <c r="O15" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="P15" s="32"/>
-      <c r="Q15" s="32"/>
-      <c r="R15" s="32"/>
+      <c r="P15" s="21"/>
+      <c r="Q15" s="21"/>
+      <c r="R15" s="21"/>
       <c r="S15" s="2">
         <v>0.35499999999999998</v>
       </c>
@@ -1613,7 +1609,7 @@
       <c r="W15" s="2">
         <v>0.187</v>
       </c>
-      <c r="X15" s="31">
+      <c r="X15" s="20">
         <f>-90*LN(1-W15) / 1440</f>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -1623,17 +1619,17 @@
       <c r="Z15" s="2">
         <v>0</v>
       </c>
-      <c r="AA15" s="30">
+      <c r="AA15" s="19">
         <f>Q14</f>
         <v>7.3263888888888892E-3</v>
       </c>
-      <c r="AB15" s="30">
+      <c r="AB15" s="19">
         <v>0</v>
       </c>
       <c r="AC15" s="2">
         <v>0</v>
       </c>
-      <c r="AD15" s="33"/>
+      <c r="AD15" s="22"/>
       <c r="AE15" s="2"/>
       <c r="AF15" s="2"/>
       <c r="AG15" s="2"/>
@@ -1643,7 +1639,7 @@
       <c r="AK15" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="AL15" s="30">
+      <c r="AL15" s="19">
         <f>J15</f>
         <v>0.43664351851851851</v>
       </c>
@@ -1682,7 +1678,7 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="J16" s="30">
+      <c r="J16" s="19">
         <f>J15+X15</f>
         <v>0.44958252910816393</v>
       </c>
@@ -1690,34 +1686,34 @@
         <v>94</v>
       </c>
       <c r="L16" s="1"/>
-      <c r="M16" s="34"/>
-      <c r="N16" s="31">
+      <c r="M16" s="23"/>
+      <c r="N16" s="20">
         <f>N15</f>
         <v>0.45483104828289339</v>
       </c>
-      <c r="O16" s="30" t="s">
+      <c r="O16" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="P16" s="34"/>
-      <c r="Q16" s="34"/>
-      <c r="R16" s="34"/>
-      <c r="S16" s="34"/>
-      <c r="T16" s="34"/>
-      <c r="U16" s="34"/>
-      <c r="V16" s="34"/>
-      <c r="W16" s="34"/>
-      <c r="X16" s="30"/>
+      <c r="P16" s="23"/>
+      <c r="Q16" s="23"/>
+      <c r="R16" s="23"/>
+      <c r="S16" s="23"/>
+      <c r="T16" s="23"/>
+      <c r="U16" s="23"/>
+      <c r="V16" s="23"/>
+      <c r="W16" s="23"/>
+      <c r="X16" s="19"/>
       <c r="Y16" s="2">
         <v>0</v>
       </c>
       <c r="Z16" s="2">
         <v>0</v>
       </c>
-      <c r="AA16" s="30">
+      <c r="AA16" s="19">
         <f>AA15</f>
         <v>7.3263888888888892E-3</v>
       </c>
-      <c r="AB16" s="30">
+      <c r="AB16" s="19">
         <f>AB15+X15</f>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -1731,16 +1727,16 @@
       <c r="AH16" s="2"/>
       <c r="AI16" s="2"/>
       <c r="AJ16" s="2"/>
-      <c r="AK16" s="35"/>
-      <c r="AL16" s="30">
+      <c r="AK16" s="24"/>
+      <c r="AL16" s="19">
         <f>AL15</f>
         <v>0.43664351851851851</v>
       </c>
-      <c r="AM16" s="30">
+      <c r="AM16" s="19">
         <f>J16</f>
         <v>0.44958252910816393</v>
       </c>
-      <c r="AN16" s="30">
+      <c r="AN16" s="19">
         <f>AM16-AL16</f>
         <v>1.2939010589645417E-2</v>
       </c>
@@ -1777,7 +1773,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="J17" s="30">
+      <c r="J17" s="19">
         <f>N15</f>
         <v>0.45483104828289339</v>
       </c>
@@ -1787,11 +1783,11 @@
       <c r="L17" s="2">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="M17" s="30">
+      <c r="M17" s="19">
         <f>-$C$3*LN(1-L17) / 1440</f>
         <v>9.3890906884335122E-5</v>
       </c>
-      <c r="N17" s="31">
+      <c r="N17" s="20">
         <f>J17+M17</f>
         <v>0.45492493918977772</v>
       </c>
@@ -1801,11 +1797,11 @@
       <c r="P17" s="2">
         <v>0.35799999999999998</v>
       </c>
-      <c r="Q17" s="30">
+      <c r="Q17" s="19">
         <f>($F$8+P17*($F$9-$F$8)) / 1440</f>
         <v>9.4305555555555549E-3</v>
       </c>
-      <c r="R17" s="30">
+      <c r="R17" s="19">
         <f>J17+Q17</f>
         <v>0.46426160383844894</v>
       </c>
@@ -1821,12 +1817,12 @@
       <c r="Z17" s="2">
         <v>0</v>
       </c>
-      <c r="AA17" s="30">
+      <c r="AA17" s="19">
         <f>AA16+Q18</f>
         <v>1.6756944444444442E-2</v>
       </c>
-      <c r="AB17" s="30">
-        <f>AB16</f>
+      <c r="AB17" s="19">
+        <f t="shared" ref="AB17:AB22" si="1">AB16</f>
         <v>1.2939010589645406E-2</v>
       </c>
       <c r="AC17" s="2">
@@ -1842,9 +1838,9 @@
       <c r="AI17" s="2"/>
       <c r="AJ17" s="2"/>
       <c r="AK17" s="2"/>
-      <c r="AL17" s="35"/>
-      <c r="AM17" s="35"/>
-      <c r="AN17" s="35"/>
+      <c r="AL17" s="24"/>
+      <c r="AM17" s="24"/>
+      <c r="AN17" s="24"/>
       <c r="AO17" s="2"/>
       <c r="AP17" s="2"/>
       <c r="AQ17" s="2"/>
@@ -1863,7 +1859,7 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="J18" s="30">
+      <c r="J18" s="19">
         <f>N17</f>
         <v>0.45492493918977772</v>
       </c>
@@ -1873,11 +1869,11 @@
       <c r="L18" s="2">
         <v>0.44</v>
       </c>
-      <c r="M18" s="30">
+      <c r="M18" s="19">
         <f>-$C$3*LN(1-L18) / 1440</f>
         <v>1.8119327976654439E-2</v>
       </c>
-      <c r="N18" s="30">
+      <c r="N18" s="19">
         <f>J18+M18</f>
         <v>0.47304426716643216</v>
       </c>
@@ -1885,11 +1881,11 @@
         <v>62</v>
       </c>
       <c r="P18" s="1"/>
-      <c r="Q18" s="30">
+      <c r="Q18" s="19">
         <f>Q17</f>
         <v>9.4305555555555549E-3</v>
       </c>
-      <c r="R18" s="31">
+      <c r="R18" s="20">
         <f>R17</f>
         <v>0.46426160383844894</v>
       </c>
@@ -1905,12 +1901,12 @@
       <c r="Z18" s="2">
         <v>0</v>
       </c>
-      <c r="AA18" s="30">
+      <c r="AA18" s="19">
         <f>AA17+(J18-J17)</f>
         <v>1.6850835351328773E-2</v>
       </c>
-      <c r="AB18" s="30">
-        <f>AB17</f>
+      <c r="AB18" s="19">
+        <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
       <c r="AC18" s="2">
@@ -1945,18 +1941,18 @@
       <c r="AZ18" s="2"/>
     </row>
     <row r="19" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="B19" s="9" t="s">
+      <c r="B19" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
       <c r="I19" s="2">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="J19" s="30">
+      <c r="J19" s="19">
         <f>R17</f>
         <v>0.46426160383844894</v>
       </c>
@@ -1964,22 +1960,22 @@
         <v>97</v>
       </c>
       <c r="L19" s="1"/>
-      <c r="M19" s="34"/>
-      <c r="N19" s="36">
+      <c r="M19" s="23"/>
+      <c r="N19" s="25">
         <f>N18</f>
         <v>0.47304426716643216</v>
       </c>
-      <c r="O19" s="30" t="s">
+      <c r="O19" s="19" t="s">
         <v>62</v>
       </c>
       <c r="P19" s="2">
         <v>0.61399999999999999</v>
       </c>
-      <c r="Q19" s="30">
+      <c r="Q19" s="19">
         <f>($F$8+P19*($F$9-$F$8)) / 1440</f>
         <v>1.1208333333333334E-2</v>
       </c>
-      <c r="R19" s="30">
+      <c r="R19" s="19">
         <f>J19+Q19</f>
         <v>0.47546993717178226</v>
       </c>
@@ -1993,32 +1989,27 @@
       <c r="V19" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="W19" s="2">
-        <v>0.49399999999999999</v>
-      </c>
-      <c r="X19" s="30">
-        <f>-90*LN(1-W19) / 1440</f>
-        <v>4.257616310591697E-2</v>
-      </c>
+      <c r="W19" s="2"/>
+      <c r="X19" s="19"/>
       <c r="Y19" s="2">
         <v>0</v>
       </c>
       <c r="Z19" s="2">
         <v>1</v>
       </c>
-      <c r="AA19" s="30">
+      <c r="AA19" s="19">
         <f>AA18+Q17</f>
         <v>2.6281390906884326E-2</v>
       </c>
-      <c r="AB19" s="30">
-        <f>AB18</f>
+      <c r="AB19" s="19">
+        <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
       <c r="AC19" s="2">
         <v>0</v>
       </c>
       <c r="AD19" s="2"/>
-      <c r="AE19" s="33"/>
+      <c r="AE19" s="22"/>
       <c r="AF19" s="2" t="s">
         <v>85</v>
       </c>
@@ -2033,7 +2024,7 @@
       <c r="AO19" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AP19" s="30">
+      <c r="AP19" s="19">
         <f>J19</f>
         <v>0.46426160383844894</v>
       </c>
@@ -2068,7 +2059,7 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="J20" s="30">
+      <c r="J20" s="19">
         <f>N19</f>
         <v>0.47304426716643216</v>
       </c>
@@ -2078,23 +2069,23 @@
       <c r="L20" s="2">
         <v>0.22500000000000001</v>
       </c>
-      <c r="M20" s="30">
+      <c r="M20" s="19">
         <f>-$C$3*LN(1-L20) / 1440</f>
         <v>7.9653828008996886E-3</v>
       </c>
-      <c r="N20" s="30">
+      <c r="N20" s="19">
         <f>J20+M20</f>
         <v>0.48100964996733186</v>
       </c>
-      <c r="O20" s="30" t="s">
+      <c r="O20" s="19" t="s">
         <v>62</v>
       </c>
       <c r="P20" s="2"/>
-      <c r="Q20" s="30">
+      <c r="Q20" s="19">
         <f>Q19</f>
         <v>1.1208333333333334E-2</v>
       </c>
-      <c r="R20" s="31">
+      <c r="R20" s="20">
         <f>R19</f>
         <v>0.47546993717178226</v>
       </c>
@@ -2103,22 +2094,19 @@
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
       <c r="W20" s="1"/>
-      <c r="X20" s="37">
-        <f>X19</f>
-        <v>4.257616310591697E-2</v>
-      </c>
+      <c r="X20" s="26"/>
       <c r="Y20" s="2">
         <v>1</v>
       </c>
       <c r="Z20" s="2">
         <v>1</v>
       </c>
-      <c r="AA20" s="30">
+      <c r="AA20" s="19">
         <f>AA19+Q18</f>
         <v>3.5711946462439879E-2</v>
       </c>
-      <c r="AB20" s="30">
-        <f>AB19</f>
+      <c r="AB20" s="19">
+        <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
       <c r="AC20" s="2">
@@ -2142,7 +2130,7 @@
       <c r="AO20" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AP20" s="30">
+      <c r="AP20" s="19">
         <f>AP19</f>
         <v>0.46426160383844894</v>
       </c>
@@ -2180,7 +2168,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="J21" s="30">
+      <c r="J21" s="19">
         <f>R20</f>
         <v>0.47546993717178226</v>
       </c>
@@ -2188,22 +2176,22 @@
         <v>99</v>
       </c>
       <c r="L21" s="2"/>
-      <c r="M21" s="30"/>
-      <c r="N21" s="31">
+      <c r="M21" s="19"/>
+      <c r="N21" s="20">
         <f>N20</f>
         <v>0.48100964996733186</v>
       </c>
-      <c r="O21" s="30" t="s">
+      <c r="O21" s="19" t="s">
         <v>62</v>
       </c>
       <c r="P21" s="2">
         <v>0.26900000000000002</v>
       </c>
-      <c r="Q21" s="30">
+      <c r="Q21" s="19">
         <f>($F$8+P21*($F$9-$F$8)) / 1440</f>
         <v>8.8125000000000009E-3</v>
       </c>
-      <c r="R21" s="30">
+      <c r="R21" s="19">
         <f>Q21+J21</f>
         <v>0.48428243717178227</v>
       </c>
@@ -2218,22 +2206,19 @@
         <v>56</v>
       </c>
       <c r="W21" s="2"/>
-      <c r="X21" s="30">
-        <f>X20</f>
-        <v>4.257616310591697E-2</v>
-      </c>
+      <c r="X21" s="19"/>
       <c r="Y21" s="2">
         <v>0</v>
       </c>
       <c r="Z21" s="2">
         <v>2</v>
       </c>
-      <c r="AA21" s="30">
+      <c r="AA21" s="19">
         <f>AA20+(J21-J20)</f>
         <v>3.813761646778998E-2</v>
       </c>
-      <c r="AB21" s="30">
-        <f>AB20</f>
+      <c r="AB21" s="19">
+        <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
       <c r="AC21" s="2">
@@ -2241,7 +2226,7 @@
       </c>
       <c r="AD21" s="2"/>
       <c r="AE21" s="2"/>
-      <c r="AF21" s="33"/>
+      <c r="AF21" s="22"/>
       <c r="AG21" s="2" t="s">
         <v>88</v>
       </c>
@@ -2255,8 +2240,8 @@
       <c r="AO21" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AP21" s="30">
-        <f t="shared" ref="AP21:AP22" si="1">AP20</f>
+      <c r="AP21" s="19">
+        <f t="shared" ref="AP21:AP22" si="2">AP20</f>
         <v>0.46426160383844894</v>
       </c>
       <c r="AQ21" s="2"/>
@@ -2264,7 +2249,7 @@
       <c r="AS21" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AT21" s="30">
+      <c r="AT21" s="19">
         <f>J21</f>
         <v>0.47546993717178226</v>
       </c>
@@ -2295,7 +2280,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="J22" s="30">
+      <c r="J22" s="19">
         <f>N21</f>
         <v>0.48100964996733186</v>
       </c>
@@ -2305,23 +2290,23 @@
       <c r="L22" s="2">
         <v>0.57099999999999995</v>
       </c>
-      <c r="M22" s="30">
+      <c r="M22" s="19">
         <f>-$C$3*LN(1-L22) / 1440</f>
         <v>2.6446823751691249E-2</v>
       </c>
-      <c r="N22" s="30">
+      <c r="N22" s="19">
         <f>J22+M22</f>
         <v>0.50745647371902314</v>
       </c>
-      <c r="O22" s="30" t="s">
+      <c r="O22" s="19" t="s">
         <v>62</v>
       </c>
       <c r="P22" s="2"/>
-      <c r="Q22" s="30">
+      <c r="Q22" s="19">
         <f>Q21</f>
         <v>8.8125000000000009E-3</v>
       </c>
-      <c r="R22" s="30">
+      <c r="R22" s="19">
         <f>R21</f>
         <v>0.48428243717178227</v>
       </c>
@@ -2330,22 +2315,19 @@
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
       <c r="W22" s="2"/>
-      <c r="X22" s="30">
-        <f>X21</f>
-        <v>4.257616310591697E-2</v>
-      </c>
+      <c r="X22" s="19"/>
       <c r="Y22" s="2">
         <v>1</v>
       </c>
       <c r="Z22" s="2">
         <v>2</v>
       </c>
-      <c r="AA22" s="30">
+      <c r="AA22" s="19">
         <f>AA21++J22-J21</f>
         <v>4.3677329263339615E-2</v>
       </c>
-      <c r="AB22" s="30">
-        <f>AB21</f>
+      <c r="AB22" s="19">
+        <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
       <c r="AC22" s="2">
@@ -2369,8 +2351,8 @@
       <c r="AO22" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AP22" s="30">
-        <f t="shared" si="1"/>
+      <c r="AP22" s="19">
+        <f t="shared" si="2"/>
         <v>0.46426160383844894</v>
       </c>
       <c r="AQ22" s="2"/>
@@ -2378,7 +2360,7 @@
       <c r="AS22" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AT22" s="30">
+      <c r="AT22" s="19">
         <f>AT21</f>
         <v>0.47546993717178226</v>
       </c>
@@ -2398,21 +2380,21 @@
       </c>
     </row>
     <row r="24" spans="2:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="34"/>
+      <c r="F24" s="34"/>
       <c r="J24" s="3"/>
     </row>
     <row r="25" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
+      <c r="B25" s="34"/>
+      <c r="C25" s="34"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="34"/>
       <c r="J25" s="3"/>
     </row>
     <row r="26" spans="2:52" x14ac:dyDescent="0.25">
@@ -2422,25 +2404,7 @@
       <c r="J27" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
-    <mergeCell ref="AO11:AR11"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="AD10:AI10"/>
-    <mergeCell ref="O11:V11"/>
-    <mergeCell ref="AA11:AC11"/>
-    <mergeCell ref="Y11:Z11"/>
-    <mergeCell ref="AK11:AN11"/>
-    <mergeCell ref="B24:F25"/>
-    <mergeCell ref="G8:H9"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B19:F19"/>
+  <mergeCells count="33">
     <mergeCell ref="E2:H2"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="E5:F5"/>
@@ -2454,9 +2418,26 @@
     <mergeCell ref="Q3:R3"/>
     <mergeCell ref="Q4:R4"/>
     <mergeCell ref="S4:T4"/>
+    <mergeCell ref="Q2:T2"/>
     <mergeCell ref="S3:T3"/>
-    <mergeCell ref="Q2:T2"/>
-    <mergeCell ref="Q5:R5"/>
+    <mergeCell ref="B24:F25"/>
+    <mergeCell ref="G8:H9"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="AO11:AR11"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="AD10:AI10"/>
+    <mergeCell ref="O11:V11"/>
+    <mergeCell ref="AA11:AC11"/>
+    <mergeCell ref="Y11:Z11"/>
+    <mergeCell ref="AK11:AN11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Añadí filas y comencé el camino de la tienda cerrada
</commit_message>
<xml_diff>
--- a/1er Entrega/Plantilla.xlsx
+++ b/1er Entrega/Plantilla.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\UTN\Simulación\TP 4\Tp4-Simulacion-G5\1er Entrega\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{146DAC6F-4680-4A94-A8CA-610AED6A1729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F7D5A6-70D8-467E-97E8-13468611C6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="111">
   <si>
     <t>Horario Apertura</t>
   </si>
@@ -342,6 +342,33 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Fin_Atención_CL4</t>
+  </si>
+  <si>
+    <t>Elevado</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>Fin_Atencion_CL5</t>
+  </si>
+  <si>
+    <t>Fin_Reparacion_CL2</t>
+  </si>
+  <si>
+    <t>Llegada_Cliente 6</t>
+  </si>
+  <si>
+    <t>Fin_Atencion_CL6</t>
+  </si>
+  <si>
+    <t>Fin_Reparacion_CL3</t>
+  </si>
+  <si>
+    <t>Llega_Cliente_7</t>
   </si>
 </sst>
 </file>
@@ -352,7 +379,7 @@
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -371,6 +398,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -489,13 +522,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -553,28 +585,10 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -594,6 +608,28 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -874,14 +910,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:AZ27"/>
+  <dimension ref="B2:BD52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
     <col min="3" max="3" width="8.5703125" customWidth="1"/>
     <col min="4" max="4" width="13.5703125" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="11" max="11" width="18.140625" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" customWidth="1"/>
     <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="17.5703125" customWidth="1"/>
     <col min="19" max="20" width="12.42578125" customWidth="1"/>
@@ -894,47 +930,47 @@
     <col min="29" max="29" width="10.28515625" customWidth="1"/>
     <col min="32" max="32" width="15.28515625" customWidth="1"/>
     <col min="33" max="33" width="16.28515625" customWidth="1"/>
-    <col min="34" max="34" width="12" customWidth="1"/>
-    <col min="36" max="36" width="1.140625" customWidth="1"/>
-    <col min="37" max="39" width="15.5703125" customWidth="1"/>
-    <col min="40" max="40" width="11.7109375" customWidth="1"/>
-    <col min="43" max="43" width="12.42578125" customWidth="1"/>
-    <col min="44" max="44" width="12.28515625" customWidth="1"/>
-    <col min="47" max="47" width="12.28515625" customWidth="1"/>
-    <col min="48" max="48" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="11.7109375" customWidth="1"/>
-    <col min="52" max="52" width="12" customWidth="1"/>
+    <col min="34" max="38" width="12" customWidth="1"/>
+    <col min="40" max="40" width="1.140625" customWidth="1"/>
+    <col min="41" max="43" width="15.5703125" customWidth="1"/>
+    <col min="44" max="44" width="11.7109375" customWidth="1"/>
+    <col min="47" max="47" width="12.42578125" customWidth="1"/>
+    <col min="48" max="48" width="12.28515625" customWidth="1"/>
+    <col min="51" max="51" width="12.28515625" customWidth="1"/>
+    <col min="52" max="52" width="11.42578125" customWidth="1"/>
+    <col min="55" max="55" width="11.7109375" customWidth="1"/>
+    <col min="56" max="56" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:56" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2"/>
-      <c r="E2" s="35" t="s">
+      <c r="E2" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
       <c r="J2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="38" t="s">
+      <c r="K2" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="L2" s="38"/>
-      <c r="M2" s="38"/>
-      <c r="N2" s="38"/>
-      <c r="O2" s="38"/>
-      <c r="Q2" s="41" t="s">
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
+      <c r="Q2" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="R2" s="41"/>
-      <c r="S2" s="41"/>
-      <c r="T2" s="41"/>
-    </row>
-    <row r="3" spans="2:52" x14ac:dyDescent="0.25">
+      <c r="R2" s="34"/>
+      <c r="S2" s="34"/>
+      <c r="T2" s="34"/>
+    </row>
+    <row r="3" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -956,7 +992,7 @@
       </c>
       <c r="T3" s="28"/>
     </row>
-    <row r="4" spans="2:52" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B4" s="28" t="s">
         <v>27</v>
       </c>
@@ -972,15 +1008,15 @@
         <v>2</v>
       </c>
       <c r="J4" s="2"/>
-      <c r="K4" s="4" t="s">
+      <c r="K4" s="3" t="s">
         <v>35</v>
       </c>
       <c r="L4" s="2"/>
-      <c r="M4" s="4" t="s">
+      <c r="M4" s="3" t="s">
         <v>36</v>
       </c>
       <c r="N4" s="2"/>
-      <c r="O4" s="4" t="s">
+      <c r="O4" s="3" t="s">
         <v>68</v>
       </c>
       <c r="Q4" s="28" t="s">
@@ -992,7 +1028,7 @@
       </c>
       <c r="T4" s="28"/>
     </row>
-    <row r="5" spans="2:52" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:56" x14ac:dyDescent="0.25">
       <c r="E5" s="28" t="s">
         <v>1</v>
       </c>
@@ -1003,7 +1039,7 @@
       <c r="H5" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="J5" s="4" t="s">
         <v>59</v>
       </c>
       <c r="K5" s="2" t="s">
@@ -1018,23 +1054,23 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="2:52" ht="60" x14ac:dyDescent="0.25">
-      <c r="J6" s="6" t="s">
+    <row r="6" spans="2:56" ht="60" x14ac:dyDescent="0.25">
+      <c r="J6" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="K6" s="6" t="s">
+      <c r="K6" s="5" t="s">
         <v>86</v>
       </c>
       <c r="L6" s="2"/>
-      <c r="M6" s="6" t="s">
+      <c r="M6" s="5" t="s">
         <v>67</v>
       </c>
       <c r="N6" s="2"/>
-      <c r="O6" s="6" t="s">
+      <c r="O6" s="5" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="2:52" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1052,15 +1088,8 @@
         <v>31</v>
       </c>
       <c r="H7" s="28"/>
-      <c r="S7" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="T7" s="27">
-        <f ca="1">RAND()</f>
-        <v>0.98911930971154549</v>
-      </c>
-    </row>
-    <row r="8" spans="2:52" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B8" s="28" t="s">
         <v>6</v>
       </c>
@@ -1076,12 +1105,12 @@
       <c r="F8" s="2">
         <v>10</v>
       </c>
-      <c r="G8" s="29" t="s">
+      <c r="G8" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="H8" s="29"/>
-    </row>
-    <row r="9" spans="2:52" x14ac:dyDescent="0.25">
+      <c r="H8" s="36"/>
+    </row>
+    <row r="9" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B9" s="28"/>
       <c r="C9" s="28"/>
       <c r="D9" s="28"/>
@@ -1091,55 +1120,59 @@
       <c r="F9" s="2">
         <v>20</v>
       </c>
-      <c r="G9" s="29"/>
-      <c r="H9" s="29"/>
-      <c r="J9" s="37" t="s">
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="J9" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="37"/>
-      <c r="L9" s="37"/>
-      <c r="M9" s="37"/>
-      <c r="N9" s="37"/>
-      <c r="O9" s="37"/>
-      <c r="P9" s="37"/>
-      <c r="Q9" s="37"/>
-      <c r="R9" s="37"/>
-      <c r="S9" s="37"/>
-      <c r="T9" s="37"/>
-      <c r="U9" s="37"/>
-      <c r="V9" s="37"/>
-      <c r="W9" s="37"/>
-      <c r="X9" s="37"/>
-      <c r="Y9" s="37"/>
-      <c r="Z9" s="37"/>
-      <c r="AA9" s="37"/>
-      <c r="AB9" s="37"/>
-      <c r="AC9" s="37"/>
-      <c r="AD9" s="37"/>
-      <c r="AE9" s="37"/>
-      <c r="AF9" s="37"/>
-      <c r="AG9" s="37"/>
-      <c r="AH9" s="37"/>
-      <c r="AI9" s="37"/>
-      <c r="AJ9" s="37"/>
-      <c r="AK9" s="37"/>
-      <c r="AL9" s="37"/>
-      <c r="AM9" s="37"/>
-      <c r="AN9" s="37"/>
-      <c r="AO9" s="37"/>
-      <c r="AP9" s="37"/>
-      <c r="AQ9" s="37"/>
-      <c r="AR9" s="37"/>
-      <c r="AS9" s="37"/>
-      <c r="AT9" s="37"/>
-      <c r="AU9" s="37"/>
-      <c r="AV9" s="37"/>
-      <c r="AW9" s="37"/>
-      <c r="AX9" s="37"/>
-      <c r="AY9" s="37"/>
-      <c r="AZ9" s="37"/>
-    </row>
-    <row r="10" spans="2:52" x14ac:dyDescent="0.25">
+      <c r="K9" s="30"/>
+      <c r="L9" s="30"/>
+      <c r="M9" s="30"/>
+      <c r="N9" s="30"/>
+      <c r="O9" s="30"/>
+      <c r="P9" s="30"/>
+      <c r="Q9" s="30"/>
+      <c r="R9" s="30"/>
+      <c r="S9" s="30"/>
+      <c r="T9" s="30"/>
+      <c r="U9" s="30"/>
+      <c r="V9" s="30"/>
+      <c r="W9" s="30"/>
+      <c r="X9" s="30"/>
+      <c r="Y9" s="30"/>
+      <c r="Z9" s="30"/>
+      <c r="AA9" s="30"/>
+      <c r="AB9" s="30"/>
+      <c r="AC9" s="30"/>
+      <c r="AD9" s="30"/>
+      <c r="AE9" s="30"/>
+      <c r="AF9" s="30"/>
+      <c r="AG9" s="30"/>
+      <c r="AH9" s="30"/>
+      <c r="AI9" s="30"/>
+      <c r="AJ9" s="30"/>
+      <c r="AK9" s="30"/>
+      <c r="AL9" s="30"/>
+      <c r="AM9" s="30"/>
+      <c r="AN9" s="30"/>
+      <c r="AO9" s="30"/>
+      <c r="AP9" s="30"/>
+      <c r="AQ9" s="30"/>
+      <c r="AR9" s="30"/>
+      <c r="AS9" s="30"/>
+      <c r="AT9" s="30"/>
+      <c r="AU9" s="30"/>
+      <c r="AV9" s="30"/>
+      <c r="AW9" s="30"/>
+      <c r="AX9" s="30"/>
+      <c r="AY9" s="30"/>
+      <c r="AZ9" s="30"/>
+      <c r="BA9" s="30"/>
+      <c r="BB9" s="30"/>
+      <c r="BC9" s="30"/>
+      <c r="BD9" s="30"/>
+    </row>
+    <row r="10" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>7</v>
       </c>
@@ -1159,68 +1192,72 @@
         <v>29</v>
       </c>
       <c r="H10" s="28"/>
-      <c r="AD10" s="30" t="s">
+      <c r="AD10" s="37" t="s">
         <v>63</v>
       </c>
-      <c r="AE10" s="30"/>
-      <c r="AF10" s="30"/>
-      <c r="AG10" s="30"/>
-      <c r="AH10" s="30"/>
-      <c r="AI10" s="30"/>
-      <c r="AJ10" s="2"/>
-      <c r="AK10" s="36" t="s">
+      <c r="AE10" s="37"/>
+      <c r="AF10" s="37"/>
+      <c r="AG10" s="37"/>
+      <c r="AH10" s="37"/>
+      <c r="AI10" s="37"/>
+      <c r="AJ10" s="37"/>
+      <c r="AK10" s="37"/>
+      <c r="AL10" s="37"/>
+      <c r="AM10" s="37"/>
+      <c r="AN10" s="2"/>
+      <c r="AO10" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="AL10" s="36"/>
-      <c r="AM10" s="36"/>
-      <c r="AN10" s="36"/>
-      <c r="AO10" s="36"/>
-      <c r="AP10" s="36"/>
-      <c r="AQ10" s="36"/>
-      <c r="AR10" s="36"/>
-      <c r="AS10" s="36"/>
-      <c r="AT10" s="36"/>
-      <c r="AU10" s="36"/>
-      <c r="AV10" s="36"/>
-      <c r="AW10" s="36"/>
-      <c r="AX10" s="36"/>
-      <c r="AY10" s="36"/>
-      <c r="AZ10" s="36"/>
-    </row>
-    <row r="11" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="I11" s="29" t="s">
+      <c r="AP10" s="29"/>
+      <c r="AQ10" s="29"/>
+      <c r="AR10" s="29"/>
+      <c r="AS10" s="29"/>
+      <c r="AT10" s="29"/>
+      <c r="AU10" s="29"/>
+      <c r="AV10" s="29"/>
+      <c r="AW10" s="29"/>
+      <c r="AX10" s="29"/>
+      <c r="AY10" s="29"/>
+      <c r="AZ10" s="29"/>
+      <c r="BA10" s="29"/>
+      <c r="BB10" s="29"/>
+      <c r="BC10" s="29"/>
+      <c r="BD10" s="29"/>
+    </row>
+    <row r="11" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="I11" s="36" t="s">
         <v>84</v>
       </c>
-      <c r="J11" s="9"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="39" t="s">
+      <c r="J11" s="8"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="M11" s="39"/>
-      <c r="N11" s="39"/>
-      <c r="O11" s="31" t="s">
+      <c r="M11" s="32"/>
+      <c r="N11" s="32"/>
+      <c r="O11" s="38" t="s">
         <v>77</v>
       </c>
-      <c r="P11" s="31"/>
-      <c r="Q11" s="31"/>
-      <c r="R11" s="31"/>
-      <c r="S11" s="31"/>
-      <c r="T11" s="31"/>
-      <c r="U11" s="31"/>
-      <c r="V11" s="31"/>
-      <c r="W11" s="40" t="s">
+      <c r="P11" s="38"/>
+      <c r="Q11" s="38"/>
+      <c r="R11" s="38"/>
+      <c r="S11" s="38"/>
+      <c r="T11" s="38"/>
+      <c r="U11" s="38"/>
+      <c r="V11" s="38"/>
+      <c r="W11" s="33" t="s">
         <v>78</v>
       </c>
-      <c r="X11" s="40"/>
-      <c r="Y11" s="33" t="s">
+      <c r="X11" s="33"/>
+      <c r="Y11" s="40" t="s">
         <v>69</v>
       </c>
-      <c r="Z11" s="33"/>
-      <c r="AA11" s="32" t="s">
+      <c r="Z11" s="40"/>
+      <c r="AA11" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="AB11" s="32"/>
-      <c r="AC11" s="32"/>
+      <c r="AB11" s="39"/>
+      <c r="AC11" s="39"/>
       <c r="AD11" s="2">
         <v>1</v>
       </c>
@@ -1236,170 +1273,186 @@
       <c r="AH11" s="1">
         <v>5</v>
       </c>
-      <c r="AI11" s="1" t="s">
+      <c r="AI11" s="1">
+        <v>6</v>
+      </c>
+      <c r="AJ11" s="1">
+        <v>7</v>
+      </c>
+      <c r="AK11" s="1">
+        <v>8</v>
+      </c>
+      <c r="AL11" s="1">
+        <v>9</v>
+      </c>
+      <c r="AM11" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="AJ11" s="2"/>
-      <c r="AK11" s="28">
+      <c r="AN11" s="2"/>
+      <c r="AO11" s="28">
         <v>1</v>
-      </c>
-      <c r="AL11" s="28"/>
-      <c r="AM11" s="28"/>
-      <c r="AN11" s="28"/>
-      <c r="AO11" s="28">
-        <v>2</v>
       </c>
       <c r="AP11" s="28"/>
       <c r="AQ11" s="28"/>
       <c r="AR11" s="28"/>
       <c r="AS11" s="28">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AT11" s="28"/>
       <c r="AU11" s="28"/>
       <c r="AV11" s="28"/>
-      <c r="AW11" s="28" t="s">
-        <v>79</v>
+      <c r="AW11" s="28">
+        <v>3</v>
       </c>
       <c r="AX11" s="28"/>
       <c r="AY11" s="28"/>
       <c r="AZ11" s="28"/>
-    </row>
-    <row r="12" spans="2:52" ht="60" x14ac:dyDescent="0.25">
-      <c r="I12" s="29"/>
-      <c r="J12" s="11" t="s">
+      <c r="BA11" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="BB11" s="28"/>
+      <c r="BC11" s="28"/>
+      <c r="BD11" s="28"/>
+    </row>
+    <row r="12" spans="2:56" ht="60" x14ac:dyDescent="0.25">
+      <c r="I12" s="36"/>
+      <c r="J12" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="K12" s="12" t="s">
+      <c r="K12" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="L12" s="13" t="s">
+      <c r="L12" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="M12" s="13" t="s">
+      <c r="M12" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="N12" s="14" t="s">
+      <c r="N12" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="O12" s="15" t="s">
+      <c r="O12" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="P12" s="15" t="s">
+      <c r="P12" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="Q12" s="15" t="s">
+      <c r="Q12" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="R12" s="14" t="s">
+      <c r="R12" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="S12" s="15" t="s">
+      <c r="S12" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="T12" s="15" t="s">
+      <c r="T12" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="U12" s="15" t="s">
+      <c r="U12" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="V12" s="15" t="s">
+      <c r="V12" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="W12" s="16" t="s">
+      <c r="W12" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="X12" s="16" t="s">
+      <c r="X12" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="Y12" s="17" t="s">
+      <c r="Y12" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="Z12" s="17" t="s">
+      <c r="Z12" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="AA12" s="18" t="s">
+      <c r="AA12" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="AB12" s="18" t="s">
+      <c r="AB12" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="AC12" s="18" t="s">
+      <c r="AC12" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="AD12" s="8" t="s">
+      <c r="AD12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="AE12" s="8" t="s">
+      <c r="AE12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="AF12" s="8" t="s">
+      <c r="AF12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="AG12" s="8" t="s">
+      <c r="AG12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="AH12" s="8" t="s">
+      <c r="AH12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="AI12" s="8" t="s">
+      <c r="AI12" s="7"/>
+      <c r="AJ12" s="7"/>
+      <c r="AK12" s="7"/>
+      <c r="AL12" s="7"/>
+      <c r="AM12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="AJ12" s="1"/>
-      <c r="AK12" s="8" t="s">
+      <c r="AN12" s="1"/>
+      <c r="AO12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="AL12" s="7" t="s">
+      <c r="AP12" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="AM12" s="7" t="s">
+      <c r="AQ12" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="AN12" s="7" t="s">
+      <c r="AR12" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="AO12" s="8" t="s">
+      <c r="AS12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="AP12" s="7" t="s">
+      <c r="AT12" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="AQ12" s="7" t="s">
+      <c r="AU12" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="AR12" s="7" t="s">
+      <c r="AV12" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="AS12" s="8" t="s">
+      <c r="AW12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="AT12" s="7" t="s">
+      <c r="AX12" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="AU12" s="7" t="s">
+      <c r="AY12" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="AV12" s="7" t="s">
+      <c r="AZ12" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="AW12" s="8" t="s">
+      <c r="BA12" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="AX12" s="7" t="s">
+      <c r="BB12" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="AY12" s="7" t="s">
+      <c r="BC12" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="AZ12" s="7" t="s">
+      <c r="BD12" s="6" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="2:52" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:56" x14ac:dyDescent="0.25">
       <c r="I13" s="2">
         <v>1</v>
       </c>
-      <c r="J13" s="19">
+      <c r="J13" s="18">
         <v>0.41666666666666669</v>
       </c>
       <c r="K13" s="2" t="s">
@@ -1408,11 +1461,11 @@
       <c r="L13" s="2">
         <v>0.33300000000000002</v>
       </c>
-      <c r="M13" s="19">
+      <c r="M13" s="18">
         <f>-$C$3*(LN(1-L13)) / 1440</f>
         <v>1.265516353332854E-2</v>
       </c>
-      <c r="N13" s="20">
+      <c r="N13" s="19">
         <f>J13+M13</f>
         <v>0.4293218301999952</v>
       </c>
@@ -1420,24 +1473,24 @@
         <v>54</v>
       </c>
       <c r="P13" s="2"/>
-      <c r="Q13" s="19"/>
+      <c r="Q13" s="18"/>
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
-      <c r="X13" s="19"/>
+      <c r="X13" s="18"/>
       <c r="Y13" s="2">
         <v>0</v>
       </c>
       <c r="Z13" s="2">
         <v>0</v>
       </c>
-      <c r="AA13" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="19">
+      <c r="AA13" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="18">
         <v>0</v>
       </c>
       <c r="AC13" s="2">
@@ -1466,8 +1519,12 @@
       <c r="AX13" s="2"/>
       <c r="AY13" s="2"/>
       <c r="AZ13" s="2"/>
-    </row>
-    <row r="14" spans="2:52" x14ac:dyDescent="0.25">
+      <c r="BA13" s="2"/>
+      <c r="BB13" s="2"/>
+      <c r="BC13" s="2"/>
+      <c r="BD13" s="2"/>
+    </row>
+    <row r="14" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B14" s="28" t="s">
         <v>17</v>
       </c>
@@ -1479,7 +1536,7 @@
         <f>I13+1</f>
         <v>2</v>
       </c>
-      <c r="J14" s="19">
+      <c r="J14" s="18">
         <v>0.42931712962962965</v>
       </c>
       <c r="K14" s="2" t="s">
@@ -1488,11 +1545,11 @@
       <c r="L14" s="2">
         <v>0.55800000000000005</v>
       </c>
-      <c r="M14" s="19">
+      <c r="M14" s="18">
         <f>-$C$3*(LN(1-L14)) / 1440</f>
         <v>2.5513918653263721E-2</v>
       </c>
-      <c r="N14" s="19">
+      <c r="N14" s="18">
         <f>J14+M14</f>
         <v>0.45483104828289339</v>
       </c>
@@ -1502,11 +1559,11 @@
       <c r="P14" s="2">
         <v>5.5E-2</v>
       </c>
-      <c r="Q14" s="19">
+      <c r="Q14" s="18">
         <f>($F$8+P14*($F$9-$F$8)) / 1440</f>
         <v>7.3263888888888892E-3</v>
       </c>
-      <c r="R14" s="20">
+      <c r="R14" s="19">
         <f>J14+Q14</f>
         <v>0.43664351851851851</v>
       </c>
@@ -1522,10 +1579,10 @@
       <c r="Z14" s="2">
         <v>0</v>
       </c>
-      <c r="AA14" s="19">
-        <v>0</v>
-      </c>
-      <c r="AB14" s="19">
+      <c r="AA14" s="18">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="18">
         <v>0</v>
       </c>
       <c r="AC14" s="2">
@@ -1556,8 +1613,12 @@
       <c r="AX14" s="2"/>
       <c r="AY14" s="2"/>
       <c r="AZ14" s="2"/>
-    </row>
-    <row r="15" spans="2:52" x14ac:dyDescent="0.25">
+      <c r="BA14" s="2"/>
+      <c r="BB14" s="2"/>
+      <c r="BC14" s="2"/>
+      <c r="BD14" s="2"/>
+    </row>
+    <row r="15" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
         <v>24</v>
       </c>
@@ -1574,28 +1635,28 @@
         <v>23</v>
       </c>
       <c r="I15" s="2">
-        <f t="shared" ref="I15:I22" si="0">I14+1</f>
+        <f t="shared" ref="I15:I52" si="0">I14+1</f>
         <v>3</v>
       </c>
-      <c r="J15" s="19">
+      <c r="J15" s="18">
         <f>R14</f>
         <v>0.43664351851851851</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="L15" s="8"/>
-      <c r="M15" s="21"/>
-      <c r="N15" s="19">
+      <c r="L15" s="7"/>
+      <c r="M15" s="20"/>
+      <c r="N15" s="18">
         <f>N14</f>
         <v>0.45483104828289339</v>
       </c>
-      <c r="O15" s="19" t="s">
+      <c r="O15" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="P15" s="21"/>
-      <c r="Q15" s="21"/>
-      <c r="R15" s="21"/>
+      <c r="P15" s="20"/>
+      <c r="Q15" s="20"/>
+      <c r="R15" s="20"/>
       <c r="S15" s="2">
         <v>0.35499999999999998</v>
       </c>
@@ -1609,7 +1670,7 @@
       <c r="W15" s="2">
         <v>0.187</v>
       </c>
-      <c r="X15" s="20">
+      <c r="X15" s="19">
         <f>-90*LN(1-W15) / 1440</f>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -1619,34 +1680,34 @@
       <c r="Z15" s="2">
         <v>0</v>
       </c>
-      <c r="AA15" s="19">
+      <c r="AA15" s="18">
         <f>Q14</f>
         <v>7.3263888888888892E-3</v>
       </c>
-      <c r="AB15" s="19">
+      <c r="AB15" s="18">
         <v>0</v>
       </c>
       <c r="AC15" s="2">
         <v>0</v>
       </c>
-      <c r="AD15" s="22"/>
+      <c r="AD15" s="21"/>
       <c r="AE15" s="2"/>
       <c r="AF15" s="2"/>
       <c r="AG15" s="2"/>
       <c r="AH15" s="2"/>
       <c r="AI15" s="2"/>
       <c r="AJ15" s="2"/>
-      <c r="AK15" s="2" t="s">
+      <c r="AK15" s="2"/>
+      <c r="AL15" s="2"/>
+      <c r="AM15" s="2"/>
+      <c r="AN15" s="2"/>
+      <c r="AO15" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="AL15" s="19">
+      <c r="AP15" s="18">
         <f>J15</f>
         <v>0.43664351851851851</v>
       </c>
-      <c r="AM15" s="2"/>
-      <c r="AN15" s="2"/>
-      <c r="AO15" s="2"/>
-      <c r="AP15" s="2"/>
       <c r="AQ15" s="2"/>
       <c r="AR15" s="2"/>
       <c r="AS15" s="2"/>
@@ -1657,8 +1718,12 @@
       <c r="AX15" s="2"/>
       <c r="AY15" s="2"/>
       <c r="AZ15" s="2"/>
-    </row>
-    <row r="16" spans="2:52" x14ac:dyDescent="0.25">
+      <c r="BA15" s="2"/>
+      <c r="BB15" s="2"/>
+      <c r="BC15" s="2"/>
+      <c r="BD15" s="2"/>
+    </row>
+    <row r="16" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
         <v>19</v>
       </c>
@@ -1678,7 +1743,7 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="J16" s="19">
+      <c r="J16" s="18">
         <f>J15+X15</f>
         <v>0.44958252910816393</v>
       </c>
@@ -1686,34 +1751,34 @@
         <v>94</v>
       </c>
       <c r="L16" s="1"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="20">
+      <c r="M16" s="22"/>
+      <c r="N16" s="19">
         <f>N15</f>
         <v>0.45483104828289339</v>
       </c>
-      <c r="O16" s="19" t="s">
+      <c r="O16" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="P16" s="23"/>
-      <c r="Q16" s="23"/>
-      <c r="R16" s="23"/>
-      <c r="S16" s="23"/>
-      <c r="T16" s="23"/>
-      <c r="U16" s="23"/>
-      <c r="V16" s="23"/>
-      <c r="W16" s="23"/>
-      <c r="X16" s="19"/>
+      <c r="P16" s="22"/>
+      <c r="Q16" s="22"/>
+      <c r="R16" s="22"/>
+      <c r="S16" s="22"/>
+      <c r="T16" s="22"/>
+      <c r="U16" s="22"/>
+      <c r="V16" s="22"/>
+      <c r="W16" s="22"/>
+      <c r="X16" s="18"/>
       <c r="Y16" s="2">
         <v>0</v>
       </c>
       <c r="Z16" s="2">
         <v>0</v>
       </c>
-      <c r="AA16" s="19">
+      <c r="AA16" s="18">
         <f>AA15</f>
         <v>7.3263888888888892E-3</v>
       </c>
-      <c r="AB16" s="19">
+      <c r="AB16" s="18">
         <f>AB15+X15</f>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -1727,23 +1792,23 @@
       <c r="AH16" s="2"/>
       <c r="AI16" s="2"/>
       <c r="AJ16" s="2"/>
-      <c r="AK16" s="24"/>
-      <c r="AL16" s="19">
-        <f>AL15</f>
+      <c r="AK16" s="2"/>
+      <c r="AL16" s="2"/>
+      <c r="AM16" s="2"/>
+      <c r="AN16" s="2"/>
+      <c r="AO16" s="23"/>
+      <c r="AP16" s="18">
+        <f>AP15</f>
         <v>0.43664351851851851</v>
       </c>
-      <c r="AM16" s="19">
+      <c r="AQ16" s="18">
         <f>J16</f>
         <v>0.44958252910816393</v>
       </c>
-      <c r="AN16" s="19">
-        <f>AM16-AL16</f>
+      <c r="AR16" s="18">
+        <f>AQ16-AP16</f>
         <v>1.2939010589645417E-2</v>
       </c>
-      <c r="AO16" s="2"/>
-      <c r="AP16" s="2"/>
-      <c r="AQ16" s="2"/>
-      <c r="AR16" s="2"/>
       <c r="AS16" s="2"/>
       <c r="AT16" s="2"/>
       <c r="AU16" s="2"/>
@@ -1752,8 +1817,12 @@
       <c r="AX16" s="2"/>
       <c r="AY16" s="2"/>
       <c r="AZ16" s="2"/>
-    </row>
-    <row r="17" spans="2:52" x14ac:dyDescent="0.25">
+      <c r="BA16" s="2"/>
+      <c r="BB16" s="2"/>
+      <c r="BC16" s="2"/>
+      <c r="BD16" s="2"/>
+    </row>
+    <row r="17" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
         <v>20</v>
       </c>
@@ -1773,7 +1842,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="J17" s="19">
+      <c r="J17" s="18">
         <f>N15</f>
         <v>0.45483104828289339</v>
       </c>
@@ -1783,11 +1852,11 @@
       <c r="L17" s="2">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="M17" s="19">
+      <c r="M17" s="18">
         <f>-$C$3*LN(1-L17) / 1440</f>
         <v>9.3890906884335122E-5</v>
       </c>
-      <c r="N17" s="20">
+      <c r="N17" s="19">
         <f>J17+M17</f>
         <v>0.45492493918977772</v>
       </c>
@@ -1797,11 +1866,11 @@
       <c r="P17" s="2">
         <v>0.35799999999999998</v>
       </c>
-      <c r="Q17" s="19">
+      <c r="Q17" s="18">
         <f>($F$8+P17*($F$9-$F$8)) / 1440</f>
         <v>9.4305555555555549E-3</v>
       </c>
-      <c r="R17" s="19">
+      <c r="R17" s="18">
         <f>J17+Q17</f>
         <v>0.46426160383844894</v>
       </c>
@@ -1817,11 +1886,11 @@
       <c r="Z17" s="2">
         <v>0</v>
       </c>
-      <c r="AA17" s="19">
+      <c r="AA17" s="18">
         <f>AA16+Q18</f>
         <v>1.6756944444444442E-2</v>
       </c>
-      <c r="AB17" s="19">
+      <c r="AB17" s="18">
         <f t="shared" ref="AB17:AB22" si="1">AB16</f>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -1838,13 +1907,13 @@
       <c r="AI17" s="2"/>
       <c r="AJ17" s="2"/>
       <c r="AK17" s="2"/>
-      <c r="AL17" s="24"/>
-      <c r="AM17" s="24"/>
-      <c r="AN17" s="24"/>
+      <c r="AL17" s="2"/>
+      <c r="AM17" s="2"/>
+      <c r="AN17" s="2"/>
       <c r="AO17" s="2"/>
-      <c r="AP17" s="2"/>
-      <c r="AQ17" s="2"/>
-      <c r="AR17" s="2"/>
+      <c r="AP17" s="23"/>
+      <c r="AQ17" s="23"/>
+      <c r="AR17" s="23"/>
       <c r="AS17" s="2"/>
       <c r="AT17" s="2"/>
       <c r="AU17" s="2"/>
@@ -1853,13 +1922,17 @@
       <c r="AX17" s="2"/>
       <c r="AY17" s="2"/>
       <c r="AZ17" s="2"/>
-    </row>
-    <row r="18" spans="2:52" x14ac:dyDescent="0.25">
+      <c r="BA17" s="2"/>
+      <c r="BB17" s="2"/>
+      <c r="BC17" s="2"/>
+      <c r="BD17" s="2"/>
+    </row>
+    <row r="18" spans="2:56" x14ac:dyDescent="0.25">
       <c r="I18" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="J18" s="19">
+      <c r="J18" s="18">
         <f>N17</f>
         <v>0.45492493918977772</v>
       </c>
@@ -1869,11 +1942,11 @@
       <c r="L18" s="2">
         <v>0.44</v>
       </c>
-      <c r="M18" s="19">
+      <c r="M18" s="18">
         <f>-$C$3*LN(1-L18) / 1440</f>
         <v>1.8119327976654439E-2</v>
       </c>
-      <c r="N18" s="19">
+      <c r="N18" s="18">
         <f>J18+M18</f>
         <v>0.47304426716643216</v>
       </c>
@@ -1881,11 +1954,11 @@
         <v>62</v>
       </c>
       <c r="P18" s="1"/>
-      <c r="Q18" s="19">
+      <c r="Q18" s="18">
         <f>Q17</f>
         <v>9.4305555555555549E-3</v>
       </c>
-      <c r="R18" s="20">
+      <c r="R18" s="19">
         <f>R17</f>
         <v>0.46426160383844894</v>
       </c>
@@ -1901,11 +1974,11 @@
       <c r="Z18" s="2">
         <v>0</v>
       </c>
-      <c r="AA18" s="19">
+      <c r="AA18" s="18">
         <f>AA17+(J18-J17)</f>
         <v>1.6850835351328773E-2</v>
       </c>
-      <c r="AB18" s="19">
+      <c r="AB18" s="18">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -1939,8 +2012,12 @@
       <c r="AX18" s="2"/>
       <c r="AY18" s="2"/>
       <c r="AZ18" s="2"/>
-    </row>
-    <row r="19" spans="2:52" x14ac:dyDescent="0.25">
+      <c r="BA18" s="2"/>
+      <c r="BB18" s="2"/>
+      <c r="BC18" s="2"/>
+      <c r="BD18" s="2"/>
+    </row>
+    <row r="19" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B19" s="28" t="s">
         <v>25</v>
       </c>
@@ -1952,7 +2029,7 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="J19" s="19">
+      <c r="J19" s="18">
         <f>R17</f>
         <v>0.46426160383844894</v>
       </c>
@@ -1960,22 +2037,22 @@
         <v>97</v>
       </c>
       <c r="L19" s="1"/>
-      <c r="M19" s="23"/>
-      <c r="N19" s="25">
+      <c r="M19" s="22"/>
+      <c r="N19" s="24">
         <f>N18</f>
         <v>0.47304426716643216</v>
       </c>
-      <c r="O19" s="19" t="s">
+      <c r="O19" s="18" t="s">
         <v>62</v>
       </c>
       <c r="P19" s="2">
         <v>0.61399999999999999</v>
       </c>
-      <c r="Q19" s="19">
+      <c r="Q19" s="18">
         <f>($F$8+P19*($F$9-$F$8)) / 1440</f>
         <v>1.1208333333333334E-2</v>
       </c>
-      <c r="R19" s="19">
+      <c r="R19" s="18">
         <f>J19+Q19</f>
         <v>0.47546993717178226</v>
       </c>
@@ -1990,18 +2067,18 @@
         <v>56</v>
       </c>
       <c r="W19" s="2"/>
-      <c r="X19" s="19"/>
+      <c r="X19" s="18"/>
       <c r="Y19" s="2">
         <v>0</v>
       </c>
       <c r="Z19" s="2">
         <v>1</v>
       </c>
-      <c r="AA19" s="19">
+      <c r="AA19" s="18">
         <f>AA18+Q17</f>
         <v>2.6281390906884326E-2</v>
       </c>
-      <c r="AB19" s="19">
+      <c r="AB19" s="18">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2009,7 +2086,7 @@
         <v>0</v>
       </c>
       <c r="AD19" s="2"/>
-      <c r="AE19" s="22"/>
+      <c r="AE19" s="21"/>
       <c r="AF19" s="2" t="s">
         <v>85</v>
       </c>
@@ -2021,25 +2098,29 @@
       <c r="AL19" s="2"/>
       <c r="AM19" s="2"/>
       <c r="AN19" s="2"/>
-      <c r="AO19" s="2" t="s">
+      <c r="AO19" s="2"/>
+      <c r="AP19" s="2"/>
+      <c r="AQ19" s="2"/>
+      <c r="AR19" s="2"/>
+      <c r="AS19" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AP19" s="19">
+      <c r="AT19" s="18">
         <f>J19</f>
         <v>0.46426160383844894</v>
       </c>
-      <c r="AQ19" s="2"/>
-      <c r="AR19" s="2"/>
-      <c r="AS19" s="2"/>
-      <c r="AT19" s="2"/>
       <c r="AU19" s="2"/>
       <c r="AV19" s="2"/>
       <c r="AW19" s="2"/>
       <c r="AX19" s="2"/>
       <c r="AY19" s="2"/>
       <c r="AZ19" s="2"/>
-    </row>
-    <row r="20" spans="2:52" x14ac:dyDescent="0.25">
+      <c r="BA19" s="2"/>
+      <c r="BB19" s="2"/>
+      <c r="BC19" s="2"/>
+      <c r="BD19" s="2"/>
+    </row>
+    <row r="20" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
         <v>24</v>
       </c>
@@ -2059,7 +2140,7 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="J20" s="19">
+      <c r="J20" s="18">
         <f>N19</f>
         <v>0.47304426716643216</v>
       </c>
@@ -2069,23 +2150,23 @@
       <c r="L20" s="2">
         <v>0.22500000000000001</v>
       </c>
-      <c r="M20" s="19">
+      <c r="M20" s="18">
         <f>-$C$3*LN(1-L20) / 1440</f>
         <v>7.9653828008996886E-3</v>
       </c>
-      <c r="N20" s="19">
+      <c r="N20" s="18">
         <f>J20+M20</f>
         <v>0.48100964996733186</v>
       </c>
-      <c r="O20" s="19" t="s">
+      <c r="O20" s="18" t="s">
         <v>62</v>
       </c>
       <c r="P20" s="2"/>
-      <c r="Q20" s="19">
+      <c r="Q20" s="18">
         <f>Q19</f>
         <v>1.1208333333333334E-2</v>
       </c>
-      <c r="R20" s="20">
+      <c r="R20" s="19">
         <f>R19</f>
         <v>0.47546993717178226</v>
       </c>
@@ -2094,18 +2175,18 @@
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
       <c r="W20" s="1"/>
-      <c r="X20" s="26"/>
+      <c r="X20" s="25"/>
       <c r="Y20" s="2">
         <v>1</v>
       </c>
       <c r="Z20" s="2">
         <v>1</v>
       </c>
-      <c r="AA20" s="19">
+      <c r="AA20" s="18">
         <f>AA19+Q18</f>
         <v>3.5711946462439879E-2</v>
       </c>
-      <c r="AB20" s="19">
+      <c r="AB20" s="18">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2127,25 +2208,29 @@
       <c r="AL20" s="2"/>
       <c r="AM20" s="2"/>
       <c r="AN20" s="2"/>
-      <c r="AO20" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AP20" s="19">
-        <f>AP19</f>
-        <v>0.46426160383844894</v>
-      </c>
+      <c r="AO20" s="2"/>
+      <c r="AP20" s="2"/>
       <c r="AQ20" s="2"/>
       <c r="AR20" s="2"/>
-      <c r="AS20" s="2"/>
-      <c r="AT20" s="2"/>
+      <c r="AS20" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AT20" s="18">
+        <f>AT19</f>
+        <v>0.46426160383844894</v>
+      </c>
       <c r="AU20" s="2"/>
       <c r="AV20" s="2"/>
       <c r="AW20" s="2"/>
       <c r="AX20" s="2"/>
       <c r="AY20" s="2"/>
       <c r="AZ20" s="2"/>
-    </row>
-    <row r="21" spans="2:52" x14ac:dyDescent="0.25">
+      <c r="BA20" s="2"/>
+      <c r="BB20" s="2"/>
+      <c r="BC20" s="2"/>
+      <c r="BD20" s="2"/>
+    </row>
+    <row r="21" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>89</v>
       </c>
@@ -2168,7 +2253,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="J21" s="19">
+      <c r="J21" s="18">
         <f>R20</f>
         <v>0.47546993717178226</v>
       </c>
@@ -2176,22 +2261,22 @@
         <v>99</v>
       </c>
       <c r="L21" s="2"/>
-      <c r="M21" s="19"/>
-      <c r="N21" s="20">
+      <c r="M21" s="18"/>
+      <c r="N21" s="19">
         <f>N20</f>
         <v>0.48100964996733186</v>
       </c>
-      <c r="O21" s="19" t="s">
+      <c r="O21" s="18" t="s">
         <v>62</v>
       </c>
       <c r="P21" s="2">
         <v>0.26900000000000002</v>
       </c>
-      <c r="Q21" s="19">
+      <c r="Q21" s="18">
         <f>($F$8+P21*($F$9-$F$8)) / 1440</f>
         <v>8.8125000000000009E-3</v>
       </c>
-      <c r="R21" s="19">
+      <c r="R21" s="18">
         <f>Q21+J21</f>
         <v>0.48428243717178227</v>
       </c>
@@ -2206,18 +2291,18 @@
         <v>56</v>
       </c>
       <c r="W21" s="2"/>
-      <c r="X21" s="19"/>
+      <c r="X21" s="18"/>
       <c r="Y21" s="2">
         <v>0</v>
       </c>
       <c r="Z21" s="2">
         <v>2</v>
       </c>
-      <c r="AA21" s="19">
+      <c r="AA21" s="18">
         <f>AA20+(J21-J20)</f>
         <v>3.813761646778998E-2</v>
       </c>
-      <c r="AB21" s="19">
+      <c r="AB21" s="18">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2226,7 +2311,7 @@
       </c>
       <c r="AD21" s="2"/>
       <c r="AE21" s="2"/>
-      <c r="AF21" s="22"/>
+      <c r="AF21" s="21"/>
       <c r="AG21" s="2" t="s">
         <v>88</v>
       </c>
@@ -2237,30 +2322,34 @@
       <c r="AL21" s="2"/>
       <c r="AM21" s="2"/>
       <c r="AN21" s="2"/>
-      <c r="AO21" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AP21" s="19">
-        <f t="shared" ref="AP21:AP22" si="2">AP20</f>
-        <v>0.46426160383844894</v>
-      </c>
+      <c r="AO21" s="2"/>
+      <c r="AP21" s="2"/>
       <c r="AQ21" s="2"/>
       <c r="AR21" s="2"/>
       <c r="AS21" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AT21" s="19">
+      <c r="AT21" s="18">
+        <f t="shared" ref="AT21:AT22" si="2">AT20</f>
+        <v>0.46426160383844894</v>
+      </c>
+      <c r="AU21" s="2"/>
+      <c r="AV21" s="2"/>
+      <c r="AW21" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AX21" s="18">
         <f>J21</f>
         <v>0.47546993717178226</v>
       </c>
-      <c r="AU21" s="2"/>
-      <c r="AV21" s="2"/>
-      <c r="AW21" s="2"/>
-      <c r="AX21" s="2"/>
       <c r="AY21" s="2"/>
       <c r="AZ21" s="2"/>
-    </row>
-    <row r="22" spans="2:52" x14ac:dyDescent="0.25">
+      <c r="BA21" s="2"/>
+      <c r="BB21" s="2"/>
+      <c r="BC21" s="2"/>
+      <c r="BD21" s="2"/>
+    </row>
+    <row r="22" spans="2:56" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
         <v>90</v>
       </c>
@@ -2280,7 +2369,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="J22" s="19">
+      <c r="J22" s="18">
         <f>N21</f>
         <v>0.48100964996733186</v>
       </c>
@@ -2290,19 +2379,19 @@
       <c r="L22" s="2">
         <v>0.57099999999999995</v>
       </c>
-      <c r="M22" s="19">
+      <c r="M22" s="18">
         <f>-$C$3*LN(1-L22) / 1440</f>
         <v>2.6446823751691249E-2</v>
       </c>
-      <c r="N22" s="19">
+      <c r="N22" s="18">
         <f>J22+M22</f>
         <v>0.50745647371902314</v>
       </c>
-      <c r="O22" s="19" t="s">
+      <c r="O22" s="18" t="s">
         <v>62</v>
       </c>
       <c r="P22" s="2"/>
-      <c r="Q22" s="19">
+      <c r="Q22" s="18">
         <f>Q21</f>
         <v>8.8125000000000009E-3</v>
       </c>
@@ -2315,18 +2404,18 @@
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
       <c r="W22" s="2"/>
-      <c r="X22" s="19"/>
+      <c r="X22" s="18"/>
       <c r="Y22" s="2">
         <v>1</v>
       </c>
       <c r="Z22" s="2">
         <v>2</v>
       </c>
-      <c r="AA22" s="19">
+      <c r="AA22" s="18">
         <f>AA21++J22-J21</f>
         <v>4.3677329263339615E-2</v>
       </c>
-      <c r="AB22" s="19">
+      <c r="AB22" s="18">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2348,78 +2437,843 @@
       <c r="AL22" s="2"/>
       <c r="AM22" s="2"/>
       <c r="AN22" s="2"/>
-      <c r="AO22" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AP22" s="19">
-        <f t="shared" si="2"/>
-        <v>0.46426160383844894</v>
-      </c>
+      <c r="AO22" s="2"/>
+      <c r="AP22" s="2"/>
       <c r="AQ22" s="2"/>
       <c r="AR22" s="2"/>
       <c r="AS22" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="AT22" s="19">
-        <f>AT21</f>
-        <v>0.47546993717178226</v>
+      <c r="AT22" s="18">
+        <f t="shared" si="2"/>
+        <v>0.46426160383844894</v>
       </c>
       <c r="AU22" s="2"/>
       <c r="AV22" s="2"/>
-      <c r="AW22" s="2"/>
-      <c r="AX22" s="2"/>
+      <c r="AW22" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AX22" s="18">
+        <f>AX21</f>
+        <v>0.47546993717178226</v>
+      </c>
       <c r="AY22" s="2"/>
       <c r="AZ22" s="2"/>
-    </row>
-    <row r="23" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="J23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
+      <c r="BA22" s="2"/>
+      <c r="BB22" s="2"/>
+      <c r="BC22" s="2"/>
+      <c r="BD22" s="2"/>
+    </row>
+    <row r="23" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="I23" s="2">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="J23" s="18">
+        <f>R22</f>
+        <v>0.48428243717178227</v>
+      </c>
+      <c r="K23" s="42" t="s">
+        <v>102</v>
+      </c>
+      <c r="L23" s="2"/>
+      <c r="M23" s="18"/>
+      <c r="N23" s="18">
+        <f>N22</f>
+        <v>0.50745647371902314</v>
+      </c>
+      <c r="O23" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="P23" s="2">
+        <v>0.81699999999999995</v>
+      </c>
+      <c r="Q23" s="18">
+        <f>($F$8+P23*($F$9-$F$8)) / 1440</f>
+        <v>1.2618055555555556E-2</v>
+      </c>
+      <c r="R23" s="19">
+        <f>Q23+J23</f>
+        <v>0.49690049272733783</v>
+      </c>
+      <c r="S23" s="2">
+        <v>0.125</v>
+      </c>
+      <c r="T23" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="U23" s="2">
+        <v>0.34100000000000003</v>
+      </c>
+      <c r="V23" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="W23" s="2"/>
+      <c r="X23" s="2"/>
+      <c r="Y23" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="42">
+        <v>2</v>
+      </c>
       <c r="AA23" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="24" spans="2:52" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="34" t="s">
+      <c r="AD23" s="2"/>
+      <c r="AE23" s="2"/>
+      <c r="AF23" s="2"/>
+      <c r="AG23" s="21"/>
+      <c r="AH23" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="AI23" s="2"/>
+      <c r="AJ23" s="2"/>
+      <c r="AK23" s="2"/>
+      <c r="AL23" s="2"/>
+      <c r="AM23" s="2"/>
+      <c r="AN23" s="2"/>
+      <c r="AO23" s="2"/>
+      <c r="AP23" s="2"/>
+      <c r="AQ23" s="2"/>
+      <c r="AR23" s="2"/>
+      <c r="AS23" s="42" t="s">
+        <v>88</v>
+      </c>
+      <c r="AT23" s="18">
+        <f>AT22</f>
+        <v>0.46426160383844894</v>
+      </c>
+      <c r="AU23" s="2"/>
+      <c r="AV23" s="2"/>
+      <c r="AW23" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AX23" s="18">
+        <f>AX22</f>
+        <v>0.47546993717178226</v>
+      </c>
+      <c r="AY23" s="2"/>
+      <c r="AZ23" s="2"/>
+    </row>
+    <row r="24" spans="2:56" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="34"/>
-      <c r="D24" s="34"/>
-      <c r="E24" s="34"/>
-      <c r="F24" s="34"/>
-      <c r="J24" s="3"/>
-    </row>
-    <row r="25" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="B25" s="34"/>
-      <c r="C25" s="34"/>
-      <c r="D25" s="34"/>
-      <c r="E25" s="34"/>
-      <c r="F25" s="34"/>
-      <c r="J25" s="3"/>
-    </row>
-    <row r="26" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="J26" s="3"/>
-    </row>
-    <row r="27" spans="2:52" x14ac:dyDescent="0.25">
-      <c r="J27" s="3"/>
+      <c r="C24" s="35"/>
+      <c r="D24" s="35"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="35"/>
+      <c r="I24" s="2">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="J24" s="18">
+        <f>R23</f>
+        <v>0.49690049272733783</v>
+      </c>
+      <c r="K24" s="42" t="s">
+        <v>105</v>
+      </c>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
+      <c r="N24" s="18">
+        <f>N23</f>
+        <v>0.50745647371902314</v>
+      </c>
+      <c r="O24" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="P24" s="2"/>
+      <c r="Q24" s="2"/>
+      <c r="R24" s="2"/>
+      <c r="S24" s="2">
+        <v>4.3999999999999997E-2</v>
+      </c>
+      <c r="T24" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="U24" s="2">
+        <v>0.122</v>
+      </c>
+      <c r="V24" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="W24" s="2">
+        <v>5.5E-2</v>
+      </c>
+      <c r="X24" s="19">
+        <f>-90*LN(1-W24) / 1440</f>
+        <v>3.5356469680246473E-3</v>
+      </c>
+      <c r="Y24" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z24" s="42">
+        <v>1</v>
+      </c>
+      <c r="AD24" s="2"/>
+      <c r="AE24" s="2"/>
+      <c r="AF24" s="2"/>
+      <c r="AG24" s="2"/>
+      <c r="AH24" s="21"/>
+      <c r="AI24" s="42"/>
+      <c r="AJ24" s="42"/>
+      <c r="AK24" s="42"/>
+      <c r="AL24" s="42"/>
+      <c r="AM24" s="2"/>
+      <c r="AN24" s="2"/>
+      <c r="AO24" s="2"/>
+      <c r="AP24" s="2"/>
+      <c r="AQ24" s="2"/>
+      <c r="AR24" s="2"/>
+      <c r="AS24" s="42" t="s">
+        <v>91</v>
+      </c>
+      <c r="AT24" s="18">
+        <f>AT23</f>
+        <v>0.46426160383844894</v>
+      </c>
+      <c r="AU24" s="18">
+        <v>0.50043981481481481</v>
+      </c>
+      <c r="AV24" s="18"/>
+      <c r="AW24" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AX24" s="18">
+        <f t="shared" ref="AX24:AX28" si="3">AX23</f>
+        <v>0.47546993717178226</v>
+      </c>
+      <c r="AY24" s="2"/>
+      <c r="AZ24" s="2"/>
+    </row>
+    <row r="25" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="B25" s="35"/>
+      <c r="C25" s="35"/>
+      <c r="D25" s="35"/>
+      <c r="E25" s="35"/>
+      <c r="F25" s="35"/>
+      <c r="I25" s="2">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="J25" s="18">
+        <f>J24+X24</f>
+        <v>0.50043613969536249</v>
+      </c>
+      <c r="K25" s="42" t="s">
+        <v>106</v>
+      </c>
+      <c r="L25" s="2"/>
+      <c r="M25" s="2"/>
+      <c r="N25" s="19">
+        <f>N24</f>
+        <v>0.50745647371902314</v>
+      </c>
+      <c r="O25" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="P25" s="2"/>
+      <c r="Q25" s="2"/>
+      <c r="R25" s="2"/>
+      <c r="S25" s="2"/>
+      <c r="T25" s="2"/>
+      <c r="U25" s="2"/>
+      <c r="V25" s="2"/>
+      <c r="W25" s="2">
+        <v>0.20899999999999999</v>
+      </c>
+      <c r="X25" s="41">
+        <f>-90*LN(1-W25) / 1440</f>
+        <v>1.4653581950905195E-2</v>
+      </c>
+      <c r="Y25" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="42">
+        <v>0</v>
+      </c>
+      <c r="AD25" s="2"/>
+      <c r="AE25" s="2"/>
+      <c r="AF25" s="2"/>
+      <c r="AG25" s="2"/>
+      <c r="AH25" s="2"/>
+      <c r="AI25" s="2"/>
+      <c r="AJ25" s="2"/>
+      <c r="AK25" s="2"/>
+      <c r="AL25" s="2"/>
+      <c r="AM25" s="2"/>
+      <c r="AN25" s="2"/>
+      <c r="AO25" s="2"/>
+      <c r="AP25" s="2"/>
+      <c r="AQ25" s="2"/>
+      <c r="AR25" s="2"/>
+      <c r="AS25" s="23"/>
+      <c r="AT25" s="18">
+        <f>AT24</f>
+        <v>0.46426160383844894</v>
+      </c>
+      <c r="AU25" s="18">
+        <f>AU24</f>
+        <v>0.50043981481481481</v>
+      </c>
+      <c r="AV25" s="18">
+        <v>3.5300925925925925E-3</v>
+      </c>
+      <c r="AW25" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AX25" s="18">
+        <f t="shared" si="3"/>
+        <v>0.47546993717178226</v>
+      </c>
+      <c r="AY25" s="2"/>
+      <c r="AZ25" s="2"/>
+    </row>
+    <row r="26" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="I26" s="2">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="J26" s="18">
+        <v>0.50745370370370368</v>
+      </c>
+      <c r="K26" s="42" t="s">
+        <v>107</v>
+      </c>
+      <c r="L26" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="M26" s="18">
+        <f>-$C$3*LN(1-L26) / 1440</f>
+        <v>7.1955784156063934E-2</v>
+      </c>
+      <c r="N26" s="18">
+        <f>M26++J26</f>
+        <v>0.57940948785976765</v>
+      </c>
+      <c r="O26" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="P26" s="2">
+        <v>0.89300000000000002</v>
+      </c>
+      <c r="Q26" s="18">
+        <f>($F$8+P26*($F$9-$F$8)) / 1440</f>
+        <v>1.3145833333333332E-2</v>
+      </c>
+      <c r="R26" s="19">
+        <f>Q26+J26</f>
+        <v>0.52059953703703699</v>
+      </c>
+      <c r="S26" s="2"/>
+      <c r="T26" s="2"/>
+      <c r="U26" s="2"/>
+      <c r="V26" s="2"/>
+      <c r="W26" s="2"/>
+      <c r="X26" s="41">
+        <f>AZ26</f>
+        <v>7.6332479272445495E-3</v>
+      </c>
+      <c r="Y26" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z26" s="2">
+        <v>1</v>
+      </c>
+      <c r="AD26" s="2"/>
+      <c r="AE26" s="2"/>
+      <c r="AF26" s="2"/>
+      <c r="AG26" s="2"/>
+      <c r="AH26" s="2"/>
+      <c r="AI26" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="AJ26" s="2"/>
+      <c r="AK26" s="2"/>
+      <c r="AL26" s="2"/>
+      <c r="AM26" s="2"/>
+      <c r="AN26" s="2"/>
+      <c r="AO26" s="2"/>
+      <c r="AP26" s="2"/>
+      <c r="AQ26" s="2"/>
+      <c r="AR26" s="2"/>
+      <c r="AS26" s="2"/>
+      <c r="AT26" s="23"/>
+      <c r="AU26" s="23"/>
+      <c r="AV26" s="23"/>
+      <c r="AW26" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AX26" s="18">
+        <f t="shared" si="3"/>
+        <v>0.47546993717178226</v>
+      </c>
+      <c r="AY26" s="2"/>
+      <c r="AZ26" s="18">
+        <f>X25-(N25-J25)</f>
+        <v>7.6332479272445495E-3</v>
+      </c>
+    </row>
+    <row r="27" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="I27" s="2">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="J27" s="18">
+        <f>R26</f>
+        <v>0.52059953703703699</v>
+      </c>
+      <c r="K27" s="42" t="s">
+        <v>108</v>
+      </c>
+      <c r="L27" s="2"/>
+      <c r="M27" s="2"/>
+      <c r="N27" s="18">
+        <f>N26</f>
+        <v>0.57940948785976765</v>
+      </c>
+      <c r="O27" s="43" t="s">
+        <v>61</v>
+      </c>
+      <c r="P27" s="2"/>
+      <c r="Q27" s="2"/>
+      <c r="R27" s="2"/>
+      <c r="S27" s="2">
+        <v>0.89900000000000002</v>
+      </c>
+      <c r="T27" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="U27" s="2"/>
+      <c r="V27" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="W27" s="2"/>
+      <c r="X27" s="19">
+        <f>X26</f>
+        <v>7.6332479272445495E-3</v>
+      </c>
+      <c r="Y27" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="42">
+        <v>0</v>
+      </c>
+      <c r="AD27" s="2"/>
+      <c r="AE27" s="2"/>
+      <c r="AF27" s="2"/>
+      <c r="AG27" s="2"/>
+      <c r="AH27" s="2"/>
+      <c r="AI27" s="21"/>
+      <c r="AJ27" s="42"/>
+      <c r="AK27" s="42"/>
+      <c r="AL27" s="42"/>
+      <c r="AM27" s="2"/>
+      <c r="AN27" s="2"/>
+      <c r="AO27" s="2"/>
+      <c r="AP27" s="2"/>
+      <c r="AQ27" s="2"/>
+      <c r="AR27" s="2"/>
+      <c r="AS27" s="2"/>
+      <c r="AT27" s="2"/>
+      <c r="AU27" s="2"/>
+      <c r="AV27" s="2"/>
+      <c r="AW27" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AX27" s="18">
+        <f t="shared" si="3"/>
+        <v>0.47546993717178226</v>
+      </c>
+      <c r="AY27" s="2"/>
+      <c r="AZ27" s="18">
+        <f>AZ26</f>
+        <v>7.6332479272445495E-3</v>
+      </c>
+    </row>
+    <row r="28" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="I28" s="2">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="J28" s="18">
+        <f>J27+X27</f>
+        <v>0.5282327849642815</v>
+      </c>
+      <c r="K28" s="42" t="s">
+        <v>109</v>
+      </c>
+      <c r="L28" s="2"/>
+      <c r="M28" s="2"/>
+      <c r="N28" s="19">
+        <f>N27</f>
+        <v>0.57940948785976765</v>
+      </c>
+      <c r="O28" s="43" t="s">
+        <v>54</v>
+      </c>
+      <c r="P28" s="2"/>
+      <c r="Q28" s="2"/>
+      <c r="R28" s="2"/>
+      <c r="S28" s="2"/>
+      <c r="T28" s="2"/>
+      <c r="U28" s="2"/>
+      <c r="V28" s="2"/>
+      <c r="W28" s="2"/>
+      <c r="X28" s="2"/>
+      <c r="Y28" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="42">
+        <v>0</v>
+      </c>
+      <c r="AD28" s="2"/>
+      <c r="AE28" s="2"/>
+      <c r="AF28" s="2"/>
+      <c r="AG28" s="2"/>
+      <c r="AH28" s="2"/>
+      <c r="AI28" s="2"/>
+      <c r="AJ28" s="2"/>
+      <c r="AK28" s="2"/>
+      <c r="AL28" s="2"/>
+      <c r="AM28" s="2"/>
+      <c r="AN28" s="2"/>
+      <c r="AO28" s="2"/>
+      <c r="AP28" s="2"/>
+      <c r="AQ28" s="2"/>
+      <c r="AR28" s="2"/>
+      <c r="AS28" s="2"/>
+      <c r="AT28" s="2"/>
+      <c r="AU28" s="2"/>
+      <c r="AV28" s="2"/>
+      <c r="AW28" s="23"/>
+      <c r="AX28" s="18">
+        <f t="shared" si="3"/>
+        <v>0.47546993717178226</v>
+      </c>
+      <c r="AY28" s="18">
+        <v>0.52822916666666664</v>
+      </c>
+      <c r="AZ28" s="18">
+        <f>AZ27</f>
+        <v>7.6332479272445495E-3</v>
+      </c>
+    </row>
+    <row r="29" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="I29" s="2">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="J29" s="18">
+        <f>N28</f>
+        <v>0.57940948785976765</v>
+      </c>
+      <c r="K29" s="42" t="s">
+        <v>110</v>
+      </c>
+      <c r="L29" s="2">
+        <v>0.87</v>
+      </c>
+      <c r="M29" s="18">
+        <f>-$C$3*LN(1-L29) / 1440</f>
+        <v>6.3756900891454832E-2</v>
+      </c>
+      <c r="N29" s="18">
+        <f>M29++J29</f>
+        <v>0.64316638875122245</v>
+      </c>
+      <c r="O29" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="P29" s="2">
+        <v>0.93</v>
+      </c>
+      <c r="Q29" s="18">
+        <f>($F$8+P29*($F$9-$F$8)) / 1440</f>
+        <v>1.3402777777777779E-2</v>
+      </c>
+      <c r="R29" s="19">
+        <f>Q29+J29</f>
+        <v>0.59281226563754541</v>
+      </c>
+      <c r="S29" s="2"/>
+      <c r="T29" s="2"/>
+      <c r="U29" s="2"/>
+      <c r="V29" s="2"/>
+      <c r="W29" s="2"/>
+      <c r="X29" s="2"/>
+      <c r="Y29" s="42">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="42">
+        <v>0</v>
+      </c>
+      <c r="AD29" s="2"/>
+      <c r="AE29" s="2"/>
+      <c r="AF29" s="2"/>
+      <c r="AG29" s="2"/>
+      <c r="AH29" s="2"/>
+      <c r="AI29" s="2"/>
+      <c r="AJ29" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="AK29" s="2"/>
+      <c r="AL29" s="2"/>
+      <c r="AM29" s="2"/>
+      <c r="AN29" s="2"/>
+      <c r="AO29" s="2"/>
+      <c r="AP29" s="2"/>
+      <c r="AQ29" s="2"/>
+      <c r="AR29" s="2"/>
+      <c r="AS29" s="2"/>
+      <c r="AT29" s="2"/>
+      <c r="AU29" s="2"/>
+      <c r="AV29" s="2"/>
+      <c r="AW29" s="2"/>
+      <c r="AX29" s="23"/>
+      <c r="AY29" s="23"/>
+      <c r="AZ29" s="23"/>
+    </row>
+    <row r="30" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="I30" s="2">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="J30" s="18"/>
+      <c r="K30" s="42"/>
+      <c r="L30" s="2"/>
+      <c r="M30" s="2"/>
+      <c r="N30" s="2"/>
+      <c r="O30" s="2"/>
+      <c r="P30" s="2"/>
+      <c r="Q30" s="2"/>
+      <c r="R30" s="2"/>
+      <c r="S30" s="2"/>
+      <c r="T30" s="2"/>
+      <c r="U30" s="2"/>
+      <c r="V30" s="2"/>
+      <c r="W30" s="2"/>
+      <c r="X30" s="2"/>
+      <c r="Y30" s="2"/>
+      <c r="Z30" s="2"/>
+      <c r="AD30" s="2"/>
+      <c r="AE30" s="2"/>
+      <c r="AF30" s="2"/>
+      <c r="AG30" s="2"/>
+      <c r="AH30" s="2"/>
+      <c r="AI30" s="2"/>
+      <c r="AJ30" s="42"/>
+      <c r="AK30" s="42"/>
+      <c r="AL30" s="42"/>
+      <c r="AM30" s="2"/>
+      <c r="AN30" s="2"/>
+      <c r="AO30" s="2"/>
+      <c r="AP30" s="2"/>
+      <c r="AQ30" s="2"/>
+      <c r="AR30" s="2"/>
+      <c r="AS30" s="2"/>
+      <c r="AT30" s="2"/>
+      <c r="AU30" s="2"/>
+      <c r="AV30" s="2"/>
+      <c r="AW30" s="2"/>
+      <c r="AX30" s="2"/>
+      <c r="AY30" s="2"/>
+      <c r="AZ30" s="2"/>
+    </row>
+    <row r="31" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="I31" s="2">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="AD31" s="44"/>
+      <c r="AE31" s="44"/>
+      <c r="AF31" s="44"/>
+      <c r="AG31" s="44"/>
+      <c r="AH31" s="44"/>
+      <c r="AI31" s="44"/>
+      <c r="AJ31" s="44"/>
+      <c r="AK31" s="44"/>
+      <c r="AL31" s="44"/>
+      <c r="AM31" s="44"/>
+      <c r="AN31" s="44"/>
+      <c r="AO31" s="44"/>
+      <c r="AP31" s="44"/>
+      <c r="AQ31" s="44"/>
+      <c r="AR31" s="44"/>
+      <c r="AS31" s="44"/>
+      <c r="AT31" s="44"/>
+      <c r="AU31" s="44"/>
+      <c r="AV31" s="44"/>
+      <c r="AW31" s="44"/>
+      <c r="AX31" s="44"/>
+      <c r="AY31" s="44"/>
+      <c r="AZ31" s="44"/>
+    </row>
+    <row r="32" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="I32" s="2">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="R32" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="S32" s="26">
+        <f ca="1">RAND()</f>
+        <v>0.57786729470145815</v>
+      </c>
+      <c r="AD32" s="44"/>
+      <c r="AE32" s="44"/>
+      <c r="AF32" s="44"/>
+      <c r="AG32" s="44"/>
+      <c r="AH32" s="44"/>
+      <c r="AI32" s="44"/>
+      <c r="AJ32" s="44"/>
+      <c r="AK32" s="44"/>
+      <c r="AL32" s="44"/>
+      <c r="AM32" s="44"/>
+      <c r="AN32" s="44"/>
+      <c r="AO32" s="44"/>
+      <c r="AP32" s="44"/>
+      <c r="AQ32" s="44"/>
+      <c r="AR32" s="44"/>
+      <c r="AS32" s="44"/>
+      <c r="AT32" s="44"/>
+      <c r="AU32" s="44"/>
+      <c r="AV32" s="44"/>
+      <c r="AW32" s="44"/>
+      <c r="AX32" s="44"/>
+      <c r="AY32" s="44"/>
+      <c r="AZ32" s="44"/>
+    </row>
+    <row r="33" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I33" s="2">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I34" s="2">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I35" s="2">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="36" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I36" s="2">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="37" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I37" s="2">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I38" s="2">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="39" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I39" s="2">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="40" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I40" s="2">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="41" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I41" s="2">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="42" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I42" s="2">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I43" s="2">
+        <f t="shared" si="0"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="44" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I44" s="2">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="45" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I45" s="2">
+        <f t="shared" si="0"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="46" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I46" s="2">
+        <f t="shared" si="0"/>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="47" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I47" s="2">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I48" s="2">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="49" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I49" s="2">
+        <f t="shared" si="0"/>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="50" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I50" s="2">
+        <f t="shared" si="0"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="51" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I51" s="2">
+        <f t="shared" si="0"/>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="52" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="I52" s="2">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="AS11:AV11"/>
-    <mergeCell ref="AW11:AZ11"/>
-    <mergeCell ref="AK10:AZ10"/>
-    <mergeCell ref="J9:AZ9"/>
-    <mergeCell ref="K2:O2"/>
-    <mergeCell ref="L11:N11"/>
-    <mergeCell ref="W11:X11"/>
-    <mergeCell ref="Q3:R3"/>
-    <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="Q2:T2"/>
-    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="AO11:AR11"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="AD10:AM10"/>
+    <mergeCell ref="O11:V11"/>
+    <mergeCell ref="AA11:AC11"/>
+    <mergeCell ref="Y11:Z11"/>
     <mergeCell ref="B24:F25"/>
     <mergeCell ref="G8:H9"/>
     <mergeCell ref="B4:C4"/>
@@ -2431,13 +3285,22 @@
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B19:F19"/>
-    <mergeCell ref="AO11:AR11"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="AD10:AI10"/>
-    <mergeCell ref="O11:V11"/>
-    <mergeCell ref="AA11:AC11"/>
-    <mergeCell ref="Y11:Z11"/>
-    <mergeCell ref="AK11:AN11"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="AW11:AZ11"/>
+    <mergeCell ref="BA11:BD11"/>
+    <mergeCell ref="AO10:BD10"/>
+    <mergeCell ref="J9:BD9"/>
+    <mergeCell ref="K2:O2"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="W11:X11"/>
+    <mergeCell ref="Q3:R3"/>
+    <mergeCell ref="Q4:R4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="Q2:T2"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="AS11:AV11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel terminado de nuevo hasta el dia de Cierre más los cambios en el Front
</commit_message>
<xml_diff>
--- a/1er Entrega/Plantilla.xlsx
+++ b/1er Entrega/Plantilla.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\UTN\Simulación\TP 4\Tp4-Simulacion-G5\1er Entrega\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc_ju\OneDrive\Escritorio\Tp4-Simulacion-G5\1er Entrega\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F7D5A6-70D8-467E-97E8-13468611C6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3F41667-2752-4B13-AF08-5E6A00266121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="119">
   <si>
     <t>Horario Apertura</t>
   </si>
@@ -194,9 +194,6 @@
     <t>RND Duracion Reparacion</t>
   </si>
   <si>
-    <t>Randoms</t>
-  </si>
-  <si>
     <t>Tiempo entre Llegadas</t>
   </si>
   <si>
@@ -368,7 +365,34 @@
     <t>Fin_Reparacion_CL3</t>
   </si>
   <si>
-    <t>Llega_Cliente_7</t>
+    <t>Llegada_Cliente_7</t>
+  </si>
+  <si>
+    <t>Fin_Atencion_CL7</t>
+  </si>
+  <si>
+    <t>Llegada_Cliente_8</t>
+  </si>
+  <si>
+    <t>Fin_Atencion_CL8</t>
+  </si>
+  <si>
+    <t>Llegada_Cliente_9</t>
+  </si>
+  <si>
+    <t>Fin_Atencion_CL9</t>
+  </si>
+  <si>
+    <t>Llegada_Cliente_10</t>
+  </si>
+  <si>
+    <t>Fin_Atencion_CL10</t>
+  </si>
+  <si>
+    <t>Fin_Reparacion_CL4</t>
+  </si>
+  <si>
+    <t>c</t>
   </si>
 </sst>
 </file>
@@ -379,7 +403,7 @@
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -404,6 +428,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1" tint="4.9989318521683403E-2"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -495,7 +526,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -518,11 +549,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -580,15 +648,30 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -608,28 +691,35 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="46" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="46" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="46" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -910,67 +1000,77 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:BD52"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:BH182"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" customWidth="1"/>
+    <col min="3" max="3" width="8.54296875" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="11" max="11" width="19.42578125" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.5703125" customWidth="1"/>
-    <col min="19" max="20" width="12.42578125" customWidth="1"/>
-    <col min="21" max="21" width="12.5703125" customWidth="1"/>
-    <col min="23" max="23" width="11.28515625" customWidth="1"/>
-    <col min="25" max="25" width="9.85546875" customWidth="1"/>
-    <col min="26" max="26" width="11.5703125" customWidth="1"/>
-    <col min="27" max="27" width="10.140625" customWidth="1"/>
-    <col min="28" max="28" width="10.85546875" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="32" max="32" width="15.28515625" customWidth="1"/>
-    <col min="33" max="33" width="16.28515625" customWidth="1"/>
+    <col min="9" max="9" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" customWidth="1"/>
+    <col min="11" max="11" width="19.453125" customWidth="1"/>
+    <col min="12" max="12" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="17.54296875" customWidth="1"/>
+    <col min="16" max="16" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.54296875" customWidth="1"/>
+    <col min="18" max="18" width="16.81640625" customWidth="1"/>
+    <col min="19" max="20" width="12.453125" customWidth="1"/>
+    <col min="21" max="21" width="12.54296875" customWidth="1"/>
+    <col min="23" max="23" width="11.26953125" customWidth="1"/>
+    <col min="25" max="25" width="9.81640625" customWidth="1"/>
+    <col min="26" max="26" width="11.54296875" customWidth="1"/>
+    <col min="27" max="27" width="12.7265625" customWidth="1"/>
+    <col min="28" max="28" width="10.81640625" customWidth="1"/>
+    <col min="29" max="29" width="10.26953125" customWidth="1"/>
+    <col min="32" max="32" width="15.26953125" customWidth="1"/>
+    <col min="33" max="33" width="16.26953125" customWidth="1"/>
     <col min="34" max="38" width="12" customWidth="1"/>
-    <col min="40" max="40" width="1.140625" customWidth="1"/>
-    <col min="41" max="43" width="15.5703125" customWidth="1"/>
-    <col min="44" max="44" width="11.7109375" customWidth="1"/>
-    <col min="47" max="47" width="12.42578125" customWidth="1"/>
-    <col min="48" max="48" width="12.28515625" customWidth="1"/>
-    <col min="51" max="51" width="12.28515625" customWidth="1"/>
-    <col min="52" max="52" width="11.42578125" customWidth="1"/>
-    <col min="55" max="55" width="11.7109375" customWidth="1"/>
+    <col min="40" max="40" width="1.1796875" customWidth="1"/>
+    <col min="41" max="43" width="15.54296875" customWidth="1"/>
+    <col min="44" max="44" width="11.7265625" customWidth="1"/>
+    <col min="46" max="46" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="12.453125" customWidth="1"/>
+    <col min="48" max="48" width="12.26953125" customWidth="1"/>
+    <col min="50" max="50" width="11.1796875" customWidth="1"/>
+    <col min="51" max="51" width="12.26953125" customWidth="1"/>
+    <col min="52" max="52" width="11.453125" customWidth="1"/>
+    <col min="54" max="54" width="13.453125" customWidth="1"/>
+    <col min="55" max="55" width="11.7265625" customWidth="1"/>
     <col min="56" max="56" width="12" customWidth="1"/>
+    <col min="58" max="58" width="11.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:56" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:60" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2"/>
-      <c r="E2" s="27" t="s">
+      <c r="E2" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="33"/>
+      <c r="H2" s="33"/>
       <c r="J2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="31" t="s">
+      <c r="K2" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="31"/>
-      <c r="O2" s="31"/>
-      <c r="Q2" s="34" t="s">
-        <v>73</v>
-      </c>
-      <c r="R2" s="34"/>
-      <c r="S2" s="34"/>
-      <c r="T2" s="34"/>
-    </row>
-    <row r="3" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
+      <c r="N2" s="36"/>
+      <c r="O2" s="36"/>
+      <c r="Q2" s="39" t="s">
+        <v>72</v>
+      </c>
+      <c r="R2" s="39"/>
+      <c r="S2" s="39"/>
+      <c r="T2" s="39"/>
+    </row>
+    <row r="3" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -983,24 +1083,24 @@
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
-      <c r="Q3" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="R3" s="28"/>
-      <c r="S3" s="28" t="s">
-        <v>78</v>
-      </c>
-      <c r="T3" s="28"/>
-    </row>
-    <row r="4" spans="2:56" x14ac:dyDescent="0.25">
-      <c r="B4" s="28" t="s">
+      <c r="Q3" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="R3" s="26"/>
+      <c r="S3" s="26" t="s">
+        <v>77</v>
+      </c>
+      <c r="T3" s="26"/>
+    </row>
+    <row r="4" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="B4" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="28"/>
-      <c r="E4" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="F4" s="28"/>
+      <c r="C4" s="26"/>
+      <c r="E4" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" s="26"/>
       <c r="G4" s="2">
         <v>10</v>
       </c>
@@ -1017,22 +1117,22 @@
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q4" s="28" t="s">
-        <v>74</v>
-      </c>
-      <c r="R4" s="28"/>
-      <c r="S4" s="28" t="s">
-        <v>76</v>
-      </c>
-      <c r="T4" s="28"/>
-    </row>
-    <row r="5" spans="2:56" x14ac:dyDescent="0.25">
-      <c r="E5" s="28" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q4" s="26" t="s">
+        <v>73</v>
+      </c>
+      <c r="R4" s="26"/>
+      <c r="S4" s="26" t="s">
+        <v>75</v>
+      </c>
+      <c r="T4" s="26"/>
+    </row>
+    <row r="5" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="E5" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="28"/>
+      <c r="F5" s="26"/>
       <c r="G5" s="2">
         <v>18</v>
       </c>
@@ -1040,37 +1140,37 @@
         <v>2</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L5" s="2"/>
       <c r="M5" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="6" spans="2:56" ht="60" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="2:60" ht="58" x14ac:dyDescent="0.35">
       <c r="J6" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="7" spans="2:56" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1080,23 +1180,23 @@
       <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="28" t="s">
+      <c r="E7" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28" t="s">
+      <c r="F7" s="26"/>
+      <c r="G7" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="28"/>
-    </row>
-    <row r="8" spans="2:56" x14ac:dyDescent="0.25">
-      <c r="B8" s="28" t="s">
+      <c r="H7" s="26"/>
+    </row>
+    <row r="8" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="B8" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="28" t="s">
+      <c r="D8" s="26" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -1105,74 +1205,74 @@
       <c r="F8" s="2">
         <v>10</v>
       </c>
-      <c r="G8" s="36" t="s">
+      <c r="G8" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="H8" s="36"/>
-    </row>
-    <row r="9" spans="2:56" x14ac:dyDescent="0.25">
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
+      <c r="H8" s="27"/>
+    </row>
+    <row r="9" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="B9" s="26"/>
+      <c r="C9" s="26"/>
+      <c r="D9" s="26"/>
       <c r="E9" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="2">
         <v>20</v>
       </c>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="J9" s="30" t="s">
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="J9" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="30"/>
-      <c r="L9" s="30"/>
-      <c r="M9" s="30"/>
-      <c r="N9" s="30"/>
-      <c r="O9" s="30"/>
-      <c r="P9" s="30"/>
-      <c r="Q9" s="30"/>
-      <c r="R9" s="30"/>
-      <c r="S9" s="30"/>
-      <c r="T9" s="30"/>
-      <c r="U9" s="30"/>
-      <c r="V9" s="30"/>
-      <c r="W9" s="30"/>
-      <c r="X9" s="30"/>
-      <c r="Y9" s="30"/>
-      <c r="Z9" s="30"/>
-      <c r="AA9" s="30"/>
-      <c r="AB9" s="30"/>
-      <c r="AC9" s="30"/>
-      <c r="AD9" s="30"/>
-      <c r="AE9" s="30"/>
-      <c r="AF9" s="30"/>
-      <c r="AG9" s="30"/>
-      <c r="AH9" s="30"/>
-      <c r="AI9" s="30"/>
-      <c r="AJ9" s="30"/>
-      <c r="AK9" s="30"/>
-      <c r="AL9" s="30"/>
-      <c r="AM9" s="30"/>
-      <c r="AN9" s="30"/>
-      <c r="AO9" s="30"/>
-      <c r="AP9" s="30"/>
-      <c r="AQ9" s="30"/>
-      <c r="AR9" s="30"/>
-      <c r="AS9" s="30"/>
-      <c r="AT9" s="30"/>
-      <c r="AU9" s="30"/>
-      <c r="AV9" s="30"/>
-      <c r="AW9" s="30"/>
-      <c r="AX9" s="30"/>
-      <c r="AY9" s="30"/>
-      <c r="AZ9" s="30"/>
-      <c r="BA9" s="30"/>
-      <c r="BB9" s="30"/>
-      <c r="BC9" s="30"/>
-      <c r="BD9" s="30"/>
-    </row>
-    <row r="10" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="K9" s="35"/>
+      <c r="L9" s="35"/>
+      <c r="M9" s="35"/>
+      <c r="N9" s="35"/>
+      <c r="O9" s="35"/>
+      <c r="P9" s="35"/>
+      <c r="Q9" s="35"/>
+      <c r="R9" s="35"/>
+      <c r="S9" s="35"/>
+      <c r="T9" s="35"/>
+      <c r="U9" s="35"/>
+      <c r="V9" s="35"/>
+      <c r="W9" s="35"/>
+      <c r="X9" s="35"/>
+      <c r="Y9" s="35"/>
+      <c r="Z9" s="35"/>
+      <c r="AA9" s="35"/>
+      <c r="AB9" s="35"/>
+      <c r="AC9" s="35"/>
+      <c r="AD9" s="35"/>
+      <c r="AE9" s="35"/>
+      <c r="AF9" s="35"/>
+      <c r="AG9" s="35"/>
+      <c r="AH9" s="35"/>
+      <c r="AI9" s="35"/>
+      <c r="AJ9" s="35"/>
+      <c r="AK9" s="35"/>
+      <c r="AL9" s="35"/>
+      <c r="AM9" s="35"/>
+      <c r="AN9" s="35"/>
+      <c r="AO9" s="35"/>
+      <c r="AP9" s="35"/>
+      <c r="AQ9" s="35"/>
+      <c r="AR9" s="35"/>
+      <c r="AS9" s="35"/>
+      <c r="AT9" s="35"/>
+      <c r="AU9" s="35"/>
+      <c r="AV9" s="35"/>
+      <c r="AW9" s="35"/>
+      <c r="AX9" s="35"/>
+      <c r="AY9" s="35"/>
+      <c r="AZ9" s="35"/>
+      <c r="BA9" s="35"/>
+      <c r="BB9" s="35"/>
+      <c r="BC9" s="35"/>
+      <c r="BD9" s="35"/>
+    </row>
+    <row r="10" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
         <v>7</v>
       </c>
@@ -1188,76 +1288,76 @@
       <c r="F10" s="2">
         <v>90</v>
       </c>
-      <c r="G10" s="28" t="s">
+      <c r="G10" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="H10" s="28"/>
-      <c r="AD10" s="37" t="s">
-        <v>63</v>
-      </c>
-      <c r="AE10" s="37"/>
-      <c r="AF10" s="37"/>
-      <c r="AG10" s="37"/>
-      <c r="AH10" s="37"/>
-      <c r="AI10" s="37"/>
-      <c r="AJ10" s="37"/>
-      <c r="AK10" s="37"/>
-      <c r="AL10" s="37"/>
-      <c r="AM10" s="37"/>
+      <c r="H10" s="26"/>
+      <c r="AD10" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="AE10" s="28"/>
+      <c r="AF10" s="28"/>
+      <c r="AG10" s="28"/>
+      <c r="AH10" s="28"/>
+      <c r="AI10" s="28"/>
+      <c r="AJ10" s="28"/>
+      <c r="AK10" s="28"/>
+      <c r="AL10" s="28"/>
+      <c r="AM10" s="28"/>
       <c r="AN10" s="2"/>
-      <c r="AO10" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="AP10" s="29"/>
-      <c r="AQ10" s="29"/>
-      <c r="AR10" s="29"/>
-      <c r="AS10" s="29"/>
-      <c r="AT10" s="29"/>
-      <c r="AU10" s="29"/>
-      <c r="AV10" s="29"/>
-      <c r="AW10" s="29"/>
-      <c r="AX10" s="29"/>
-      <c r="AY10" s="29"/>
-      <c r="AZ10" s="29"/>
-      <c r="BA10" s="29"/>
-      <c r="BB10" s="29"/>
-      <c r="BC10" s="29"/>
-      <c r="BD10" s="29"/>
-    </row>
-    <row r="11" spans="2:56" x14ac:dyDescent="0.25">
-      <c r="I11" s="36" t="s">
-        <v>84</v>
+      <c r="AO10" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="AP10" s="34"/>
+      <c r="AQ10" s="34"/>
+      <c r="AR10" s="34"/>
+      <c r="AS10" s="34"/>
+      <c r="AT10" s="34"/>
+      <c r="AU10" s="34"/>
+      <c r="AV10" s="34"/>
+      <c r="AW10" s="34"/>
+      <c r="AX10" s="34"/>
+      <c r="AY10" s="34"/>
+      <c r="AZ10" s="34"/>
+      <c r="BA10" s="34"/>
+      <c r="BB10" s="34"/>
+      <c r="BC10" s="34"/>
+      <c r="BD10" s="34"/>
+    </row>
+    <row r="11" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="I11" s="27" t="s">
+        <v>83</v>
       </c>
       <c r="J11" s="8"/>
       <c r="K11" s="9"/>
-      <c r="L11" s="32" t="s">
-        <v>72</v>
-      </c>
-      <c r="M11" s="32"/>
-      <c r="N11" s="32"/>
-      <c r="O11" s="38" t="s">
+      <c r="L11" s="37" t="s">
+        <v>71</v>
+      </c>
+      <c r="M11" s="37"/>
+      <c r="N11" s="37"/>
+      <c r="O11" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="P11" s="29"/>
+      <c r="Q11" s="29"/>
+      <c r="R11" s="29"/>
+      <c r="S11" s="29"/>
+      <c r="T11" s="29"/>
+      <c r="U11" s="29"/>
+      <c r="V11" s="29"/>
+      <c r="W11" s="38" t="s">
         <v>77</v>
       </c>
-      <c r="P11" s="38"/>
-      <c r="Q11" s="38"/>
-      <c r="R11" s="38"/>
-      <c r="S11" s="38"/>
-      <c r="T11" s="38"/>
-      <c r="U11" s="38"/>
-      <c r="V11" s="38"/>
-      <c r="W11" s="33" t="s">
-        <v>78</v>
-      </c>
-      <c r="X11" s="33"/>
-      <c r="Y11" s="40" t="s">
-        <v>69</v>
-      </c>
-      <c r="Z11" s="40"/>
-      <c r="AA11" s="39" t="s">
+      <c r="X11" s="38"/>
+      <c r="Y11" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="Z11" s="31"/>
+      <c r="AA11" s="30" t="s">
         <v>46</v>
       </c>
-      <c r="AB11" s="39"/>
-      <c r="AC11" s="39"/>
+      <c r="AB11" s="30"/>
+      <c r="AC11" s="30"/>
       <c r="AD11" s="2">
         <v>1</v>
       </c>
@@ -1286,36 +1386,42 @@
         <v>9</v>
       </c>
       <c r="AM11" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="AN11" s="2"/>
-      <c r="AO11" s="28">
+      <c r="AO11" s="26">
         <v>1</v>
       </c>
-      <c r="AP11" s="28"/>
-      <c r="AQ11" s="28"/>
-      <c r="AR11" s="28"/>
-      <c r="AS11" s="28">
+      <c r="AP11" s="26"/>
+      <c r="AQ11" s="26"/>
+      <c r="AR11" s="26"/>
+      <c r="AS11" s="26">
         <v>2</v>
       </c>
-      <c r="AT11" s="28"/>
-      <c r="AU11" s="28"/>
-      <c r="AV11" s="28"/>
-      <c r="AW11" s="28">
+      <c r="AT11" s="26"/>
+      <c r="AU11" s="26"/>
+      <c r="AV11" s="26"/>
+      <c r="AW11" s="26">
         <v>3</v>
       </c>
-      <c r="AX11" s="28"/>
-      <c r="AY11" s="28"/>
-      <c r="AZ11" s="28"/>
-      <c r="BA11" s="28" t="s">
-        <v>79</v>
-      </c>
-      <c r="BB11" s="28"/>
-      <c r="BC11" s="28"/>
-      <c r="BD11" s="28"/>
-    </row>
-    <row r="12" spans="2:56" ht="60" x14ac:dyDescent="0.25">
-      <c r="I12" s="36"/>
+      <c r="AX11" s="26"/>
+      <c r="AY11" s="26"/>
+      <c r="AZ11" s="26"/>
+      <c r="BA11" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="BB11" s="26"/>
+      <c r="BC11" s="26"/>
+      <c r="BD11" s="26"/>
+      <c r="BE11" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="BF11" s="26"/>
+      <c r="BG11" s="26"/>
+      <c r="BH11" s="26"/>
+    </row>
+    <row r="12" spans="2:60" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="I12" s="27"/>
       <c r="J12" s="10" t="s">
         <v>39</v>
       </c>
@@ -1326,7 +1432,7 @@
         <v>50</v>
       </c>
       <c r="M12" s="12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="N12" s="13" t="s">
         <v>40</v>
@@ -1341,7 +1447,7 @@
         <v>43</v>
       </c>
       <c r="R12" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="S12" s="14" t="s">
         <v>44</v>
@@ -1350,24 +1456,24 @@
         <v>45</v>
       </c>
       <c r="U12" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="V12" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="W12" s="15" t="s">
         <v>51</v>
       </c>
       <c r="X12" s="15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Y12" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="Z12" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="AA12" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="AA12" s="56" t="s">
         <v>47</v>
       </c>
       <c r="AB12" s="17" t="s">
@@ -1403,52 +1509,64 @@
         <v>41</v>
       </c>
       <c r="AP12" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AQ12" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AR12" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AS12" s="7" t="s">
         <v>41</v>
       </c>
       <c r="AT12" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AU12" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AV12" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="AW12" s="7" t="s">
         <v>41</v>
       </c>
       <c r="AX12" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AY12" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="AZ12" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="BA12" s="7" t="s">
         <v>41</v>
       </c>
       <c r="BB12" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="BC12" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="BD12" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="BE12" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="BF12" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="BD12" s="6" t="s">
+      <c r="BG12" s="6" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="13" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BH12" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I13" s="2">
         <v>1</v>
       </c>
@@ -1456,12 +1574,12 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L13" s="2">
         <v>0.33300000000000002</v>
       </c>
-      <c r="M13" s="18">
+      <c r="M13" s="40">
         <f>-$C$3*(LN(1-L13)) / 1440</f>
         <v>1.265516353332854E-2</v>
       </c>
@@ -1470,27 +1588,27 @@
         <v>0.4293218301999952</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P13" s="2"/>
-      <c r="Q13" s="18"/>
+      <c r="Q13" s="40"/>
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
-      <c r="X13" s="18"/>
+      <c r="X13" s="40"/>
       <c r="Y13" s="2">
         <v>0</v>
       </c>
       <c r="Z13" s="2">
         <v>0</v>
       </c>
-      <c r="AA13" s="18">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="18">
+      <c r="AA13" s="57">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="40">
         <v>0</v>
       </c>
       <c r="AC13" s="2">
@@ -1523,15 +1641,19 @@
       <c r="BB13" s="2"/>
       <c r="BC13" s="2"/>
       <c r="BD13" s="2"/>
-    </row>
-    <row r="14" spans="2:56" x14ac:dyDescent="0.25">
-      <c r="B14" s="28" t="s">
+      <c r="BE13" s="2"/>
+      <c r="BF13" s="2"/>
+      <c r="BG13" s="2"/>
+      <c r="BH13" s="2"/>
+    </row>
+    <row r="14" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="B14" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
       <c r="I14" s="2">
         <f>I13+1</f>
         <v>2</v>
@@ -1540,12 +1662,12 @@
         <v>0.42931712962962965</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="L14" s="2">
         <v>0.55800000000000005</v>
       </c>
-      <c r="M14" s="18">
+      <c r="M14" s="40">
         <f>-$C$3*(LN(1-L14)) / 1440</f>
         <v>2.5513918653263721E-2</v>
       </c>
@@ -1554,12 +1676,12 @@
         <v>0.45483104828289339</v>
       </c>
       <c r="O14" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P14" s="2">
         <v>5.5E-2</v>
       </c>
-      <c r="Q14" s="18">
+      <c r="Q14" s="40">
         <f>($F$8+P14*($F$9-$F$8)) / 1440</f>
         <v>7.3263888888888892E-3</v>
       </c>
@@ -1572,24 +1694,24 @@
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
-      <c r="X14" s="2"/>
+      <c r="X14" s="40"/>
       <c r="Y14" s="2">
         <v>0</v>
       </c>
       <c r="Z14" s="2">
         <v>0</v>
       </c>
-      <c r="AA14" s="18">
-        <v>0</v>
-      </c>
-      <c r="AB14" s="18">
+      <c r="AA14" s="57">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="40">
         <v>0</v>
       </c>
       <c r="AC14" s="2">
         <v>0</v>
       </c>
       <c r="AD14" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AE14" s="2"/>
       <c r="AF14" s="2"/>
@@ -1617,8 +1739,12 @@
       <c r="BB14" s="2"/>
       <c r="BC14" s="2"/>
       <c r="BD14" s="2"/>
-    </row>
-    <row r="15" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BE14" s="2"/>
+      <c r="BF14" s="2"/>
+      <c r="BG14" s="2"/>
+      <c r="BH14" s="2"/>
+    </row>
+    <row r="15" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B15" s="2" t="s">
         <v>24</v>
       </c>
@@ -1642,35 +1768,35 @@
         <f>R14</f>
         <v>0.43664351851851851</v>
       </c>
-      <c r="K15" s="2" t="s">
-        <v>93</v>
+      <c r="K15" s="47" t="s">
+        <v>92</v>
       </c>
       <c r="L15" s="7"/>
-      <c r="M15" s="20"/>
+      <c r="M15" s="41"/>
       <c r="N15" s="18">
         <f>N14</f>
         <v>0.45483104828289339</v>
       </c>
       <c r="O15" s="18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P15" s="20"/>
-      <c r="Q15" s="20"/>
+      <c r="Q15" s="41"/>
       <c r="R15" s="20"/>
       <c r="S15" s="2">
         <v>0.35499999999999998</v>
       </c>
       <c r="T15" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="U15" s="1"/>
       <c r="V15" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="W15" s="2">
         <v>0.187</v>
       </c>
-      <c r="X15" s="19">
+      <c r="X15" s="44">
         <f>-90*LN(1-W15) / 1440</f>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -1680,11 +1806,11 @@
       <c r="Z15" s="2">
         <v>0</v>
       </c>
-      <c r="AA15" s="18">
+      <c r="AA15" s="57">
         <f>Q14</f>
         <v>7.3263888888888892E-3</v>
       </c>
-      <c r="AB15" s="18">
+      <c r="AB15" s="40">
         <v>0</v>
       </c>
       <c r="AC15" s="2">
@@ -1702,7 +1828,7 @@
       <c r="AM15" s="2"/>
       <c r="AN15" s="2"/>
       <c r="AO15" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AP15" s="18">
         <f>J15</f>
@@ -1722,8 +1848,12 @@
       <c r="BB15" s="2"/>
       <c r="BC15" s="2"/>
       <c r="BD15" s="2"/>
-    </row>
-    <row r="16" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BE15" s="2"/>
+      <c r="BF15" s="2"/>
+      <c r="BG15" s="2"/>
+      <c r="BH15" s="2"/>
+    </row>
+    <row r="16" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B16" s="2" t="s">
         <v>19</v>
       </c>
@@ -1748,37 +1878,37 @@
         <v>0.44958252910816393</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L16" s="1"/>
-      <c r="M16" s="22"/>
+      <c r="M16" s="42"/>
       <c r="N16" s="19">
         <f>N15</f>
         <v>0.45483104828289339</v>
       </c>
       <c r="O16" s="18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="P16" s="22"/>
-      <c r="Q16" s="22"/>
+      <c r="Q16" s="42"/>
       <c r="R16" s="22"/>
       <c r="S16" s="22"/>
       <c r="T16" s="22"/>
       <c r="U16" s="22"/>
       <c r="V16" s="22"/>
       <c r="W16" s="22"/>
-      <c r="X16" s="18"/>
+      <c r="X16" s="40"/>
       <c r="Y16" s="2">
         <v>0</v>
       </c>
       <c r="Z16" s="2">
         <v>0</v>
       </c>
-      <c r="AA16" s="18">
+      <c r="AA16" s="57">
         <f>AA15</f>
         <v>7.3263888888888892E-3</v>
       </c>
-      <c r="AB16" s="18">
+      <c r="AB16" s="40">
         <f>AB15+X15</f>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -1821,8 +1951,12 @@
       <c r="BB16" s="2"/>
       <c r="BC16" s="2"/>
       <c r="BD16" s="2"/>
-    </row>
-    <row r="17" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BE16" s="2"/>
+      <c r="BF16" s="2"/>
+      <c r="BG16" s="2"/>
+      <c r="BH16" s="2"/>
+    </row>
+    <row r="17" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B17" s="2" t="s">
         <v>20</v>
       </c>
@@ -1847,12 +1981,12 @@
         <v>0.45483104828289339</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L17" s="2">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="M17" s="18">
+      <c r="M17" s="40">
         <f>-$C$3*LN(1-L17) / 1440</f>
         <v>9.3890906884335122E-5</v>
       </c>
@@ -1861,12 +1995,12 @@
         <v>0.45492493918977772</v>
       </c>
       <c r="O17" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P17" s="2">
         <v>0.35799999999999998</v>
       </c>
-      <c r="Q17" s="18">
+      <c r="Q17" s="40">
         <f>($F$8+P17*($F$9-$F$8)) / 1440</f>
         <v>9.4305555555555549E-3</v>
       </c>
@@ -1879,19 +2013,19 @@
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
       <c r="W17" s="2"/>
-      <c r="X17" s="2"/>
+      <c r="X17" s="40"/>
       <c r="Y17" s="2">
         <v>0</v>
       </c>
       <c r="Z17" s="2">
         <v>0</v>
       </c>
-      <c r="AA17" s="18">
+      <c r="AA17" s="57">
         <f>AA16+Q18</f>
         <v>1.6756944444444442E-2</v>
       </c>
-      <c r="AB17" s="18">
-        <f t="shared" ref="AB17:AB22" si="1">AB16</f>
+      <c r="AB17" s="40">
+        <f t="shared" ref="AB17:AB24" si="1">AB16</f>
         <v>1.2939010589645406E-2</v>
       </c>
       <c r="AC17" s="2">
@@ -1899,7 +2033,7 @@
       </c>
       <c r="AD17" s="2"/>
       <c r="AE17" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AF17" s="2"/>
       <c r="AG17" s="2"/>
@@ -1926,8 +2060,12 @@
       <c r="BB17" s="2"/>
       <c r="BC17" s="2"/>
       <c r="BD17" s="2"/>
-    </row>
-    <row r="18" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BE17" s="2"/>
+      <c r="BF17" s="2"/>
+      <c r="BG17" s="2"/>
+      <c r="BH17" s="2"/>
+    </row>
+    <row r="18" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I18" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1937,12 +2075,12 @@
         <v>0.45492493918977772</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L18" s="2">
         <v>0.44</v>
       </c>
-      <c r="M18" s="18">
+      <c r="M18" s="40">
         <f>-$C$3*LN(1-L18) / 1440</f>
         <v>1.8119327976654439E-2</v>
       </c>
@@ -1951,10 +2089,10 @@
         <v>0.47304426716643216</v>
       </c>
       <c r="O18" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P18" s="1"/>
-      <c r="Q18" s="18">
+      <c r="Q18" s="40">
         <f>Q17</f>
         <v>9.4305555555555549E-3</v>
       </c>
@@ -1967,18 +2105,18 @@
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
       <c r="W18" s="2"/>
-      <c r="X18" s="2"/>
+      <c r="X18" s="40"/>
       <c r="Y18" s="2">
         <v>1</v>
       </c>
       <c r="Z18" s="2">
         <v>0</v>
       </c>
-      <c r="AA18" s="18">
+      <c r="AA18" s="57">
         <f>AA17+(J18-J17)</f>
         <v>1.6850835351328773E-2</v>
       </c>
-      <c r="AB18" s="18">
+      <c r="AB18" s="40">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -1987,10 +2125,10 @@
       </c>
       <c r="AD18" s="2"/>
       <c r="AE18" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AF18" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AG18" s="2"/>
       <c r="AH18" s="2"/>
@@ -2016,15 +2154,19 @@
       <c r="BB18" s="2"/>
       <c r="BC18" s="2"/>
       <c r="BD18" s="2"/>
-    </row>
-    <row r="19" spans="2:56" x14ac:dyDescent="0.25">
-      <c r="B19" s="28" t="s">
+      <c r="BE18" s="2"/>
+      <c r="BF18" s="2"/>
+      <c r="BG18" s="2"/>
+      <c r="BH18" s="2"/>
+    </row>
+    <row r="19" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="B19" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
       <c r="I19" s="2">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2033,22 +2175,22 @@
         <f>R17</f>
         <v>0.46426160383844894</v>
       </c>
-      <c r="K19" s="2" t="s">
-        <v>97</v>
+      <c r="K19" s="47" t="s">
+        <v>96</v>
       </c>
       <c r="L19" s="1"/>
-      <c r="M19" s="22"/>
+      <c r="M19" s="42"/>
       <c r="N19" s="24">
         <f>N18</f>
         <v>0.47304426716643216</v>
       </c>
       <c r="O19" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P19" s="2">
         <v>0.61399999999999999</v>
       </c>
-      <c r="Q19" s="18">
+      <c r="Q19" s="40">
         <f>($F$8+P19*($F$9-$F$8)) / 1440</f>
         <v>1.1208333333333334E-2</v>
       </c>
@@ -2060,25 +2202,25 @@
         <v>0.34499999999999997</v>
       </c>
       <c r="T19" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="U19" s="1"/>
       <c r="V19" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="W19" s="2"/>
-      <c r="X19" s="18"/>
+      <c r="X19" s="40"/>
       <c r="Y19" s="2">
         <v>0</v>
       </c>
       <c r="Z19" s="2">
         <v>1</v>
       </c>
-      <c r="AA19" s="18">
+      <c r="AA19" s="57">
         <f>AA18+Q17</f>
         <v>2.6281390906884326E-2</v>
       </c>
-      <c r="AB19" s="18">
+      <c r="AB19" s="40">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2088,7 +2230,7 @@
       <c r="AD19" s="2"/>
       <c r="AE19" s="21"/>
       <c r="AF19" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AG19" s="2"/>
       <c r="AH19" s="2"/>
@@ -2103,7 +2245,7 @@
       <c r="AQ19" s="2"/>
       <c r="AR19" s="2"/>
       <c r="AS19" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AT19" s="18">
         <f>J19</f>
@@ -2119,8 +2261,12 @@
       <c r="BB19" s="2"/>
       <c r="BC19" s="2"/>
       <c r="BD19" s="2"/>
-    </row>
-    <row r="20" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BE19" s="2"/>
+      <c r="BF19" s="2"/>
+      <c r="BG19" s="2"/>
+      <c r="BH19" s="2"/>
+    </row>
+    <row r="20" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B20" s="2" t="s">
         <v>24</v>
       </c>
@@ -2145,12 +2291,12 @@
         <v>0.47304426716643216</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L20" s="2">
         <v>0.22500000000000001</v>
       </c>
-      <c r="M20" s="18">
+      <c r="M20" s="40">
         <f>-$C$3*LN(1-L20) / 1440</f>
         <v>7.9653828008996886E-3</v>
       </c>
@@ -2159,10 +2305,10 @@
         <v>0.48100964996733186</v>
       </c>
       <c r="O20" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P20" s="2"/>
-      <c r="Q20" s="18">
+      <c r="Q20" s="40">
         <f>Q19</f>
         <v>1.1208333333333334E-2</v>
       </c>
@@ -2175,18 +2321,18 @@
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
       <c r="W20" s="1"/>
-      <c r="X20" s="25"/>
+      <c r="X20" s="45"/>
       <c r="Y20" s="2">
         <v>1</v>
       </c>
       <c r="Z20" s="2">
         <v>1</v>
       </c>
-      <c r="AA20" s="18">
+      <c r="AA20" s="57">
         <f>AA19+Q18</f>
         <v>3.5711946462439879E-2</v>
       </c>
-      <c r="AB20" s="18">
+      <c r="AB20" s="40">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2196,10 +2342,10 @@
       <c r="AD20" s="2"/>
       <c r="AE20" s="2"/>
       <c r="AF20" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AG20" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AH20" s="2"/>
       <c r="AI20" s="2"/>
@@ -2213,7 +2359,7 @@
       <c r="AQ20" s="2"/>
       <c r="AR20" s="2"/>
       <c r="AS20" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AT20" s="18">
         <f>AT19</f>
@@ -2229,10 +2375,14 @@
       <c r="BB20" s="2"/>
       <c r="BC20" s="2"/>
       <c r="BD20" s="2"/>
-    </row>
-    <row r="21" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BE20" s="2"/>
+      <c r="BF20" s="2"/>
+      <c r="BG20" s="2"/>
+      <c r="BH20" s="2"/>
+    </row>
+    <row r="21" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B21" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C21" s="2">
         <v>0.5</v>
@@ -2257,22 +2407,22 @@
         <f>R20</f>
         <v>0.47546993717178226</v>
       </c>
-      <c r="K21" s="2" t="s">
-        <v>99</v>
+      <c r="K21" s="47" t="s">
+        <v>98</v>
       </c>
       <c r="L21" s="2"/>
-      <c r="M21" s="18"/>
+      <c r="M21" s="40"/>
       <c r="N21" s="19">
         <f>N20</f>
         <v>0.48100964996733186</v>
       </c>
       <c r="O21" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P21" s="2">
         <v>0.26900000000000002</v>
       </c>
-      <c r="Q21" s="18">
+      <c r="Q21" s="40">
         <f>($F$8+P21*($F$9-$F$8)) / 1440</f>
         <v>8.8125000000000009E-3</v>
       </c>
@@ -2284,25 +2434,25 @@
         <v>0.35299999999999998</v>
       </c>
       <c r="T21" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="U21" s="2"/>
       <c r="V21" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="W21" s="2"/>
-      <c r="X21" s="18"/>
+      <c r="X21" s="40"/>
       <c r="Y21" s="2">
         <v>0</v>
       </c>
       <c r="Z21" s="2">
         <v>2</v>
       </c>
-      <c r="AA21" s="18">
+      <c r="AA21" s="57">
         <f>AA20+(J21-J20)</f>
         <v>3.813761646778998E-2</v>
       </c>
-      <c r="AB21" s="18">
+      <c r="AB21" s="40">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2313,7 +2463,7 @@
       <c r="AE21" s="2"/>
       <c r="AF21" s="21"/>
       <c r="AG21" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AH21" s="2"/>
       <c r="AI21" s="2"/>
@@ -2327,7 +2477,7 @@
       <c r="AQ21" s="2"/>
       <c r="AR21" s="2"/>
       <c r="AS21" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AT21" s="18">
         <f t="shared" ref="AT21:AT22" si="2">AT20</f>
@@ -2336,7 +2486,7 @@
       <c r="AU21" s="2"/>
       <c r="AV21" s="2"/>
       <c r="AW21" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AX21" s="18">
         <f>J21</f>
@@ -2348,10 +2498,14 @@
       <c r="BB21" s="2"/>
       <c r="BC21" s="2"/>
       <c r="BD21" s="2"/>
-    </row>
-    <row r="22" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BE21" s="2"/>
+      <c r="BF21" s="2"/>
+      <c r="BG21" s="2"/>
+      <c r="BH21" s="2"/>
+    </row>
+    <row r="22" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B22" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C22" s="2">
         <v>0.5</v>
@@ -2374,12 +2528,12 @@
         <v>0.48100964996733186</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L22" s="2">
         <v>0.57099999999999995</v>
       </c>
-      <c r="M22" s="18">
+      <c r="M22" s="40">
         <f>-$C$3*LN(1-L22) / 1440</f>
         <v>2.6446823751691249E-2</v>
       </c>
@@ -2388,10 +2542,10 @@
         <v>0.50745647371902314</v>
       </c>
       <c r="O22" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P22" s="2"/>
-      <c r="Q22" s="18">
+      <c r="Q22" s="40">
         <f>Q21</f>
         <v>8.8125000000000009E-3</v>
       </c>
@@ -2404,18 +2558,18 @@
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
       <c r="W22" s="2"/>
-      <c r="X22" s="18"/>
+      <c r="X22" s="40"/>
       <c r="Y22" s="2">
         <v>1</v>
       </c>
       <c r="Z22" s="2">
         <v>2</v>
       </c>
-      <c r="AA22" s="18">
+      <c r="AA22" s="57">
         <f>AA21++J22-J21</f>
         <v>4.3677329263339615E-2</v>
       </c>
-      <c r="AB22" s="18">
+      <c r="AB22" s="40">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2426,10 +2580,10 @@
       <c r="AE22" s="2"/>
       <c r="AF22" s="2"/>
       <c r="AG22" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AH22" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AI22" s="2"/>
       <c r="AJ22" s="2"/>
@@ -2442,7 +2596,7 @@
       <c r="AQ22" s="2"/>
       <c r="AR22" s="2"/>
       <c r="AS22" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AT22" s="18">
         <f t="shared" si="2"/>
@@ -2451,7 +2605,7 @@
       <c r="AU22" s="2"/>
       <c r="AV22" s="2"/>
       <c r="AW22" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AX22" s="18">
         <f>AX21</f>
@@ -2463,8 +2617,12 @@
       <c r="BB22" s="2"/>
       <c r="BC22" s="2"/>
       <c r="BD22" s="2"/>
-    </row>
-    <row r="23" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BE22" s="2"/>
+      <c r="BF22" s="2"/>
+      <c r="BG22" s="2"/>
+      <c r="BH22" s="2"/>
+    </row>
+    <row r="23" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I23" s="2">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2473,22 +2631,22 @@
         <f>R22</f>
         <v>0.48428243717178227</v>
       </c>
-      <c r="K23" s="42" t="s">
-        <v>102</v>
+      <c r="K23" s="47" t="s">
+        <v>101</v>
       </c>
       <c r="L23" s="2"/>
-      <c r="M23" s="18"/>
+      <c r="M23" s="40"/>
       <c r="N23" s="18">
         <f>N22</f>
         <v>0.50745647371902314</v>
       </c>
-      <c r="O23" s="43" t="s">
-        <v>62</v>
+      <c r="O23" s="18" t="s">
+        <v>61</v>
       </c>
       <c r="P23" s="2">
         <v>0.81699999999999995</v>
       </c>
-      <c r="Q23" s="18">
+      <c r="Q23" s="40">
         <f>($F$8+P23*($F$9-$F$8)) / 1440</f>
         <v>1.2618055555555556E-2</v>
       </c>
@@ -2500,31 +2658,38 @@
         <v>0.125</v>
       </c>
       <c r="T23" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="U23" s="2">
         <v>0.34100000000000003</v>
       </c>
       <c r="V23" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="W23" s="2"/>
-      <c r="X23" s="2"/>
-      <c r="Y23" s="42">
-        <v>0</v>
-      </c>
-      <c r="Z23" s="42">
+      <c r="X23" s="40"/>
+      <c r="Y23" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="2">
         <v>2</v>
       </c>
-      <c r="AA23" t="s">
-        <v>101</v>
+      <c r="AA23" s="43" t="s">
+        <v>100</v>
+      </c>
+      <c r="AB23" s="40">
+        <f t="shared" si="1"/>
+        <v>1.2939010589645406E-2</v>
+      </c>
+      <c r="AC23" s="52">
+        <v>0</v>
       </c>
       <c r="AD23" s="2"/>
       <c r="AE23" s="2"/>
       <c r="AF23" s="2"/>
       <c r="AG23" s="21"/>
       <c r="AH23" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AI23" s="2"/>
       <c r="AJ23" s="2"/>
@@ -2536,8 +2701,8 @@
       <c r="AP23" s="2"/>
       <c r="AQ23" s="2"/>
       <c r="AR23" s="2"/>
-      <c r="AS23" s="42" t="s">
-        <v>88</v>
+      <c r="AS23" s="2" t="s">
+        <v>87</v>
       </c>
       <c r="AT23" s="18">
         <f>AT22</f>
@@ -2546,7 +2711,7 @@
       <c r="AU23" s="2"/>
       <c r="AV23" s="2"/>
       <c r="AW23" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AX23" s="18">
         <f>AX22</f>
@@ -2554,15 +2719,23 @@
       </c>
       <c r="AY23" s="2"/>
       <c r="AZ23" s="2"/>
-    </row>
-    <row r="24" spans="2:56" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="35" t="s">
+      <c r="BA23" s="2"/>
+      <c r="BB23" s="2"/>
+      <c r="BC23" s="2"/>
+      <c r="BD23" s="2"/>
+      <c r="BE23" s="2"/>
+      <c r="BF23" s="2"/>
+      <c r="BG23" s="2"/>
+      <c r="BH23" s="2"/>
+    </row>
+    <row r="24" spans="2:60" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
       <c r="I24" s="2">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2571,63 +2744,71 @@
         <f>R23</f>
         <v>0.49690049272733783</v>
       </c>
-      <c r="K24" s="42" t="s">
-        <v>105</v>
+      <c r="K24" s="47" t="s">
+        <v>104</v>
       </c>
       <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
+      <c r="M24" s="40"/>
       <c r="N24" s="18">
         <f>N23</f>
         <v>0.50745647371902314</v>
       </c>
-      <c r="O24" s="43" t="s">
-        <v>61</v>
+      <c r="O24" s="18" t="s">
+        <v>60</v>
       </c>
       <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
+      <c r="Q24" s="40"/>
       <c r="R24" s="2"/>
       <c r="S24" s="2">
         <v>4.3999999999999997E-2</v>
       </c>
       <c r="T24" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="U24" s="2">
         <v>0.122</v>
       </c>
       <c r="V24" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="W24" s="2">
         <v>5.5E-2</v>
       </c>
-      <c r="X24" s="19">
+      <c r="X24" s="44">
         <f>-90*LN(1-W24) / 1440</f>
         <v>3.5356469680246473E-3</v>
       </c>
-      <c r="Y24" s="42">
-        <v>0</v>
-      </c>
-      <c r="Z24" s="42">
+      <c r="Y24" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z24" s="2">
         <v>1</v>
+      </c>
+      <c r="AA24" s="43"/>
+      <c r="AB24" s="40">
+        <f t="shared" si="1"/>
+        <v>1.2939010589645406E-2</v>
+      </c>
+      <c r="AC24" s="52">
+        <v>0</v>
       </c>
       <c r="AD24" s="2"/>
       <c r="AE24" s="2"/>
       <c r="AF24" s="2"/>
       <c r="AG24" s="2"/>
       <c r="AH24" s="21"/>
-      <c r="AI24" s="42"/>
-      <c r="AJ24" s="42"/>
-      <c r="AK24" s="42"/>
-      <c r="AL24" s="42"/>
+      <c r="AI24" s="2"/>
+      <c r="AJ24" s="2"/>
+      <c r="AK24" s="2"/>
+      <c r="AL24" s="2"/>
       <c r="AM24" s="2"/>
       <c r="AN24" s="2"/>
       <c r="AO24" s="2"/>
       <c r="AP24" s="2"/>
       <c r="AQ24" s="2"/>
       <c r="AR24" s="2"/>
-      <c r="AS24" s="42" t="s">
-        <v>91</v>
+      <c r="AS24" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="AT24" s="18">
         <f>AT23</f>
@@ -2638,7 +2819,7 @@
       </c>
       <c r="AV24" s="18"/>
       <c r="AW24" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AX24" s="18">
         <f t="shared" ref="AX24:AX28" si="3">AX23</f>
@@ -2646,13 +2827,21 @@
       </c>
       <c r="AY24" s="2"/>
       <c r="AZ24" s="2"/>
-    </row>
-    <row r="25" spans="2:56" x14ac:dyDescent="0.25">
-      <c r="B25" s="35"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="35"/>
-      <c r="E25" s="35"/>
-      <c r="F25" s="35"/>
+      <c r="BA24" s="2"/>
+      <c r="BB24" s="2"/>
+      <c r="BC24" s="2"/>
+      <c r="BD24" s="2"/>
+      <c r="BE24" s="2"/>
+      <c r="BF24" s="2"/>
+      <c r="BG24" s="2"/>
+      <c r="BH24" s="2"/>
+    </row>
+    <row r="25" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
       <c r="I25" s="2">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2661,20 +2850,20 @@
         <f>J24+X24</f>
         <v>0.50043613969536249</v>
       </c>
-      <c r="K25" s="42" t="s">
-        <v>106</v>
+      <c r="K25" s="2" t="s">
+        <v>105</v>
       </c>
       <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
+      <c r="M25" s="40"/>
       <c r="N25" s="19">
         <f>N24</f>
         <v>0.50745647371902314</v>
       </c>
-      <c r="O25" s="43" t="s">
-        <v>61</v>
+      <c r="O25" s="18" t="s">
+        <v>60</v>
       </c>
       <c r="P25" s="2"/>
-      <c r="Q25" s="2"/>
+      <c r="Q25" s="40"/>
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
       <c r="T25" s="2"/>
@@ -2683,14 +2872,22 @@
       <c r="W25" s="2">
         <v>0.20899999999999999</v>
       </c>
-      <c r="X25" s="41">
+      <c r="X25" s="46">
         <f>-90*LN(1-W25) / 1440</f>
         <v>1.4653581950905195E-2</v>
       </c>
-      <c r="Y25" s="42">
-        <v>0</v>
-      </c>
-      <c r="Z25" s="42">
+      <c r="Y25" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z25" s="2">
+        <v>0</v>
+      </c>
+      <c r="AA25" s="43"/>
+      <c r="AB25" s="43">
+        <f>AB24+X24</f>
+        <v>1.6474657557670053E-2</v>
+      </c>
+      <c r="AC25" s="52">
         <v>0</v>
       </c>
       <c r="AD25" s="2"/>
@@ -2721,7 +2918,7 @@
         <v>3.5300925925925925E-3</v>
       </c>
       <c r="AW25" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AX25" s="18">
         <f t="shared" si="3"/>
@@ -2729,8 +2926,16 @@
       </c>
       <c r="AY25" s="2"/>
       <c r="AZ25" s="2"/>
-    </row>
-    <row r="26" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BA25" s="2"/>
+      <c r="BB25" s="2"/>
+      <c r="BC25" s="2"/>
+      <c r="BD25" s="2"/>
+      <c r="BE25" s="2"/>
+      <c r="BF25" s="2"/>
+      <c r="BG25" s="2"/>
+      <c r="BH25" s="2"/>
+    </row>
+    <row r="26" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I26" s="2">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2738,13 +2943,13 @@
       <c r="J26" s="18">
         <v>0.50745370370370368</v>
       </c>
-      <c r="K26" s="42" t="s">
-        <v>107</v>
+      <c r="K26" s="2" t="s">
+        <v>106</v>
       </c>
       <c r="L26" s="2">
         <v>0.9</v>
       </c>
-      <c r="M26" s="18">
+      <c r="M26" s="40">
         <f>-$C$3*LN(1-L26) / 1440</f>
         <v>7.1955784156063934E-2</v>
       </c>
@@ -2752,13 +2957,13 @@
         <f>M26++J26</f>
         <v>0.57940948785976765</v>
       </c>
-      <c r="O26" s="43" t="s">
-        <v>62</v>
+      <c r="O26" s="18" t="s">
+        <v>61</v>
       </c>
       <c r="P26" s="2">
         <v>0.89300000000000002</v>
       </c>
-      <c r="Q26" s="18">
+      <c r="Q26" s="40">
         <f>($F$8+P26*($F$9-$F$8)) / 1440</f>
         <v>1.3145833333333332E-2</v>
       </c>
@@ -2771,7 +2976,7 @@
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
       <c r="W26" s="2"/>
-      <c r="X26" s="41">
+      <c r="X26" s="46">
         <f>AZ26</f>
         <v>7.6332479272445495E-3</v>
       </c>
@@ -2780,6 +2985,14 @@
       </c>
       <c r="Z26" s="2">
         <v>1</v>
+      </c>
+      <c r="AA26" s="43"/>
+      <c r="AB26" s="43">
+        <f>AB25</f>
+        <v>1.6474657557670053E-2</v>
+      </c>
+      <c r="AC26" s="52">
+        <v>0</v>
       </c>
       <c r="AD26" s="2"/>
       <c r="AE26" s="2"/>
@@ -2787,7 +3000,7 @@
       <c r="AG26" s="2"/>
       <c r="AH26" s="2"/>
       <c r="AI26" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AJ26" s="2"/>
       <c r="AK26" s="2"/>
@@ -2803,7 +3016,7 @@
       <c r="AU26" s="23"/>
       <c r="AV26" s="23"/>
       <c r="AW26" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="AX26" s="18">
         <f t="shared" si="3"/>
@@ -2814,8 +3027,16 @@
         <f>X25-(N25-J25)</f>
         <v>7.6332479272445495E-3</v>
       </c>
-    </row>
-    <row r="27" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BA26" s="2"/>
+      <c r="BB26" s="2"/>
+      <c r="BC26" s="2"/>
+      <c r="BD26" s="2"/>
+      <c r="BE26" s="2"/>
+      <c r="BF26" s="2"/>
+      <c r="BG26" s="2"/>
+      <c r="BH26" s="2"/>
+    </row>
+    <row r="27" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I27" s="2">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -2824,40 +3045,48 @@
         <f>R26</f>
         <v>0.52059953703703699</v>
       </c>
-      <c r="K27" s="42" t="s">
-        <v>108</v>
+      <c r="K27" s="47" t="s">
+        <v>107</v>
       </c>
       <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
+      <c r="M27" s="40"/>
       <c r="N27" s="18">
         <f>N26</f>
         <v>0.57940948785976765</v>
       </c>
-      <c r="O27" s="43" t="s">
-        <v>61</v>
+      <c r="O27" s="18" t="s">
+        <v>60</v>
       </c>
       <c r="P27" s="2"/>
-      <c r="Q27" s="2"/>
+      <c r="Q27" s="40"/>
       <c r="R27" s="2"/>
       <c r="S27" s="2">
         <v>0.89900000000000002</v>
       </c>
       <c r="T27" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="U27" s="2"/>
       <c r="V27" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="W27" s="2"/>
-      <c r="X27" s="19">
+      <c r="X27" s="44">
         <f>X26</f>
         <v>7.6332479272445495E-3</v>
       </c>
-      <c r="Y27" s="42">
-        <v>0</v>
-      </c>
-      <c r="Z27" s="42">
+      <c r="Y27" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z27" s="2">
+        <v>0</v>
+      </c>
+      <c r="AA27" s="43"/>
+      <c r="AB27" s="43">
+        <f>AB26</f>
+        <v>1.6474657557670053E-2</v>
+      </c>
+      <c r="AC27" s="52">
         <v>0</v>
       </c>
       <c r="AD27" s="2"/>
@@ -2866,9 +3095,9 @@
       <c r="AG27" s="2"/>
       <c r="AH27" s="2"/>
       <c r="AI27" s="21"/>
-      <c r="AJ27" s="42"/>
-      <c r="AK27" s="42"/>
-      <c r="AL27" s="42"/>
+      <c r="AJ27" s="2"/>
+      <c r="AK27" s="2"/>
+      <c r="AL27" s="2"/>
       <c r="AM27" s="2"/>
       <c r="AN27" s="2"/>
       <c r="AO27" s="2"/>
@@ -2880,7 +3109,7 @@
       <c r="AU27" s="2"/>
       <c r="AV27" s="2"/>
       <c r="AW27" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="AX27" s="18">
         <f t="shared" si="3"/>
@@ -2891,8 +3120,16 @@
         <f>AZ26</f>
         <v>7.6332479272445495E-3</v>
       </c>
-    </row>
-    <row r="28" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BA27" s="2"/>
+      <c r="BB27" s="2"/>
+      <c r="BC27" s="2"/>
+      <c r="BD27" s="2"/>
+      <c r="BE27" s="2"/>
+      <c r="BF27" s="2"/>
+      <c r="BG27" s="2"/>
+      <c r="BH27" s="2"/>
+    </row>
+    <row r="28" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I28" s="2">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -2901,31 +3138,39 @@
         <f>J27+X27</f>
         <v>0.5282327849642815</v>
       </c>
-      <c r="K28" s="42" t="s">
-        <v>109</v>
+      <c r="K28" s="48" t="s">
+        <v>108</v>
       </c>
       <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
+      <c r="M28" s="40"/>
       <c r="N28" s="19">
         <f>N27</f>
         <v>0.57940948785976765</v>
       </c>
-      <c r="O28" s="43" t="s">
-        <v>54</v>
+      <c r="O28" s="18" t="s">
+        <v>53</v>
       </c>
       <c r="P28" s="2"/>
-      <c r="Q28" s="2"/>
+      <c r="Q28" s="40"/>
       <c r="R28" s="2"/>
       <c r="S28" s="2"/>
       <c r="T28" s="2"/>
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
       <c r="W28" s="2"/>
-      <c r="X28" s="2"/>
-      <c r="Y28" s="42">
-        <v>0</v>
-      </c>
-      <c r="Z28" s="42">
+      <c r="X28" s="40"/>
+      <c r="Y28" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z28" s="2">
+        <v>0</v>
+      </c>
+      <c r="AA28" s="43"/>
+      <c r="AB28" s="43">
+        <f>X25+AB27</f>
+        <v>3.1128239508575246E-2</v>
+      </c>
+      <c r="AC28" s="52">
         <v>0</v>
       </c>
       <c r="AD28" s="2"/>
@@ -2959,8 +3204,16 @@
         <f>AZ27</f>
         <v>7.6332479272445495E-3</v>
       </c>
-    </row>
-    <row r="29" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BA28" s="2"/>
+      <c r="BB28" s="2"/>
+      <c r="BC28" s="2"/>
+      <c r="BD28" s="2"/>
+      <c r="BE28" s="2"/>
+      <c r="BF28" s="2"/>
+      <c r="BG28" s="2"/>
+      <c r="BH28" s="2"/>
+    </row>
+    <row r="29" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I29" s="2">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -2969,13 +3222,13 @@
         <f>N28</f>
         <v>0.57940948785976765</v>
       </c>
-      <c r="K29" s="42" t="s">
-        <v>110</v>
+      <c r="K29" s="2" t="s">
+        <v>109</v>
       </c>
       <c r="L29" s="2">
         <v>0.87</v>
       </c>
-      <c r="M29" s="18">
+      <c r="M29" s="40">
         <f>-$C$3*LN(1-L29) / 1440</f>
         <v>6.3756900891454832E-2</v>
       </c>
@@ -2983,13 +3236,13 @@
         <f>M29++J29</f>
         <v>0.64316638875122245</v>
       </c>
-      <c r="O29" s="43" t="s">
-        <v>62</v>
+      <c r="O29" s="18" t="s">
+        <v>61</v>
       </c>
       <c r="P29" s="2">
         <v>0.93</v>
       </c>
-      <c r="Q29" s="18">
+      <c r="Q29" s="40">
         <f>($F$8+P29*($F$9-$F$8)) / 1440</f>
         <v>1.3402777777777779E-2</v>
       </c>
@@ -3002,11 +3255,19 @@
       <c r="U29" s="2"/>
       <c r="V29" s="2"/>
       <c r="W29" s="2"/>
-      <c r="X29" s="2"/>
-      <c r="Y29" s="42">
-        <v>0</v>
-      </c>
-      <c r="Z29" s="42">
+      <c r="X29" s="40"/>
+      <c r="Y29" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="2">
+        <v>0</v>
+      </c>
+      <c r="AA29" s="43"/>
+      <c r="AB29" s="43">
+        <f>AB28</f>
+        <v>3.1128239508575246E-2</v>
+      </c>
+      <c r="AC29" s="52">
         <v>0</v>
       </c>
       <c r="AD29" s="2"/>
@@ -3016,7 +3277,7 @@
       <c r="AH29" s="2"/>
       <c r="AI29" s="2"/>
       <c r="AJ29" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="AK29" s="2"/>
       <c r="AL29" s="2"/>
@@ -3034,38 +3295,82 @@
       <c r="AX29" s="23"/>
       <c r="AY29" s="23"/>
       <c r="AZ29" s="23"/>
-    </row>
-    <row r="30" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BA29" s="2"/>
+      <c r="BB29" s="2"/>
+      <c r="BC29" s="2"/>
+      <c r="BD29" s="2"/>
+      <c r="BE29" s="2"/>
+      <c r="BF29" s="2"/>
+      <c r="BG29" s="2"/>
+      <c r="BH29" s="2"/>
+    </row>
+    <row r="30" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I30" s="2">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="J30" s="18"/>
-      <c r="K30" s="42"/>
+      <c r="J30" s="51">
+        <f>R29</f>
+        <v>0.59281226563754541</v>
+      </c>
+      <c r="K30" s="47" t="s">
+        <v>110</v>
+      </c>
       <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2"/>
+      <c r="M30" s="40"/>
+      <c r="N30" s="19">
+        <f>N29</f>
+        <v>0.64316638875122245</v>
+      </c>
+      <c r="O30" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="P30" s="2"/>
-      <c r="Q30" s="2"/>
-      <c r="R30" s="2"/>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2"/>
-      <c r="U30" s="2"/>
-      <c r="V30" s="2"/>
-      <c r="W30" s="2"/>
-      <c r="X30" s="2"/>
-      <c r="Y30" s="2"/>
-      <c r="Z30" s="2"/>
+      <c r="Q30" s="40"/>
+      <c r="R30" s="18"/>
+      <c r="S30" s="2">
+        <v>0.23300000000000001</v>
+      </c>
+      <c r="T30" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="U30" s="2">
+        <v>0.81200000000000006</v>
+      </c>
+      <c r="V30" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="W30" s="2">
+        <f>0.882</f>
+        <v>0.88200000000000001</v>
+      </c>
+      <c r="X30" s="40">
+        <f>-90*LN(1-W30) / 1440</f>
+        <v>0.13356691590727951</v>
+      </c>
+      <c r="Y30" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="2">
+        <v>0</v>
+      </c>
+      <c r="AA30" s="43"/>
+      <c r="AB30" s="43">
+        <f t="shared" ref="AB30:AB36" si="4">AB29</f>
+        <v>3.1128239508575246E-2</v>
+      </c>
+      <c r="AC30" s="52">
+        <v>0</v>
+      </c>
       <c r="AD30" s="2"/>
       <c r="AE30" s="2"/>
       <c r="AF30" s="2"/>
       <c r="AG30" s="2"/>
       <c r="AH30" s="2"/>
       <c r="AI30" s="2"/>
-      <c r="AJ30" s="42"/>
-      <c r="AK30" s="42"/>
-      <c r="AL30" s="42"/>
+      <c r="AJ30" s="21"/>
+      <c r="AK30" s="2"/>
+      <c r="AL30" s="2"/>
       <c r="AM30" s="2"/>
       <c r="AN30" s="2"/>
       <c r="AO30" s="2"/>
@@ -3080,211 +3385,1556 @@
       <c r="AX30" s="2"/>
       <c r="AY30" s="2"/>
       <c r="AZ30" s="2"/>
-    </row>
-    <row r="31" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="BA30" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="BB30" s="18">
+        <f>J30</f>
+        <v>0.59281226563754541</v>
+      </c>
+      <c r="BC30" s="2"/>
+      <c r="BD30" s="2"/>
+      <c r="BE30" s="2"/>
+      <c r="BF30" s="2"/>
+      <c r="BG30" s="2"/>
+      <c r="BH30" s="2"/>
+    </row>
+    <row r="31" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I31" s="2">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="AD31" s="44"/>
-      <c r="AE31" s="44"/>
-      <c r="AF31" s="44"/>
-      <c r="AG31" s="44"/>
-      <c r="AH31" s="44"/>
-      <c r="AI31" s="44"/>
-      <c r="AJ31" s="44"/>
-      <c r="AK31" s="44"/>
-      <c r="AL31" s="44"/>
-      <c r="AM31" s="44"/>
-      <c r="AN31" s="44"/>
-      <c r="AO31" s="44"/>
-      <c r="AP31" s="44"/>
-      <c r="AQ31" s="44"/>
-      <c r="AR31" s="44"/>
-      <c r="AS31" s="44"/>
-      <c r="AT31" s="44"/>
-      <c r="AU31" s="44"/>
-      <c r="AV31" s="44"/>
-      <c r="AW31" s="44"/>
-      <c r="AX31" s="44"/>
-      <c r="AY31" s="44"/>
-      <c r="AZ31" s="44"/>
-    </row>
-    <row r="32" spans="2:56" x14ac:dyDescent="0.25">
+      <c r="J31" s="51">
+        <f>N30</f>
+        <v>0.64316638875122245</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="L31" s="2">
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="M31" s="40">
+        <f>-$C$3*LN(1-L31) / 1440</f>
+        <v>7.4455371601330599E-3</v>
+      </c>
+      <c r="N31" s="19">
+        <f>J31+M31</f>
+        <v>0.65061192591135553</v>
+      </c>
+      <c r="O31" s="51" t="s">
+        <v>61</v>
+      </c>
+      <c r="P31" s="2">
+        <v>0.51200000000000001</v>
+      </c>
+      <c r="Q31" s="40">
+        <f>($F$8+P31*($F$9-$F$8)) / 1440</f>
+        <v>1.0500000000000001E-2</v>
+      </c>
+      <c r="R31" s="58">
+        <f>Q31+J31</f>
+        <v>0.6536663887512224</v>
+      </c>
+      <c r="S31" s="2"/>
+      <c r="T31" s="2"/>
+      <c r="U31" s="2"/>
+      <c r="V31" s="2"/>
+      <c r="W31" s="2"/>
+      <c r="X31" s="40">
+        <f>BD31</f>
+        <v>8.3212792793602469E-2</v>
+      </c>
+      <c r="Y31" s="48">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="48">
+        <v>0</v>
+      </c>
+      <c r="AA31" s="43"/>
+      <c r="AB31" s="43">
+        <f t="shared" si="4"/>
+        <v>3.1128239508575246E-2</v>
+      </c>
+      <c r="AC31" s="52">
+        <v>0</v>
+      </c>
+      <c r="AD31" s="2"/>
+      <c r="AE31" s="2"/>
+      <c r="AF31" s="2"/>
+      <c r="AG31" s="2"/>
+      <c r="AH31" s="2"/>
+      <c r="AI31" s="2"/>
+      <c r="AJ31" s="2"/>
+      <c r="AK31" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AL31" s="2"/>
+      <c r="AM31" s="2"/>
+      <c r="AN31" s="2"/>
+      <c r="AO31" s="2"/>
+      <c r="AP31" s="2"/>
+      <c r="AQ31" s="2"/>
+      <c r="AR31" s="2"/>
+      <c r="AS31" s="2"/>
+      <c r="AT31" s="2"/>
+      <c r="AU31" s="2"/>
+      <c r="AV31" s="2"/>
+      <c r="AW31" s="2"/>
+      <c r="AX31" s="2"/>
+      <c r="AY31" s="2"/>
+      <c r="AZ31" s="2"/>
+      <c r="BA31" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="BB31" s="18">
+        <f>BB30</f>
+        <v>0.59281226563754541</v>
+      </c>
+      <c r="BC31" s="2"/>
+      <c r="BD31" s="40">
+        <f>X30-(J31-BB30)</f>
+        <v>8.3212792793602469E-2</v>
+      </c>
+      <c r="BE31" s="2"/>
+      <c r="BF31" s="2"/>
+      <c r="BG31" s="2"/>
+      <c r="BH31" s="2"/>
+    </row>
+    <row r="32" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I32" s="2">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="R32" s="18" t="s">
-        <v>52</v>
-      </c>
-      <c r="S32" s="26">
-        <f ca="1">RAND()</f>
-        <v>0.57786729470145815</v>
-      </c>
-      <c r="AD32" s="44"/>
-      <c r="AE32" s="44"/>
-      <c r="AF32" s="44"/>
-      <c r="AG32" s="44"/>
-      <c r="AH32" s="44"/>
-      <c r="AI32" s="44"/>
-      <c r="AJ32" s="44"/>
-      <c r="AK32" s="44"/>
-      <c r="AL32" s="44"/>
-      <c r="AM32" s="44"/>
-      <c r="AN32" s="44"/>
-      <c r="AO32" s="44"/>
-      <c r="AP32" s="44"/>
-      <c r="AQ32" s="44"/>
-      <c r="AR32" s="44"/>
-      <c r="AS32" s="44"/>
-      <c r="AT32" s="44"/>
-      <c r="AU32" s="44"/>
-      <c r="AV32" s="44"/>
-      <c r="AW32" s="44"/>
-      <c r="AX32" s="44"/>
-      <c r="AY32" s="44"/>
-      <c r="AZ32" s="44"/>
-    </row>
-    <row r="33" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="J32" s="51">
+        <f>N31</f>
+        <v>0.65061192591135553</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="L32" s="2">
+        <v>0.91200000000000003</v>
+      </c>
+      <c r="M32" s="40">
+        <f>-$C$3*LN(1-L32) / 1440</f>
+        <v>7.5950577015747839E-2</v>
+      </c>
+      <c r="N32" s="18">
+        <f>M32+J32</f>
+        <v>0.72656250292710334</v>
+      </c>
+      <c r="O32" s="51" t="s">
+        <v>61</v>
+      </c>
+      <c r="P32" s="2"/>
+      <c r="Q32" s="40"/>
+      <c r="R32" s="19">
+        <f>R31</f>
+        <v>0.6536663887512224</v>
+      </c>
+      <c r="S32" s="25"/>
+      <c r="T32" s="2"/>
+      <c r="U32" s="2"/>
+      <c r="V32" s="2"/>
+      <c r="W32" s="2"/>
+      <c r="X32" s="40">
+        <f>X31</f>
+        <v>8.3212792793602469E-2</v>
+      </c>
+      <c r="Y32" s="48">
+        <v>1</v>
+      </c>
+      <c r="Z32" s="2">
+        <v>0</v>
+      </c>
+      <c r="AA32" s="43"/>
+      <c r="AB32" s="43">
+        <f t="shared" si="4"/>
+        <v>3.1128239508575246E-2</v>
+      </c>
+      <c r="AC32" s="52">
+        <v>0</v>
+      </c>
+      <c r="AD32" s="2"/>
+      <c r="AE32" s="2"/>
+      <c r="AF32" s="2"/>
+      <c r="AG32" s="2"/>
+      <c r="AH32" s="2"/>
+      <c r="AI32" s="2"/>
+      <c r="AJ32" s="2"/>
+      <c r="AK32" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AL32" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AM32" s="2"/>
+      <c r="AN32" s="2"/>
+      <c r="AO32" s="2"/>
+      <c r="AP32" s="2"/>
+      <c r="AQ32" s="2"/>
+      <c r="AR32" s="2"/>
+      <c r="AS32" s="2"/>
+      <c r="AT32" s="2"/>
+      <c r="AU32" s="2"/>
+      <c r="AV32" s="2"/>
+      <c r="AW32" s="2"/>
+      <c r="AX32" s="2"/>
+      <c r="AY32" s="2"/>
+      <c r="AZ32" s="2"/>
+      <c r="BA32" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="BB32" s="18">
+        <f t="shared" ref="BB32:BB35" si="5">BB31</f>
+        <v>0.59281226563754541</v>
+      </c>
+      <c r="BC32" s="2"/>
+      <c r="BD32" s="2"/>
+      <c r="BE32" s="2"/>
+      <c r="BF32" s="2"/>
+      <c r="BG32" s="2"/>
+      <c r="BH32" s="2"/>
+    </row>
+    <row r="33" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I33" s="2">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-    </row>
-    <row r="34" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="J33" s="51">
+        <f>R32</f>
+        <v>0.6536663887512224</v>
+      </c>
+      <c r="K33" s="47" t="s">
+        <v>112</v>
+      </c>
+      <c r="L33" s="2"/>
+      <c r="M33" s="40"/>
+      <c r="N33" s="18">
+        <f>N32</f>
+        <v>0.72656250292710334</v>
+      </c>
+      <c r="O33" s="51" t="s">
+        <v>61</v>
+      </c>
+      <c r="P33" s="2">
+        <v>0.314</v>
+      </c>
+      <c r="Q33" s="40">
+        <f>($F$8+P33*($F$9-$F$8)) / 1440</f>
+        <v>9.1250000000000012E-3</v>
+      </c>
+      <c r="R33" s="18">
+        <f>Q33+J33</f>
+        <v>0.66279138875122245</v>
+      </c>
+      <c r="S33" s="2">
+        <v>0.121</v>
+      </c>
+      <c r="T33" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="U33" s="2">
+        <v>0.161</v>
+      </c>
+      <c r="V33" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="W33" s="2"/>
+      <c r="X33" s="40">
+        <f>X32</f>
+        <v>8.3212792793602469E-2</v>
+      </c>
+      <c r="Y33" s="48">
+        <v>0</v>
+      </c>
+      <c r="Z33" s="2">
+        <v>0</v>
+      </c>
+      <c r="AA33" s="43"/>
+      <c r="AB33" s="43">
+        <f t="shared" si="4"/>
+        <v>3.1128239508575246E-2</v>
+      </c>
+      <c r="AC33" s="52">
+        <v>0</v>
+      </c>
+      <c r="AD33" s="2"/>
+      <c r="AE33" s="2"/>
+      <c r="AF33" s="2"/>
+      <c r="AG33" s="2"/>
+      <c r="AH33" s="2"/>
+      <c r="AI33" s="2"/>
+      <c r="AJ33" s="2"/>
+      <c r="AK33" s="59"/>
+      <c r="AL33" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AM33" s="2"/>
+      <c r="AN33" s="2"/>
+      <c r="AO33" s="2"/>
+      <c r="AP33" s="2"/>
+      <c r="AQ33" s="2"/>
+      <c r="AR33" s="2"/>
+      <c r="AS33" s="2"/>
+      <c r="AT33" s="2"/>
+      <c r="AU33" s="2"/>
+      <c r="AV33" s="2"/>
+      <c r="AW33" s="2"/>
+      <c r="AX33" s="2"/>
+      <c r="AY33" s="2"/>
+      <c r="AZ33" s="2"/>
+      <c r="BA33" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="BB33" s="18">
+        <f t="shared" si="5"/>
+        <v>0.59281226563754541</v>
+      </c>
+      <c r="BC33" s="2"/>
+      <c r="BD33" s="2"/>
+      <c r="BE33" s="2"/>
+      <c r="BF33" s="2"/>
+      <c r="BG33" s="2"/>
+      <c r="BH33" s="2"/>
+    </row>
+    <row r="34" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I34" s="2">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-    </row>
-    <row r="35" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="J34" s="18">
+        <f>R33</f>
+        <v>0.66279138875122245</v>
+      </c>
+      <c r="K34" s="47" t="s">
+        <v>114</v>
+      </c>
+      <c r="L34" s="2"/>
+      <c r="M34" s="40"/>
+      <c r="N34" s="19">
+        <f>N33</f>
+        <v>0.72656250292710334</v>
+      </c>
+      <c r="O34" s="51" t="s">
+        <v>60</v>
+      </c>
+      <c r="P34" s="2"/>
+      <c r="Q34" s="40"/>
+      <c r="R34" s="18"/>
+      <c r="S34" s="2">
+        <v>0.40300000000000002</v>
+      </c>
+      <c r="T34" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="U34" s="2"/>
+      <c r="V34" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="W34" s="2"/>
+      <c r="X34" s="40">
+        <f>X33</f>
+        <v>8.3212792793602469E-2</v>
+      </c>
+      <c r="Y34" s="48">
+        <v>0</v>
+      </c>
+      <c r="Z34" s="2">
+        <v>1</v>
+      </c>
+      <c r="AA34" s="43"/>
+      <c r="AB34" s="43">
+        <f t="shared" si="4"/>
+        <v>3.1128239508575246E-2</v>
+      </c>
+      <c r="AC34" s="52">
+        <v>0</v>
+      </c>
+      <c r="AD34" s="2"/>
+      <c r="AE34" s="2"/>
+      <c r="AF34" s="2"/>
+      <c r="AG34" s="2"/>
+      <c r="AH34" s="2"/>
+      <c r="AI34" s="2"/>
+      <c r="AJ34" s="2"/>
+      <c r="AK34" s="2"/>
+      <c r="AL34" s="21"/>
+      <c r="AM34" s="2"/>
+      <c r="AN34" s="2"/>
+      <c r="AO34" s="2"/>
+      <c r="AP34" s="2"/>
+      <c r="AQ34" s="2"/>
+      <c r="AR34" s="2"/>
+      <c r="AS34" s="2"/>
+      <c r="AT34" s="2"/>
+      <c r="AU34" s="2"/>
+      <c r="AV34" s="2"/>
+      <c r="AW34" s="2"/>
+      <c r="AX34" s="2"/>
+      <c r="AY34" s="2"/>
+      <c r="AZ34" s="2"/>
+      <c r="BA34" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="BB34" s="18">
+        <f t="shared" si="5"/>
+        <v>0.59281226563754541</v>
+      </c>
+      <c r="BC34" s="2"/>
+      <c r="BD34" s="2"/>
+      <c r="BE34" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="BF34" s="18">
+        <f>J34</f>
+        <v>0.66279138875122245</v>
+      </c>
+      <c r="BG34" s="2"/>
+      <c r="BH34" s="2"/>
+    </row>
+    <row r="35" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I35" s="2">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-    </row>
-    <row r="36" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="J35" s="51">
+        <f>N34</f>
+        <v>0.72656250292710334</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="L35" s="2">
+        <v>0.69299999999999995</v>
+      </c>
+      <c r="M35" s="40">
+        <f>-$C$3*LN(1-L35) / 1440</f>
+        <v>3.6903360356091867E-2</v>
+      </c>
+      <c r="N35" s="18">
+        <f>M35+J35</f>
+        <v>0.76346586328319521</v>
+      </c>
+      <c r="O35" s="51" t="s">
+        <v>61</v>
+      </c>
+      <c r="P35" s="2">
+        <v>0.12</v>
+      </c>
+      <c r="Q35" s="40">
+        <f>($F$8+P35*($F$9-$F$8)) / 1440</f>
+        <v>7.7777777777777776E-3</v>
+      </c>
+      <c r="R35" s="19">
+        <f>Q35+J35</f>
+        <v>0.73434028070488111</v>
+      </c>
+      <c r="S35" s="2"/>
+      <c r="T35" s="2"/>
+      <c r="U35" s="2"/>
+      <c r="V35" s="2"/>
+      <c r="W35" s="2"/>
+      <c r="X35" s="40">
+        <f>BD35</f>
+        <v>1.9441678617721586E-2</v>
+      </c>
+      <c r="Y35" s="48">
+        <v>0</v>
+      </c>
+      <c r="Z35" s="2">
+        <v>1</v>
+      </c>
+      <c r="AA35" s="43"/>
+      <c r="AB35" s="43">
+        <f t="shared" si="4"/>
+        <v>3.1128239508575246E-2</v>
+      </c>
+      <c r="AC35" s="52">
+        <v>0</v>
+      </c>
+      <c r="AD35" s="2"/>
+      <c r="AE35" s="2"/>
+      <c r="AF35" s="2"/>
+      <c r="AG35" s="2"/>
+      <c r="AH35" s="2"/>
+      <c r="AI35" s="2"/>
+      <c r="AJ35" s="2"/>
+      <c r="AK35" s="2"/>
+      <c r="AL35" s="2"/>
+      <c r="AM35" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AN35" s="2"/>
+      <c r="AO35" s="2"/>
+      <c r="AP35" s="2"/>
+      <c r="AQ35" s="2"/>
+      <c r="AR35" s="2"/>
+      <c r="AS35" s="2"/>
+      <c r="AT35" s="2"/>
+      <c r="AU35" s="2"/>
+      <c r="AV35" s="2"/>
+      <c r="AW35" s="2"/>
+      <c r="AX35" s="2"/>
+      <c r="AY35" s="2"/>
+      <c r="AZ35" s="2"/>
+      <c r="BA35" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="BB35" s="18">
+        <f t="shared" si="5"/>
+        <v>0.59281226563754541</v>
+      </c>
+      <c r="BC35" s="2"/>
+      <c r="BD35" s="40">
+        <f>X34-(J35-J34)</f>
+        <v>1.9441678617721586E-2</v>
+      </c>
+      <c r="BE35" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="BF35" s="18">
+        <f>BF34</f>
+        <v>0.66279138875122245</v>
+      </c>
+      <c r="BG35" s="2"/>
+      <c r="BH35" s="2"/>
+    </row>
+    <row r="36" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I36" s="2">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-    </row>
-    <row r="37" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="J36" s="51">
+        <f>R35</f>
+        <v>0.73434028070488111</v>
+      </c>
+      <c r="K36" s="47" t="s">
+        <v>116</v>
+      </c>
+      <c r="L36" s="2"/>
+      <c r="M36" s="40"/>
+      <c r="N36" s="18">
+        <f>N35</f>
+        <v>0.76346586328319521</v>
+      </c>
+      <c r="O36" s="51" t="s">
+        <v>60</v>
+      </c>
+      <c r="P36" s="2"/>
+      <c r="Q36" s="40"/>
+      <c r="R36" s="18"/>
+      <c r="S36" s="2"/>
+      <c r="T36" s="2"/>
+      <c r="U36" s="2"/>
+      <c r="V36" s="2"/>
+      <c r="W36" s="2"/>
+      <c r="X36" s="40"/>
+      <c r="Y36" s="48">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="2">
+        <v>1</v>
+      </c>
+      <c r="AA36" s="43"/>
+      <c r="AB36" s="43">
+        <f t="shared" si="4"/>
+        <v>3.1128239508575246E-2</v>
+      </c>
+      <c r="AC36" s="52">
+        <v>0</v>
+      </c>
+      <c r="AD36" s="2"/>
+      <c r="AE36" s="2"/>
+      <c r="AF36" s="2"/>
+      <c r="AG36" s="2"/>
+      <c r="AH36" s="2"/>
+      <c r="AI36" s="2"/>
+      <c r="AJ36" s="2"/>
+      <c r="AK36" s="2"/>
+      <c r="AL36" s="2"/>
+      <c r="AM36" s="2"/>
+      <c r="AN36" s="2"/>
+      <c r="AO36" s="2"/>
+      <c r="AP36" s="2"/>
+      <c r="AQ36" s="2"/>
+      <c r="AR36" s="2"/>
+      <c r="AS36" s="2"/>
+      <c r="AT36" s="2"/>
+      <c r="AU36" s="2"/>
+      <c r="AV36" s="2"/>
+      <c r="AW36" s="2"/>
+      <c r="AX36" s="2"/>
+      <c r="AY36" s="2"/>
+      <c r="AZ36" s="2"/>
+      <c r="BA36" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="BB36" s="18">
+        <f>BB35</f>
+        <v>0.59281226563754541</v>
+      </c>
+      <c r="BC36" s="2"/>
+      <c r="BD36" s="2"/>
+      <c r="BE36" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="BF36" s="18">
+        <f>BF35</f>
+        <v>0.66279138875122245</v>
+      </c>
+      <c r="BG36" s="2"/>
+      <c r="BH36" s="2"/>
+    </row>
+    <row r="37" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I37" s="2">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-    </row>
-    <row r="38" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="J37" s="50">
+        <f>J36+X35</f>
+        <v>0.75378195932260272</v>
+      </c>
+      <c r="K37" s="60" t="s">
+        <v>117</v>
+      </c>
+      <c r="L37" s="53"/>
+      <c r="M37" s="55"/>
+      <c r="N37" s="50">
+        <f>N36</f>
+        <v>0.76346586328319521</v>
+      </c>
+      <c r="O37" s="53" t="s">
+        <v>60</v>
+      </c>
+      <c r="P37" s="53"/>
+      <c r="Q37" s="55"/>
+      <c r="R37" s="50"/>
+      <c r="S37" s="53"/>
+      <c r="T37" s="53"/>
+      <c r="U37" s="53"/>
+      <c r="V37" s="53"/>
+      <c r="W37" s="53"/>
+      <c r="X37" s="55"/>
+      <c r="Y37" s="53">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA37" s="55"/>
+      <c r="AB37" s="55">
+        <f>AB36+X30</f>
+        <v>0.16469515541585475</v>
+      </c>
+      <c r="AC37" s="53"/>
+      <c r="AD37" s="53"/>
+      <c r="AE37" s="53"/>
+      <c r="AF37" s="53"/>
+      <c r="AG37" s="53"/>
+      <c r="AH37" s="53"/>
+      <c r="AI37" s="53"/>
+      <c r="AJ37" s="53"/>
+      <c r="AK37" s="53"/>
+      <c r="AL37" s="53"/>
+      <c r="AM37" s="53"/>
+      <c r="AN37" s="53"/>
+      <c r="AO37" s="53"/>
+      <c r="AP37" s="53"/>
+      <c r="AQ37" s="53"/>
+      <c r="AR37" s="53"/>
+      <c r="AS37" s="53"/>
+      <c r="AT37" s="53"/>
+      <c r="AU37" s="53"/>
+      <c r="AV37" s="53"/>
+      <c r="AW37" s="53"/>
+      <c r="AX37" s="53"/>
+      <c r="AY37" s="53"/>
+      <c r="AZ37" s="53"/>
+      <c r="BA37" s="53"/>
+      <c r="BB37" s="50">
+        <f>BB36</f>
+        <v>0.59281226563754541</v>
+      </c>
+      <c r="BC37" s="50">
+        <f>J37</f>
+        <v>0.75378195932260272</v>
+      </c>
+      <c r="BD37" s="53"/>
+      <c r="BE37" s="53" t="s">
+        <v>90</v>
+      </c>
+      <c r="BF37" s="50">
+        <f>BF36</f>
+        <v>0.66279138875122245</v>
+      </c>
+      <c r="BG37" s="53"/>
+      <c r="BH37" s="53"/>
+    </row>
+    <row r="38" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I38" s="2">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-    </row>
-    <row r="39" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M38" s="43"/>
+      <c r="Q38" s="43"/>
+      <c r="R38" s="49"/>
+      <c r="T38" s="49"/>
+      <c r="X38" s="43"/>
+      <c r="AA38" s="43"/>
+      <c r="AB38" s="43"/>
+      <c r="BB38" s="54"/>
+      <c r="BC38" s="54"/>
+      <c r="BD38" s="54"/>
+    </row>
+    <row r="39" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I39" s="2">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-    </row>
-    <row r="40" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M39" s="43"/>
+      <c r="Q39" s="43"/>
+      <c r="R39" s="49"/>
+      <c r="X39" s="43"/>
+      <c r="AA39" s="43"/>
+      <c r="AB39" s="43"/>
+    </row>
+    <row r="40" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I40" s="2">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-    </row>
-    <row r="41" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M40" s="43"/>
+      <c r="Q40" s="43"/>
+      <c r="R40" s="49"/>
+      <c r="T40" s="49"/>
+      <c r="X40" s="43"/>
+      <c r="AA40" s="43"/>
+      <c r="AB40" s="43"/>
+    </row>
+    <row r="41" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I41" s="2">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-    </row>
-    <row r="42" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="N41" t="s">
+        <v>118</v>
+      </c>
+      <c r="Q41" s="43"/>
+      <c r="R41" s="49"/>
+      <c r="X41" s="43"/>
+      <c r="AA41" s="43"/>
+      <c r="AB41" s="43"/>
+    </row>
+    <row r="42" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I42" s="2">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-    </row>
-    <row r="43" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M42" s="43"/>
+      <c r="Q42" s="43"/>
+      <c r="R42" s="49"/>
+      <c r="X42" s="43"/>
+      <c r="AA42" s="43"/>
+      <c r="AB42" s="43"/>
+    </row>
+    <row r="43" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I43" s="2">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-    </row>
-    <row r="44" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M43" s="43"/>
+      <c r="Q43" s="43"/>
+      <c r="R43" s="49"/>
+      <c r="X43" s="43"/>
+      <c r="AA43" s="43"/>
+      <c r="AB43" s="43"/>
+    </row>
+    <row r="44" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I44" s="2">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-    </row>
-    <row r="45" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M44" s="43"/>
+      <c r="Q44" s="43"/>
+      <c r="R44" s="49"/>
+      <c r="X44" s="43"/>
+      <c r="AA44" s="43"/>
+      <c r="AB44" s="43"/>
+    </row>
+    <row r="45" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I45" s="2">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-    </row>
-    <row r="46" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M45" s="43"/>
+      <c r="Q45" s="43"/>
+      <c r="R45" s="49"/>
+      <c r="X45" s="43"/>
+      <c r="AA45" s="43"/>
+      <c r="AB45" s="43"/>
+    </row>
+    <row r="46" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I46" s="2">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-    </row>
-    <row r="47" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M46" s="43"/>
+      <c r="Q46" s="43"/>
+      <c r="R46" s="49"/>
+      <c r="X46" s="43"/>
+      <c r="AA46" s="43"/>
+      <c r="AB46" s="43"/>
+    </row>
+    <row r="47" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I47" s="2">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-    </row>
-    <row r="48" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M47" s="43"/>
+      <c r="Q47" s="43"/>
+      <c r="R47" s="49"/>
+      <c r="X47" s="43"/>
+      <c r="AA47" s="43"/>
+      <c r="AB47" s="43"/>
+    </row>
+    <row r="48" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I48" s="2">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-    </row>
-    <row r="49" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M48" s="43"/>
+      <c r="Q48" s="43"/>
+      <c r="R48" s="49"/>
+      <c r="X48" s="43"/>
+      <c r="AA48" s="43"/>
+      <c r="AB48" s="43"/>
+    </row>
+    <row r="49" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I49" s="2">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-    </row>
-    <row r="50" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M49" s="43"/>
+      <c r="Q49" s="43"/>
+      <c r="R49" s="49"/>
+      <c r="X49" s="43"/>
+      <c r="AA49" s="43"/>
+      <c r="AB49" s="43"/>
+    </row>
+    <row r="50" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I50" s="2">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-    </row>
-    <row r="51" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M50" s="43"/>
+      <c r="Q50" s="43"/>
+      <c r="R50" s="49"/>
+      <c r="X50" s="43"/>
+      <c r="AA50" s="43"/>
+      <c r="AB50" s="43"/>
+    </row>
+    <row r="51" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I51" s="2">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-    </row>
-    <row r="52" spans="9:9" x14ac:dyDescent="0.25">
+      <c r="M51" s="43"/>
+      <c r="Q51" s="43"/>
+      <c r="R51" s="49"/>
+      <c r="X51" s="43"/>
+      <c r="AA51" s="43"/>
+      <c r="AB51" s="43"/>
+    </row>
+    <row r="52" spans="9:36" x14ac:dyDescent="0.35">
       <c r="I52" s="2">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
+      <c r="M52" s="43"/>
+      <c r="Q52" s="43"/>
+      <c r="X52" s="43"/>
+      <c r="AA52" s="43"/>
+      <c r="AB52" s="43"/>
+      <c r="AE52" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF52" s="26"/>
+      <c r="AG52" s="26"/>
+      <c r="AH52" s="26"/>
+      <c r="AI52" s="26"/>
+    </row>
+    <row r="53" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M53" s="43"/>
+      <c r="Q53" s="43"/>
+      <c r="X53" s="43"/>
+      <c r="AB53" s="43"/>
+      <c r="AE53" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AF53" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="AG53" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="AH53" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="AI53" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="54" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M54" s="43"/>
+      <c r="Q54" s="43"/>
+      <c r="X54" s="43"/>
+      <c r="AB54" s="43"/>
+      <c r="AE54" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="AF54" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="AG54" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="AH54" s="2">
+        <v>0</v>
+      </c>
+      <c r="AI54" s="2">
+        <v>0.29899999999999999</v>
+      </c>
+    </row>
+    <row r="55" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M55" s="43"/>
+      <c r="X55" s="43"/>
+      <c r="AB55" s="43"/>
+      <c r="AE55" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF55" s="2">
+        <v>0.7</v>
+      </c>
+      <c r="AG55" s="2">
+        <v>1</v>
+      </c>
+      <c r="AH55" s="2">
+        <v>0.3</v>
+      </c>
+      <c r="AI55" s="2">
+        <v>0.999</v>
+      </c>
+    </row>
+    <row r="56" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M56" s="43"/>
+      <c r="X56" s="43"/>
+      <c r="AB56" s="43"/>
+    </row>
+    <row r="57" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M57" s="43"/>
+      <c r="X57" s="43"/>
+      <c r="AB57" s="43"/>
+      <c r="AE57" s="26" t="s">
+        <v>25</v>
+      </c>
+      <c r="AF57" s="26"/>
+      <c r="AG57" s="26"/>
+      <c r="AH57" s="26"/>
+      <c r="AI57" s="26"/>
+    </row>
+    <row r="58" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M58" s="43"/>
+      <c r="X58" s="43"/>
+      <c r="AB58" s="43"/>
+      <c r="AE58" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="AF58" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="AG58" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="AH58" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="AI58" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="59" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M59" s="43"/>
+      <c r="X59" s="43"/>
+      <c r="AB59" s="43"/>
+      <c r="AE59" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="AF59" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="AG59" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="AH59" s="2">
+        <v>0</v>
+      </c>
+      <c r="AI59" s="2">
+        <v>0.499</v>
+      </c>
+      <c r="AJ59" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="60" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M60" s="43"/>
+      <c r="X60" s="43"/>
+      <c r="AB60" s="43"/>
+      <c r="AE60" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="AF60" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="AG60" s="2">
+        <v>1</v>
+      </c>
+      <c r="AH60" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="AI60" s="2">
+        <v>0.999</v>
+      </c>
+    </row>
+    <row r="61" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M61" s="43"/>
+      <c r="X61" s="43"/>
+      <c r="AB61" s="43"/>
+    </row>
+    <row r="62" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M62" s="43"/>
+      <c r="X62" s="43"/>
+      <c r="AB62" s="43"/>
+      <c r="AE62" s="32" t="s">
+        <v>26</v>
+      </c>
+      <c r="AF62" s="32"/>
+      <c r="AG62" s="32"/>
+      <c r="AH62" s="32"/>
+      <c r="AI62" s="32"/>
+    </row>
+    <row r="63" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M63" s="43"/>
+      <c r="X63" s="43"/>
+      <c r="AB63" s="43"/>
+      <c r="AE63" s="32"/>
+      <c r="AF63" s="32"/>
+      <c r="AG63" s="32"/>
+      <c r="AH63" s="32"/>
+      <c r="AI63" s="32"/>
+    </row>
+    <row r="64" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M64" s="43"/>
+      <c r="X64" s="43"/>
+      <c r="AB64" s="43"/>
+    </row>
+    <row r="65" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M65" s="43"/>
+      <c r="X65" s="43"/>
+      <c r="AB65" s="43"/>
+    </row>
+    <row r="66" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M66" s="43"/>
+      <c r="X66" s="43"/>
+      <c r="AB66" s="43"/>
+    </row>
+    <row r="67" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M67" s="43"/>
+      <c r="X67" s="43"/>
+      <c r="AB67" s="43"/>
+    </row>
+    <row r="68" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M68" s="43"/>
+      <c r="X68" s="43"/>
+      <c r="AB68" s="43"/>
+    </row>
+    <row r="69" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M69" s="43"/>
+      <c r="X69" s="43"/>
+      <c r="AB69" s="43"/>
+    </row>
+    <row r="70" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M70" s="43"/>
+      <c r="X70" s="43"/>
+      <c r="AB70" s="43"/>
+    </row>
+    <row r="71" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M71" s="43"/>
+      <c r="X71" s="43"/>
+      <c r="AB71" s="43"/>
+    </row>
+    <row r="72" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M72" s="43"/>
+      <c r="X72" s="43"/>
+      <c r="AB72" s="43"/>
+    </row>
+    <row r="73" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M73" s="43"/>
+      <c r="X73" s="43"/>
+      <c r="AB73" s="43"/>
+    </row>
+    <row r="74" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M74" s="43"/>
+      <c r="X74" s="43"/>
+      <c r="AB74" s="43"/>
+    </row>
+    <row r="75" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M75" s="43"/>
+      <c r="X75" s="43"/>
+      <c r="AB75" s="43"/>
+    </row>
+    <row r="76" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M76" s="43"/>
+      <c r="X76" s="43"/>
+      <c r="AB76" s="43"/>
+    </row>
+    <row r="77" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M77" s="43"/>
+      <c r="X77" s="43"/>
+      <c r="AB77" s="43"/>
+    </row>
+    <row r="78" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M78" s="43"/>
+      <c r="X78" s="43"/>
+      <c r="AB78" s="43"/>
+    </row>
+    <row r="79" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M79" s="43"/>
+      <c r="X79" s="43"/>
+      <c r="AB79" s="43"/>
+    </row>
+    <row r="80" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M80" s="43"/>
+      <c r="X80" s="43"/>
+      <c r="AB80" s="43"/>
+    </row>
+    <row r="81" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M81" s="43"/>
+      <c r="X81" s="43"/>
+      <c r="AB81" s="43"/>
+    </row>
+    <row r="82" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M82" s="43"/>
+      <c r="X82" s="43"/>
+      <c r="AB82" s="43"/>
+    </row>
+    <row r="83" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M83" s="43"/>
+      <c r="X83" s="43"/>
+      <c r="AB83" s="43"/>
+    </row>
+    <row r="84" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M84" s="43"/>
+      <c r="X84" s="43"/>
+      <c r="AB84" s="43"/>
+    </row>
+    <row r="85" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M85" s="43"/>
+      <c r="X85" s="43"/>
+      <c r="AB85" s="43"/>
+    </row>
+    <row r="86" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M86" s="43"/>
+      <c r="X86" s="43"/>
+      <c r="AB86" s="43"/>
+    </row>
+    <row r="87" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M87" s="43"/>
+      <c r="X87" s="43"/>
+      <c r="AB87" s="43"/>
+    </row>
+    <row r="88" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M88" s="43"/>
+      <c r="X88" s="43"/>
+      <c r="AB88" s="43"/>
+    </row>
+    <row r="89" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M89" s="43"/>
+      <c r="AB89" s="43"/>
+    </row>
+    <row r="90" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M90" s="43"/>
+      <c r="AB90" s="43"/>
+    </row>
+    <row r="91" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M91" s="43"/>
+      <c r="AB91" s="43"/>
+    </row>
+    <row r="92" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M92" s="43"/>
+      <c r="AB92" s="43"/>
+    </row>
+    <row r="93" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M93" s="43"/>
+      <c r="AB93" s="43"/>
+    </row>
+    <row r="94" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M94" s="43"/>
+      <c r="AB94" s="43"/>
+    </row>
+    <row r="95" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M95" s="43"/>
+      <c r="AB95" s="43"/>
+    </row>
+    <row r="96" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M96" s="43"/>
+      <c r="AB96" s="43"/>
+    </row>
+    <row r="97" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M97" s="43"/>
+      <c r="AB97" s="43"/>
+    </row>
+    <row r="98" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M98" s="43"/>
+      <c r="AB98" s="43"/>
+    </row>
+    <row r="99" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M99" s="43"/>
+      <c r="AB99" s="43"/>
+    </row>
+    <row r="100" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M100" s="43"/>
+      <c r="AB100" s="43"/>
+    </row>
+    <row r="101" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M101" s="43"/>
+      <c r="AB101" s="43"/>
+    </row>
+    <row r="102" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M102" s="43"/>
+      <c r="AB102" s="43"/>
+    </row>
+    <row r="103" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M103" s="43"/>
+      <c r="AB103" s="43"/>
+    </row>
+    <row r="104" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M104" s="43"/>
+      <c r="AB104" s="43"/>
+    </row>
+    <row r="105" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M105" s="43"/>
+      <c r="AB105" s="43"/>
+    </row>
+    <row r="106" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M106" s="43"/>
+      <c r="AB106" s="43"/>
+    </row>
+    <row r="107" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M107" s="43"/>
+      <c r="AB107" s="43"/>
+    </row>
+    <row r="108" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M108" s="43"/>
+      <c r="AB108" s="43"/>
+    </row>
+    <row r="109" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M109" s="43"/>
+      <c r="AB109" s="43"/>
+    </row>
+    <row r="110" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M110" s="43"/>
+      <c r="AB110" s="43"/>
+    </row>
+    <row r="111" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M111" s="43"/>
+      <c r="AB111" s="43"/>
+    </row>
+    <row r="112" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M112" s="43"/>
+      <c r="AB112" s="43"/>
+    </row>
+    <row r="113" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M113" s="43"/>
+      <c r="AB113" s="43"/>
+    </row>
+    <row r="114" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M114" s="43"/>
+      <c r="AB114" s="43"/>
+    </row>
+    <row r="115" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M115" s="43"/>
+      <c r="AB115" s="43"/>
+    </row>
+    <row r="116" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M116" s="43"/>
+      <c r="AB116" s="43"/>
+    </row>
+    <row r="117" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M117" s="43"/>
+      <c r="AB117" s="43"/>
+    </row>
+    <row r="118" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M118" s="43"/>
+      <c r="AB118" s="43"/>
+    </row>
+    <row r="119" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M119" s="43"/>
+      <c r="AB119" s="43"/>
+    </row>
+    <row r="120" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M120" s="43"/>
+      <c r="AB120" s="43"/>
+    </row>
+    <row r="121" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M121" s="43"/>
+      <c r="AB121" s="43"/>
+    </row>
+    <row r="122" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M122" s="43"/>
+      <c r="AB122" s="43"/>
+    </row>
+    <row r="123" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M123" s="43"/>
+      <c r="AB123" s="43"/>
+    </row>
+    <row r="124" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M124" s="43"/>
+      <c r="AB124" s="43"/>
+    </row>
+    <row r="125" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M125" s="43"/>
+      <c r="AB125" s="43"/>
+    </row>
+    <row r="126" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M126" s="43"/>
+      <c r="AB126" s="43"/>
+    </row>
+    <row r="127" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M127" s="43"/>
+      <c r="AB127" s="43"/>
+    </row>
+    <row r="128" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M128" s="43"/>
+      <c r="AB128" s="43"/>
+    </row>
+    <row r="129" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M129" s="43"/>
+      <c r="AB129" s="43"/>
+    </row>
+    <row r="130" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M130" s="43"/>
+      <c r="AB130" s="43"/>
+    </row>
+    <row r="131" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M131" s="43"/>
+      <c r="AB131" s="43"/>
+    </row>
+    <row r="132" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M132" s="43"/>
+      <c r="AB132" s="43"/>
+    </row>
+    <row r="133" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M133" s="43"/>
+      <c r="AB133" s="43"/>
+    </row>
+    <row r="134" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M134" s="43"/>
+      <c r="AB134" s="43"/>
+    </row>
+    <row r="135" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M135" s="43"/>
+      <c r="AB135" s="43"/>
+    </row>
+    <row r="136" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M136" s="43"/>
+      <c r="AB136" s="43"/>
+    </row>
+    <row r="137" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M137" s="43"/>
+      <c r="AB137" s="43"/>
+    </row>
+    <row r="138" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M138" s="43"/>
+      <c r="AB138" s="43"/>
+    </row>
+    <row r="139" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M139" s="43"/>
+      <c r="AB139" s="43"/>
+    </row>
+    <row r="140" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M140" s="43"/>
+      <c r="AB140" s="43"/>
+    </row>
+    <row r="141" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M141" s="43"/>
+      <c r="AB141" s="43"/>
+    </row>
+    <row r="142" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M142" s="43"/>
+      <c r="AB142" s="43"/>
+    </row>
+    <row r="143" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M143" s="43"/>
+      <c r="AB143" s="43"/>
+    </row>
+    <row r="144" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M144" s="43"/>
+      <c r="AB144" s="43"/>
+    </row>
+    <row r="145" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M145" s="43"/>
+      <c r="AB145" s="43"/>
+    </row>
+    <row r="146" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M146" s="43"/>
+      <c r="AB146" s="43"/>
+    </row>
+    <row r="147" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M147" s="43"/>
+      <c r="AB147" s="43"/>
+    </row>
+    <row r="148" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M148" s="43"/>
+      <c r="AB148" s="43"/>
+    </row>
+    <row r="149" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M149" s="43"/>
+      <c r="AB149" s="43"/>
+    </row>
+    <row r="150" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M150" s="43"/>
+      <c r="AB150" s="43"/>
+    </row>
+    <row r="151" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M151" s="43"/>
+      <c r="AB151" s="43"/>
+    </row>
+    <row r="152" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M152" s="43"/>
+      <c r="AB152" s="43"/>
+    </row>
+    <row r="153" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M153" s="43"/>
+      <c r="AB153" s="43"/>
+    </row>
+    <row r="154" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M154" s="43"/>
+      <c r="AB154" s="43"/>
+    </row>
+    <row r="155" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M155" s="43"/>
+      <c r="AB155" s="43"/>
+    </row>
+    <row r="156" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M156" s="43"/>
+      <c r="AB156" s="43"/>
+    </row>
+    <row r="157" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M157" s="43"/>
+      <c r="AB157" s="43"/>
+    </row>
+    <row r="158" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M158" s="43"/>
+      <c r="AB158" s="43"/>
+    </row>
+    <row r="159" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M159" s="43"/>
+      <c r="AB159" s="43"/>
+    </row>
+    <row r="160" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M160" s="43"/>
+      <c r="AB160" s="43"/>
+    </row>
+    <row r="161" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M161" s="43"/>
+      <c r="AB161" s="43"/>
+    </row>
+    <row r="162" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M162" s="43"/>
+      <c r="AB162" s="43"/>
+    </row>
+    <row r="163" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M163" s="43"/>
+      <c r="AB163" s="43"/>
+    </row>
+    <row r="164" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M164" s="43"/>
+      <c r="AB164" s="43"/>
+    </row>
+    <row r="165" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M165" s="43"/>
+      <c r="AB165" s="43"/>
+    </row>
+    <row r="166" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M166" s="43"/>
+      <c r="AB166" s="43"/>
+    </row>
+    <row r="167" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M167" s="43"/>
+      <c r="AB167" s="43"/>
+    </row>
+    <row r="168" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M168" s="43"/>
+      <c r="AB168" s="43"/>
+    </row>
+    <row r="169" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M169" s="43"/>
+      <c r="AB169" s="43"/>
+    </row>
+    <row r="170" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M170" s="43"/>
+      <c r="AB170" s="43"/>
+    </row>
+    <row r="171" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M171" s="43"/>
+      <c r="AB171" s="43"/>
+    </row>
+    <row r="172" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M172" s="43"/>
+      <c r="AB172" s="43"/>
+    </row>
+    <row r="173" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M173" s="43"/>
+      <c r="AB173" s="43"/>
+    </row>
+    <row r="174" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M174" s="43"/>
+      <c r="AB174" s="43"/>
+    </row>
+    <row r="175" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M175" s="43"/>
+      <c r="AB175" s="43"/>
+    </row>
+    <row r="176" spans="13:28" x14ac:dyDescent="0.35">
+      <c r="M176" s="43"/>
+      <c r="AB176" s="43"/>
+    </row>
+    <row r="177" spans="13:13" x14ac:dyDescent="0.35">
+      <c r="M177" s="43"/>
+    </row>
+    <row r="178" spans="13:13" x14ac:dyDescent="0.35">
+      <c r="M178" s="43"/>
+    </row>
+    <row r="179" spans="13:13" x14ac:dyDescent="0.35">
+      <c r="M179" s="43"/>
+    </row>
+    <row r="180" spans="13:13" x14ac:dyDescent="0.35">
+      <c r="M180" s="43"/>
+    </row>
+    <row r="181" spans="13:13" x14ac:dyDescent="0.35">
+      <c r="M181" s="43"/>
+    </row>
+    <row r="182" spans="13:13" x14ac:dyDescent="0.35">
+      <c r="M182" s="43"/>
     </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="AO11:AR11"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="AD10:AM10"/>
-    <mergeCell ref="O11:V11"/>
-    <mergeCell ref="AA11:AC11"/>
-    <mergeCell ref="Y11:Z11"/>
-    <mergeCell ref="B24:F25"/>
-    <mergeCell ref="G8:H9"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B19:F19"/>
+  <mergeCells count="37">
+    <mergeCell ref="AE52:AI52"/>
+    <mergeCell ref="AE57:AI57"/>
+    <mergeCell ref="AE62:AI63"/>
+    <mergeCell ref="BE11:BH11"/>
     <mergeCell ref="E2:H2"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="E5:F5"/>
@@ -3301,6 +4951,23 @@
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="S3:T3"/>
     <mergeCell ref="AS11:AV11"/>
+    <mergeCell ref="B24:F25"/>
+    <mergeCell ref="G8:H9"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="AO11:AR11"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="AD10:AM10"/>
+    <mergeCell ref="O11:V11"/>
+    <mergeCell ref="AA11:AC11"/>
+    <mergeCell ref="Y11:Z11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Arreglé cosas sobre Nones en casos particulares
</commit_message>
<xml_diff>
--- a/1er Entrega/Plantilla.xlsx
+++ b/1er Entrega/Plantilla.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc_ju\OneDrive\Escritorio\Tp4-Simulacion-G5\1er Entrega\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\UTN\Simulación\TP 4\Tp4-Simulacion-G5\1er Entrega\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3F41667-2752-4B13-AF08-5E6A00266121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01A6CCB0-D28D-4191-8DCD-B02B2B795742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -590,7 +590,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -645,26 +645,35 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="46" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="46" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="46" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -691,35 +700,22 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="46" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="46" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="46" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="46" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="46" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1001,76 +997,76 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:BH182"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="8.54296875" customWidth="1"/>
-    <col min="4" max="4" width="13.54296875" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="9" max="9" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.453125" customWidth="1"/>
-    <col min="11" max="11" width="19.453125" customWidth="1"/>
-    <col min="12" max="12" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="17.54296875" customWidth="1"/>
-    <col min="16" max="16" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.54296875" customWidth="1"/>
-    <col min="18" max="18" width="16.81640625" customWidth="1"/>
-    <col min="19" max="20" width="12.453125" customWidth="1"/>
-    <col min="21" max="21" width="12.54296875" customWidth="1"/>
-    <col min="23" max="23" width="11.26953125" customWidth="1"/>
-    <col min="25" max="25" width="9.81640625" customWidth="1"/>
-    <col min="26" max="26" width="11.54296875" customWidth="1"/>
-    <col min="27" max="27" width="12.7265625" customWidth="1"/>
-    <col min="28" max="28" width="10.81640625" customWidth="1"/>
-    <col min="29" max="29" width="10.26953125" customWidth="1"/>
-    <col min="32" max="32" width="15.26953125" customWidth="1"/>
-    <col min="33" max="33" width="16.26953125" customWidth="1"/>
+    <col min="9" max="9" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.42578125" customWidth="1"/>
+    <col min="11" max="11" width="19.42578125" customWidth="1"/>
+    <col min="12" max="12" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="17.5703125" customWidth="1"/>
+    <col min="16" max="16" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.5703125" customWidth="1"/>
+    <col min="18" max="18" width="16.85546875" customWidth="1"/>
+    <col min="19" max="20" width="12.42578125" customWidth="1"/>
+    <col min="21" max="21" width="12.5703125" customWidth="1"/>
+    <col min="23" max="23" width="11.28515625" customWidth="1"/>
+    <col min="25" max="25" width="9.85546875" customWidth="1"/>
+    <col min="26" max="26" width="11.5703125" customWidth="1"/>
+    <col min="27" max="27" width="12.7109375" customWidth="1"/>
+    <col min="28" max="28" width="10.85546875" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="32" max="32" width="15.28515625" customWidth="1"/>
+    <col min="33" max="33" width="16.28515625" customWidth="1"/>
     <col min="34" max="38" width="12" customWidth="1"/>
-    <col min="40" max="40" width="1.1796875" customWidth="1"/>
-    <col min="41" max="43" width="15.54296875" customWidth="1"/>
-    <col min="44" max="44" width="11.7265625" customWidth="1"/>
-    <col min="46" max="46" width="12.36328125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="12.453125" customWidth="1"/>
-    <col min="48" max="48" width="12.26953125" customWidth="1"/>
-    <col min="50" max="50" width="11.1796875" customWidth="1"/>
-    <col min="51" max="51" width="12.26953125" customWidth="1"/>
-    <col min="52" max="52" width="11.453125" customWidth="1"/>
-    <col min="54" max="54" width="13.453125" customWidth="1"/>
-    <col min="55" max="55" width="11.7265625" customWidth="1"/>
+    <col min="40" max="40" width="1.140625" customWidth="1"/>
+    <col min="41" max="43" width="15.5703125" customWidth="1"/>
+    <col min="44" max="44" width="11.7109375" customWidth="1"/>
+    <col min="46" max="46" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="12.42578125" customWidth="1"/>
+    <col min="48" max="48" width="12.28515625" customWidth="1"/>
+    <col min="50" max="50" width="11.140625" customWidth="1"/>
+    <col min="51" max="51" width="12.28515625" customWidth="1"/>
+    <col min="52" max="52" width="11.42578125" customWidth="1"/>
+    <col min="54" max="54" width="13.42578125" customWidth="1"/>
+    <col min="55" max="55" width="11.7109375" customWidth="1"/>
     <col min="56" max="56" width="12" customWidth="1"/>
-    <col min="58" max="58" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:60" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:60" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2"/>
-      <c r="E2" s="33" t="s">
+      <c r="E2" s="46" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="33"/>
-      <c r="G2" s="33"/>
-      <c r="H2" s="33"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
       <c r="J2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="36" t="s">
+      <c r="K2" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="Q2" s="39" t="s">
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="49"/>
+      <c r="Q2" s="52" t="s">
         <v>72</v>
       </c>
-      <c r="R2" s="39"/>
-      <c r="S2" s="39"/>
-      <c r="T2" s="39"/>
-    </row>
-    <row r="3" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="R2" s="52"/>
+      <c r="S2" s="52"/>
+      <c r="T2" s="52"/>
+    </row>
+    <row r="3" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -1083,24 +1079,24 @@
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
-      <c r="Q3" s="26" t="s">
+      <c r="Q3" s="44" t="s">
         <v>71</v>
       </c>
-      <c r="R3" s="26"/>
-      <c r="S3" s="26" t="s">
+      <c r="R3" s="44"/>
+      <c r="S3" s="44" t="s">
         <v>77</v>
       </c>
-      <c r="T3" s="26"/>
-    </row>
-    <row r="4" spans="2:60" x14ac:dyDescent="0.35">
-      <c r="B4" s="26" t="s">
+      <c r="T3" s="44"/>
+    </row>
+    <row r="4" spans="2:60" x14ac:dyDescent="0.25">
+      <c r="B4" s="44" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="26"/>
-      <c r="E4" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="F4" s="26"/>
+      <c r="C4" s="44"/>
+      <c r="E4" s="44" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" s="44"/>
       <c r="G4" s="2">
         <v>10</v>
       </c>
@@ -1119,20 +1115,20 @@
       <c r="O4" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="Q4" s="26" t="s">
+      <c r="Q4" s="44" t="s">
         <v>73</v>
       </c>
-      <c r="R4" s="26"/>
-      <c r="S4" s="26" t="s">
+      <c r="R4" s="44"/>
+      <c r="S4" s="44" t="s">
         <v>75</v>
       </c>
-      <c r="T4" s="26"/>
-    </row>
-    <row r="5" spans="2:60" x14ac:dyDescent="0.35">
-      <c r="E5" s="26" t="s">
+      <c r="T4" s="44"/>
+    </row>
+    <row r="5" spans="2:60" x14ac:dyDescent="0.25">
+      <c r="E5" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="26"/>
+      <c r="F5" s="44"/>
       <c r="G5" s="2">
         <v>18</v>
       </c>
@@ -1154,7 +1150,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="2:60" ht="58" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:60" ht="60" x14ac:dyDescent="0.25">
       <c r="J6" s="5" t="s">
         <v>65</v>
       </c>
@@ -1170,7 +1166,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1180,23 +1176,23 @@
       <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="E7" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26" t="s">
+      <c r="F7" s="44"/>
+      <c r="G7" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="26"/>
-    </row>
-    <row r="8" spans="2:60" x14ac:dyDescent="0.35">
-      <c r="B8" s="26" t="s">
+      <c r="H7" s="44"/>
+    </row>
+    <row r="8" spans="2:60" x14ac:dyDescent="0.25">
+      <c r="B8" s="44" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="44" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -1205,74 +1201,74 @@
       <c r="F8" s="2">
         <v>10</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="53" t="s">
         <v>28</v>
       </c>
-      <c r="H8" s="27"/>
-    </row>
-    <row r="9" spans="2:60" x14ac:dyDescent="0.35">
-      <c r="B9" s="26"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
+      <c r="H8" s="53"/>
+    </row>
+    <row r="9" spans="2:60" x14ac:dyDescent="0.25">
+      <c r="B9" s="44"/>
+      <c r="C9" s="44"/>
+      <c r="D9" s="44"/>
       <c r="E9" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="2">
         <v>20</v>
       </c>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="J9" s="35" t="s">
+      <c r="G9" s="53"/>
+      <c r="H9" s="53"/>
+      <c r="J9" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="35"/>
-      <c r="L9" s="35"/>
-      <c r="M9" s="35"/>
-      <c r="N9" s="35"/>
-      <c r="O9" s="35"/>
-      <c r="P9" s="35"/>
-      <c r="Q9" s="35"/>
-      <c r="R9" s="35"/>
-      <c r="S9" s="35"/>
-      <c r="T9" s="35"/>
-      <c r="U9" s="35"/>
-      <c r="V9" s="35"/>
-      <c r="W9" s="35"/>
-      <c r="X9" s="35"/>
-      <c r="Y9" s="35"/>
-      <c r="Z9" s="35"/>
-      <c r="AA9" s="35"/>
-      <c r="AB9" s="35"/>
-      <c r="AC9" s="35"/>
-      <c r="AD9" s="35"/>
-      <c r="AE9" s="35"/>
-      <c r="AF9" s="35"/>
-      <c r="AG9" s="35"/>
-      <c r="AH9" s="35"/>
-      <c r="AI9" s="35"/>
-      <c r="AJ9" s="35"/>
-      <c r="AK9" s="35"/>
-      <c r="AL9" s="35"/>
-      <c r="AM9" s="35"/>
-      <c r="AN9" s="35"/>
-      <c r="AO9" s="35"/>
-      <c r="AP9" s="35"/>
-      <c r="AQ9" s="35"/>
-      <c r="AR9" s="35"/>
-      <c r="AS9" s="35"/>
-      <c r="AT9" s="35"/>
-      <c r="AU9" s="35"/>
-      <c r="AV9" s="35"/>
-      <c r="AW9" s="35"/>
-      <c r="AX9" s="35"/>
-      <c r="AY9" s="35"/>
-      <c r="AZ9" s="35"/>
-      <c r="BA9" s="35"/>
-      <c r="BB9" s="35"/>
-      <c r="BC9" s="35"/>
-      <c r="BD9" s="35"/>
-    </row>
-    <row r="10" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="K9" s="48"/>
+      <c r="L9" s="48"/>
+      <c r="M9" s="48"/>
+      <c r="N9" s="48"/>
+      <c r="O9" s="48"/>
+      <c r="P9" s="48"/>
+      <c r="Q9" s="48"/>
+      <c r="R9" s="48"/>
+      <c r="S9" s="48"/>
+      <c r="T9" s="48"/>
+      <c r="U9" s="48"/>
+      <c r="V9" s="48"/>
+      <c r="W9" s="48"/>
+      <c r="X9" s="48"/>
+      <c r="Y9" s="48"/>
+      <c r="Z9" s="48"/>
+      <c r="AA9" s="48"/>
+      <c r="AB9" s="48"/>
+      <c r="AC9" s="48"/>
+      <c r="AD9" s="48"/>
+      <c r="AE9" s="48"/>
+      <c r="AF9" s="48"/>
+      <c r="AG9" s="48"/>
+      <c r="AH9" s="48"/>
+      <c r="AI9" s="48"/>
+      <c r="AJ9" s="48"/>
+      <c r="AK9" s="48"/>
+      <c r="AL9" s="48"/>
+      <c r="AM9" s="48"/>
+      <c r="AN9" s="48"/>
+      <c r="AO9" s="48"/>
+      <c r="AP9" s="48"/>
+      <c r="AQ9" s="48"/>
+      <c r="AR9" s="48"/>
+      <c r="AS9" s="48"/>
+      <c r="AT9" s="48"/>
+      <c r="AU9" s="48"/>
+      <c r="AV9" s="48"/>
+      <c r="AW9" s="48"/>
+      <c r="AX9" s="48"/>
+      <c r="AY9" s="48"/>
+      <c r="AZ9" s="48"/>
+      <c r="BA9" s="48"/>
+      <c r="BB9" s="48"/>
+      <c r="BC9" s="48"/>
+      <c r="BD9" s="48"/>
+    </row>
+    <row r="10" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>7</v>
       </c>
@@ -1288,76 +1284,76 @@
       <c r="F10" s="2">
         <v>90</v>
       </c>
-      <c r="G10" s="26" t="s">
+      <c r="G10" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="H10" s="26"/>
-      <c r="AD10" s="28" t="s">
+      <c r="H10" s="44"/>
+      <c r="AD10" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="AE10" s="28"/>
-      <c r="AF10" s="28"/>
-      <c r="AG10" s="28"/>
-      <c r="AH10" s="28"/>
-      <c r="AI10" s="28"/>
-      <c r="AJ10" s="28"/>
-      <c r="AK10" s="28"/>
-      <c r="AL10" s="28"/>
-      <c r="AM10" s="28"/>
+      <c r="AE10" s="54"/>
+      <c r="AF10" s="54"/>
+      <c r="AG10" s="54"/>
+      <c r="AH10" s="54"/>
+      <c r="AI10" s="54"/>
+      <c r="AJ10" s="54"/>
+      <c r="AK10" s="54"/>
+      <c r="AL10" s="54"/>
+      <c r="AM10" s="54"/>
       <c r="AN10" s="2"/>
-      <c r="AO10" s="34" t="s">
+      <c r="AO10" s="47" t="s">
         <v>79</v>
       </c>
-      <c r="AP10" s="34"/>
-      <c r="AQ10" s="34"/>
-      <c r="AR10" s="34"/>
-      <c r="AS10" s="34"/>
-      <c r="AT10" s="34"/>
-      <c r="AU10" s="34"/>
-      <c r="AV10" s="34"/>
-      <c r="AW10" s="34"/>
-      <c r="AX10" s="34"/>
-      <c r="AY10" s="34"/>
-      <c r="AZ10" s="34"/>
-      <c r="BA10" s="34"/>
-      <c r="BB10" s="34"/>
-      <c r="BC10" s="34"/>
-      <c r="BD10" s="34"/>
-    </row>
-    <row r="11" spans="2:60" x14ac:dyDescent="0.35">
-      <c r="I11" s="27" t="s">
+      <c r="AP10" s="47"/>
+      <c r="AQ10" s="47"/>
+      <c r="AR10" s="47"/>
+      <c r="AS10" s="47"/>
+      <c r="AT10" s="47"/>
+      <c r="AU10" s="47"/>
+      <c r="AV10" s="47"/>
+      <c r="AW10" s="47"/>
+      <c r="AX10" s="47"/>
+      <c r="AY10" s="47"/>
+      <c r="AZ10" s="47"/>
+      <c r="BA10" s="47"/>
+      <c r="BB10" s="47"/>
+      <c r="BC10" s="47"/>
+      <c r="BD10" s="47"/>
+    </row>
+    <row r="11" spans="2:60" x14ac:dyDescent="0.25">
+      <c r="I11" s="53" t="s">
         <v>83</v>
       </c>
       <c r="J11" s="8"/>
       <c r="K11" s="9"/>
-      <c r="L11" s="37" t="s">
+      <c r="L11" s="50" t="s">
         <v>71</v>
       </c>
-      <c r="M11" s="37"/>
-      <c r="N11" s="37"/>
-      <c r="O11" s="29" t="s">
+      <c r="M11" s="50"/>
+      <c r="N11" s="50"/>
+      <c r="O11" s="55" t="s">
         <v>76</v>
       </c>
-      <c r="P11" s="29"/>
-      <c r="Q11" s="29"/>
-      <c r="R11" s="29"/>
-      <c r="S11" s="29"/>
-      <c r="T11" s="29"/>
-      <c r="U11" s="29"/>
-      <c r="V11" s="29"/>
-      <c r="W11" s="38" t="s">
+      <c r="P11" s="55"/>
+      <c r="Q11" s="55"/>
+      <c r="R11" s="55"/>
+      <c r="S11" s="55"/>
+      <c r="T11" s="55"/>
+      <c r="U11" s="55"/>
+      <c r="V11" s="55"/>
+      <c r="W11" s="51" t="s">
         <v>77</v>
       </c>
-      <c r="X11" s="38"/>
-      <c r="Y11" s="31" t="s">
+      <c r="X11" s="51"/>
+      <c r="Y11" s="57" t="s">
         <v>68</v>
       </c>
-      <c r="Z11" s="31"/>
-      <c r="AA11" s="30" t="s">
+      <c r="Z11" s="57"/>
+      <c r="AA11" s="56" t="s">
         <v>46</v>
       </c>
-      <c r="AB11" s="30"/>
-      <c r="AC11" s="30"/>
+      <c r="AB11" s="56"/>
+      <c r="AC11" s="56"/>
       <c r="AD11" s="2">
         <v>1</v>
       </c>
@@ -1389,39 +1385,39 @@
         <v>78</v>
       </c>
       <c r="AN11" s="2"/>
-      <c r="AO11" s="26">
+      <c r="AO11" s="44">
         <v>1</v>
       </c>
-      <c r="AP11" s="26"/>
-      <c r="AQ11" s="26"/>
-      <c r="AR11" s="26"/>
-      <c r="AS11" s="26">
+      <c r="AP11" s="44"/>
+      <c r="AQ11" s="44"/>
+      <c r="AR11" s="44"/>
+      <c r="AS11" s="44">
         <v>2</v>
       </c>
-      <c r="AT11" s="26"/>
-      <c r="AU11" s="26"/>
-      <c r="AV11" s="26"/>
-      <c r="AW11" s="26">
+      <c r="AT11" s="44"/>
+      <c r="AU11" s="44"/>
+      <c r="AV11" s="44"/>
+      <c r="AW11" s="44">
         <v>3</v>
       </c>
-      <c r="AX11" s="26"/>
-      <c r="AY11" s="26"/>
-      <c r="AZ11" s="26"/>
-      <c r="BA11" s="26" t="s">
+      <c r="AX11" s="44"/>
+      <c r="AY11" s="44"/>
+      <c r="AZ11" s="44"/>
+      <c r="BA11" s="44" t="s">
         <v>78</v>
       </c>
-      <c r="BB11" s="26"/>
-      <c r="BC11" s="26"/>
-      <c r="BD11" s="26"/>
-      <c r="BE11" s="26" t="s">
+      <c r="BB11" s="44"/>
+      <c r="BC11" s="44"/>
+      <c r="BD11" s="44"/>
+      <c r="BE11" s="44" t="s">
         <v>78</v>
       </c>
-      <c r="BF11" s="26"/>
-      <c r="BG11" s="26"/>
-      <c r="BH11" s="26"/>
-    </row>
-    <row r="12" spans="2:60" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="I12" s="27"/>
+      <c r="BF11" s="44"/>
+      <c r="BG11" s="44"/>
+      <c r="BH11" s="44"/>
+    </row>
+    <row r="12" spans="2:60" ht="60" x14ac:dyDescent="0.25">
+      <c r="I12" s="53"/>
       <c r="J12" s="10" t="s">
         <v>39</v>
       </c>
@@ -1473,7 +1469,7 @@
       <c r="Z12" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="AA12" s="56" t="s">
+      <c r="AA12" s="39" t="s">
         <v>47</v>
       </c>
       <c r="AB12" s="17" t="s">
@@ -1566,7 +1562,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="13" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:60" x14ac:dyDescent="0.25">
       <c r="I13" s="2">
         <v>1</v>
       </c>
@@ -1579,7 +1575,7 @@
       <c r="L13" s="2">
         <v>0.33300000000000002</v>
       </c>
-      <c r="M13" s="40">
+      <c r="M13" s="25">
         <f>-$C$3*(LN(1-L13)) / 1440</f>
         <v>1.265516353332854E-2</v>
       </c>
@@ -1591,24 +1587,24 @@
         <v>53</v>
       </c>
       <c r="P13" s="2"/>
-      <c r="Q13" s="40"/>
+      <c r="Q13" s="25"/>
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
-      <c r="X13" s="40"/>
+      <c r="X13" s="25"/>
       <c r="Y13" s="2">
         <v>0</v>
       </c>
       <c r="Z13" s="2">
         <v>0</v>
       </c>
-      <c r="AA13" s="57">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="40">
+      <c r="AA13" s="40">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="25">
         <v>0</v>
       </c>
       <c r="AC13" s="2">
@@ -1646,14 +1642,14 @@
       <c r="BG13" s="2"/>
       <c r="BH13" s="2"/>
     </row>
-    <row r="14" spans="2:60" x14ac:dyDescent="0.35">
-      <c r="B14" s="26" t="s">
+    <row r="14" spans="2:60" x14ac:dyDescent="0.25">
+      <c r="B14" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="26"/>
-      <c r="F14" s="26"/>
+      <c r="C14" s="44"/>
+      <c r="D14" s="44"/>
+      <c r="E14" s="44"/>
+      <c r="F14" s="44"/>
       <c r="I14" s="2">
         <f>I13+1</f>
         <v>2</v>
@@ -1667,7 +1663,7 @@
       <c r="L14" s="2">
         <v>0.55800000000000005</v>
       </c>
-      <c r="M14" s="40">
+      <c r="M14" s="25">
         <f>-$C$3*(LN(1-L14)) / 1440</f>
         <v>2.5513918653263721E-2</v>
       </c>
@@ -1681,7 +1677,7 @@
       <c r="P14" s="2">
         <v>5.5E-2</v>
       </c>
-      <c r="Q14" s="40">
+      <c r="Q14" s="25">
         <f>($F$8+P14*($F$9-$F$8)) / 1440</f>
         <v>7.3263888888888892E-3</v>
       </c>
@@ -1694,17 +1690,17 @@
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
-      <c r="X14" s="40"/>
+      <c r="X14" s="25"/>
       <c r="Y14" s="2">
         <v>0</v>
       </c>
       <c r="Z14" s="2">
         <v>0</v>
       </c>
-      <c r="AA14" s="57">
-        <v>0</v>
-      </c>
-      <c r="AB14" s="40">
+      <c r="AA14" s="40">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="25">
         <v>0</v>
       </c>
       <c r="AC14" s="2">
@@ -1744,7 +1740,7 @@
       <c r="BG14" s="2"/>
       <c r="BH14" s="2"/>
     </row>
-    <row r="15" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
         <v>24</v>
       </c>
@@ -1768,11 +1764,11 @@
         <f>R14</f>
         <v>0.43664351851851851</v>
       </c>
-      <c r="K15" s="47" t="s">
+      <c r="K15" s="32" t="s">
         <v>92</v>
       </c>
       <c r="L15" s="7"/>
-      <c r="M15" s="41"/>
+      <c r="M15" s="26"/>
       <c r="N15" s="18">
         <f>N14</f>
         <v>0.45483104828289339</v>
@@ -1781,7 +1777,7 @@
         <v>60</v>
       </c>
       <c r="P15" s="20"/>
-      <c r="Q15" s="41"/>
+      <c r="Q15" s="26"/>
       <c r="R15" s="20"/>
       <c r="S15" s="2">
         <v>0.35499999999999998</v>
@@ -1796,7 +1792,7 @@
       <c r="W15" s="2">
         <v>0.187</v>
       </c>
-      <c r="X15" s="44">
+      <c r="X15" s="29">
         <f>-90*LN(1-W15) / 1440</f>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -1806,11 +1802,11 @@
       <c r="Z15" s="2">
         <v>0</v>
       </c>
-      <c r="AA15" s="57">
+      <c r="AA15" s="40">
         <f>Q14</f>
         <v>7.3263888888888892E-3</v>
       </c>
-      <c r="AB15" s="40">
+      <c r="AB15" s="25">
         <v>0</v>
       </c>
       <c r="AC15" s="2">
@@ -1853,7 +1849,7 @@
       <c r="BG15" s="2"/>
       <c r="BH15" s="2"/>
     </row>
-    <row r="16" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
         <v>19</v>
       </c>
@@ -1881,7 +1877,7 @@
         <v>93</v>
       </c>
       <c r="L16" s="1"/>
-      <c r="M16" s="42"/>
+      <c r="M16" s="27"/>
       <c r="N16" s="19">
         <f>N15</f>
         <v>0.45483104828289339</v>
@@ -1890,25 +1886,25 @@
         <v>53</v>
       </c>
       <c r="P16" s="22"/>
-      <c r="Q16" s="42"/>
+      <c r="Q16" s="27"/>
       <c r="R16" s="22"/>
       <c r="S16" s="22"/>
       <c r="T16" s="22"/>
       <c r="U16" s="22"/>
       <c r="V16" s="22"/>
       <c r="W16" s="22"/>
-      <c r="X16" s="40"/>
+      <c r="X16" s="25"/>
       <c r="Y16" s="2">
         <v>0</v>
       </c>
       <c r="Z16" s="2">
         <v>0</v>
       </c>
-      <c r="AA16" s="57">
+      <c r="AA16" s="40">
         <f>AA15</f>
         <v>7.3263888888888892E-3</v>
       </c>
-      <c r="AB16" s="40">
+      <c r="AB16" s="25">
         <f>AB15+X15</f>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -1956,7 +1952,7 @@
       <c r="BG16" s="2"/>
       <c r="BH16" s="2"/>
     </row>
-    <row r="17" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
         <v>20</v>
       </c>
@@ -1986,7 +1982,7 @@
       <c r="L17" s="2">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="M17" s="40">
+      <c r="M17" s="25">
         <f>-$C$3*LN(1-L17) / 1440</f>
         <v>9.3890906884335122E-5</v>
       </c>
@@ -2000,7 +1996,7 @@
       <c r="P17" s="2">
         <v>0.35799999999999998</v>
       </c>
-      <c r="Q17" s="40">
+      <c r="Q17" s="25">
         <f>($F$8+P17*($F$9-$F$8)) / 1440</f>
         <v>9.4305555555555549E-3</v>
       </c>
@@ -2013,18 +2009,18 @@
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
       <c r="W17" s="2"/>
-      <c r="X17" s="40"/>
+      <c r="X17" s="25"/>
       <c r="Y17" s="2">
         <v>0</v>
       </c>
       <c r="Z17" s="2">
         <v>0</v>
       </c>
-      <c r="AA17" s="57">
+      <c r="AA17" s="40">
         <f>AA16+Q18</f>
         <v>1.6756944444444442E-2</v>
       </c>
-      <c r="AB17" s="40">
+      <c r="AB17" s="25">
         <f t="shared" ref="AB17:AB24" si="1">AB16</f>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2065,7 +2061,7 @@
       <c r="BG17" s="2"/>
       <c r="BH17" s="2"/>
     </row>
-    <row r="18" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:60" x14ac:dyDescent="0.25">
       <c r="I18" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -2080,7 +2076,7 @@
       <c r="L18" s="2">
         <v>0.44</v>
       </c>
-      <c r="M18" s="40">
+      <c r="M18" s="25">
         <f>-$C$3*LN(1-L18) / 1440</f>
         <v>1.8119327976654439E-2</v>
       </c>
@@ -2092,7 +2088,7 @@
         <v>61</v>
       </c>
       <c r="P18" s="1"/>
-      <c r="Q18" s="40">
+      <c r="Q18" s="25">
         <f>Q17</f>
         <v>9.4305555555555549E-3</v>
       </c>
@@ -2105,18 +2101,18 @@
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
       <c r="W18" s="2"/>
-      <c r="X18" s="40"/>
+      <c r="X18" s="25"/>
       <c r="Y18" s="2">
         <v>1</v>
       </c>
       <c r="Z18" s="2">
         <v>0</v>
       </c>
-      <c r="AA18" s="57">
+      <c r="AA18" s="40">
         <f>AA17+(J18-J17)</f>
         <v>1.6850835351328773E-2</v>
       </c>
-      <c r="AB18" s="40">
+      <c r="AB18" s="25">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2159,14 +2155,14 @@
       <c r="BG18" s="2"/>
       <c r="BH18" s="2"/>
     </row>
-    <row r="19" spans="2:60" x14ac:dyDescent="0.35">
-      <c r="B19" s="26" t="s">
+    <row r="19" spans="2:60" x14ac:dyDescent="0.25">
+      <c r="B19" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
+      <c r="C19" s="44"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="44"/>
+      <c r="F19" s="44"/>
       <c r="I19" s="2">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2175,12 +2171,12 @@
         <f>R17</f>
         <v>0.46426160383844894</v>
       </c>
-      <c r="K19" s="47" t="s">
+      <c r="K19" s="32" t="s">
         <v>96</v>
       </c>
       <c r="L19" s="1"/>
-      <c r="M19" s="42"/>
-      <c r="N19" s="24">
+      <c r="M19" s="27"/>
+      <c r="N19" s="58">
         <f>N18</f>
         <v>0.47304426716643216</v>
       </c>
@@ -2190,7 +2186,7 @@
       <c r="P19" s="2">
         <v>0.61399999999999999</v>
       </c>
-      <c r="Q19" s="40">
+      <c r="Q19" s="25">
         <f>($F$8+P19*($F$9-$F$8)) / 1440</f>
         <v>1.1208333333333334E-2</v>
       </c>
@@ -2209,18 +2205,18 @@
         <v>55</v>
       </c>
       <c r="W19" s="2"/>
-      <c r="X19" s="40"/>
+      <c r="X19" s="25"/>
       <c r="Y19" s="2">
         <v>0</v>
       </c>
       <c r="Z19" s="2">
         <v>1</v>
       </c>
-      <c r="AA19" s="57">
+      <c r="AA19" s="40">
         <f>AA18+Q17</f>
         <v>2.6281390906884326E-2</v>
       </c>
-      <c r="AB19" s="40">
+      <c r="AB19" s="25">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2266,7 +2262,7 @@
       <c r="BG19" s="2"/>
       <c r="BH19" s="2"/>
     </row>
-    <row r="20" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
         <v>24</v>
       </c>
@@ -2296,7 +2292,7 @@
       <c r="L20" s="2">
         <v>0.22500000000000001</v>
       </c>
-      <c r="M20" s="40">
+      <c r="M20" s="25">
         <f>-$C$3*LN(1-L20) / 1440</f>
         <v>7.9653828008996886E-3</v>
       </c>
@@ -2308,7 +2304,7 @@
         <v>61</v>
       </c>
       <c r="P20" s="2"/>
-      <c r="Q20" s="40">
+      <c r="Q20" s="25">
         <f>Q19</f>
         <v>1.1208333333333334E-2</v>
       </c>
@@ -2321,18 +2317,18 @@
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
       <c r="W20" s="1"/>
-      <c r="X20" s="45"/>
+      <c r="X20" s="30"/>
       <c r="Y20" s="2">
         <v>1</v>
       </c>
       <c r="Z20" s="2">
         <v>1</v>
       </c>
-      <c r="AA20" s="57">
+      <c r="AA20" s="40">
         <f>AA19+Q18</f>
         <v>3.5711946462439879E-2</v>
       </c>
-      <c r="AB20" s="40">
+      <c r="AB20" s="25">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2380,7 +2376,7 @@
       <c r="BG20" s="2"/>
       <c r="BH20" s="2"/>
     </row>
-    <row r="21" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>88</v>
       </c>
@@ -2407,11 +2403,11 @@
         <f>R20</f>
         <v>0.47546993717178226</v>
       </c>
-      <c r="K21" s="47" t="s">
+      <c r="K21" s="32" t="s">
         <v>98</v>
       </c>
       <c r="L21" s="2"/>
-      <c r="M21" s="40"/>
+      <c r="M21" s="25"/>
       <c r="N21" s="19">
         <f>N20</f>
         <v>0.48100964996733186</v>
@@ -2422,7 +2418,7 @@
       <c r="P21" s="2">
         <v>0.26900000000000002</v>
       </c>
-      <c r="Q21" s="40">
+      <c r="Q21" s="25">
         <f>($F$8+P21*($F$9-$F$8)) / 1440</f>
         <v>8.8125000000000009E-3</v>
       </c>
@@ -2441,18 +2437,18 @@
         <v>55</v>
       </c>
       <c r="W21" s="2"/>
-      <c r="X21" s="40"/>
+      <c r="X21" s="25"/>
       <c r="Y21" s="2">
         <v>0</v>
       </c>
       <c r="Z21" s="2">
         <v>2</v>
       </c>
-      <c r="AA21" s="57">
+      <c r="AA21" s="40">
         <f>AA20+(J21-J20)</f>
         <v>3.813761646778998E-2</v>
       </c>
-      <c r="AB21" s="40">
+      <c r="AB21" s="25">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2503,7 +2499,7 @@
       <c r="BG21" s="2"/>
       <c r="BH21" s="2"/>
     </row>
-    <row r="22" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:60" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
         <v>89</v>
       </c>
@@ -2533,7 +2529,7 @@
       <c r="L22" s="2">
         <v>0.57099999999999995</v>
       </c>
-      <c r="M22" s="40">
+      <c r="M22" s="25">
         <f>-$C$3*LN(1-L22) / 1440</f>
         <v>2.6446823751691249E-2</v>
       </c>
@@ -2545,7 +2541,7 @@
         <v>61</v>
       </c>
       <c r="P22" s="2"/>
-      <c r="Q22" s="40">
+      <c r="Q22" s="25">
         <f>Q21</f>
         <v>8.8125000000000009E-3</v>
       </c>
@@ -2558,18 +2554,18 @@
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
       <c r="W22" s="2"/>
-      <c r="X22" s="40"/>
+      <c r="X22" s="25"/>
       <c r="Y22" s="2">
         <v>1</v>
       </c>
       <c r="Z22" s="2">
         <v>2</v>
       </c>
-      <c r="AA22" s="57">
+      <c r="AA22" s="40">
         <f>AA21++J22-J21</f>
         <v>4.3677329263339615E-2</v>
       </c>
-      <c r="AB22" s="40">
+      <c r="AB22" s="25">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
@@ -2622,7 +2618,7 @@
       <c r="BG22" s="2"/>
       <c r="BH22" s="2"/>
     </row>
-    <row r="23" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:60" x14ac:dyDescent="0.25">
       <c r="I23" s="2">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2631,11 +2627,11 @@
         <f>R22</f>
         <v>0.48428243717178227</v>
       </c>
-      <c r="K23" s="47" t="s">
+      <c r="K23" s="32" t="s">
         <v>101</v>
       </c>
       <c r="L23" s="2"/>
-      <c r="M23" s="40"/>
+      <c r="M23" s="25"/>
       <c r="N23" s="18">
         <f>N22</f>
         <v>0.50745647371902314</v>
@@ -2646,7 +2642,7 @@
       <c r="P23" s="2">
         <v>0.81699999999999995</v>
       </c>
-      <c r="Q23" s="40">
+      <c r="Q23" s="25">
         <f>($F$8+P23*($F$9-$F$8)) / 1440</f>
         <v>1.2618055555555556E-2</v>
       </c>
@@ -2667,21 +2663,21 @@
         <v>103</v>
       </c>
       <c r="W23" s="2"/>
-      <c r="X23" s="40"/>
+      <c r="X23" s="25"/>
       <c r="Y23" s="2">
         <v>0</v>
       </c>
       <c r="Z23" s="2">
         <v>2</v>
       </c>
-      <c r="AA23" s="43" t="s">
+      <c r="AA23" s="28" t="s">
         <v>100</v>
       </c>
-      <c r="AB23" s="40">
+      <c r="AB23" s="25">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
-      <c r="AC23" s="52">
+      <c r="AC23" s="35">
         <v>0</v>
       </c>
       <c r="AD23" s="2"/>
@@ -2728,14 +2724,14 @@
       <c r="BG23" s="2"/>
       <c r="BH23" s="2"/>
     </row>
-    <row r="24" spans="2:60" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="32" t="s">
+    <row r="24" spans="2:60" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="32"/>
+      <c r="C24" s="45"/>
+      <c r="D24" s="45"/>
+      <c r="E24" s="45"/>
+      <c r="F24" s="45"/>
       <c r="I24" s="2">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2744,11 +2740,11 @@
         <f>R23</f>
         <v>0.49690049272733783</v>
       </c>
-      <c r="K24" s="47" t="s">
+      <c r="K24" s="32" t="s">
         <v>104</v>
       </c>
       <c r="L24" s="2"/>
-      <c r="M24" s="40"/>
+      <c r="M24" s="25"/>
       <c r="N24" s="18">
         <f>N23</f>
         <v>0.50745647371902314</v>
@@ -2757,7 +2753,7 @@
         <v>60</v>
       </c>
       <c r="P24" s="2"/>
-      <c r="Q24" s="40"/>
+      <c r="Q24" s="25"/>
       <c r="R24" s="2"/>
       <c r="S24" s="2">
         <v>4.3999999999999997E-2</v>
@@ -2774,7 +2770,7 @@
       <c r="W24" s="2">
         <v>5.5E-2</v>
       </c>
-      <c r="X24" s="44">
+      <c r="X24" s="29">
         <f>-90*LN(1-W24) / 1440</f>
         <v>3.5356469680246473E-3</v>
       </c>
@@ -2784,12 +2780,12 @@
       <c r="Z24" s="2">
         <v>1</v>
       </c>
-      <c r="AA24" s="43"/>
-      <c r="AB24" s="40">
+      <c r="AA24" s="28"/>
+      <c r="AB24" s="25">
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
-      <c r="AC24" s="52">
+      <c r="AC24" s="35">
         <v>0</v>
       </c>
       <c r="AD24" s="2"/>
@@ -2836,12 +2832,12 @@
       <c r="BG24" s="2"/>
       <c r="BH24" s="2"/>
     </row>
-    <row r="25" spans="2:60" x14ac:dyDescent="0.35">
-      <c r="B25" s="32"/>
-      <c r="C25" s="32"/>
-      <c r="D25" s="32"/>
-      <c r="E25" s="32"/>
-      <c r="F25" s="32"/>
+    <row r="25" spans="2:60" x14ac:dyDescent="0.25">
+      <c r="B25" s="45"/>
+      <c r="C25" s="45"/>
+      <c r="D25" s="45"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="45"/>
       <c r="I25" s="2">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2854,7 +2850,7 @@
         <v>105</v>
       </c>
       <c r="L25" s="2"/>
-      <c r="M25" s="40"/>
+      <c r="M25" s="25"/>
       <c r="N25" s="19">
         <f>N24</f>
         <v>0.50745647371902314</v>
@@ -2863,7 +2859,7 @@
         <v>60</v>
       </c>
       <c r="P25" s="2"/>
-      <c r="Q25" s="40"/>
+      <c r="Q25" s="25"/>
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
       <c r="T25" s="2"/>
@@ -2872,7 +2868,7 @@
       <c r="W25" s="2">
         <v>0.20899999999999999</v>
       </c>
-      <c r="X25" s="46">
+      <c r="X25" s="31">
         <f>-90*LN(1-W25) / 1440</f>
         <v>1.4653581950905195E-2</v>
       </c>
@@ -2882,12 +2878,12 @@
       <c r="Z25" s="2">
         <v>0</v>
       </c>
-      <c r="AA25" s="43"/>
-      <c r="AB25" s="43">
+      <c r="AA25" s="28"/>
+      <c r="AB25" s="28">
         <f>AB24+X24</f>
         <v>1.6474657557670053E-2</v>
       </c>
-      <c r="AC25" s="52">
+      <c r="AC25" s="35">
         <v>0</v>
       </c>
       <c r="AD25" s="2"/>
@@ -2935,7 +2931,7 @@
       <c r="BG25" s="2"/>
       <c r="BH25" s="2"/>
     </row>
-    <row r="26" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:60" x14ac:dyDescent="0.25">
       <c r="I26" s="2">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2949,7 +2945,7 @@
       <c r="L26" s="2">
         <v>0.9</v>
       </c>
-      <c r="M26" s="40">
+      <c r="M26" s="25">
         <f>-$C$3*LN(1-L26) / 1440</f>
         <v>7.1955784156063934E-2</v>
       </c>
@@ -2963,7 +2959,7 @@
       <c r="P26" s="2">
         <v>0.89300000000000002</v>
       </c>
-      <c r="Q26" s="40">
+      <c r="Q26" s="25">
         <f>($F$8+P26*($F$9-$F$8)) / 1440</f>
         <v>1.3145833333333332E-2</v>
       </c>
@@ -2976,7 +2972,7 @@
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
       <c r="W26" s="2"/>
-      <c r="X26" s="46">
+      <c r="X26" s="31">
         <f>AZ26</f>
         <v>7.6332479272445495E-3</v>
       </c>
@@ -2986,12 +2982,12 @@
       <c r="Z26" s="2">
         <v>1</v>
       </c>
-      <c r="AA26" s="43"/>
-      <c r="AB26" s="43">
+      <c r="AA26" s="28"/>
+      <c r="AB26" s="28">
         <f>AB25</f>
         <v>1.6474657557670053E-2</v>
       </c>
-      <c r="AC26" s="52">
+      <c r="AC26" s="35">
         <v>0</v>
       </c>
       <c r="AD26" s="2"/>
@@ -3036,7 +3032,7 @@
       <c r="BG26" s="2"/>
       <c r="BH26" s="2"/>
     </row>
-    <row r="27" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:60" x14ac:dyDescent="0.25">
       <c r="I27" s="2">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -3045,11 +3041,11 @@
         <f>R26</f>
         <v>0.52059953703703699</v>
       </c>
-      <c r="K27" s="47" t="s">
+      <c r="K27" s="32" t="s">
         <v>107</v>
       </c>
       <c r="L27" s="2"/>
-      <c r="M27" s="40"/>
+      <c r="M27" s="25"/>
       <c r="N27" s="18">
         <f>N26</f>
         <v>0.57940948785976765</v>
@@ -3058,7 +3054,7 @@
         <v>60</v>
       </c>
       <c r="P27" s="2"/>
-      <c r="Q27" s="40"/>
+      <c r="Q27" s="25"/>
       <c r="R27" s="2"/>
       <c r="S27" s="2">
         <v>0.89900000000000002</v>
@@ -3071,7 +3067,7 @@
         <v>55</v>
       </c>
       <c r="W27" s="2"/>
-      <c r="X27" s="44">
+      <c r="X27" s="29">
         <f>X26</f>
         <v>7.6332479272445495E-3</v>
       </c>
@@ -3081,12 +3077,12 @@
       <c r="Z27" s="2">
         <v>0</v>
       </c>
-      <c r="AA27" s="43"/>
-      <c r="AB27" s="43">
+      <c r="AA27" s="28"/>
+      <c r="AB27" s="28">
         <f>AB26</f>
         <v>1.6474657557670053E-2</v>
       </c>
-      <c r="AC27" s="52">
+      <c r="AC27" s="35">
         <v>0</v>
       </c>
       <c r="AD27" s="2"/>
@@ -3129,7 +3125,7 @@
       <c r="BG27" s="2"/>
       <c r="BH27" s="2"/>
     </row>
-    <row r="28" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:60" x14ac:dyDescent="0.25">
       <c r="I28" s="2">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -3138,11 +3134,11 @@
         <f>J27+X27</f>
         <v>0.5282327849642815</v>
       </c>
-      <c r="K28" s="48" t="s">
+      <c r="K28" s="2" t="s">
         <v>108</v>
       </c>
       <c r="L28" s="2"/>
-      <c r="M28" s="40"/>
+      <c r="M28" s="25"/>
       <c r="N28" s="19">
         <f>N27</f>
         <v>0.57940948785976765</v>
@@ -3151,26 +3147,26 @@
         <v>53</v>
       </c>
       <c r="P28" s="2"/>
-      <c r="Q28" s="40"/>
+      <c r="Q28" s="25"/>
       <c r="R28" s="2"/>
       <c r="S28" s="2"/>
       <c r="T28" s="2"/>
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
       <c r="W28" s="2"/>
-      <c r="X28" s="40"/>
+      <c r="X28" s="25"/>
       <c r="Y28" s="2">
         <v>0</v>
       </c>
       <c r="Z28" s="2">
         <v>0</v>
       </c>
-      <c r="AA28" s="43"/>
-      <c r="AB28" s="43">
+      <c r="AA28" s="28"/>
+      <c r="AB28" s="28">
         <f>X25+AB27</f>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC28" s="52">
+      <c r="AC28" s="35">
         <v>0</v>
       </c>
       <c r="AD28" s="2"/>
@@ -3213,7 +3209,7 @@
       <c r="BG28" s="2"/>
       <c r="BH28" s="2"/>
     </row>
-    <row r="29" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:60" x14ac:dyDescent="0.25">
       <c r="I29" s="2">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -3228,7 +3224,7 @@
       <c r="L29" s="2">
         <v>0.87</v>
       </c>
-      <c r="M29" s="40">
+      <c r="M29" s="25">
         <f>-$C$3*LN(1-L29) / 1440</f>
         <v>6.3756900891454832E-2</v>
       </c>
@@ -3242,7 +3238,7 @@
       <c r="P29" s="2">
         <v>0.93</v>
       </c>
-      <c r="Q29" s="40">
+      <c r="Q29" s="25">
         <f>($F$8+P29*($F$9-$F$8)) / 1440</f>
         <v>1.3402777777777779E-2</v>
       </c>
@@ -3255,19 +3251,19 @@
       <c r="U29" s="2"/>
       <c r="V29" s="2"/>
       <c r="W29" s="2"/>
-      <c r="X29" s="40"/>
+      <c r="X29" s="25"/>
       <c r="Y29" s="2">
         <v>0</v>
       </c>
       <c r="Z29" s="2">
         <v>0</v>
       </c>
-      <c r="AA29" s="43"/>
-      <c r="AB29" s="43">
+      <c r="AA29" s="28"/>
+      <c r="AB29" s="28">
         <f>AB28</f>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC29" s="52">
+      <c r="AC29" s="35">
         <v>0</v>
       </c>
       <c r="AD29" s="2"/>
@@ -3304,20 +3300,20 @@
       <c r="BG29" s="2"/>
       <c r="BH29" s="2"/>
     </row>
-    <row r="30" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:60" x14ac:dyDescent="0.25">
       <c r="I30" s="2">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="J30" s="51">
+      <c r="J30" s="18">
         <f>R29</f>
         <v>0.59281226563754541</v>
       </c>
-      <c r="K30" s="47" t="s">
+      <c r="K30" s="32" t="s">
         <v>110</v>
       </c>
       <c r="L30" s="2"/>
-      <c r="M30" s="40"/>
+      <c r="M30" s="25"/>
       <c r="N30" s="19">
         <f>N29</f>
         <v>0.64316638875122245</v>
@@ -3326,7 +3322,7 @@
         <v>60</v>
       </c>
       <c r="P30" s="2"/>
-      <c r="Q30" s="40"/>
+      <c r="Q30" s="25"/>
       <c r="R30" s="18"/>
       <c r="S30" s="2">
         <v>0.23300000000000001</v>
@@ -3344,7 +3340,7 @@
         <f>0.882</f>
         <v>0.88200000000000001</v>
       </c>
-      <c r="X30" s="40">
+      <c r="X30" s="25">
         <f>-90*LN(1-W30) / 1440</f>
         <v>0.13356691590727951</v>
       </c>
@@ -3354,12 +3350,12 @@
       <c r="Z30" s="2">
         <v>0</v>
       </c>
-      <c r="AA30" s="43"/>
-      <c r="AB30" s="43">
+      <c r="AA30" s="28"/>
+      <c r="AB30" s="28">
         <f t="shared" ref="AB30:AB36" si="4">AB29</f>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC30" s="52">
+      <c r="AC30" s="35">
         <v>0</v>
       </c>
       <c r="AD30" s="2"/>
@@ -3399,12 +3395,12 @@
       <c r="BG30" s="2"/>
       <c r="BH30" s="2"/>
     </row>
-    <row r="31" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:60" x14ac:dyDescent="0.25">
       <c r="I31" s="2">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="J31" s="51">
+      <c r="J31" s="18">
         <f>N30</f>
         <v>0.64316638875122245</v>
       </c>
@@ -3414,7 +3410,7 @@
       <c r="L31" s="2">
         <v>0.21199999999999999</v>
       </c>
-      <c r="M31" s="40">
+      <c r="M31" s="25">
         <f>-$C$3*LN(1-L31) / 1440</f>
         <v>7.4455371601330599E-3</v>
       </c>
@@ -3422,17 +3418,17 @@
         <f>J31+M31</f>
         <v>0.65061192591135553</v>
       </c>
-      <c r="O31" s="51" t="s">
+      <c r="O31" s="18" t="s">
         <v>61</v>
       </c>
       <c r="P31" s="2">
         <v>0.51200000000000001</v>
       </c>
-      <c r="Q31" s="40">
+      <c r="Q31" s="25">
         <f>($F$8+P31*($F$9-$F$8)) / 1440</f>
         <v>1.0500000000000001E-2</v>
       </c>
-      <c r="R31" s="58">
+      <c r="R31" s="41">
         <f>Q31+J31</f>
         <v>0.6536663887512224</v>
       </c>
@@ -3441,22 +3437,22 @@
       <c r="U31" s="2"/>
       <c r="V31" s="2"/>
       <c r="W31" s="2"/>
-      <c r="X31" s="40">
+      <c r="X31" s="25">
         <f>BD31</f>
         <v>8.3212792793602469E-2</v>
       </c>
-      <c r="Y31" s="48">
-        <v>0</v>
-      </c>
-      <c r="Z31" s="48">
-        <v>0</v>
-      </c>
-      <c r="AA31" s="43"/>
-      <c r="AB31" s="43">
+      <c r="Y31" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="2">
+        <v>0</v>
+      </c>
+      <c r="AA31" s="28"/>
+      <c r="AB31" s="28">
         <f t="shared" si="4"/>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC31" s="52">
+      <c r="AC31" s="35">
         <v>0</v>
       </c>
       <c r="AD31" s="2"/>
@@ -3492,7 +3488,7 @@
         <v>0.59281226563754541</v>
       </c>
       <c r="BC31" s="2"/>
-      <c r="BD31" s="40">
+      <c r="BD31" s="25">
         <f>X30-(J31-BB30)</f>
         <v>8.3212792793602469E-2</v>
       </c>
@@ -3501,12 +3497,12 @@
       <c r="BG31" s="2"/>
       <c r="BH31" s="2"/>
     </row>
-    <row r="32" spans="2:60" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:60" x14ac:dyDescent="0.25">
       <c r="I32" s="2">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="J32" s="51">
+      <c r="J32" s="18">
         <f>N31</f>
         <v>0.65061192591135553</v>
       </c>
@@ -3516,7 +3512,7 @@
       <c r="L32" s="2">
         <v>0.91200000000000003</v>
       </c>
-      <c r="M32" s="40">
+      <c r="M32" s="25">
         <f>-$C$3*LN(1-L32) / 1440</f>
         <v>7.5950577015747839E-2</v>
       </c>
@@ -3524,36 +3520,36 @@
         <f>M32+J32</f>
         <v>0.72656250292710334</v>
       </c>
-      <c r="O32" s="51" t="s">
+      <c r="O32" s="18" t="s">
         <v>61</v>
       </c>
       <c r="P32" s="2"/>
-      <c r="Q32" s="40"/>
+      <c r="Q32" s="25"/>
       <c r="R32" s="19">
         <f>R31</f>
         <v>0.6536663887512224</v>
       </c>
-      <c r="S32" s="25"/>
+      <c r="S32" s="24"/>
       <c r="T32" s="2"/>
       <c r="U32" s="2"/>
       <c r="V32" s="2"/>
       <c r="W32" s="2"/>
-      <c r="X32" s="40">
+      <c r="X32" s="25">
         <f>X31</f>
         <v>8.3212792793602469E-2</v>
       </c>
-      <c r="Y32" s="48">
+      <c r="Y32" s="2">
         <v>1</v>
       </c>
       <c r="Z32" s="2">
         <v>0</v>
       </c>
-      <c r="AA32" s="43"/>
-      <c r="AB32" s="43">
+      <c r="AA32" s="28"/>
+      <c r="AB32" s="28">
         <f t="shared" si="4"/>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC32" s="52">
+      <c r="AC32" s="35">
         <v>0</v>
       </c>
       <c r="AD32" s="2"/>
@@ -3597,31 +3593,31 @@
       <c r="BG32" s="2"/>
       <c r="BH32" s="2"/>
     </row>
-    <row r="33" spans="9:60" x14ac:dyDescent="0.35">
+    <row r="33" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I33" s="2">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="J33" s="51">
+      <c r="J33" s="18">
         <f>R32</f>
         <v>0.6536663887512224</v>
       </c>
-      <c r="K33" s="47" t="s">
+      <c r="K33" s="32" t="s">
         <v>112</v>
       </c>
       <c r="L33" s="2"/>
-      <c r="M33" s="40"/>
+      <c r="M33" s="25"/>
       <c r="N33" s="18">
         <f>N32</f>
         <v>0.72656250292710334</v>
       </c>
-      <c r="O33" s="51" t="s">
+      <c r="O33" s="18" t="s">
         <v>61</v>
       </c>
       <c r="P33" s="2">
         <v>0.314</v>
       </c>
-      <c r="Q33" s="40">
+      <c r="Q33" s="25">
         <f>($F$8+P33*($F$9-$F$8)) / 1440</f>
         <v>9.1250000000000012E-3</v>
       </c>
@@ -3642,22 +3638,22 @@
         <v>103</v>
       </c>
       <c r="W33" s="2"/>
-      <c r="X33" s="40">
+      <c r="X33" s="25">
         <f>X32</f>
         <v>8.3212792793602469E-2</v>
       </c>
-      <c r="Y33" s="48">
+      <c r="Y33" s="2">
         <v>0</v>
       </c>
       <c r="Z33" s="2">
         <v>0</v>
       </c>
-      <c r="AA33" s="43"/>
-      <c r="AB33" s="43">
+      <c r="AA33" s="28"/>
+      <c r="AB33" s="28">
         <f t="shared" si="4"/>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC33" s="52">
+      <c r="AC33" s="35">
         <v>0</v>
       </c>
       <c r="AD33" s="2"/>
@@ -3667,7 +3663,7 @@
       <c r="AH33" s="2"/>
       <c r="AI33" s="2"/>
       <c r="AJ33" s="2"/>
-      <c r="AK33" s="59"/>
+      <c r="AK33" s="42"/>
       <c r="AL33" s="2" t="s">
         <v>84</v>
       </c>
@@ -3699,7 +3695,7 @@
       <c r="BG33" s="2"/>
       <c r="BH33" s="2"/>
     </row>
-    <row r="34" spans="9:60" x14ac:dyDescent="0.35">
+    <row r="34" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I34" s="2">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -3708,20 +3704,20 @@
         <f>R33</f>
         <v>0.66279138875122245</v>
       </c>
-      <c r="K34" s="47" t="s">
+      <c r="K34" s="32" t="s">
         <v>114</v>
       </c>
       <c r="L34" s="2"/>
-      <c r="M34" s="40"/>
+      <c r="M34" s="25"/>
       <c r="N34" s="19">
         <f>N33</f>
         <v>0.72656250292710334</v>
       </c>
-      <c r="O34" s="51" t="s">
+      <c r="O34" s="18" t="s">
         <v>60</v>
       </c>
       <c r="P34" s="2"/>
-      <c r="Q34" s="40"/>
+      <c r="Q34" s="25"/>
       <c r="R34" s="18"/>
       <c r="S34" s="2">
         <v>0.40300000000000002</v>
@@ -3734,22 +3730,22 @@
         <v>55</v>
       </c>
       <c r="W34" s="2"/>
-      <c r="X34" s="40">
+      <c r="X34" s="25">
         <f>X33</f>
         <v>8.3212792793602469E-2</v>
       </c>
-      <c r="Y34" s="48">
+      <c r="Y34" s="2">
         <v>0</v>
       </c>
       <c r="Z34" s="2">
         <v>1</v>
       </c>
-      <c r="AA34" s="43"/>
-      <c r="AB34" s="43">
+      <c r="AA34" s="28"/>
+      <c r="AB34" s="28">
         <f t="shared" si="4"/>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC34" s="52">
+      <c r="AC34" s="35">
         <v>0</v>
       </c>
       <c r="AD34" s="2"/>
@@ -3794,12 +3790,12 @@
       <c r="BG34" s="2"/>
       <c r="BH34" s="2"/>
     </row>
-    <row r="35" spans="9:60" x14ac:dyDescent="0.35">
+    <row r="35" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I35" s="2">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="J35" s="51">
+      <c r="J35" s="18">
         <f>N34</f>
         <v>0.72656250292710334</v>
       </c>
@@ -3809,7 +3805,7 @@
       <c r="L35" s="2">
         <v>0.69299999999999995</v>
       </c>
-      <c r="M35" s="40">
+      <c r="M35" s="25">
         <f>-$C$3*LN(1-L35) / 1440</f>
         <v>3.6903360356091867E-2</v>
       </c>
@@ -3817,13 +3813,13 @@
         <f>M35+J35</f>
         <v>0.76346586328319521</v>
       </c>
-      <c r="O35" s="51" t="s">
+      <c r="O35" s="18" t="s">
         <v>61</v>
       </c>
       <c r="P35" s="2">
         <v>0.12</v>
       </c>
-      <c r="Q35" s="40">
+      <c r="Q35" s="25">
         <f>($F$8+P35*($F$9-$F$8)) / 1440</f>
         <v>7.7777777777777776E-3</v>
       </c>
@@ -3836,22 +3832,22 @@
       <c r="U35" s="2"/>
       <c r="V35" s="2"/>
       <c r="W35" s="2"/>
-      <c r="X35" s="40">
+      <c r="X35" s="25">
         <f>BD35</f>
         <v>1.9441678617721586E-2</v>
       </c>
-      <c r="Y35" s="48">
+      <c r="Y35" s="2">
         <v>0</v>
       </c>
       <c r="Z35" s="2">
         <v>1</v>
       </c>
-      <c r="AA35" s="43"/>
-      <c r="AB35" s="43">
+      <c r="AA35" s="28"/>
+      <c r="AB35" s="28">
         <f t="shared" si="4"/>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC35" s="52">
+      <c r="AC35" s="35">
         <v>0</v>
       </c>
       <c r="AD35" s="2"/>
@@ -3887,7 +3883,7 @@
         <v>0.59281226563754541</v>
       </c>
       <c r="BC35" s="2"/>
-      <c r="BD35" s="40">
+      <c r="BD35" s="25">
         <f>X34-(J35-J34)</f>
         <v>1.9441678617721586E-2</v>
       </c>
@@ -3901,48 +3897,48 @@
       <c r="BG35" s="2"/>
       <c r="BH35" s="2"/>
     </row>
-    <row r="36" spans="9:60" x14ac:dyDescent="0.35">
+    <row r="36" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I36" s="2">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="J36" s="51">
+      <c r="J36" s="18">
         <f>R35</f>
         <v>0.73434028070488111</v>
       </c>
-      <c r="K36" s="47" t="s">
+      <c r="K36" s="32" t="s">
         <v>116</v>
       </c>
       <c r="L36" s="2"/>
-      <c r="M36" s="40"/>
+      <c r="M36" s="25"/>
       <c r="N36" s="18">
         <f>N35</f>
         <v>0.76346586328319521</v>
       </c>
-      <c r="O36" s="51" t="s">
+      <c r="O36" s="18" t="s">
         <v>60</v>
       </c>
       <c r="P36" s="2"/>
-      <c r="Q36" s="40"/>
+      <c r="Q36" s="25"/>
       <c r="R36" s="18"/>
       <c r="S36" s="2"/>
       <c r="T36" s="2"/>
       <c r="U36" s="2"/>
       <c r="V36" s="2"/>
       <c r="W36" s="2"/>
-      <c r="X36" s="40"/>
-      <c r="Y36" s="48">
+      <c r="X36" s="25"/>
+      <c r="Y36" s="2">
         <v>0</v>
       </c>
       <c r="Z36" s="2">
         <v>1</v>
       </c>
-      <c r="AA36" s="43"/>
-      <c r="AB36" s="43">
+      <c r="AA36" s="28"/>
+      <c r="AB36" s="28">
         <f t="shared" si="4"/>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC36" s="52">
+      <c r="AC36" s="35">
         <v>0</v>
       </c>
       <c r="AD36" s="2"/>
@@ -3987,133 +3983,133 @@
       <c r="BG36" s="2"/>
       <c r="BH36" s="2"/>
     </row>
-    <row r="37" spans="9:60" x14ac:dyDescent="0.35">
+    <row r="37" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I37" s="2">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="J37" s="50">
+      <c r="J37" s="34">
         <f>J36+X35</f>
         <v>0.75378195932260272</v>
       </c>
-      <c r="K37" s="60" t="s">
+      <c r="K37" s="43" t="s">
         <v>117</v>
       </c>
-      <c r="L37" s="53"/>
-      <c r="M37" s="55"/>
-      <c r="N37" s="50">
+      <c r="L37" s="36"/>
+      <c r="M37" s="38"/>
+      <c r="N37" s="34">
         <f>N36</f>
         <v>0.76346586328319521</v>
       </c>
-      <c r="O37" s="53" t="s">
+      <c r="O37" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="P37" s="53"/>
-      <c r="Q37" s="55"/>
-      <c r="R37" s="50"/>
-      <c r="S37" s="53"/>
-      <c r="T37" s="53"/>
-      <c r="U37" s="53"/>
-      <c r="V37" s="53"/>
-      <c r="W37" s="53"/>
-      <c r="X37" s="55"/>
-      <c r="Y37" s="53">
-        <v>0</v>
-      </c>
-      <c r="Z37" s="53">
-        <v>0</v>
-      </c>
-      <c r="AA37" s="55"/>
-      <c r="AB37" s="55">
+      <c r="P37" s="36"/>
+      <c r="Q37" s="38"/>
+      <c r="R37" s="34"/>
+      <c r="S37" s="36"/>
+      <c r="T37" s="36"/>
+      <c r="U37" s="36"/>
+      <c r="V37" s="36"/>
+      <c r="W37" s="36"/>
+      <c r="X37" s="38"/>
+      <c r="Y37" s="36">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="36">
+        <v>0</v>
+      </c>
+      <c r="AA37" s="38"/>
+      <c r="AB37" s="38">
         <f>AB36+X30</f>
         <v>0.16469515541585475</v>
       </c>
-      <c r="AC37" s="53"/>
-      <c r="AD37" s="53"/>
-      <c r="AE37" s="53"/>
-      <c r="AF37" s="53"/>
-      <c r="AG37" s="53"/>
-      <c r="AH37" s="53"/>
-      <c r="AI37" s="53"/>
-      <c r="AJ37" s="53"/>
-      <c r="AK37" s="53"/>
-      <c r="AL37" s="53"/>
-      <c r="AM37" s="53"/>
-      <c r="AN37" s="53"/>
-      <c r="AO37" s="53"/>
-      <c r="AP37" s="53"/>
-      <c r="AQ37" s="53"/>
-      <c r="AR37" s="53"/>
-      <c r="AS37" s="53"/>
-      <c r="AT37" s="53"/>
-      <c r="AU37" s="53"/>
-      <c r="AV37" s="53"/>
-      <c r="AW37" s="53"/>
-      <c r="AX37" s="53"/>
-      <c r="AY37" s="53"/>
-      <c r="AZ37" s="53"/>
-      <c r="BA37" s="53"/>
-      <c r="BB37" s="50">
+      <c r="AC37" s="36"/>
+      <c r="AD37" s="36"/>
+      <c r="AE37" s="36"/>
+      <c r="AF37" s="36"/>
+      <c r="AG37" s="36"/>
+      <c r="AH37" s="36"/>
+      <c r="AI37" s="36"/>
+      <c r="AJ37" s="36"/>
+      <c r="AK37" s="36"/>
+      <c r="AL37" s="36"/>
+      <c r="AM37" s="36"/>
+      <c r="AN37" s="36"/>
+      <c r="AO37" s="36"/>
+      <c r="AP37" s="36"/>
+      <c r="AQ37" s="36"/>
+      <c r="AR37" s="36"/>
+      <c r="AS37" s="36"/>
+      <c r="AT37" s="36"/>
+      <c r="AU37" s="36"/>
+      <c r="AV37" s="36"/>
+      <c r="AW37" s="36"/>
+      <c r="AX37" s="36"/>
+      <c r="AY37" s="36"/>
+      <c r="AZ37" s="36"/>
+      <c r="BA37" s="36"/>
+      <c r="BB37" s="34">
         <f>BB36</f>
         <v>0.59281226563754541</v>
       </c>
-      <c r="BC37" s="50">
+      <c r="BC37" s="34">
         <f>J37</f>
         <v>0.75378195932260272</v>
       </c>
-      <c r="BD37" s="53"/>
-      <c r="BE37" s="53" t="s">
+      <c r="BD37" s="36"/>
+      <c r="BE37" s="36" t="s">
         <v>90</v>
       </c>
-      <c r="BF37" s="50">
+      <c r="BF37" s="34">
         <f>BF36</f>
         <v>0.66279138875122245</v>
       </c>
-      <c r="BG37" s="53"/>
-      <c r="BH37" s="53"/>
-    </row>
-    <row r="38" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="BG37" s="36"/>
+      <c r="BH37" s="36"/>
+    </row>
+    <row r="38" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I38" s="2">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="M38" s="43"/>
-      <c r="Q38" s="43"/>
-      <c r="R38" s="49"/>
-      <c r="T38" s="49"/>
-      <c r="X38" s="43"/>
-      <c r="AA38" s="43"/>
-      <c r="AB38" s="43"/>
-      <c r="BB38" s="54"/>
-      <c r="BC38" s="54"/>
-      <c r="BD38" s="54"/>
-    </row>
-    <row r="39" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="M38" s="28"/>
+      <c r="Q38" s="28"/>
+      <c r="R38" s="33"/>
+      <c r="T38" s="33"/>
+      <c r="X38" s="28"/>
+      <c r="AA38" s="28"/>
+      <c r="AB38" s="28"/>
+      <c r="BB38" s="37"/>
+      <c r="BC38" s="37"/>
+      <c r="BD38" s="37"/>
+    </row>
+    <row r="39" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I39" s="2">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="M39" s="43"/>
-      <c r="Q39" s="43"/>
-      <c r="R39" s="49"/>
-      <c r="X39" s="43"/>
-      <c r="AA39" s="43"/>
-      <c r="AB39" s="43"/>
-    </row>
-    <row r="40" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="M39" s="28"/>
+      <c r="Q39" s="28"/>
+      <c r="R39" s="33"/>
+      <c r="X39" s="28"/>
+      <c r="AA39" s="28"/>
+      <c r="AB39" s="28"/>
+    </row>
+    <row r="40" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I40" s="2">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="M40" s="43"/>
-      <c r="Q40" s="43"/>
-      <c r="R40" s="49"/>
-      <c r="T40" s="49"/>
-      <c r="X40" s="43"/>
-      <c r="AA40" s="43"/>
-      <c r="AB40" s="43"/>
-    </row>
-    <row r="41" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="M40" s="28"/>
+      <c r="Q40" s="28"/>
+      <c r="R40" s="33"/>
+      <c r="T40" s="33"/>
+      <c r="X40" s="28"/>
+      <c r="AA40" s="28"/>
+      <c r="AB40" s="28"/>
+    </row>
+    <row r="41" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I41" s="2">
         <f t="shared" si="0"/>
         <v>29</v>
@@ -4121,155 +4117,155 @@
       <c r="N41" t="s">
         <v>118</v>
       </c>
-      <c r="Q41" s="43"/>
-      <c r="R41" s="49"/>
-      <c r="X41" s="43"/>
-      <c r="AA41" s="43"/>
-      <c r="AB41" s="43"/>
-    </row>
-    <row r="42" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="Q41" s="28"/>
+      <c r="R41" s="33"/>
+      <c r="X41" s="28"/>
+      <c r="AA41" s="28"/>
+      <c r="AB41" s="28"/>
+    </row>
+    <row r="42" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I42" s="2">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="M42" s="43"/>
-      <c r="Q42" s="43"/>
-      <c r="R42" s="49"/>
-      <c r="X42" s="43"/>
-      <c r="AA42" s="43"/>
-      <c r="AB42" s="43"/>
-    </row>
-    <row r="43" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="M42" s="28"/>
+      <c r="Q42" s="28"/>
+      <c r="R42" s="33"/>
+      <c r="X42" s="28"/>
+      <c r="AA42" s="28"/>
+      <c r="AB42" s="28"/>
+    </row>
+    <row r="43" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I43" s="2">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="M43" s="43"/>
-      <c r="Q43" s="43"/>
-      <c r="R43" s="49"/>
-      <c r="X43" s="43"/>
-      <c r="AA43" s="43"/>
-      <c r="AB43" s="43"/>
-    </row>
-    <row r="44" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="M43" s="28"/>
+      <c r="Q43" s="28"/>
+      <c r="R43" s="33"/>
+      <c r="X43" s="28"/>
+      <c r="AA43" s="28"/>
+      <c r="AB43" s="28"/>
+    </row>
+    <row r="44" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I44" s="2">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="M44" s="43"/>
-      <c r="Q44" s="43"/>
-      <c r="R44" s="49"/>
-      <c r="X44" s="43"/>
-      <c r="AA44" s="43"/>
-      <c r="AB44" s="43"/>
-    </row>
-    <row r="45" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="M44" s="28"/>
+      <c r="Q44" s="28"/>
+      <c r="R44" s="33"/>
+      <c r="X44" s="28"/>
+      <c r="AA44" s="28"/>
+      <c r="AB44" s="28"/>
+    </row>
+    <row r="45" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I45" s="2">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="M45" s="43"/>
-      <c r="Q45" s="43"/>
-      <c r="R45" s="49"/>
-      <c r="X45" s="43"/>
-      <c r="AA45" s="43"/>
-      <c r="AB45" s="43"/>
-    </row>
-    <row r="46" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="M45" s="28"/>
+      <c r="Q45" s="28"/>
+      <c r="R45" s="33"/>
+      <c r="X45" s="28"/>
+      <c r="AA45" s="28"/>
+      <c r="AB45" s="28"/>
+    </row>
+    <row r="46" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I46" s="2">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="M46" s="43"/>
-      <c r="Q46" s="43"/>
-      <c r="R46" s="49"/>
-      <c r="X46" s="43"/>
-      <c r="AA46" s="43"/>
-      <c r="AB46" s="43"/>
-    </row>
-    <row r="47" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="M46" s="28"/>
+      <c r="Q46" s="28"/>
+      <c r="R46" s="33"/>
+      <c r="X46" s="28"/>
+      <c r="AA46" s="28"/>
+      <c r="AB46" s="28"/>
+    </row>
+    <row r="47" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I47" s="2">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="M47" s="43"/>
-      <c r="Q47" s="43"/>
-      <c r="R47" s="49"/>
-      <c r="X47" s="43"/>
-      <c r="AA47" s="43"/>
-      <c r="AB47" s="43"/>
-    </row>
-    <row r="48" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="M47" s="28"/>
+      <c r="Q47" s="28"/>
+      <c r="R47" s="33"/>
+      <c r="X47" s="28"/>
+      <c r="AA47" s="28"/>
+      <c r="AB47" s="28"/>
+    </row>
+    <row r="48" spans="9:60" x14ac:dyDescent="0.25">
       <c r="I48" s="2">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="M48" s="43"/>
-      <c r="Q48" s="43"/>
-      <c r="R48" s="49"/>
-      <c r="X48" s="43"/>
-      <c r="AA48" s="43"/>
-      <c r="AB48" s="43"/>
-    </row>
-    <row r="49" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M48" s="28"/>
+      <c r="Q48" s="28"/>
+      <c r="R48" s="33"/>
+      <c r="X48" s="28"/>
+      <c r="AA48" s="28"/>
+      <c r="AB48" s="28"/>
+    </row>
+    <row r="49" spans="9:36" x14ac:dyDescent="0.25">
       <c r="I49" s="2">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="M49" s="43"/>
-      <c r="Q49" s="43"/>
-      <c r="R49" s="49"/>
-      <c r="X49" s="43"/>
-      <c r="AA49" s="43"/>
-      <c r="AB49" s="43"/>
-    </row>
-    <row r="50" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M49" s="28"/>
+      <c r="Q49" s="28"/>
+      <c r="R49" s="33"/>
+      <c r="X49" s="28"/>
+      <c r="AA49" s="28"/>
+      <c r="AB49" s="28"/>
+    </row>
+    <row r="50" spans="9:36" x14ac:dyDescent="0.25">
       <c r="I50" s="2">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="M50" s="43"/>
-      <c r="Q50" s="43"/>
-      <c r="R50" s="49"/>
-      <c r="X50" s="43"/>
-      <c r="AA50" s="43"/>
-      <c r="AB50" s="43"/>
-    </row>
-    <row r="51" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M50" s="28"/>
+      <c r="Q50" s="28"/>
+      <c r="R50" s="33"/>
+      <c r="X50" s="28"/>
+      <c r="AA50" s="28"/>
+      <c r="AB50" s="28"/>
+    </row>
+    <row r="51" spans="9:36" x14ac:dyDescent="0.25">
       <c r="I51" s="2">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="M51" s="43"/>
-      <c r="Q51" s="43"/>
-      <c r="R51" s="49"/>
-      <c r="X51" s="43"/>
-      <c r="AA51" s="43"/>
-      <c r="AB51" s="43"/>
-    </row>
-    <row r="52" spans="9:36" x14ac:dyDescent="0.35">
+      <c r="M51" s="28"/>
+      <c r="Q51" s="28"/>
+      <c r="R51" s="33"/>
+      <c r="X51" s="28"/>
+      <c r="AA51" s="28"/>
+      <c r="AB51" s="28"/>
+    </row>
+    <row r="52" spans="9:36" x14ac:dyDescent="0.25">
       <c r="I52" s="2">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="M52" s="43"/>
-      <c r="Q52" s="43"/>
-      <c r="X52" s="43"/>
-      <c r="AA52" s="43"/>
-      <c r="AB52" s="43"/>
-      <c r="AE52" s="26" t="s">
+      <c r="M52" s="28"/>
+      <c r="Q52" s="28"/>
+      <c r="X52" s="28"/>
+      <c r="AA52" s="28"/>
+      <c r="AB52" s="28"/>
+      <c r="AE52" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="AF52" s="26"/>
-      <c r="AG52" s="26"/>
-      <c r="AH52" s="26"/>
-      <c r="AI52" s="26"/>
-    </row>
-    <row r="53" spans="9:36" x14ac:dyDescent="0.35">
-      <c r="M53" s="43"/>
-      <c r="Q53" s="43"/>
-      <c r="X53" s="43"/>
-      <c r="AB53" s="43"/>
+      <c r="AF52" s="44"/>
+      <c r="AG52" s="44"/>
+      <c r="AH52" s="44"/>
+      <c r="AI52" s="44"/>
+    </row>
+    <row r="53" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="M53" s="28"/>
+      <c r="Q53" s="28"/>
+      <c r="X53" s="28"/>
+      <c r="AB53" s="28"/>
       <c r="AE53" s="2" t="s">
         <v>24</v>
       </c>
@@ -4286,11 +4282,11 @@
         <v>23</v>
       </c>
     </row>
-    <row r="54" spans="9:36" x14ac:dyDescent="0.35">
-      <c r="M54" s="43"/>
-      <c r="Q54" s="43"/>
-      <c r="X54" s="43"/>
-      <c r="AB54" s="43"/>
+    <row r="54" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="M54" s="28"/>
+      <c r="Q54" s="28"/>
+      <c r="X54" s="28"/>
+      <c r="AB54" s="28"/>
       <c r="AE54" s="2" t="s">
         <v>19</v>
       </c>
@@ -4307,10 +4303,10 @@
         <v>0.29899999999999999</v>
       </c>
     </row>
-    <row r="55" spans="9:36" x14ac:dyDescent="0.35">
-      <c r="M55" s="43"/>
-      <c r="X55" s="43"/>
-      <c r="AB55" s="43"/>
+    <row r="55" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="M55" s="28"/>
+      <c r="X55" s="28"/>
+      <c r="AB55" s="28"/>
       <c r="AE55" s="2" t="s">
         <v>20</v>
       </c>
@@ -4327,27 +4323,27 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="56" spans="9:36" x14ac:dyDescent="0.35">
-      <c r="M56" s="43"/>
-      <c r="X56" s="43"/>
-      <c r="AB56" s="43"/>
-    </row>
-    <row r="57" spans="9:36" x14ac:dyDescent="0.35">
-      <c r="M57" s="43"/>
-      <c r="X57" s="43"/>
-      <c r="AB57" s="43"/>
-      <c r="AE57" s="26" t="s">
+    <row r="56" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="M56" s="28"/>
+      <c r="X56" s="28"/>
+      <c r="AB56" s="28"/>
+    </row>
+    <row r="57" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="M57" s="28"/>
+      <c r="X57" s="28"/>
+      <c r="AB57" s="28"/>
+      <c r="AE57" s="44" t="s">
         <v>25</v>
       </c>
-      <c r="AF57" s="26"/>
-      <c r="AG57" s="26"/>
-      <c r="AH57" s="26"/>
-      <c r="AI57" s="26"/>
-    </row>
-    <row r="58" spans="9:36" x14ac:dyDescent="0.35">
-      <c r="M58" s="43"/>
-      <c r="X58" s="43"/>
-      <c r="AB58" s="43"/>
+      <c r="AF57" s="44"/>
+      <c r="AG57" s="44"/>
+      <c r="AH57" s="44"/>
+      <c r="AI57" s="44"/>
+    </row>
+    <row r="58" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="M58" s="28"/>
+      <c r="X58" s="28"/>
+      <c r="AB58" s="28"/>
       <c r="AE58" s="2" t="s">
         <v>24</v>
       </c>
@@ -4364,10 +4360,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="59" spans="9:36" x14ac:dyDescent="0.35">
-      <c r="M59" s="43"/>
-      <c r="X59" s="43"/>
-      <c r="AB59" s="43"/>
+    <row r="59" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="M59" s="28"/>
+      <c r="X59" s="28"/>
+      <c r="AB59" s="28"/>
       <c r="AE59" s="2" t="s">
         <v>88</v>
       </c>
@@ -4387,10 +4383,10 @@
         <v>30</v>
       </c>
     </row>
-    <row r="60" spans="9:36" x14ac:dyDescent="0.35">
-      <c r="M60" s="43"/>
-      <c r="X60" s="43"/>
-      <c r="AB60" s="43"/>
+    <row r="60" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="M60" s="28"/>
+      <c r="X60" s="28"/>
+      <c r="AB60" s="28"/>
       <c r="AE60" s="2" t="s">
         <v>89</v>
       </c>
@@ -4407,530 +4403,551 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="61" spans="9:36" x14ac:dyDescent="0.35">
-      <c r="M61" s="43"/>
-      <c r="X61" s="43"/>
-      <c r="AB61" s="43"/>
-    </row>
-    <row r="62" spans="9:36" x14ac:dyDescent="0.35">
-      <c r="M62" s="43"/>
-      <c r="X62" s="43"/>
-      <c r="AB62" s="43"/>
-      <c r="AE62" s="32" t="s">
+    <row r="61" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="M61" s="28"/>
+      <c r="X61" s="28"/>
+      <c r="AB61" s="28"/>
+    </row>
+    <row r="62" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="M62" s="28"/>
+      <c r="X62" s="28"/>
+      <c r="AB62" s="28"/>
+      <c r="AE62" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="AF62" s="32"/>
-      <c r="AG62" s="32"/>
-      <c r="AH62" s="32"/>
-      <c r="AI62" s="32"/>
-    </row>
-    <row r="63" spans="9:36" x14ac:dyDescent="0.35">
-      <c r="M63" s="43"/>
-      <c r="X63" s="43"/>
-      <c r="AB63" s="43"/>
-      <c r="AE63" s="32"/>
-      <c r="AF63" s="32"/>
-      <c r="AG63" s="32"/>
-      <c r="AH63" s="32"/>
-      <c r="AI63" s="32"/>
-    </row>
-    <row r="64" spans="9:36" x14ac:dyDescent="0.35">
-      <c r="M64" s="43"/>
-      <c r="X64" s="43"/>
-      <c r="AB64" s="43"/>
-    </row>
-    <row r="65" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M65" s="43"/>
-      <c r="X65" s="43"/>
-      <c r="AB65" s="43"/>
-    </row>
-    <row r="66" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M66" s="43"/>
-      <c r="X66" s="43"/>
-      <c r="AB66" s="43"/>
-    </row>
-    <row r="67" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M67" s="43"/>
-      <c r="X67" s="43"/>
-      <c r="AB67" s="43"/>
-    </row>
-    <row r="68" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M68" s="43"/>
-      <c r="X68" s="43"/>
-      <c r="AB68" s="43"/>
-    </row>
-    <row r="69" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M69" s="43"/>
-      <c r="X69" s="43"/>
-      <c r="AB69" s="43"/>
-    </row>
-    <row r="70" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M70" s="43"/>
-      <c r="X70" s="43"/>
-      <c r="AB70" s="43"/>
-    </row>
-    <row r="71" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M71" s="43"/>
-      <c r="X71" s="43"/>
-      <c r="AB71" s="43"/>
-    </row>
-    <row r="72" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M72" s="43"/>
-      <c r="X72" s="43"/>
-      <c r="AB72" s="43"/>
-    </row>
-    <row r="73" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M73" s="43"/>
-      <c r="X73" s="43"/>
-      <c r="AB73" s="43"/>
-    </row>
-    <row r="74" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M74" s="43"/>
-      <c r="X74" s="43"/>
-      <c r="AB74" s="43"/>
-    </row>
-    <row r="75" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M75" s="43"/>
-      <c r="X75" s="43"/>
-      <c r="AB75" s="43"/>
-    </row>
-    <row r="76" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M76" s="43"/>
-      <c r="X76" s="43"/>
-      <c r="AB76" s="43"/>
-    </row>
-    <row r="77" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M77" s="43"/>
-      <c r="X77" s="43"/>
-      <c r="AB77" s="43"/>
-    </row>
-    <row r="78" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M78" s="43"/>
-      <c r="X78" s="43"/>
-      <c r="AB78" s="43"/>
-    </row>
-    <row r="79" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M79" s="43"/>
-      <c r="X79" s="43"/>
-      <c r="AB79" s="43"/>
-    </row>
-    <row r="80" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M80" s="43"/>
-      <c r="X80" s="43"/>
-      <c r="AB80" s="43"/>
-    </row>
-    <row r="81" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M81" s="43"/>
-      <c r="X81" s="43"/>
-      <c r="AB81" s="43"/>
-    </row>
-    <row r="82" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M82" s="43"/>
-      <c r="X82" s="43"/>
-      <c r="AB82" s="43"/>
-    </row>
-    <row r="83" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M83" s="43"/>
-      <c r="X83" s="43"/>
-      <c r="AB83" s="43"/>
-    </row>
-    <row r="84" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M84" s="43"/>
-      <c r="X84" s="43"/>
-      <c r="AB84" s="43"/>
-    </row>
-    <row r="85" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M85" s="43"/>
-      <c r="X85" s="43"/>
-      <c r="AB85" s="43"/>
-    </row>
-    <row r="86" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M86" s="43"/>
-      <c r="X86" s="43"/>
-      <c r="AB86" s="43"/>
-    </row>
-    <row r="87" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M87" s="43"/>
-      <c r="X87" s="43"/>
-      <c r="AB87" s="43"/>
-    </row>
-    <row r="88" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M88" s="43"/>
-      <c r="X88" s="43"/>
-      <c r="AB88" s="43"/>
-    </row>
-    <row r="89" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M89" s="43"/>
-      <c r="AB89" s="43"/>
-    </row>
-    <row r="90" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M90" s="43"/>
-      <c r="AB90" s="43"/>
-    </row>
-    <row r="91" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M91" s="43"/>
-      <c r="AB91" s="43"/>
-    </row>
-    <row r="92" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M92" s="43"/>
-      <c r="AB92" s="43"/>
-    </row>
-    <row r="93" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M93" s="43"/>
-      <c r="AB93" s="43"/>
-    </row>
-    <row r="94" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M94" s="43"/>
-      <c r="AB94" s="43"/>
-    </row>
-    <row r="95" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M95" s="43"/>
-      <c r="AB95" s="43"/>
-    </row>
-    <row r="96" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M96" s="43"/>
-      <c r="AB96" s="43"/>
-    </row>
-    <row r="97" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M97" s="43"/>
-      <c r="AB97" s="43"/>
-    </row>
-    <row r="98" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M98" s="43"/>
-      <c r="AB98" s="43"/>
-    </row>
-    <row r="99" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M99" s="43"/>
-      <c r="AB99" s="43"/>
-    </row>
-    <row r="100" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M100" s="43"/>
-      <c r="AB100" s="43"/>
-    </row>
-    <row r="101" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M101" s="43"/>
-      <c r="AB101" s="43"/>
-    </row>
-    <row r="102" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M102" s="43"/>
-      <c r="AB102" s="43"/>
-    </row>
-    <row r="103" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M103" s="43"/>
-      <c r="AB103" s="43"/>
-    </row>
-    <row r="104" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M104" s="43"/>
-      <c r="AB104" s="43"/>
-    </row>
-    <row r="105" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M105" s="43"/>
-      <c r="AB105" s="43"/>
-    </row>
-    <row r="106" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M106" s="43"/>
-      <c r="AB106" s="43"/>
-    </row>
-    <row r="107" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M107" s="43"/>
-      <c r="AB107" s="43"/>
-    </row>
-    <row r="108" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M108" s="43"/>
-      <c r="AB108" s="43"/>
-    </row>
-    <row r="109" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M109" s="43"/>
-      <c r="AB109" s="43"/>
-    </row>
-    <row r="110" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M110" s="43"/>
-      <c r="AB110" s="43"/>
-    </row>
-    <row r="111" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M111" s="43"/>
-      <c r="AB111" s="43"/>
-    </row>
-    <row r="112" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M112" s="43"/>
-      <c r="AB112" s="43"/>
-    </row>
-    <row r="113" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M113" s="43"/>
-      <c r="AB113" s="43"/>
-    </row>
-    <row r="114" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M114" s="43"/>
-      <c r="AB114" s="43"/>
-    </row>
-    <row r="115" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M115" s="43"/>
-      <c r="AB115" s="43"/>
-    </row>
-    <row r="116" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M116" s="43"/>
-      <c r="AB116" s="43"/>
-    </row>
-    <row r="117" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M117" s="43"/>
-      <c r="AB117" s="43"/>
-    </row>
-    <row r="118" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M118" s="43"/>
-      <c r="AB118" s="43"/>
-    </row>
-    <row r="119" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M119" s="43"/>
-      <c r="AB119" s="43"/>
-    </row>
-    <row r="120" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M120" s="43"/>
-      <c r="AB120" s="43"/>
-    </row>
-    <row r="121" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M121" s="43"/>
-      <c r="AB121" s="43"/>
-    </row>
-    <row r="122" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M122" s="43"/>
-      <c r="AB122" s="43"/>
-    </row>
-    <row r="123" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M123" s="43"/>
-      <c r="AB123" s="43"/>
-    </row>
-    <row r="124" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M124" s="43"/>
-      <c r="AB124" s="43"/>
-    </row>
-    <row r="125" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M125" s="43"/>
-      <c r="AB125" s="43"/>
-    </row>
-    <row r="126" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M126" s="43"/>
-      <c r="AB126" s="43"/>
-    </row>
-    <row r="127" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M127" s="43"/>
-      <c r="AB127" s="43"/>
-    </row>
-    <row r="128" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M128" s="43"/>
-      <c r="AB128" s="43"/>
-    </row>
-    <row r="129" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M129" s="43"/>
-      <c r="AB129" s="43"/>
-    </row>
-    <row r="130" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M130" s="43"/>
-      <c r="AB130" s="43"/>
-    </row>
-    <row r="131" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M131" s="43"/>
-      <c r="AB131" s="43"/>
-    </row>
-    <row r="132" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M132" s="43"/>
-      <c r="AB132" s="43"/>
-    </row>
-    <row r="133" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M133" s="43"/>
-      <c r="AB133" s="43"/>
-    </row>
-    <row r="134" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M134" s="43"/>
-      <c r="AB134" s="43"/>
-    </row>
-    <row r="135" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M135" s="43"/>
-      <c r="AB135" s="43"/>
-    </row>
-    <row r="136" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M136" s="43"/>
-      <c r="AB136" s="43"/>
-    </row>
-    <row r="137" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M137" s="43"/>
-      <c r="AB137" s="43"/>
-    </row>
-    <row r="138" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M138" s="43"/>
-      <c r="AB138" s="43"/>
-    </row>
-    <row r="139" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M139" s="43"/>
-      <c r="AB139" s="43"/>
-    </row>
-    <row r="140" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M140" s="43"/>
-      <c r="AB140" s="43"/>
-    </row>
-    <row r="141" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M141" s="43"/>
-      <c r="AB141" s="43"/>
-    </row>
-    <row r="142" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M142" s="43"/>
-      <c r="AB142" s="43"/>
-    </row>
-    <row r="143" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M143" s="43"/>
-      <c r="AB143" s="43"/>
-    </row>
-    <row r="144" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M144" s="43"/>
-      <c r="AB144" s="43"/>
-    </row>
-    <row r="145" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M145" s="43"/>
-      <c r="AB145" s="43"/>
-    </row>
-    <row r="146" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M146" s="43"/>
-      <c r="AB146" s="43"/>
-    </row>
-    <row r="147" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M147" s="43"/>
-      <c r="AB147" s="43"/>
-    </row>
-    <row r="148" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M148" s="43"/>
-      <c r="AB148" s="43"/>
-    </row>
-    <row r="149" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M149" s="43"/>
-      <c r="AB149" s="43"/>
-    </row>
-    <row r="150" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M150" s="43"/>
-      <c r="AB150" s="43"/>
-    </row>
-    <row r="151" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M151" s="43"/>
-      <c r="AB151" s="43"/>
-    </row>
-    <row r="152" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M152" s="43"/>
-      <c r="AB152" s="43"/>
-    </row>
-    <row r="153" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M153" s="43"/>
-      <c r="AB153" s="43"/>
-    </row>
-    <row r="154" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M154" s="43"/>
-      <c r="AB154" s="43"/>
-    </row>
-    <row r="155" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M155" s="43"/>
-      <c r="AB155" s="43"/>
-    </row>
-    <row r="156" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M156" s="43"/>
-      <c r="AB156" s="43"/>
-    </row>
-    <row r="157" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M157" s="43"/>
-      <c r="AB157" s="43"/>
-    </row>
-    <row r="158" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M158" s="43"/>
-      <c r="AB158" s="43"/>
-    </row>
-    <row r="159" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M159" s="43"/>
-      <c r="AB159" s="43"/>
-    </row>
-    <row r="160" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M160" s="43"/>
-      <c r="AB160" s="43"/>
-    </row>
-    <row r="161" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M161" s="43"/>
-      <c r="AB161" s="43"/>
-    </row>
-    <row r="162" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M162" s="43"/>
-      <c r="AB162" s="43"/>
-    </row>
-    <row r="163" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M163" s="43"/>
-      <c r="AB163" s="43"/>
-    </row>
-    <row r="164" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M164" s="43"/>
-      <c r="AB164" s="43"/>
-    </row>
-    <row r="165" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M165" s="43"/>
-      <c r="AB165" s="43"/>
-    </row>
-    <row r="166" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M166" s="43"/>
-      <c r="AB166" s="43"/>
-    </row>
-    <row r="167" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M167" s="43"/>
-      <c r="AB167" s="43"/>
-    </row>
-    <row r="168" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M168" s="43"/>
-      <c r="AB168" s="43"/>
-    </row>
-    <row r="169" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M169" s="43"/>
-      <c r="AB169" s="43"/>
-    </row>
-    <row r="170" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M170" s="43"/>
-      <c r="AB170" s="43"/>
-    </row>
-    <row r="171" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M171" s="43"/>
-      <c r="AB171" s="43"/>
-    </row>
-    <row r="172" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M172" s="43"/>
-      <c r="AB172" s="43"/>
-    </row>
-    <row r="173" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M173" s="43"/>
-      <c r="AB173" s="43"/>
-    </row>
-    <row r="174" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M174" s="43"/>
-      <c r="AB174" s="43"/>
-    </row>
-    <row r="175" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M175" s="43"/>
-      <c r="AB175" s="43"/>
-    </row>
-    <row r="176" spans="13:28" x14ac:dyDescent="0.35">
-      <c r="M176" s="43"/>
-      <c r="AB176" s="43"/>
-    </row>
-    <row r="177" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M177" s="43"/>
-    </row>
-    <row r="178" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M178" s="43"/>
-    </row>
-    <row r="179" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M179" s="43"/>
-    </row>
-    <row r="180" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M180" s="43"/>
-    </row>
-    <row r="181" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M181" s="43"/>
-    </row>
-    <row r="182" spans="13:13" x14ac:dyDescent="0.35">
-      <c r="M182" s="43"/>
+      <c r="AF62" s="45"/>
+      <c r="AG62" s="45"/>
+      <c r="AH62" s="45"/>
+      <c r="AI62" s="45"/>
+    </row>
+    <row r="63" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="M63" s="28"/>
+      <c r="X63" s="28"/>
+      <c r="AB63" s="28"/>
+      <c r="AE63" s="45"/>
+      <c r="AF63" s="45"/>
+      <c r="AG63" s="45"/>
+      <c r="AH63" s="45"/>
+      <c r="AI63" s="45"/>
+    </row>
+    <row r="64" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="M64" s="28"/>
+      <c r="X64" s="28"/>
+      <c r="AB64" s="28"/>
+    </row>
+    <row r="65" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M65" s="28"/>
+      <c r="X65" s="28"/>
+      <c r="AB65" s="28"/>
+    </row>
+    <row r="66" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M66" s="28"/>
+      <c r="X66" s="28"/>
+      <c r="AB66" s="28"/>
+    </row>
+    <row r="67" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M67" s="28"/>
+      <c r="X67" s="28"/>
+      <c r="AB67" s="28"/>
+    </row>
+    <row r="68" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M68" s="28"/>
+      <c r="X68" s="28"/>
+      <c r="AB68" s="28"/>
+    </row>
+    <row r="69" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M69" s="28"/>
+      <c r="X69" s="28"/>
+      <c r="AB69" s="28"/>
+    </row>
+    <row r="70" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M70" s="28"/>
+      <c r="X70" s="28"/>
+      <c r="AB70" s="28"/>
+    </row>
+    <row r="71" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M71" s="28"/>
+      <c r="X71" s="28"/>
+      <c r="AB71" s="28"/>
+    </row>
+    <row r="72" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M72" s="28"/>
+      <c r="X72" s="28"/>
+      <c r="AB72" s="28"/>
+    </row>
+    <row r="73" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M73" s="28"/>
+      <c r="X73" s="28"/>
+      <c r="AB73" s="28"/>
+    </row>
+    <row r="74" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M74" s="28"/>
+      <c r="X74" s="28"/>
+      <c r="AB74" s="28"/>
+    </row>
+    <row r="75" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M75" s="28"/>
+      <c r="X75" s="28"/>
+      <c r="AB75" s="28"/>
+    </row>
+    <row r="76" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M76" s="28"/>
+      <c r="X76" s="28"/>
+      <c r="AB76" s="28"/>
+    </row>
+    <row r="77" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M77" s="28"/>
+      <c r="X77" s="28"/>
+      <c r="AB77" s="28"/>
+    </row>
+    <row r="78" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M78" s="28"/>
+      <c r="X78" s="28"/>
+      <c r="AB78" s="28"/>
+    </row>
+    <row r="79" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M79" s="28"/>
+      <c r="X79" s="28"/>
+      <c r="AB79" s="28"/>
+    </row>
+    <row r="80" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M80" s="28"/>
+      <c r="X80" s="28"/>
+      <c r="AB80" s="28"/>
+    </row>
+    <row r="81" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M81" s="28"/>
+      <c r="X81" s="28"/>
+      <c r="AB81" s="28"/>
+    </row>
+    <row r="82" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M82" s="28"/>
+      <c r="X82" s="28"/>
+      <c r="AB82" s="28"/>
+    </row>
+    <row r="83" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M83" s="28"/>
+      <c r="X83" s="28"/>
+      <c r="AB83" s="28"/>
+    </row>
+    <row r="84" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M84" s="28"/>
+      <c r="X84" s="28"/>
+      <c r="AB84" s="28"/>
+    </row>
+    <row r="85" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M85" s="28"/>
+      <c r="X85" s="28"/>
+      <c r="AB85" s="28"/>
+    </row>
+    <row r="86" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M86" s="28"/>
+      <c r="X86" s="28"/>
+      <c r="AB86" s="28"/>
+    </row>
+    <row r="87" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M87" s="28"/>
+      <c r="X87" s="28"/>
+      <c r="AB87" s="28"/>
+    </row>
+    <row r="88" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M88" s="28"/>
+      <c r="X88" s="28"/>
+      <c r="AB88" s="28"/>
+    </row>
+    <row r="89" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M89" s="28"/>
+      <c r="AB89" s="28"/>
+    </row>
+    <row r="90" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M90" s="28"/>
+      <c r="AB90" s="28"/>
+    </row>
+    <row r="91" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M91" s="28"/>
+      <c r="AB91" s="28"/>
+    </row>
+    <row r="92" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M92" s="28"/>
+      <c r="AB92" s="28"/>
+    </row>
+    <row r="93" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M93" s="28"/>
+      <c r="AB93" s="28"/>
+    </row>
+    <row r="94" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M94" s="28"/>
+      <c r="AB94" s="28"/>
+    </row>
+    <row r="95" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M95" s="28"/>
+      <c r="AB95" s="28"/>
+    </row>
+    <row r="96" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M96" s="28"/>
+      <c r="AB96" s="28"/>
+    </row>
+    <row r="97" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M97" s="28"/>
+      <c r="AB97" s="28"/>
+    </row>
+    <row r="98" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M98" s="28"/>
+      <c r="AB98" s="28"/>
+    </row>
+    <row r="99" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M99" s="28"/>
+      <c r="AB99" s="28"/>
+    </row>
+    <row r="100" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M100" s="28"/>
+      <c r="AB100" s="28"/>
+    </row>
+    <row r="101" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M101" s="28"/>
+      <c r="AB101" s="28"/>
+    </row>
+    <row r="102" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M102" s="28"/>
+      <c r="AB102" s="28"/>
+    </row>
+    <row r="103" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M103" s="28"/>
+      <c r="AB103" s="28"/>
+    </row>
+    <row r="104" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M104" s="28"/>
+      <c r="AB104" s="28"/>
+    </row>
+    <row r="105" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M105" s="28"/>
+      <c r="AB105" s="28"/>
+    </row>
+    <row r="106" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M106" s="28"/>
+      <c r="AB106" s="28"/>
+    </row>
+    <row r="107" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M107" s="28"/>
+      <c r="AB107" s="28"/>
+    </row>
+    <row r="108" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M108" s="28"/>
+      <c r="AB108" s="28"/>
+    </row>
+    <row r="109" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M109" s="28"/>
+      <c r="AB109" s="28"/>
+    </row>
+    <row r="110" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M110" s="28"/>
+      <c r="AB110" s="28"/>
+    </row>
+    <row r="111" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M111" s="28"/>
+      <c r="AB111" s="28"/>
+    </row>
+    <row r="112" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M112" s="28"/>
+      <c r="AB112" s="28"/>
+    </row>
+    <row r="113" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M113" s="28"/>
+      <c r="AB113" s="28"/>
+    </row>
+    <row r="114" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M114" s="28"/>
+      <c r="AB114" s="28"/>
+    </row>
+    <row r="115" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M115" s="28"/>
+      <c r="AB115" s="28"/>
+    </row>
+    <row r="116" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M116" s="28"/>
+      <c r="AB116" s="28"/>
+    </row>
+    <row r="117" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M117" s="28"/>
+      <c r="AB117" s="28"/>
+    </row>
+    <row r="118" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M118" s="28"/>
+      <c r="AB118" s="28"/>
+    </row>
+    <row r="119" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M119" s="28"/>
+      <c r="AB119" s="28"/>
+    </row>
+    <row r="120" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M120" s="28"/>
+      <c r="AB120" s="28"/>
+    </row>
+    <row r="121" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M121" s="28"/>
+      <c r="AB121" s="28"/>
+    </row>
+    <row r="122" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M122" s="28"/>
+      <c r="AB122" s="28"/>
+    </row>
+    <row r="123" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M123" s="28"/>
+      <c r="AB123" s="28"/>
+    </row>
+    <row r="124" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M124" s="28"/>
+      <c r="AB124" s="28"/>
+    </row>
+    <row r="125" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M125" s="28"/>
+      <c r="AB125" s="28"/>
+    </row>
+    <row r="126" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M126" s="28"/>
+      <c r="AB126" s="28"/>
+    </row>
+    <row r="127" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M127" s="28"/>
+      <c r="AB127" s="28"/>
+    </row>
+    <row r="128" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M128" s="28"/>
+      <c r="AB128" s="28"/>
+    </row>
+    <row r="129" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M129" s="28"/>
+      <c r="AB129" s="28"/>
+    </row>
+    <row r="130" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M130" s="28"/>
+      <c r="AB130" s="28"/>
+    </row>
+    <row r="131" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M131" s="28"/>
+      <c r="AB131" s="28"/>
+    </row>
+    <row r="132" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M132" s="28"/>
+      <c r="AB132" s="28"/>
+    </row>
+    <row r="133" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M133" s="28"/>
+      <c r="AB133" s="28"/>
+    </row>
+    <row r="134" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M134" s="28"/>
+      <c r="AB134" s="28"/>
+    </row>
+    <row r="135" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M135" s="28"/>
+      <c r="AB135" s="28"/>
+    </row>
+    <row r="136" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M136" s="28"/>
+      <c r="AB136" s="28"/>
+    </row>
+    <row r="137" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M137" s="28"/>
+      <c r="AB137" s="28"/>
+    </row>
+    <row r="138" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M138" s="28"/>
+      <c r="AB138" s="28"/>
+    </row>
+    <row r="139" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M139" s="28"/>
+      <c r="AB139" s="28"/>
+    </row>
+    <row r="140" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M140" s="28"/>
+      <c r="AB140" s="28"/>
+    </row>
+    <row r="141" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M141" s="28"/>
+      <c r="AB141" s="28"/>
+    </row>
+    <row r="142" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M142" s="28"/>
+      <c r="AB142" s="28"/>
+    </row>
+    <row r="143" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M143" s="28"/>
+      <c r="AB143" s="28"/>
+    </row>
+    <row r="144" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M144" s="28"/>
+      <c r="AB144" s="28"/>
+    </row>
+    <row r="145" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M145" s="28"/>
+      <c r="AB145" s="28"/>
+    </row>
+    <row r="146" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M146" s="28"/>
+      <c r="AB146" s="28"/>
+    </row>
+    <row r="147" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M147" s="28"/>
+      <c r="AB147" s="28"/>
+    </row>
+    <row r="148" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M148" s="28"/>
+      <c r="AB148" s="28"/>
+    </row>
+    <row r="149" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M149" s="28"/>
+      <c r="AB149" s="28"/>
+    </row>
+    <row r="150" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M150" s="28"/>
+      <c r="AB150" s="28"/>
+    </row>
+    <row r="151" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M151" s="28"/>
+      <c r="AB151" s="28"/>
+    </row>
+    <row r="152" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M152" s="28"/>
+      <c r="AB152" s="28"/>
+    </row>
+    <row r="153" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M153" s="28"/>
+      <c r="AB153" s="28"/>
+    </row>
+    <row r="154" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M154" s="28"/>
+      <c r="AB154" s="28"/>
+    </row>
+    <row r="155" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M155" s="28"/>
+      <c r="AB155" s="28"/>
+    </row>
+    <row r="156" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M156" s="28"/>
+      <c r="AB156" s="28"/>
+    </row>
+    <row r="157" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M157" s="28"/>
+      <c r="AB157" s="28"/>
+    </row>
+    <row r="158" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M158" s="28"/>
+      <c r="AB158" s="28"/>
+    </row>
+    <row r="159" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M159" s="28"/>
+      <c r="AB159" s="28"/>
+    </row>
+    <row r="160" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M160" s="28"/>
+      <c r="AB160" s="28"/>
+    </row>
+    <row r="161" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M161" s="28"/>
+      <c r="AB161" s="28"/>
+    </row>
+    <row r="162" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M162" s="28"/>
+      <c r="AB162" s="28"/>
+    </row>
+    <row r="163" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M163" s="28"/>
+      <c r="AB163" s="28"/>
+    </row>
+    <row r="164" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M164" s="28"/>
+      <c r="AB164" s="28"/>
+    </row>
+    <row r="165" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M165" s="28"/>
+      <c r="AB165" s="28"/>
+    </row>
+    <row r="166" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M166" s="28"/>
+      <c r="AB166" s="28"/>
+    </row>
+    <row r="167" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M167" s="28"/>
+      <c r="AB167" s="28"/>
+    </row>
+    <row r="168" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M168" s="28"/>
+      <c r="AB168" s="28"/>
+    </row>
+    <row r="169" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M169" s="28"/>
+      <c r="AB169" s="28"/>
+    </row>
+    <row r="170" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M170" s="28"/>
+      <c r="AB170" s="28"/>
+    </row>
+    <row r="171" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M171" s="28"/>
+      <c r="AB171" s="28"/>
+    </row>
+    <row r="172" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M172" s="28"/>
+      <c r="AB172" s="28"/>
+    </row>
+    <row r="173" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M173" s="28"/>
+      <c r="AB173" s="28"/>
+    </row>
+    <row r="174" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M174" s="28"/>
+      <c r="AB174" s="28"/>
+    </row>
+    <row r="175" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M175" s="28"/>
+      <c r="AB175" s="28"/>
+    </row>
+    <row r="176" spans="13:28" x14ac:dyDescent="0.25">
+      <c r="M176" s="28"/>
+      <c r="AB176" s="28"/>
+    </row>
+    <row r="177" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M177" s="28"/>
+    </row>
+    <row r="178" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M178" s="28"/>
+    </row>
+    <row r="179" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M179" s="28"/>
+    </row>
+    <row r="180" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M180" s="28"/>
+    </row>
+    <row r="181" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M181" s="28"/>
+    </row>
+    <row r="182" spans="13:13" x14ac:dyDescent="0.25">
+      <c r="M182" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="37">
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="AD10:AM10"/>
+    <mergeCell ref="O11:V11"/>
+    <mergeCell ref="AA11:AC11"/>
+    <mergeCell ref="Y11:Z11"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="Q2:T2"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="AS11:AV11"/>
+    <mergeCell ref="B24:F25"/>
+    <mergeCell ref="G8:H9"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="AO11:AR11"/>
     <mergeCell ref="AE52:AI52"/>
     <mergeCell ref="AE57:AI57"/>
     <mergeCell ref="AE62:AI63"/>
@@ -4947,27 +4964,6 @@
     <mergeCell ref="W11:X11"/>
     <mergeCell ref="Q3:R3"/>
     <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="Q2:T2"/>
-    <mergeCell ref="S3:T3"/>
-    <mergeCell ref="AS11:AV11"/>
-    <mergeCell ref="B24:F25"/>
-    <mergeCell ref="G8:H9"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="AO11:AR11"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="AD10:AM10"/>
-    <mergeCell ref="O11:V11"/>
-    <mergeCell ref="AA11:AC11"/>
-    <mergeCell ref="Y11:Z11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fin de la 2da simulacion excel
</commit_message>
<xml_diff>
--- a/1er Entrega/Plantilla.xlsx
+++ b/1er Entrega/Plantilla.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\UTN\Simulación\TP 4\Tp4-Simulacion-G5\1er Entrega\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc_ju\OneDrive\Escritorio\Tp4-Simulacion-G5\1er Entrega\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01A6CCB0-D28D-4191-8DCD-B02B2B795742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6B2A8D-1238-4D27-BE9E-CBA640B0621A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="120">
   <si>
     <t>Horario Apertura</t>
   </si>
@@ -392,7 +392,10 @@
     <t>Fin_Reparacion_CL4</t>
   </si>
   <si>
-    <t>c</t>
+    <t xml:space="preserve">Inicializacion </t>
+  </si>
+  <si>
+    <t>Fin_Atencion_CL4</t>
   </si>
 </sst>
 </file>
@@ -403,7 +406,7 @@
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -439,8 +442,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -525,8 +534,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -586,11 +601,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -660,11 +712,9 @@
     </xf>
     <xf numFmtId="46" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="46" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -672,8 +722,25 @@
     <xf numFmtId="46" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -697,25 +764,42 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="19" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="46" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -997,76 +1081,76 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:BH182"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="17" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" customWidth="1"/>
+    <col min="3" max="3" width="8.54296875" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="9" max="9" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.42578125" customWidth="1"/>
-    <col min="11" max="11" width="19.42578125" customWidth="1"/>
-    <col min="12" max="12" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="17.5703125" customWidth="1"/>
-    <col min="16" max="16" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="12.5703125" customWidth="1"/>
-    <col min="18" max="18" width="16.85546875" customWidth="1"/>
-    <col min="19" max="20" width="12.42578125" customWidth="1"/>
-    <col min="21" max="21" width="12.5703125" customWidth="1"/>
-    <col min="23" max="23" width="11.28515625" customWidth="1"/>
-    <col min="25" max="25" width="9.85546875" customWidth="1"/>
-    <col min="26" max="26" width="11.5703125" customWidth="1"/>
-    <col min="27" max="27" width="12.7109375" customWidth="1"/>
-    <col min="28" max="28" width="10.85546875" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="32" max="32" width="15.28515625" customWidth="1"/>
-    <col min="33" max="33" width="16.28515625" customWidth="1"/>
+    <col min="9" max="9" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.453125" customWidth="1"/>
+    <col min="11" max="11" width="19.453125" customWidth="1"/>
+    <col min="12" max="12" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="17.54296875" customWidth="1"/>
+    <col min="16" max="16" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.54296875" customWidth="1"/>
+    <col min="18" max="18" width="16.81640625" customWidth="1"/>
+    <col min="19" max="20" width="12.453125" customWidth="1"/>
+    <col min="21" max="21" width="12.54296875" customWidth="1"/>
+    <col min="23" max="23" width="11.26953125" customWidth="1"/>
+    <col min="25" max="25" width="9.81640625" customWidth="1"/>
+    <col min="26" max="26" width="11.54296875" customWidth="1"/>
+    <col min="27" max="27" width="12.7265625" customWidth="1"/>
+    <col min="28" max="28" width="10.81640625" customWidth="1"/>
+    <col min="29" max="29" width="10.26953125" customWidth="1"/>
+    <col min="32" max="32" width="15.26953125" customWidth="1"/>
+    <col min="33" max="33" width="16.26953125" customWidth="1"/>
     <col min="34" max="38" width="12" customWidth="1"/>
-    <col min="40" max="40" width="1.140625" customWidth="1"/>
-    <col min="41" max="43" width="15.5703125" customWidth="1"/>
-    <col min="44" max="44" width="11.7109375" customWidth="1"/>
-    <col min="46" max="46" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="12.42578125" customWidth="1"/>
-    <col min="48" max="48" width="12.28515625" customWidth="1"/>
-    <col min="50" max="50" width="11.140625" customWidth="1"/>
-    <col min="51" max="51" width="12.28515625" customWidth="1"/>
-    <col min="52" max="52" width="11.42578125" customWidth="1"/>
-    <col min="54" max="54" width="13.42578125" customWidth="1"/>
-    <col min="55" max="55" width="11.7109375" customWidth="1"/>
+    <col min="40" max="40" width="1.1796875" customWidth="1"/>
+    <col min="41" max="43" width="15.54296875" customWidth="1"/>
+    <col min="44" max="44" width="11.7265625" customWidth="1"/>
+    <col min="46" max="46" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="12.453125" customWidth="1"/>
+    <col min="48" max="48" width="12.26953125" customWidth="1"/>
+    <col min="50" max="50" width="11.1796875" customWidth="1"/>
+    <col min="51" max="51" width="12.26953125" customWidth="1"/>
+    <col min="52" max="52" width="11.453125" customWidth="1"/>
+    <col min="54" max="54" width="13.453125" customWidth="1"/>
+    <col min="55" max="55" width="11.7265625" customWidth="1"/>
     <col min="56" max="56" width="12" customWidth="1"/>
-    <col min="58" max="58" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="11.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:60" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:60" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2"/>
-      <c r="E2" s="46" t="s">
+      <c r="E2" s="49" t="s">
         <v>32</v>
       </c>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
       <c r="J2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="K2" s="49" t="s">
+      <c r="K2" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="L2" s="49"/>
-      <c r="M2" s="49"/>
-      <c r="N2" s="49"/>
-      <c r="O2" s="49"/>
-      <c r="Q2" s="52" t="s">
+      <c r="L2" s="52"/>
+      <c r="M2" s="52"/>
+      <c r="N2" s="52"/>
+      <c r="O2" s="52"/>
+      <c r="Q2" s="47" t="s">
         <v>72</v>
       </c>
-      <c r="R2" s="52"/>
-      <c r="S2" s="52"/>
-      <c r="T2" s="52"/>
-    </row>
-    <row r="3" spans="2:60" x14ac:dyDescent="0.25">
+      <c r="R2" s="47"/>
+      <c r="S2" s="47"/>
+      <c r="T2" s="47"/>
+    </row>
+    <row r="3" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
@@ -1079,24 +1163,24 @@
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
-      <c r="Q3" s="44" t="s">
+      <c r="Q3" s="46" t="s">
         <v>71</v>
       </c>
-      <c r="R3" s="44"/>
-      <c r="S3" s="44" t="s">
+      <c r="R3" s="46"/>
+      <c r="S3" s="46" t="s">
         <v>77</v>
       </c>
-      <c r="T3" s="44"/>
-    </row>
-    <row r="4" spans="2:60" x14ac:dyDescent="0.25">
-      <c r="B4" s="44" t="s">
+      <c r="T3" s="46"/>
+    </row>
+    <row r="4" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="B4" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="44"/>
-      <c r="E4" s="44" t="s">
-        <v>0</v>
-      </c>
-      <c r="F4" s="44"/>
+      <c r="C4" s="46"/>
+      <c r="E4" s="46" t="s">
+        <v>0</v>
+      </c>
+      <c r="F4" s="46"/>
       <c r="G4" s="2">
         <v>10</v>
       </c>
@@ -1115,20 +1199,20 @@
       <c r="O4" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="Q4" s="44" t="s">
+      <c r="Q4" s="46" t="s">
         <v>73</v>
       </c>
-      <c r="R4" s="44"/>
-      <c r="S4" s="44" t="s">
+      <c r="R4" s="46"/>
+      <c r="S4" s="46" t="s">
         <v>75</v>
       </c>
-      <c r="T4" s="44"/>
-    </row>
-    <row r="5" spans="2:60" x14ac:dyDescent="0.25">
-      <c r="E5" s="44" t="s">
+      <c r="T4" s="46"/>
+    </row>
+    <row r="5" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="E5" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="44"/>
+      <c r="F5" s="46"/>
       <c r="G5" s="2">
         <v>18</v>
       </c>
@@ -1150,7 +1234,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="2:60" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:60" ht="58" x14ac:dyDescent="0.35">
       <c r="J6" s="5" t="s">
         <v>65</v>
       </c>
@@ -1166,7 +1250,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="7" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1176,23 +1260,23 @@
       <c r="D7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="44" t="s">
+      <c r="E7" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="44"/>
-      <c r="G7" s="44" t="s">
+      <c r="F7" s="46"/>
+      <c r="G7" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="H7" s="44"/>
-    </row>
-    <row r="8" spans="2:60" x14ac:dyDescent="0.25">
-      <c r="B8" s="44" t="s">
+      <c r="H7" s="46"/>
+    </row>
+    <row r="8" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="B8" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="C8" s="46" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="44" t="s">
+      <c r="D8" s="46" t="s">
         <v>12</v>
       </c>
       <c r="E8" s="2" t="s">
@@ -1201,74 +1285,74 @@
       <c r="F8" s="2">
         <v>10</v>
       </c>
-      <c r="G8" s="53" t="s">
+      <c r="G8" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="H8" s="53"/>
-    </row>
-    <row r="9" spans="2:60" x14ac:dyDescent="0.25">
-      <c r="B9" s="44"/>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
+      <c r="H8" s="41"/>
+    </row>
+    <row r="9" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="B9" s="46"/>
+      <c r="C9" s="46"/>
+      <c r="D9" s="46"/>
       <c r="E9" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F9" s="2">
         <v>20</v>
       </c>
-      <c r="G9" s="53"/>
-      <c r="H9" s="53"/>
-      <c r="J9" s="48" t="s">
+      <c r="G9" s="41"/>
+      <c r="H9" s="41"/>
+      <c r="J9" s="51" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="48"/>
-      <c r="L9" s="48"/>
-      <c r="M9" s="48"/>
-      <c r="N9" s="48"/>
-      <c r="O9" s="48"/>
-      <c r="P9" s="48"/>
-      <c r="Q9" s="48"/>
-      <c r="R9" s="48"/>
-      <c r="S9" s="48"/>
-      <c r="T9" s="48"/>
-      <c r="U9" s="48"/>
-      <c r="V9" s="48"/>
-      <c r="W9" s="48"/>
-      <c r="X9" s="48"/>
-      <c r="Y9" s="48"/>
-      <c r="Z9" s="48"/>
-      <c r="AA9" s="48"/>
-      <c r="AB9" s="48"/>
-      <c r="AC9" s="48"/>
-      <c r="AD9" s="48"/>
-      <c r="AE9" s="48"/>
-      <c r="AF9" s="48"/>
-      <c r="AG9" s="48"/>
-      <c r="AH9" s="48"/>
-      <c r="AI9" s="48"/>
-      <c r="AJ9" s="48"/>
-      <c r="AK9" s="48"/>
-      <c r="AL9" s="48"/>
-      <c r="AM9" s="48"/>
-      <c r="AN9" s="48"/>
-      <c r="AO9" s="48"/>
-      <c r="AP9" s="48"/>
-      <c r="AQ9" s="48"/>
-      <c r="AR9" s="48"/>
-      <c r="AS9" s="48"/>
-      <c r="AT9" s="48"/>
-      <c r="AU9" s="48"/>
-      <c r="AV9" s="48"/>
-      <c r="AW9" s="48"/>
-      <c r="AX9" s="48"/>
-      <c r="AY9" s="48"/>
-      <c r="AZ9" s="48"/>
-      <c r="BA9" s="48"/>
-      <c r="BB9" s="48"/>
-      <c r="BC9" s="48"/>
-      <c r="BD9" s="48"/>
-    </row>
-    <row r="10" spans="2:60" x14ac:dyDescent="0.25">
+      <c r="K9" s="51"/>
+      <c r="L9" s="51"/>
+      <c r="M9" s="51"/>
+      <c r="N9" s="51"/>
+      <c r="O9" s="51"/>
+      <c r="P9" s="51"/>
+      <c r="Q9" s="51"/>
+      <c r="R9" s="51"/>
+      <c r="S9" s="51"/>
+      <c r="T9" s="51"/>
+      <c r="U9" s="51"/>
+      <c r="V9" s="51"/>
+      <c r="W9" s="51"/>
+      <c r="X9" s="51"/>
+      <c r="Y9" s="51"/>
+      <c r="Z9" s="51"/>
+      <c r="AA9" s="51"/>
+      <c r="AB9" s="51"/>
+      <c r="AC9" s="51"/>
+      <c r="AD9" s="51"/>
+      <c r="AE9" s="51"/>
+      <c r="AF9" s="51"/>
+      <c r="AG9" s="51"/>
+      <c r="AH9" s="51"/>
+      <c r="AI9" s="51"/>
+      <c r="AJ9" s="51"/>
+      <c r="AK9" s="51"/>
+      <c r="AL9" s="51"/>
+      <c r="AM9" s="51"/>
+      <c r="AN9" s="51"/>
+      <c r="AO9" s="51"/>
+      <c r="AP9" s="51"/>
+      <c r="AQ9" s="51"/>
+      <c r="AR9" s="51"/>
+      <c r="AS9" s="51"/>
+      <c r="AT9" s="51"/>
+      <c r="AU9" s="51"/>
+      <c r="AV9" s="51"/>
+      <c r="AW9" s="51"/>
+      <c r="AX9" s="51"/>
+      <c r="AY9" s="51"/>
+      <c r="AZ9" s="51"/>
+      <c r="BA9" s="51"/>
+      <c r="BB9" s="51"/>
+      <c r="BC9" s="51"/>
+      <c r="BD9" s="51"/>
+    </row>
+    <row r="10" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B10" s="1" t="s">
         <v>7</v>
       </c>
@@ -1284,76 +1368,76 @@
       <c r="F10" s="2">
         <v>90</v>
       </c>
-      <c r="G10" s="44" t="s">
+      <c r="G10" s="46" t="s">
         <v>29</v>
       </c>
-      <c r="H10" s="44"/>
-      <c r="AD10" s="54" t="s">
+      <c r="H10" s="46"/>
+      <c r="AD10" s="42" t="s">
         <v>62</v>
       </c>
-      <c r="AE10" s="54"/>
-      <c r="AF10" s="54"/>
-      <c r="AG10" s="54"/>
-      <c r="AH10" s="54"/>
-      <c r="AI10" s="54"/>
-      <c r="AJ10" s="54"/>
-      <c r="AK10" s="54"/>
-      <c r="AL10" s="54"/>
-      <c r="AM10" s="54"/>
+      <c r="AE10" s="42"/>
+      <c r="AF10" s="42"/>
+      <c r="AG10" s="42"/>
+      <c r="AH10" s="42"/>
+      <c r="AI10" s="42"/>
+      <c r="AJ10" s="42"/>
+      <c r="AK10" s="42"/>
+      <c r="AL10" s="42"/>
+      <c r="AM10" s="42"/>
       <c r="AN10" s="2"/>
-      <c r="AO10" s="47" t="s">
+      <c r="AO10" s="50" t="s">
         <v>79</v>
       </c>
-      <c r="AP10" s="47"/>
-      <c r="AQ10" s="47"/>
-      <c r="AR10" s="47"/>
-      <c r="AS10" s="47"/>
-      <c r="AT10" s="47"/>
-      <c r="AU10" s="47"/>
-      <c r="AV10" s="47"/>
-      <c r="AW10" s="47"/>
-      <c r="AX10" s="47"/>
-      <c r="AY10" s="47"/>
-      <c r="AZ10" s="47"/>
-      <c r="BA10" s="47"/>
-      <c r="BB10" s="47"/>
-      <c r="BC10" s="47"/>
-      <c r="BD10" s="47"/>
-    </row>
-    <row r="11" spans="2:60" x14ac:dyDescent="0.25">
-      <c r="I11" s="53" t="s">
+      <c r="AP10" s="50"/>
+      <c r="AQ10" s="50"/>
+      <c r="AR10" s="50"/>
+      <c r="AS10" s="50"/>
+      <c r="AT10" s="50"/>
+      <c r="AU10" s="50"/>
+      <c r="AV10" s="50"/>
+      <c r="AW10" s="50"/>
+      <c r="AX10" s="50"/>
+      <c r="AY10" s="50"/>
+      <c r="AZ10" s="50"/>
+      <c r="BA10" s="50"/>
+      <c r="BB10" s="50"/>
+      <c r="BC10" s="50"/>
+      <c r="BD10" s="50"/>
+    </row>
+    <row r="11" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="I11" s="41" t="s">
         <v>83</v>
       </c>
       <c r="J11" s="8"/>
       <c r="K11" s="9"/>
-      <c r="L11" s="50" t="s">
+      <c r="L11" s="53" t="s">
         <v>71</v>
       </c>
-      <c r="M11" s="50"/>
-      <c r="N11" s="50"/>
-      <c r="O11" s="55" t="s">
+      <c r="M11" s="53"/>
+      <c r="N11" s="53"/>
+      <c r="O11" s="43" t="s">
         <v>76</v>
       </c>
-      <c r="P11" s="55"/>
-      <c r="Q11" s="55"/>
-      <c r="R11" s="55"/>
-      <c r="S11" s="55"/>
-      <c r="T11" s="55"/>
-      <c r="U11" s="55"/>
-      <c r="V11" s="55"/>
-      <c r="W11" s="51" t="s">
+      <c r="P11" s="43"/>
+      <c r="Q11" s="43"/>
+      <c r="R11" s="43"/>
+      <c r="S11" s="43"/>
+      <c r="T11" s="43"/>
+      <c r="U11" s="43"/>
+      <c r="V11" s="43"/>
+      <c r="W11" s="54" t="s">
         <v>77</v>
       </c>
-      <c r="X11" s="51"/>
-      <c r="Y11" s="57" t="s">
+      <c r="X11" s="54"/>
+      <c r="Y11" s="45" t="s">
         <v>68</v>
       </c>
-      <c r="Z11" s="57"/>
-      <c r="AA11" s="56" t="s">
+      <c r="Z11" s="45"/>
+      <c r="AA11" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="AB11" s="56"/>
-      <c r="AC11" s="56"/>
+      <c r="AB11" s="44"/>
+      <c r="AC11" s="44"/>
       <c r="AD11" s="2">
         <v>1</v>
       </c>
@@ -1385,39 +1469,39 @@
         <v>78</v>
       </c>
       <c r="AN11" s="2"/>
-      <c r="AO11" s="44">
+      <c r="AO11" s="46">
         <v>1</v>
       </c>
-      <c r="AP11" s="44"/>
-      <c r="AQ11" s="44"/>
-      <c r="AR11" s="44"/>
-      <c r="AS11" s="44">
+      <c r="AP11" s="46"/>
+      <c r="AQ11" s="46"/>
+      <c r="AR11" s="46"/>
+      <c r="AS11" s="46">
         <v>2</v>
       </c>
-      <c r="AT11" s="44"/>
-      <c r="AU11" s="44"/>
-      <c r="AV11" s="44"/>
-      <c r="AW11" s="44">
+      <c r="AT11" s="46"/>
+      <c r="AU11" s="46"/>
+      <c r="AV11" s="46"/>
+      <c r="AW11" s="46">
         <v>3</v>
       </c>
-      <c r="AX11" s="44"/>
-      <c r="AY11" s="44"/>
-      <c r="AZ11" s="44"/>
-      <c r="BA11" s="44" t="s">
+      <c r="AX11" s="46"/>
+      <c r="AY11" s="46"/>
+      <c r="AZ11" s="46"/>
+      <c r="BA11" s="46" t="s">
         <v>78</v>
       </c>
-      <c r="BB11" s="44"/>
-      <c r="BC11" s="44"/>
-      <c r="BD11" s="44"/>
-      <c r="BE11" s="44" t="s">
+      <c r="BB11" s="46"/>
+      <c r="BC11" s="46"/>
+      <c r="BD11" s="46"/>
+      <c r="BE11" s="46" t="s">
         <v>78</v>
       </c>
-      <c r="BF11" s="44"/>
-      <c r="BG11" s="44"/>
-      <c r="BH11" s="44"/>
-    </row>
-    <row r="12" spans="2:60" ht="60" x14ac:dyDescent="0.25">
-      <c r="I12" s="53"/>
+      <c r="BF11" s="46"/>
+      <c r="BG11" s="46"/>
+      <c r="BH11" s="46"/>
+    </row>
+    <row r="12" spans="2:60" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="I12" s="41"/>
       <c r="J12" s="10" t="s">
         <v>39</v>
       </c>
@@ -1448,7 +1532,7 @@
       <c r="S12" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="T12" s="14" t="s">
+      <c r="T12" s="61" t="s">
         <v>45</v>
       </c>
       <c r="U12" s="14" t="s">
@@ -1460,16 +1544,16 @@
       <c r="W12" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="X12" s="15" t="s">
+      <c r="X12" s="62" t="s">
         <v>58</v>
       </c>
-      <c r="Y12" s="16" t="s">
+      <c r="Y12" s="63" t="s">
         <v>70</v>
       </c>
       <c r="Z12" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="AA12" s="39" t="s">
+      <c r="AA12" s="37" t="s">
         <v>47</v>
       </c>
       <c r="AB12" s="17" t="s">
@@ -1562,7 +1646,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="13" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I13" s="2">
         <v>1</v>
       </c>
@@ -1601,7 +1685,7 @@
       <c r="Z13" s="2">
         <v>0</v>
       </c>
-      <c r="AA13" s="40">
+      <c r="AA13" s="38">
         <v>0</v>
       </c>
       <c r="AB13" s="25">
@@ -1642,14 +1726,14 @@
       <c r="BG13" s="2"/>
       <c r="BH13" s="2"/>
     </row>
-    <row r="14" spans="2:60" x14ac:dyDescent="0.25">
-      <c r="B14" s="44" t="s">
+    <row r="14" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="B14" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="44"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
+      <c r="C14" s="46"/>
+      <c r="D14" s="46"/>
+      <c r="E14" s="46"/>
+      <c r="F14" s="46"/>
       <c r="I14" s="2">
         <f>I13+1</f>
         <v>2</v>
@@ -1697,7 +1781,7 @@
       <c r="Z14" s="2">
         <v>0</v>
       </c>
-      <c r="AA14" s="40">
+      <c r="AA14" s="38">
         <v>0</v>
       </c>
       <c r="AB14" s="25">
@@ -1740,9 +1824,9 @@
       <c r="BG14" s="2"/>
       <c r="BH14" s="2"/>
     </row>
-    <row r="15" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B15" s="2" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>18</v>
@@ -1756,8 +1840,9 @@
       <c r="F15" s="1" t="s">
         <v>23</v>
       </c>
+      <c r="G15" s="64"/>
       <c r="I15" s="2">
-        <f t="shared" ref="I15:I52" si="0">I14+1</f>
+        <f t="shared" ref="I15:I54" si="0">I14+1</f>
         <v>3</v>
       </c>
       <c r="J15" s="18">
@@ -1802,7 +1887,7 @@
       <c r="Z15" s="2">
         <v>0</v>
       </c>
-      <c r="AA15" s="40">
+      <c r="AA15" s="38">
         <f>Q14</f>
         <v>7.3263888888888892E-3</v>
       </c>
@@ -1849,7 +1934,7 @@
       <c r="BG15" s="2"/>
       <c r="BH15" s="2"/>
     </row>
-    <row r="16" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B16" s="2" t="s">
         <v>19</v>
       </c>
@@ -1900,7 +1985,7 @@
       <c r="Z16" s="2">
         <v>0</v>
       </c>
-      <c r="AA16" s="40">
+      <c r="AA16" s="38">
         <f>AA15</f>
         <v>7.3263888888888892E-3</v>
       </c>
@@ -1952,7 +2037,7 @@
       <c r="BG16" s="2"/>
       <c r="BH16" s="2"/>
     </row>
-    <row r="17" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B17" s="2" t="s">
         <v>20</v>
       </c>
@@ -2016,7 +2101,7 @@
       <c r="Z17" s="2">
         <v>0</v>
       </c>
-      <c r="AA17" s="40">
+      <c r="AA17" s="38">
         <f>AA16+Q18</f>
         <v>1.6756944444444442E-2</v>
       </c>
@@ -2061,7 +2146,7 @@
       <c r="BG17" s="2"/>
       <c r="BH17" s="2"/>
     </row>
-    <row r="18" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I18" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -2108,7 +2193,7 @@
       <c r="Z18" s="2">
         <v>0</v>
       </c>
-      <c r="AA18" s="40">
+      <c r="AA18" s="38">
         <f>AA17+(J18-J17)</f>
         <v>1.6850835351328773E-2</v>
       </c>
@@ -2155,14 +2240,14 @@
       <c r="BG18" s="2"/>
       <c r="BH18" s="2"/>
     </row>
-    <row r="19" spans="2:60" x14ac:dyDescent="0.25">
-      <c r="B19" s="44" t="s">
+    <row r="19" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="B19" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="C19" s="44"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="44"/>
-      <c r="F19" s="44"/>
+      <c r="C19" s="46"/>
+      <c r="D19" s="46"/>
+      <c r="E19" s="46"/>
+      <c r="F19" s="46"/>
       <c r="I19" s="2">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -2176,7 +2261,7 @@
       </c>
       <c r="L19" s="1"/>
       <c r="M19" s="27"/>
-      <c r="N19" s="58">
+      <c r="N19" s="19">
         <f>N18</f>
         <v>0.47304426716643216</v>
       </c>
@@ -2212,7 +2297,7 @@
       <c r="Z19" s="2">
         <v>1</v>
       </c>
-      <c r="AA19" s="40">
+      <c r="AA19" s="38">
         <f>AA18+Q17</f>
         <v>2.6281390906884326E-2</v>
       </c>
@@ -2262,7 +2347,7 @@
       <c r="BG19" s="2"/>
       <c r="BH19" s="2"/>
     </row>
-    <row r="20" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B20" s="2" t="s">
         <v>24</v>
       </c>
@@ -2324,7 +2409,7 @@
       <c r="Z20" s="2">
         <v>1</v>
       </c>
-      <c r="AA20" s="40">
+      <c r="AA20" s="38">
         <f>AA19+Q18</f>
         <v>3.5711946462439879E-2</v>
       </c>
@@ -2376,7 +2461,7 @@
       <c r="BG20" s="2"/>
       <c r="BH20" s="2"/>
     </row>
-    <row r="21" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B21" s="2" t="s">
         <v>88</v>
       </c>
@@ -2444,7 +2529,7 @@
       <c r="Z21" s="2">
         <v>2</v>
       </c>
-      <c r="AA21" s="40">
+      <c r="AA21" s="38">
         <f>AA20+(J21-J20)</f>
         <v>3.813761646778998E-2</v>
       </c>
@@ -2499,7 +2584,7 @@
       <c r="BG21" s="2"/>
       <c r="BH21" s="2"/>
     </row>
-    <row r="22" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:60" x14ac:dyDescent="0.35">
       <c r="B22" s="2" t="s">
         <v>89</v>
       </c>
@@ -2561,7 +2646,7 @@
       <c r="Z22" s="2">
         <v>2</v>
       </c>
-      <c r="AA22" s="40">
+      <c r="AA22" s="38">
         <f>AA21++J22-J21</f>
         <v>4.3677329263339615E-2</v>
       </c>
@@ -2618,7 +2703,7 @@
       <c r="BG22" s="2"/>
       <c r="BH22" s="2"/>
     </row>
-    <row r="23" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I23" s="2">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -2677,7 +2762,7 @@
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
-      <c r="AC23" s="35">
+      <c r="AC23" s="34">
         <v>0</v>
       </c>
       <c r="AD23" s="2"/>
@@ -2724,14 +2809,14 @@
       <c r="BG23" s="2"/>
       <c r="BH23" s="2"/>
     </row>
-    <row r="24" spans="2:60" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="45" t="s">
+    <row r="24" spans="2:60" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="48" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="45"/>
-      <c r="D24" s="45"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="45"/>
+      <c r="C24" s="48"/>
+      <c r="D24" s="48"/>
+      <c r="E24" s="48"/>
+      <c r="F24" s="48"/>
       <c r="I24" s="2">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -2785,7 +2870,7 @@
         <f t="shared" si="1"/>
         <v>1.2939010589645406E-2</v>
       </c>
-      <c r="AC24" s="35">
+      <c r="AC24" s="34">
         <v>0</v>
       </c>
       <c r="AD24" s="2"/>
@@ -2832,12 +2917,12 @@
       <c r="BG24" s="2"/>
       <c r="BH24" s="2"/>
     </row>
-    <row r="25" spans="2:60" x14ac:dyDescent="0.25">
-      <c r="B25" s="45"/>
-      <c r="C25" s="45"/>
-      <c r="D25" s="45"/>
-      <c r="E25" s="45"/>
-      <c r="F25" s="45"/>
+    <row r="25" spans="2:60" x14ac:dyDescent="0.35">
+      <c r="B25" s="48"/>
+      <c r="C25" s="48"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="48"/>
+      <c r="F25" s="48"/>
       <c r="I25" s="2">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -2883,7 +2968,7 @@
         <f>AB24+X24</f>
         <v>1.6474657557670053E-2</v>
       </c>
-      <c r="AC25" s="35">
+      <c r="AC25" s="34">
         <v>0</v>
       </c>
       <c r="AD25" s="2"/>
@@ -2931,7 +3016,7 @@
       <c r="BG25" s="2"/>
       <c r="BH25" s="2"/>
     </row>
-    <row r="26" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I26" s="2">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -2987,7 +3072,7 @@
         <f>AB25</f>
         <v>1.6474657557670053E-2</v>
       </c>
-      <c r="AC26" s="35">
+      <c r="AC26" s="34">
         <v>0</v>
       </c>
       <c r="AD26" s="2"/>
@@ -3032,7 +3117,7 @@
       <c r="BG26" s="2"/>
       <c r="BH26" s="2"/>
     </row>
-    <row r="27" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I27" s="2">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -3082,7 +3167,7 @@
         <f>AB26</f>
         <v>1.6474657557670053E-2</v>
       </c>
-      <c r="AC27" s="35">
+      <c r="AC27" s="34">
         <v>0</v>
       </c>
       <c r="AD27" s="2"/>
@@ -3125,7 +3210,7 @@
       <c r="BG27" s="2"/>
       <c r="BH27" s="2"/>
     </row>
-    <row r="28" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I28" s="2">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -3166,7 +3251,7 @@
         <f>X25+AB27</f>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC28" s="35">
+      <c r="AC28" s="34">
         <v>0</v>
       </c>
       <c r="AD28" s="2"/>
@@ -3209,7 +3294,7 @@
       <c r="BG28" s="2"/>
       <c r="BH28" s="2"/>
     </row>
-    <row r="29" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I29" s="2">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -3263,7 +3348,7 @@
         <f>AB28</f>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC29" s="35">
+      <c r="AC29" s="34">
         <v>0</v>
       </c>
       <c r="AD29" s="2"/>
@@ -3300,7 +3385,7 @@
       <c r="BG29" s="2"/>
       <c r="BH29" s="2"/>
     </row>
-    <row r="30" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I30" s="2">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -3355,7 +3440,7 @@
         <f t="shared" ref="AB30:AB36" si="4">AB29</f>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC30" s="35">
+      <c r="AC30" s="34">
         <v>0</v>
       </c>
       <c r="AD30" s="2"/>
@@ -3395,7 +3480,7 @@
       <c r="BG30" s="2"/>
       <c r="BH30" s="2"/>
     </row>
-    <row r="31" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I31" s="2">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -3428,7 +3513,7 @@
         <f>($F$8+P31*($F$9-$F$8)) / 1440</f>
         <v>1.0500000000000001E-2</v>
       </c>
-      <c r="R31" s="41">
+      <c r="R31" s="39">
         <f>Q31+J31</f>
         <v>0.6536663887512224</v>
       </c>
@@ -3452,7 +3537,7 @@
         <f t="shared" si="4"/>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC31" s="35">
+      <c r="AC31" s="34">
         <v>0</v>
       </c>
       <c r="AD31" s="2"/>
@@ -3497,7 +3582,7 @@
       <c r="BG31" s="2"/>
       <c r="BH31" s="2"/>
     </row>
-    <row r="32" spans="2:60" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:60" x14ac:dyDescent="0.35">
       <c r="I32" s="2">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -3549,7 +3634,7 @@
         <f t="shared" si="4"/>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC32" s="35">
+      <c r="AC32" s="34">
         <v>0</v>
       </c>
       <c r="AD32" s="2"/>
@@ -3593,7 +3678,7 @@
       <c r="BG32" s="2"/>
       <c r="BH32" s="2"/>
     </row>
-    <row r="33" spans="9:60" x14ac:dyDescent="0.25">
+    <row r="33" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I33" s="2">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -3653,7 +3738,7 @@
         <f t="shared" si="4"/>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC33" s="35">
+      <c r="AC33" s="34">
         <v>0</v>
       </c>
       <c r="AD33" s="2"/>
@@ -3663,7 +3748,7 @@
       <c r="AH33" s="2"/>
       <c r="AI33" s="2"/>
       <c r="AJ33" s="2"/>
-      <c r="AK33" s="42"/>
+      <c r="AK33" s="40"/>
       <c r="AL33" s="2" t="s">
         <v>84</v>
       </c>
@@ -3695,7 +3780,7 @@
       <c r="BG33" s="2"/>
       <c r="BH33" s="2"/>
     </row>
-    <row r="34" spans="9:60" x14ac:dyDescent="0.25">
+    <row r="34" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I34" s="2">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -3745,7 +3830,7 @@
         <f t="shared" si="4"/>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC34" s="35">
+      <c r="AC34" s="34">
         <v>0</v>
       </c>
       <c r="AD34" s="2"/>
@@ -3790,7 +3875,7 @@
       <c r="BG34" s="2"/>
       <c r="BH34" s="2"/>
     </row>
-    <row r="35" spans="9:60" x14ac:dyDescent="0.25">
+    <row r="35" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I35" s="2">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -3847,7 +3932,7 @@
         <f t="shared" si="4"/>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC35" s="35">
+      <c r="AC35" s="34">
         <v>0</v>
       </c>
       <c r="AD35" s="2"/>
@@ -3897,7 +3982,7 @@
       <c r="BG35" s="2"/>
       <c r="BH35" s="2"/>
     </row>
-    <row r="36" spans="9:60" x14ac:dyDescent="0.25">
+    <row r="36" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I36" s="2">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -3938,7 +4023,7 @@
         <f t="shared" si="4"/>
         <v>3.1128239508575246E-2</v>
       </c>
-      <c r="AC36" s="35">
+      <c r="AC36" s="34">
         <v>0</v>
       </c>
       <c r="AD36" s="2"/>
@@ -3983,955 +4068,2119 @@
       <c r="BG36" s="2"/>
       <c r="BH36" s="2"/>
     </row>
-    <row r="37" spans="9:60" x14ac:dyDescent="0.25">
+    <row r="37" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I37" s="2">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="J37" s="34">
+      <c r="J37" s="33">
         <f>J36+X35</f>
         <v>0.75378195932260272</v>
       </c>
-      <c r="K37" s="43" t="s">
+      <c r="K37" s="56" t="s">
         <v>117</v>
       </c>
-      <c r="L37" s="36"/>
-      <c r="M37" s="38"/>
-      <c r="N37" s="34">
+      <c r="L37" s="35"/>
+      <c r="M37" s="36"/>
+      <c r="N37" s="33">
         <f>N36</f>
         <v>0.76346586328319521</v>
       </c>
-      <c r="O37" s="36" t="s">
+      <c r="O37" s="35" t="s">
         <v>60</v>
       </c>
-      <c r="P37" s="36"/>
-      <c r="Q37" s="38"/>
-      <c r="R37" s="34"/>
-      <c r="S37" s="36"/>
-      <c r="T37" s="36"/>
-      <c r="U37" s="36"/>
-      <c r="V37" s="36"/>
-      <c r="W37" s="36"/>
-      <c r="X37" s="38"/>
-      <c r="Y37" s="36">
-        <v>0</v>
-      </c>
-      <c r="Z37" s="36">
-        <v>0</v>
-      </c>
-      <c r="AA37" s="38"/>
-      <c r="AB37" s="38">
+      <c r="P37" s="35"/>
+      <c r="Q37" s="36"/>
+      <c r="R37" s="33"/>
+      <c r="S37" s="35"/>
+      <c r="T37" s="35"/>
+      <c r="U37" s="35"/>
+      <c r="V37" s="35"/>
+      <c r="W37" s="35"/>
+      <c r="X37" s="36"/>
+      <c r="Y37" s="35">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="35">
+        <v>0</v>
+      </c>
+      <c r="AA37" s="36"/>
+      <c r="AB37" s="36">
         <f>AB36+X30</f>
         <v>0.16469515541585475</v>
       </c>
-      <c r="AC37" s="36"/>
-      <c r="AD37" s="36"/>
-      <c r="AE37" s="36"/>
-      <c r="AF37" s="36"/>
-      <c r="AG37" s="36"/>
-      <c r="AH37" s="36"/>
-      <c r="AI37" s="36"/>
-      <c r="AJ37" s="36"/>
-      <c r="AK37" s="36"/>
-      <c r="AL37" s="36"/>
-      <c r="AM37" s="36"/>
-      <c r="AN37" s="36"/>
-      <c r="AO37" s="36"/>
-      <c r="AP37" s="36"/>
-      <c r="AQ37" s="36"/>
-      <c r="AR37" s="36"/>
-      <c r="AS37" s="36"/>
-      <c r="AT37" s="36"/>
-      <c r="AU37" s="36"/>
-      <c r="AV37" s="36"/>
-      <c r="AW37" s="36"/>
-      <c r="AX37" s="36"/>
-      <c r="AY37" s="36"/>
-      <c r="AZ37" s="36"/>
-      <c r="BA37" s="36"/>
-      <c r="BB37" s="34">
+      <c r="AC37" s="35"/>
+      <c r="AD37" s="35"/>
+      <c r="AE37" s="35"/>
+      <c r="AF37" s="35"/>
+      <c r="AG37" s="35"/>
+      <c r="AH37" s="35"/>
+      <c r="AI37" s="35"/>
+      <c r="AJ37" s="35"/>
+      <c r="AK37" s="35"/>
+      <c r="AL37" s="35"/>
+      <c r="AM37" s="35"/>
+      <c r="AN37" s="35"/>
+      <c r="AO37" s="35"/>
+      <c r="AP37" s="35"/>
+      <c r="AQ37" s="35"/>
+      <c r="AR37" s="35"/>
+      <c r="AS37" s="35"/>
+      <c r="AT37" s="35"/>
+      <c r="AU37" s="35"/>
+      <c r="AV37" s="35"/>
+      <c r="AW37" s="35"/>
+      <c r="AX37" s="35"/>
+      <c r="AY37" s="35"/>
+      <c r="AZ37" s="35"/>
+      <c r="BA37" s="35"/>
+      <c r="BB37" s="33">
         <f>BB36</f>
         <v>0.59281226563754541</v>
       </c>
-      <c r="BC37" s="34">
+      <c r="BC37" s="33">
         <f>J37</f>
         <v>0.75378195932260272</v>
       </c>
-      <c r="BD37" s="36"/>
-      <c r="BE37" s="36" t="s">
+      <c r="BD37" s="35"/>
+      <c r="BE37" s="35" t="s">
         <v>90</v>
       </c>
-      <c r="BF37" s="34">
+      <c r="BF37" s="33">
         <f>BF36</f>
         <v>0.66279138875122245</v>
       </c>
-      <c r="BG37" s="36"/>
-      <c r="BH37" s="36"/>
-    </row>
-    <row r="38" spans="9:60" x14ac:dyDescent="0.25">
+      <c r="BG37" s="35"/>
+      <c r="BH37" s="35"/>
+    </row>
+    <row r="38" spans="9:60" x14ac:dyDescent="0.35">
       <c r="I38" s="2">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="M38" s="28"/>
-      <c r="Q38" s="28"/>
-      <c r="R38" s="33"/>
-      <c r="T38" s="33"/>
-      <c r="X38" s="28"/>
-      <c r="AA38" s="28"/>
-      <c r="AB38" s="28"/>
-      <c r="BB38" s="37"/>
-      <c r="BC38" s="37"/>
-      <c r="BD38" s="37"/>
-    </row>
-    <row r="39" spans="9:60" x14ac:dyDescent="0.25">
-      <c r="I39" s="2">
+      <c r="J38" s="57"/>
+      <c r="K38" s="57"/>
+      <c r="L38" s="57"/>
+      <c r="M38" s="57"/>
+      <c r="N38" s="57"/>
+      <c r="O38" s="57"/>
+      <c r="P38" s="57"/>
+      <c r="Q38" s="57"/>
+      <c r="R38" s="57"/>
+      <c r="S38" s="57"/>
+      <c r="T38" s="57"/>
+      <c r="U38" s="57"/>
+      <c r="V38" s="57"/>
+      <c r="W38" s="57"/>
+      <c r="X38" s="57"/>
+      <c r="Y38" s="57"/>
+      <c r="Z38" s="57"/>
+      <c r="AA38" s="57"/>
+      <c r="AB38" s="57"/>
+      <c r="AC38" s="57"/>
+      <c r="AD38" s="57"/>
+      <c r="AE38" s="57"/>
+      <c r="AF38" s="57"/>
+      <c r="AG38" s="57"/>
+      <c r="AH38" s="57"/>
+      <c r="AI38" s="57"/>
+      <c r="AJ38" s="57"/>
+      <c r="AK38" s="57"/>
+      <c r="AL38" s="57"/>
+      <c r="AM38" s="57"/>
+      <c r="AN38" s="57"/>
+      <c r="AO38" s="57"/>
+      <c r="AP38" s="57"/>
+      <c r="AQ38" s="57"/>
+      <c r="AR38" s="57"/>
+      <c r="AS38" s="57"/>
+      <c r="AT38" s="57"/>
+      <c r="AU38" s="57"/>
+      <c r="AV38" s="57"/>
+      <c r="AW38" s="57"/>
+      <c r="AX38" s="57"/>
+      <c r="AY38" s="57"/>
+      <c r="AZ38" s="57"/>
+      <c r="BA38" s="57"/>
+      <c r="BB38" s="57"/>
+      <c r="BC38" s="57"/>
+      <c r="BD38" s="57"/>
+      <c r="BE38" s="57"/>
+      <c r="BF38" s="57"/>
+      <c r="BG38" s="57"/>
+      <c r="BH38" s="57"/>
+    </row>
+    <row r="39" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I39" s="68">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="M39" s="28"/>
-      <c r="Q39" s="28"/>
-      <c r="R39" s="33"/>
-      <c r="X39" s="28"/>
-      <c r="AA39" s="28"/>
-      <c r="AB39" s="28"/>
-    </row>
-    <row r="40" spans="9:60" x14ac:dyDescent="0.25">
-      <c r="I40" s="2">
+      <c r="J39" s="58">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="L39" s="2">
+        <v>0.41199999999999998</v>
+      </c>
+      <c r="M39" s="25">
+        <f>-$C$3*(LN(1-L39)) / 1440</f>
+        <v>1.6594635346359687E-2</v>
+      </c>
+      <c r="N39" s="19">
+        <f>J39+M39</f>
+        <v>0.43326130201302637</v>
+      </c>
+      <c r="O39" s="59" t="s">
+        <v>53</v>
+      </c>
+      <c r="P39" s="2"/>
+      <c r="Q39" s="25"/>
+      <c r="R39" s="18"/>
+      <c r="S39" s="2"/>
+      <c r="T39" s="2"/>
+      <c r="U39" s="2"/>
+      <c r="V39" s="2"/>
+      <c r="W39" s="2"/>
+      <c r="X39" s="25"/>
+      <c r="Y39" s="60">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="60">
+        <v>0</v>
+      </c>
+      <c r="AA39" s="74">
+        <v>0</v>
+      </c>
+      <c r="AB39" s="74">
+        <v>0</v>
+      </c>
+      <c r="AC39" s="77">
+        <v>0</v>
+      </c>
+      <c r="AD39" s="2"/>
+      <c r="AE39" s="2"/>
+      <c r="AF39" s="2"/>
+      <c r="AG39" s="2"/>
+      <c r="AH39" s="2"/>
+      <c r="AI39" s="2"/>
+      <c r="AJ39" s="2"/>
+      <c r="AK39" s="2"/>
+      <c r="AL39" s="2"/>
+      <c r="AM39" s="2"/>
+      <c r="AN39" s="2"/>
+      <c r="AO39" s="2"/>
+      <c r="AP39" s="2"/>
+      <c r="AQ39" s="2"/>
+      <c r="AR39" s="2"/>
+      <c r="AS39" s="2"/>
+      <c r="AT39" s="2"/>
+      <c r="AU39" s="2"/>
+      <c r="AV39" s="2"/>
+      <c r="AW39" s="2"/>
+      <c r="AX39" s="2"/>
+      <c r="AY39" s="2"/>
+      <c r="AZ39" s="2"/>
+      <c r="BA39" s="2"/>
+      <c r="BB39" s="69"/>
+      <c r="BC39" s="2"/>
+      <c r="BD39" s="2"/>
+      <c r="BE39" s="2"/>
+      <c r="BF39" s="2"/>
+      <c r="BG39" s="2"/>
+      <c r="BH39" s="2"/>
+    </row>
+    <row r="40" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I40" s="68">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="M40" s="28"/>
-      <c r="Q40" s="28"/>
-      <c r="R40" s="33"/>
-      <c r="T40" s="33"/>
-      <c r="X40" s="28"/>
-      <c r="AA40" s="28"/>
-      <c r="AB40" s="28"/>
-    </row>
-    <row r="41" spans="9:60" x14ac:dyDescent="0.25">
-      <c r="I41" s="2">
+      <c r="J40" s="58">
+        <f>N39</f>
+        <v>0.43326130201302637</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="L40" s="2">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="M40" s="25">
+        <f>-$C$3*(LN(1-L40)) / 1440</f>
+        <v>5.7464096148809533E-2</v>
+      </c>
+      <c r="N40" s="18">
+        <f>J40+M40</f>
+        <v>0.49072539816183591</v>
+      </c>
+      <c r="O40" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="P40" s="2">
+        <v>0.98599999999999999</v>
+      </c>
+      <c r="Q40" s="25">
+        <f>($F$8+P40*($F$9-$F$8)) / 1440</f>
+        <v>1.3791666666666666E-2</v>
+      </c>
+      <c r="R40" s="19">
+        <f>J40+Q40</f>
+        <v>0.44705296867969302</v>
+      </c>
+      <c r="S40" s="66"/>
+      <c r="T40" s="18"/>
+      <c r="U40" s="2"/>
+      <c r="V40" s="2"/>
+      <c r="W40" s="2"/>
+      <c r="X40" s="25"/>
+      <c r="Y40" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z40" s="68">
+        <v>0</v>
+      </c>
+      <c r="AA40" s="75"/>
+      <c r="AB40" s="76">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="AC40" s="75">
+        <v>0</v>
+      </c>
+      <c r="AD40" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="AE40" s="2"/>
+      <c r="AF40" s="2"/>
+      <c r="AG40" s="2"/>
+      <c r="AH40" s="2"/>
+      <c r="AI40" s="2"/>
+      <c r="AJ40" s="2"/>
+      <c r="AK40" s="2"/>
+      <c r="AL40" s="2"/>
+      <c r="AM40" s="2"/>
+      <c r="AN40" s="2"/>
+      <c r="AO40" s="2"/>
+      <c r="AP40" s="2"/>
+      <c r="AQ40" s="2"/>
+      <c r="AR40" s="2"/>
+      <c r="AS40" s="2"/>
+      <c r="AT40" s="2"/>
+      <c r="AU40" s="2"/>
+      <c r="AV40" s="2"/>
+      <c r="AW40" s="2"/>
+      <c r="AX40" s="2"/>
+      <c r="AY40" s="2"/>
+      <c r="AZ40" s="2"/>
+      <c r="BA40" s="2"/>
+      <c r="BB40" s="69"/>
+      <c r="BC40" s="2"/>
+      <c r="BD40" s="2"/>
+      <c r="BE40" s="2"/>
+      <c r="BF40" s="2"/>
+      <c r="BG40" s="2"/>
+      <c r="BH40" s="2"/>
+    </row>
+    <row r="41" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I41" s="68">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="N41" t="s">
-        <v>118</v>
-      </c>
-      <c r="Q41" s="28"/>
-      <c r="R41" s="33"/>
-      <c r="X41" s="28"/>
-      <c r="AA41" s="28"/>
-      <c r="AB41" s="28"/>
-    </row>
-    <row r="42" spans="9:60" x14ac:dyDescent="0.25">
-      <c r="I42" s="2">
+      <c r="J41" s="58">
+        <f>R40</f>
+        <v>0.44705296867969302</v>
+      </c>
+      <c r="K41" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="L41" s="2"/>
+      <c r="M41" s="25"/>
+      <c r="N41" s="65">
+        <f>N40</f>
+        <v>0.49072539816183591</v>
+      </c>
+      <c r="O41" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="P41" s="2"/>
+      <c r="Q41" s="25"/>
+      <c r="R41" s="19"/>
+      <c r="S41" s="66">
+        <f>0.853</f>
+        <v>0.85299999999999998</v>
+      </c>
+      <c r="T41" s="2" t="str">
+        <f>IF(S41&lt;$D$16,"Elevado","Normal")</f>
+        <v>Normal</v>
+      </c>
+      <c r="U41" s="2"/>
+      <c r="V41" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="W41" s="2">
+        <v>0.32300000000000001</v>
+      </c>
+      <c r="X41" s="25">
+        <f>-90*LN(1-W41) / 1440</f>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="Y41" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z41" s="68">
+        <v>0</v>
+      </c>
+      <c r="AA41" s="76"/>
+      <c r="AB41" s="76">
+        <f>0</f>
+        <v>0</v>
+      </c>
+      <c r="AC41" s="75">
+        <v>0</v>
+      </c>
+      <c r="AD41" s="21"/>
+      <c r="AE41" s="2"/>
+      <c r="AF41" s="2"/>
+      <c r="AG41" s="2"/>
+      <c r="AH41" s="2"/>
+      <c r="AI41" s="2"/>
+      <c r="AJ41" s="2"/>
+      <c r="AK41" s="2"/>
+      <c r="AL41" s="2"/>
+      <c r="AM41" s="2"/>
+      <c r="AN41" s="2"/>
+      <c r="AO41" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AP41" s="58">
+        <f>J41</f>
+        <v>0.44705296867969302</v>
+      </c>
+      <c r="AQ41" s="2"/>
+      <c r="AR41" s="25">
+        <f>X41</f>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="AS41" s="2"/>
+      <c r="AT41" s="2"/>
+      <c r="AU41" s="2"/>
+      <c r="AV41" s="2"/>
+      <c r="AW41" s="2"/>
+      <c r="AX41" s="2"/>
+      <c r="AY41" s="2"/>
+      <c r="AZ41" s="2"/>
+      <c r="BA41" s="2"/>
+      <c r="BB41" s="69"/>
+      <c r="BC41" s="2"/>
+      <c r="BD41" s="2"/>
+      <c r="BE41" s="2"/>
+      <c r="BF41" s="2"/>
+      <c r="BG41" s="2"/>
+      <c r="BH41" s="2"/>
+    </row>
+    <row r="42" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I42" s="68">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="M42" s="28"/>
-      <c r="Q42" s="28"/>
-      <c r="R42" s="33"/>
-      <c r="X42" s="28"/>
-      <c r="AA42" s="28"/>
-      <c r="AB42" s="28"/>
-    </row>
-    <row r="43" spans="9:60" x14ac:dyDescent="0.25">
-      <c r="I43" s="2">
+      <c r="J42" s="58">
+        <f>J41+AR41</f>
+        <v>0.47143321905905938</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="L42" s="2"/>
+      <c r="M42" s="25"/>
+      <c r="N42" s="19">
+        <f>N41</f>
+        <v>0.49072539816183591</v>
+      </c>
+      <c r="O42" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="P42" s="2">
+        <f>0.212</f>
+        <v>0.21199999999999999</v>
+      </c>
+      <c r="Q42" s="25">
+        <f>($F$8+P42*($F$9-$F$8)) / 1440</f>
+        <v>8.4166666666666678E-3</v>
+      </c>
+      <c r="R42" s="19">
+        <f t="shared" ref="R42" si="6">J42+Q42</f>
+        <v>0.47984988572572607</v>
+      </c>
+      <c r="S42" s="66"/>
+      <c r="T42" s="2"/>
+      <c r="U42" s="2"/>
+      <c r="V42" s="2"/>
+      <c r="W42" s="2"/>
+      <c r="X42" s="25"/>
+      <c r="Y42" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z42" s="68">
+        <v>0</v>
+      </c>
+      <c r="AA42" s="76"/>
+      <c r="AB42" s="76">
+        <f>AB40+X41</f>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="AC42" s="75">
+        <v>0</v>
+      </c>
+      <c r="AD42" s="2"/>
+      <c r="AE42" s="2"/>
+      <c r="AF42" s="2"/>
+      <c r="AG42" s="2"/>
+      <c r="AH42" s="2"/>
+      <c r="AI42" s="2"/>
+      <c r="AJ42" s="2"/>
+      <c r="AK42" s="2"/>
+      <c r="AL42" s="2"/>
+      <c r="AM42" s="2"/>
+      <c r="AN42" s="2"/>
+      <c r="AO42" s="23"/>
+      <c r="AP42" s="58">
+        <f>J42</f>
+        <v>0.47143321905905938</v>
+      </c>
+      <c r="AQ42" s="2"/>
+      <c r="AR42" s="58"/>
+      <c r="AS42" s="2"/>
+      <c r="AT42" s="2"/>
+      <c r="AU42" s="2"/>
+      <c r="AV42" s="2"/>
+      <c r="AW42" s="2"/>
+      <c r="AX42" s="2"/>
+      <c r="AY42" s="2"/>
+      <c r="AZ42" s="2"/>
+      <c r="BA42" s="2"/>
+      <c r="BB42" s="69"/>
+      <c r="BC42" s="2"/>
+      <c r="BD42" s="2"/>
+      <c r="BE42" s="2"/>
+      <c r="BF42" s="2"/>
+      <c r="BG42" s="2"/>
+      <c r="BH42" s="2"/>
+    </row>
+    <row r="43" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I43" s="68">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="M43" s="28"/>
-      <c r="Q43" s="28"/>
-      <c r="R43" s="33"/>
-      <c r="X43" s="28"/>
-      <c r="AA43" s="28"/>
-      <c r="AB43" s="28"/>
-    </row>
-    <row r="44" spans="9:60" x14ac:dyDescent="0.25">
-      <c r="I44" s="2">
+      <c r="J43" s="58">
+        <f>N42</f>
+        <v>0.49072539816183591</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="L43" s="2">
+        <v>0.92800000000000005</v>
+      </c>
+      <c r="M43" s="25">
+        <f t="shared" ref="M43:M47" si="7">-$C$3*(LN(1-L43)) / 1440</f>
+        <v>8.2221536248940075E-2</v>
+      </c>
+      <c r="N43" s="18">
+        <f>M43+J43</f>
+        <v>0.57294693441077604</v>
+      </c>
+      <c r="O43" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="P43" s="2">
+        <v>0.58199999999999996</v>
+      </c>
+      <c r="Q43" s="25">
+        <f>($F$8+P43*($F$9-$F$8)) / 1440</f>
+        <v>1.0986111111111111E-2</v>
+      </c>
+      <c r="R43" s="19">
+        <f t="shared" ref="R43" si="8">J43+Q43</f>
+        <v>0.50171150927294705</v>
+      </c>
+      <c r="S43" s="66"/>
+      <c r="T43" s="2"/>
+      <c r="U43" s="2"/>
+      <c r="V43" s="2"/>
+      <c r="W43" s="2"/>
+      <c r="X43" s="25"/>
+      <c r="Y43" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z43" s="68">
+        <v>0</v>
+      </c>
+      <c r="AA43" s="76"/>
+      <c r="AB43" s="76">
+        <f>AB42</f>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="AC43" s="55">
+        <v>0</v>
+      </c>
+      <c r="AD43" s="2"/>
+      <c r="AE43" s="2"/>
+      <c r="AF43" s="2"/>
+      <c r="AG43" s="2"/>
+      <c r="AH43" s="2"/>
+      <c r="AI43" s="2"/>
+      <c r="AJ43" s="2"/>
+      <c r="AK43" s="2"/>
+      <c r="AL43" s="2"/>
+      <c r="AM43" s="2"/>
+      <c r="AN43" s="2"/>
+      <c r="AO43" s="23"/>
+      <c r="AP43" s="23"/>
+      <c r="AQ43" s="23"/>
+      <c r="AR43" s="23"/>
+      <c r="AS43" s="2"/>
+      <c r="AT43" s="2"/>
+      <c r="AU43" s="2"/>
+      <c r="AV43" s="2"/>
+      <c r="AW43" s="2"/>
+      <c r="AX43" s="2"/>
+      <c r="AY43" s="2"/>
+      <c r="AZ43" s="2"/>
+      <c r="BA43" s="2"/>
+      <c r="BB43" s="69"/>
+      <c r="BC43" s="2"/>
+      <c r="BD43" s="2"/>
+      <c r="BE43" s="2"/>
+      <c r="BF43" s="2"/>
+      <c r="BG43" s="2"/>
+      <c r="BH43" s="2"/>
+    </row>
+    <row r="44" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I44" s="68">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="M44" s="28"/>
-      <c r="Q44" s="28"/>
-      <c r="R44" s="33"/>
-      <c r="X44" s="28"/>
-      <c r="AA44" s="28"/>
-      <c r="AB44" s="28"/>
-    </row>
-    <row r="45" spans="9:60" x14ac:dyDescent="0.25">
-      <c r="I45" s="2">
+      <c r="J44" s="18">
+        <f>R43</f>
+        <v>0.50171150927294705</v>
+      </c>
+      <c r="K44" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="L44" s="2"/>
+      <c r="M44" s="25"/>
+      <c r="N44" s="19">
+        <f>N43</f>
+        <v>0.57294693441077604</v>
+      </c>
+      <c r="O44" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="P44" s="2"/>
+      <c r="Q44" s="25"/>
+      <c r="R44" s="19"/>
+      <c r="S44" s="66">
+        <f>0.21</f>
+        <v>0.21</v>
+      </c>
+      <c r="T44" s="2" t="str">
+        <f>IF(S44&lt;$D$16,"Elevado","Normal")</f>
+        <v>Elevado</v>
+      </c>
+      <c r="U44" s="2">
+        <v>0.312</v>
+      </c>
+      <c r="V44" s="2" t="str">
+        <f>IF(U44&lt;$D$21,"NO","SI")</f>
+        <v>NO</v>
+      </c>
+      <c r="W44" s="2"/>
+      <c r="X44" s="25"/>
+      <c r="Y44" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z44" s="68">
+        <v>0</v>
+      </c>
+      <c r="AA44" s="76"/>
+      <c r="AB44" s="76">
+        <f t="shared" ref="AB44:AB52" si="9">AB43</f>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="AC44" s="55">
+        <v>0</v>
+      </c>
+      <c r="AD44" s="2"/>
+      <c r="AE44" s="2"/>
+      <c r="AF44" s="2"/>
+      <c r="AG44" s="2"/>
+      <c r="AH44" s="2"/>
+      <c r="AI44" s="2"/>
+      <c r="AJ44" s="2"/>
+      <c r="AK44" s="2"/>
+      <c r="AL44" s="2"/>
+      <c r="AM44" s="2"/>
+      <c r="AN44" s="2"/>
+      <c r="AO44" s="2"/>
+      <c r="AP44" s="2"/>
+      <c r="AQ44" s="2"/>
+      <c r="AR44" s="2"/>
+      <c r="AS44" s="2"/>
+      <c r="AT44" s="2"/>
+      <c r="AU44" s="2"/>
+      <c r="AV44" s="2"/>
+      <c r="AW44" s="2"/>
+      <c r="AX44" s="2"/>
+      <c r="AY44" s="2"/>
+      <c r="AZ44" s="2"/>
+      <c r="BA44" s="2"/>
+      <c r="BB44" s="69"/>
+      <c r="BC44" s="2"/>
+      <c r="BD44" s="2"/>
+      <c r="BE44" s="2"/>
+      <c r="BF44" s="2"/>
+      <c r="BG44" s="2"/>
+      <c r="BH44" s="2"/>
+    </row>
+    <row r="45" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I45" s="68">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="M45" s="28"/>
-      <c r="Q45" s="28"/>
-      <c r="R45" s="33"/>
-      <c r="X45" s="28"/>
-      <c r="AA45" s="28"/>
-      <c r="AB45" s="28"/>
-    </row>
-    <row r="46" spans="9:60" x14ac:dyDescent="0.25">
-      <c r="I46" s="2">
+      <c r="J45" s="18">
+        <f>N44</f>
+        <v>0.57294693441077604</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="L45" s="2">
+        <v>0.23100000000000001</v>
+      </c>
+      <c r="M45" s="25">
+        <f>-$C$3*(LN(1-L45)) / 1440</f>
+        <v>8.2082596711404079E-3</v>
+      </c>
+      <c r="N45" s="19">
+        <f>J45+M45</f>
+        <v>0.5811551940819164</v>
+      </c>
+      <c r="O45" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="P45" s="2">
+        <v>0.32100000000000001</v>
+      </c>
+      <c r="Q45" s="25">
+        <f>($F$8+P45*($F$9-$F$8)) / 1440</f>
+        <v>9.1736111111111115E-3</v>
+      </c>
+      <c r="R45" s="39">
+        <f t="shared" ref="R45" si="10">J45+Q45</f>
+        <v>0.58212054552188719</v>
+      </c>
+      <c r="S45" s="66"/>
+      <c r="T45" s="2"/>
+      <c r="U45" s="2"/>
+      <c r="V45" s="2"/>
+      <c r="W45" s="2"/>
+      <c r="X45" s="25"/>
+      <c r="Y45" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z45" s="68">
+        <v>0</v>
+      </c>
+      <c r="AA45" s="76"/>
+      <c r="AB45" s="76">
+        <f t="shared" si="9"/>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="AC45" s="55">
+        <v>0</v>
+      </c>
+      <c r="AD45" s="2"/>
+      <c r="AE45" s="2"/>
+      <c r="AF45" s="2"/>
+      <c r="AG45" s="2"/>
+      <c r="AH45" s="2"/>
+      <c r="AI45" s="2"/>
+      <c r="AJ45" s="2"/>
+      <c r="AK45" s="2"/>
+      <c r="AL45" s="2"/>
+      <c r="AM45" s="2"/>
+      <c r="AN45" s="2"/>
+      <c r="AO45" s="2"/>
+      <c r="AP45" s="2"/>
+      <c r="AQ45" s="2"/>
+      <c r="AR45" s="2"/>
+      <c r="AS45" s="2"/>
+      <c r="AT45" s="2"/>
+      <c r="AU45" s="2"/>
+      <c r="AV45" s="2"/>
+      <c r="AW45" s="2"/>
+      <c r="AX45" s="2"/>
+      <c r="AY45" s="2"/>
+      <c r="AZ45" s="2"/>
+      <c r="BA45" s="2"/>
+      <c r="BB45" s="69"/>
+      <c r="BC45" s="2"/>
+      <c r="BD45" s="2"/>
+      <c r="BE45" s="2"/>
+      <c r="BF45" s="2"/>
+      <c r="BG45" s="2"/>
+      <c r="BH45" s="2"/>
+    </row>
+    <row r="46" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I46" s="68">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="M46" s="28"/>
-      <c r="Q46" s="28"/>
-      <c r="R46" s="33"/>
-      <c r="X46" s="28"/>
-      <c r="AA46" s="28"/>
-      <c r="AB46" s="28"/>
-    </row>
-    <row r="47" spans="9:60" x14ac:dyDescent="0.25">
-      <c r="I47" s="2">
+      <c r="J46" s="18">
+        <f>N45</f>
+        <v>0.5811551940819164</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="L46" s="2">
+        <v>1.9E-2</v>
+      </c>
+      <c r="M46" s="25">
+        <f t="shared" si="7"/>
+        <v>5.994631067741871E-4</v>
+      </c>
+      <c r="N46" s="19">
+        <f>J46+M46</f>
+        <v>0.58175465718869057</v>
+      </c>
+      <c r="O46" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="P46" s="2"/>
+      <c r="Q46" s="25"/>
+      <c r="R46" s="18">
+        <f>R45</f>
+        <v>0.58212054552188719</v>
+      </c>
+      <c r="S46" s="66"/>
+      <c r="T46" s="2"/>
+      <c r="U46" s="2"/>
+      <c r="V46" s="2"/>
+      <c r="W46" s="2"/>
+      <c r="X46" s="25"/>
+      <c r="Y46" s="2">
+        <v>1</v>
+      </c>
+      <c r="Z46" s="68">
+        <v>0</v>
+      </c>
+      <c r="AA46" s="76"/>
+      <c r="AB46" s="76">
+        <f t="shared" si="9"/>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="AC46" s="55">
+        <v>0</v>
+      </c>
+      <c r="AD46" s="2"/>
+      <c r="AE46" s="2"/>
+      <c r="AF46" s="2"/>
+      <c r="AG46" s="2"/>
+      <c r="AH46" s="2"/>
+      <c r="AI46" s="2"/>
+      <c r="AJ46" s="2"/>
+      <c r="AK46" s="2"/>
+      <c r="AL46" s="2"/>
+      <c r="AM46" s="2"/>
+      <c r="AN46" s="2"/>
+      <c r="AO46" s="2"/>
+      <c r="AP46" s="2"/>
+      <c r="AQ46" s="2"/>
+      <c r="AR46" s="2"/>
+      <c r="AS46" s="2"/>
+      <c r="AT46" s="2"/>
+      <c r="AU46" s="2"/>
+      <c r="AV46" s="2"/>
+      <c r="AW46" s="2"/>
+      <c r="AX46" s="2"/>
+      <c r="AY46" s="2"/>
+      <c r="AZ46" s="2"/>
+      <c r="BA46" s="2"/>
+      <c r="BB46" s="69"/>
+      <c r="BC46" s="2"/>
+      <c r="BD46" s="2"/>
+      <c r="BE46" s="2"/>
+      <c r="BF46" s="2"/>
+      <c r="BG46" s="2"/>
+      <c r="BH46" s="2"/>
+    </row>
+    <row r="47" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I47" s="68">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="M47" s="28"/>
-      <c r="Q47" s="28"/>
-      <c r="R47" s="33"/>
-      <c r="X47" s="28"/>
-      <c r="AA47" s="28"/>
-      <c r="AB47" s="28"/>
-    </row>
-    <row r="48" spans="9:60" x14ac:dyDescent="0.25">
-      <c r="I48" s="2">
+      <c r="J47" s="18">
+        <f>N46</f>
+        <v>0.58175465718869057</v>
+      </c>
+      <c r="K47" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="L47" s="2">
+        <v>0.82899999999999996</v>
+      </c>
+      <c r="M47" s="25">
+        <f t="shared" si="7"/>
+        <v>5.5190366327483656E-2</v>
+      </c>
+      <c r="N47" s="65">
+        <f>J47+M47</f>
+        <v>0.63694502351617421</v>
+      </c>
+      <c r="O47" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="P47" s="2"/>
+      <c r="Q47" s="25"/>
+      <c r="R47" s="19">
+        <f>R46</f>
+        <v>0.58212054552188719</v>
+      </c>
+      <c r="S47" s="66"/>
+      <c r="T47" s="2"/>
+      <c r="U47" s="2"/>
+      <c r="V47" s="2"/>
+      <c r="W47" s="2"/>
+      <c r="X47" s="25"/>
+      <c r="Y47" s="2">
+        <v>2</v>
+      </c>
+      <c r="Z47" s="68">
+        <v>0</v>
+      </c>
+      <c r="AA47" s="76"/>
+      <c r="AB47" s="76">
+        <f t="shared" si="9"/>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="AC47" s="55">
+        <v>0</v>
+      </c>
+      <c r="AD47" s="2"/>
+      <c r="AE47" s="2"/>
+      <c r="AF47" s="2"/>
+      <c r="AG47" s="2"/>
+      <c r="AH47" s="2"/>
+      <c r="AI47" s="2"/>
+      <c r="AJ47" s="2"/>
+      <c r="AK47" s="2"/>
+      <c r="AL47" s="2"/>
+      <c r="AM47" s="2"/>
+      <c r="AN47" s="2"/>
+      <c r="AO47" s="2"/>
+      <c r="AP47" s="2"/>
+      <c r="AQ47" s="2"/>
+      <c r="AR47" s="2"/>
+      <c r="AS47" s="2"/>
+      <c r="AT47" s="2"/>
+      <c r="AU47" s="2"/>
+      <c r="AV47" s="2"/>
+      <c r="AW47" s="2"/>
+      <c r="AX47" s="2"/>
+      <c r="AY47" s="2"/>
+      <c r="AZ47" s="2"/>
+      <c r="BA47" s="2"/>
+      <c r="BB47" s="69"/>
+      <c r="BC47" s="2"/>
+      <c r="BD47" s="2"/>
+      <c r="BE47" s="2"/>
+      <c r="BF47" s="2"/>
+      <c r="BG47" s="2"/>
+      <c r="BH47" s="2"/>
+    </row>
+    <row r="48" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I48" s="68">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="M48" s="28"/>
-      <c r="Q48" s="28"/>
-      <c r="R48" s="33"/>
-      <c r="X48" s="28"/>
-      <c r="AA48" s="28"/>
-      <c r="AB48" s="28"/>
-    </row>
-    <row r="49" spans="9:36" x14ac:dyDescent="0.25">
-      <c r="I49" s="2">
+      <c r="J48" s="18">
+        <f>R47</f>
+        <v>0.58212054552188719</v>
+      </c>
+      <c r="K48" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="L48" s="2"/>
+      <c r="M48" s="25"/>
+      <c r="N48" s="18">
+        <f>N47</f>
+        <v>0.63694502351617421</v>
+      </c>
+      <c r="O48" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="P48" s="2">
+        <v>0.78400000000000003</v>
+      </c>
+      <c r="Q48" s="25">
+        <f>($F$8+P48*($F$9-$F$8)) / 1440</f>
+        <v>1.2388888888888889E-2</v>
+      </c>
+      <c r="R48" s="19">
+        <f>Q48+J48</f>
+        <v>0.59450943441077608</v>
+      </c>
+      <c r="S48" s="66">
+        <v>0.51200000000000001</v>
+      </c>
+      <c r="T48" s="2" t="str">
+        <f t="shared" ref="T48:T49" si="11">IF(S48&lt;$D$16,"Elevado","Normal")</f>
+        <v>Normal</v>
+      </c>
+      <c r="U48" s="2"/>
+      <c r="V48" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="W48" s="2">
+        <v>0.42299999999999999</v>
+      </c>
+      <c r="X48" s="25">
+        <f>-90*LN(1-W48) / 1440</f>
+        <v>3.4369563279627348E-2</v>
+      </c>
+      <c r="Y48" s="2">
+        <v>1</v>
+      </c>
+      <c r="Z48" s="68">
+        <v>0</v>
+      </c>
+      <c r="AA48" s="76"/>
+      <c r="AB48" s="76">
+        <f t="shared" si="9"/>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="AC48" s="55">
+        <v>0</v>
+      </c>
+      <c r="AD48" s="2"/>
+      <c r="AE48" s="2"/>
+      <c r="AF48" s="2"/>
+      <c r="AG48" s="2"/>
+      <c r="AH48" s="2"/>
+      <c r="AI48" s="2"/>
+      <c r="AJ48" s="2"/>
+      <c r="AK48" s="2"/>
+      <c r="AL48" s="2"/>
+      <c r="AM48" s="2"/>
+      <c r="AN48" s="2"/>
+      <c r="AO48" s="2"/>
+      <c r="AP48" s="2"/>
+      <c r="AQ48" s="2"/>
+      <c r="AR48" s="2"/>
+      <c r="AS48" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AT48" s="18">
+        <f>J48</f>
+        <v>0.58212054552188719</v>
+      </c>
+      <c r="AU48" s="2"/>
+      <c r="AV48" s="25">
+        <f>X48</f>
+        <v>3.4369563279627348E-2</v>
+      </c>
+      <c r="AW48" s="2"/>
+      <c r="AX48" s="2"/>
+      <c r="AY48" s="2"/>
+      <c r="AZ48" s="2"/>
+      <c r="BA48" s="2"/>
+      <c r="BB48" s="69"/>
+      <c r="BC48" s="2"/>
+      <c r="BD48" s="2"/>
+      <c r="BE48" s="2"/>
+      <c r="BF48" s="2"/>
+      <c r="BG48" s="2"/>
+      <c r="BH48" s="2"/>
+    </row>
+    <row r="49" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I49" s="68">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="M49" s="28"/>
-      <c r="Q49" s="28"/>
-      <c r="R49" s="33"/>
-      <c r="X49" s="28"/>
-      <c r="AA49" s="28"/>
-      <c r="AB49" s="28"/>
-    </row>
-    <row r="50" spans="9:36" x14ac:dyDescent="0.25">
-      <c r="I50" s="2">
+      <c r="J49" s="18">
+        <f>R48</f>
+        <v>0.59450943441077608</v>
+      </c>
+      <c r="K49" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="L49" s="2"/>
+      <c r="M49" s="25"/>
+      <c r="N49" s="18">
+        <f>N48</f>
+        <v>0.63694502351617421</v>
+      </c>
+      <c r="O49" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="P49" s="2">
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="Q49" s="25">
+        <f>($F$8+P49*($F$9-$F$8)) / 1440</f>
+        <v>9.1805555555555564E-3</v>
+      </c>
+      <c r="R49" s="19">
+        <f>Q49+J49</f>
+        <v>0.60368998996633161</v>
+      </c>
+      <c r="S49" s="66">
+        <v>0.23100000000000001</v>
+      </c>
+      <c r="T49" s="2" t="str">
+        <f t="shared" si="11"/>
+        <v>Elevado</v>
+      </c>
+      <c r="U49" s="2">
+        <v>0.43</v>
+      </c>
+      <c r="V49" s="2" t="str">
+        <f>IF(U49&lt;$D$21,"NO","SI")</f>
+        <v>NO</v>
+      </c>
+      <c r="W49" s="2"/>
+      <c r="X49" s="25"/>
+      <c r="Y49" s="2">
+        <v>0</v>
+      </c>
+      <c r="Z49" s="68">
+        <v>0</v>
+      </c>
+      <c r="AA49" s="76"/>
+      <c r="AB49" s="76">
+        <f t="shared" si="9"/>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="AC49" s="55">
+        <v>0</v>
+      </c>
+      <c r="AD49" s="2"/>
+      <c r="AE49" s="2"/>
+      <c r="AF49" s="2"/>
+      <c r="AG49" s="2"/>
+      <c r="AH49" s="2"/>
+      <c r="AI49" s="2"/>
+      <c r="AJ49" s="2"/>
+      <c r="AK49" s="2"/>
+      <c r="AL49" s="2"/>
+      <c r="AM49" s="2"/>
+      <c r="AN49" s="2"/>
+      <c r="AO49" s="2"/>
+      <c r="AP49" s="2"/>
+      <c r="AQ49" s="2"/>
+      <c r="AR49" s="2"/>
+      <c r="AS49" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AT49" s="18">
+        <f>AT48</f>
+        <v>0.58212054552188719</v>
+      </c>
+      <c r="AU49" s="2"/>
+      <c r="AV49" s="25">
+        <f>AV48</f>
+        <v>3.4369563279627348E-2</v>
+      </c>
+      <c r="AW49" s="2"/>
+      <c r="AX49" s="2"/>
+      <c r="AY49" s="2"/>
+      <c r="AZ49" s="2"/>
+      <c r="BA49" s="2"/>
+      <c r="BB49" s="69"/>
+      <c r="BC49" s="2"/>
+      <c r="BD49" s="2"/>
+      <c r="BE49" s="2"/>
+      <c r="BF49" s="2"/>
+      <c r="BG49" s="2"/>
+      <c r="BH49" s="2"/>
+    </row>
+    <row r="50" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I50" s="68">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="M50" s="28"/>
-      <c r="Q50" s="28"/>
-      <c r="R50" s="33"/>
-      <c r="X50" s="28"/>
-      <c r="AA50" s="28"/>
-      <c r="AB50" s="28"/>
-    </row>
-    <row r="51" spans="9:36" x14ac:dyDescent="0.25">
-      <c r="I51" s="2">
+      <c r="J50" s="18">
+        <f>R49</f>
+        <v>0.60368998996633161</v>
+      </c>
+      <c r="K50" s="32" t="s">
+        <v>104</v>
+      </c>
+      <c r="L50" s="2"/>
+      <c r="M50" s="25"/>
+      <c r="N50" s="19">
+        <f>N49</f>
+        <v>0.63694502351617421</v>
+      </c>
+      <c r="O50" s="60" t="s">
+        <v>60</v>
+      </c>
+      <c r="P50" s="2"/>
+      <c r="Q50" s="25"/>
+      <c r="R50" s="19"/>
+      <c r="S50" s="66"/>
+      <c r="T50" s="2"/>
+      <c r="U50" s="2"/>
+      <c r="V50" s="2"/>
+      <c r="W50" s="2"/>
+      <c r="X50" s="25"/>
+      <c r="Y50" s="60">
+        <v>0</v>
+      </c>
+      <c r="Z50" s="73">
+        <v>0</v>
+      </c>
+      <c r="AA50" s="76"/>
+      <c r="AB50" s="76">
+        <f t="shared" si="9"/>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="AC50" s="55">
+        <v>0</v>
+      </c>
+      <c r="AD50" s="2"/>
+      <c r="AE50" s="2"/>
+      <c r="AF50" s="2"/>
+      <c r="AG50" s="2"/>
+      <c r="AH50" s="2"/>
+      <c r="AI50" s="2"/>
+      <c r="AJ50" s="2"/>
+      <c r="AK50" s="2"/>
+      <c r="AL50" s="2"/>
+      <c r="AM50" s="2"/>
+      <c r="AN50" s="2"/>
+      <c r="AO50" s="2"/>
+      <c r="AP50" s="2"/>
+      <c r="AQ50" s="2"/>
+      <c r="AR50" s="2"/>
+      <c r="AS50" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AT50" s="18">
+        <f t="shared" ref="AT50:AT51" si="12">AT49</f>
+        <v>0.58212054552188719</v>
+      </c>
+      <c r="AU50" s="2"/>
+      <c r="AV50" s="25">
+        <f>AV48</f>
+        <v>3.4369563279627348E-2</v>
+      </c>
+      <c r="AW50" s="2"/>
+      <c r="AX50" s="2"/>
+      <c r="AY50" s="2"/>
+      <c r="AZ50" s="2"/>
+      <c r="BA50" s="2"/>
+    </row>
+    <row r="51" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I51" s="68">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="M51" s="28"/>
-      <c r="Q51" s="28"/>
-      <c r="R51" s="33"/>
-      <c r="X51" s="28"/>
-      <c r="AA51" s="28"/>
-      <c r="AB51" s="28"/>
-    </row>
-    <row r="52" spans="9:36" x14ac:dyDescent="0.25">
-      <c r="I52" s="2">
+      <c r="J51" s="18">
+        <f>N50</f>
+        <v>0.63694502351617421</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="L51" s="2">
+        <f>0.983</f>
+        <v>0.98299999999999998</v>
+      </c>
+      <c r="M51" s="25">
+        <f>-$C$3*(LN(1-L51)) / 1440</f>
+        <v>0.12732943546643499</v>
+      </c>
+      <c r="N51" s="18">
+        <f>M51+J51</f>
+        <v>0.76427445898260915</v>
+      </c>
+      <c r="O51" s="60" t="s">
+        <v>61</v>
+      </c>
+      <c r="P51" s="2">
+        <v>0.152</v>
+      </c>
+      <c r="Q51" s="25">
+        <f t="shared" ref="Q50:Q51" si="13">($F$8+P51*($F$9-$F$8)) / 1440</f>
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="R51" s="19">
+        <f t="shared" ref="R50:R51" si="14">Q51+J51</f>
+        <v>0.64494502351617422</v>
+      </c>
+      <c r="S51" s="66"/>
+      <c r="T51" s="2"/>
+      <c r="U51" s="2"/>
+      <c r="V51" s="2"/>
+      <c r="W51" s="2"/>
+      <c r="X51" s="25"/>
+      <c r="Y51" s="60">
+        <v>0</v>
+      </c>
+      <c r="Z51" s="73">
+        <v>0</v>
+      </c>
+      <c r="AA51" s="76"/>
+      <c r="AB51" s="76">
+        <f t="shared" si="9"/>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="AC51" s="55">
+        <v>0</v>
+      </c>
+      <c r="AD51" s="2"/>
+      <c r="AE51" s="2"/>
+      <c r="AF51" s="2"/>
+      <c r="AG51" s="2"/>
+      <c r="AH51" s="2"/>
+      <c r="AI51" s="2"/>
+      <c r="AJ51" s="2"/>
+      <c r="AK51" s="2"/>
+      <c r="AL51" s="2"/>
+      <c r="AM51" s="2"/>
+      <c r="AN51" s="2"/>
+      <c r="AO51" s="2"/>
+      <c r="AP51" s="2"/>
+      <c r="AQ51" s="2"/>
+      <c r="AR51" s="2"/>
+      <c r="AS51" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="AT51" s="18">
+        <f t="shared" si="12"/>
+        <v>0.58212054552188719</v>
+      </c>
+      <c r="AU51" s="2"/>
+      <c r="AV51" s="25">
+        <f>AV48-(J51-J50)</f>
+        <v>1.1145297297847426E-3</v>
+      </c>
+      <c r="AW51" s="2"/>
+      <c r="AX51" s="2"/>
+      <c r="AY51" s="2"/>
+      <c r="AZ51" s="2"/>
+      <c r="BA51" s="2"/>
+    </row>
+    <row r="52" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I52" s="68">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="M52" s="28"/>
-      <c r="Q52" s="28"/>
-      <c r="X52" s="28"/>
-      <c r="AA52" s="28"/>
-      <c r="AB52" s="28"/>
-      <c r="AE52" s="44" t="s">
-        <v>17</v>
-      </c>
-      <c r="AF52" s="44"/>
-      <c r="AG52" s="44"/>
-      <c r="AH52" s="44"/>
-      <c r="AI52" s="44"/>
-    </row>
-    <row r="53" spans="9:36" x14ac:dyDescent="0.25">
-      <c r="M53" s="28"/>
-      <c r="Q53" s="28"/>
-      <c r="X53" s="28"/>
-      <c r="AB53" s="28"/>
-      <c r="AE53" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AF53" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="AG53" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="AH53" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="AI53" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="54" spans="9:36" x14ac:dyDescent="0.25">
-      <c r="M54" s="28"/>
-      <c r="Q54" s="28"/>
-      <c r="X54" s="28"/>
-      <c r="AB54" s="28"/>
-      <c r="AE54" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="AF54" s="2">
-        <v>0.3</v>
-      </c>
-      <c r="AG54" s="2">
-        <v>0.3</v>
-      </c>
-      <c r="AH54" s="2">
-        <v>0</v>
-      </c>
-      <c r="AI54" s="2">
-        <v>0.29899999999999999</v>
-      </c>
-    </row>
-    <row r="55" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="J52" s="18">
+        <f>R51</f>
+        <v>0.64494502351617422</v>
+      </c>
+      <c r="K52" s="32" t="s">
+        <v>110</v>
+      </c>
+      <c r="L52" s="2"/>
+      <c r="M52" s="25"/>
+      <c r="N52" s="18">
+        <f>N51</f>
+        <v>0.76427445898260915</v>
+      </c>
+      <c r="O52" s="60" t="s">
+        <v>60</v>
+      </c>
+      <c r="P52" s="2"/>
+      <c r="Q52" s="25"/>
+      <c r="R52" s="2"/>
+      <c r="S52" s="2"/>
+      <c r="T52" s="2"/>
+      <c r="U52" s="2"/>
+      <c r="V52" s="2"/>
+      <c r="W52" s="2"/>
+      <c r="X52" s="25"/>
+      <c r="Y52" s="60">
+        <v>0</v>
+      </c>
+      <c r="Z52" s="73">
+        <v>0</v>
+      </c>
+      <c r="AA52" s="76"/>
+      <c r="AB52" s="76">
+        <f t="shared" si="9"/>
+        <v>2.4380250379366374E-2</v>
+      </c>
+      <c r="AC52" s="55">
+        <v>0</v>
+      </c>
+      <c r="AD52" s="2"/>
+      <c r="AE52" s="46"/>
+      <c r="AF52" s="46"/>
+      <c r="AG52" s="46"/>
+      <c r="AH52" s="46"/>
+      <c r="AI52" s="46"/>
+      <c r="AJ52" s="2"/>
+      <c r="AK52" s="2"/>
+      <c r="AL52" s="2"/>
+      <c r="AM52" s="2"/>
+      <c r="AN52" s="2"/>
+      <c r="AO52" s="2"/>
+      <c r="AP52" s="2"/>
+      <c r="AQ52" s="2"/>
+      <c r="AR52" s="2"/>
+      <c r="AS52" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="AT52" s="18">
+        <f>AT51</f>
+        <v>0.58212054552188719</v>
+      </c>
+      <c r="AU52" s="2"/>
+      <c r="AV52" s="25">
+        <f>AV51</f>
+        <v>1.1145297297847426E-3</v>
+      </c>
+      <c r="AW52" s="2"/>
+      <c r="AX52" s="2"/>
+      <c r="AY52" s="2"/>
+      <c r="AZ52" s="2"/>
+      <c r="BA52" s="2"/>
+    </row>
+    <row r="53" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I53" s="68">
+        <f t="shared" si="0"/>
+        <v>41</v>
+      </c>
+      <c r="J53" s="18">
+        <f>J52+AV51</f>
+        <v>0.64605955324595898</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="L53" s="2"/>
+      <c r="M53" s="25"/>
+      <c r="N53" s="19">
+        <f>N52</f>
+        <v>0.76427445898260915</v>
+      </c>
+      <c r="O53" s="60" t="s">
+        <v>53</v>
+      </c>
+      <c r="P53" s="2"/>
+      <c r="Q53" s="25"/>
+      <c r="R53" s="2"/>
+      <c r="S53" s="2"/>
+      <c r="T53" s="2"/>
+      <c r="U53" s="2"/>
+      <c r="V53" s="2"/>
+      <c r="W53" s="2"/>
+      <c r="X53" s="25"/>
+      <c r="Y53" s="60">
+        <v>0</v>
+      </c>
+      <c r="Z53" s="73">
+        <v>0</v>
+      </c>
+      <c r="AA53" s="75"/>
+      <c r="AB53" s="76">
+        <f>AB52+X48</f>
+        <v>5.8749813658993719E-2</v>
+      </c>
+      <c r="AC53" s="55">
+        <v>0</v>
+      </c>
+      <c r="AD53" s="2"/>
+      <c r="AE53" s="2"/>
+      <c r="AF53" s="1"/>
+      <c r="AG53" s="1"/>
+      <c r="AH53" s="1"/>
+      <c r="AI53" s="1"/>
+      <c r="AJ53" s="2"/>
+      <c r="AK53" s="2"/>
+      <c r="AL53" s="2"/>
+      <c r="AM53" s="2"/>
+      <c r="AN53" s="2"/>
+      <c r="AO53" s="2"/>
+      <c r="AP53" s="2"/>
+      <c r="AQ53" s="2"/>
+      <c r="AR53" s="2"/>
+      <c r="AS53" s="23"/>
+      <c r="AT53" s="18">
+        <f>AT52</f>
+        <v>0.58212054552188719</v>
+      </c>
+      <c r="AU53" s="18">
+        <f>J53</f>
+        <v>0.64605955324595898</v>
+      </c>
+      <c r="AV53" s="2">
+        <v>0</v>
+      </c>
+      <c r="AW53" s="2"/>
+      <c r="AX53" s="2"/>
+      <c r="AY53" s="2"/>
+      <c r="AZ53" s="2"/>
+      <c r="BA53" s="2"/>
+    </row>
+    <row r="54" spans="9:60" x14ac:dyDescent="0.35">
+      <c r="I54" s="68">
+        <f t="shared" si="0"/>
+        <v>42</v>
+      </c>
+      <c r="J54" s="71">
+        <f>N53</f>
+        <v>0.76427445898260915</v>
+      </c>
+      <c r="K54" s="67" t="s">
+        <v>110</v>
+      </c>
+      <c r="L54" s="67"/>
+      <c r="M54" s="72"/>
+      <c r="N54" s="67"/>
+      <c r="O54" s="67"/>
+      <c r="P54" s="67"/>
+      <c r="Q54" s="72"/>
+      <c r="R54" s="71"/>
+      <c r="S54" s="67"/>
+      <c r="T54" s="67"/>
+      <c r="U54" s="67"/>
+      <c r="V54" s="67"/>
+      <c r="W54" s="67"/>
+      <c r="X54" s="72"/>
+      <c r="Y54" s="67"/>
+      <c r="Z54" s="78"/>
+      <c r="AA54" s="79"/>
+      <c r="AB54" s="80"/>
+      <c r="AC54" s="79">
+        <v>0</v>
+      </c>
+      <c r="AD54" s="2"/>
+      <c r="AE54" s="2"/>
+      <c r="AF54" s="2"/>
+      <c r="AG54" s="2"/>
+      <c r="AH54" s="2"/>
+      <c r="AI54" s="2"/>
+      <c r="AJ54" s="2"/>
+      <c r="AK54" s="2"/>
+      <c r="AL54" s="2"/>
+      <c r="AM54" s="2"/>
+      <c r="AN54" s="2"/>
+      <c r="AO54" s="2"/>
+      <c r="AP54" s="2"/>
+      <c r="AQ54" s="2"/>
+      <c r="AR54" s="2"/>
+      <c r="AS54" s="2"/>
+      <c r="AT54" s="23"/>
+      <c r="AU54" s="23"/>
+      <c r="AV54" s="23"/>
+      <c r="AW54" s="2"/>
+      <c r="AX54" s="2"/>
+      <c r="AY54" s="2"/>
+      <c r="AZ54" s="2"/>
+      <c r="BA54" s="2"/>
+    </row>
+    <row r="55" spans="9:60" x14ac:dyDescent="0.35">
       <c r="M55" s="28"/>
       <c r="X55" s="28"/>
       <c r="AB55" s="28"/>
-      <c r="AE55" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="AF55" s="2">
-        <v>0.7</v>
-      </c>
-      <c r="AG55" s="2">
-        <v>1</v>
-      </c>
-      <c r="AH55" s="2">
-        <v>0.3</v>
-      </c>
-      <c r="AI55" s="2">
-        <v>0.999</v>
-      </c>
-    </row>
-    <row r="56" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="AD55" s="2"/>
+      <c r="AE55" s="70"/>
+      <c r="AF55" s="70"/>
+      <c r="AG55" s="70"/>
+      <c r="AH55" s="70"/>
+      <c r="AI55" s="70"/>
+    </row>
+    <row r="56" spans="9:60" x14ac:dyDescent="0.35">
       <c r="M56" s="28"/>
       <c r="X56" s="28"/>
       <c r="AB56" s="28"/>
     </row>
-    <row r="57" spans="9:36" x14ac:dyDescent="0.25">
+    <row r="57" spans="9:60" x14ac:dyDescent="0.35">
       <c r="M57" s="28"/>
       <c r="X57" s="28"/>
       <c r="AB57" s="28"/>
-      <c r="AE57" s="44" t="s">
-        <v>25</v>
-      </c>
-      <c r="AF57" s="44"/>
-      <c r="AG57" s="44"/>
-      <c r="AH57" s="44"/>
-      <c r="AI57" s="44"/>
-    </row>
-    <row r="58" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="AE57" s="46"/>
+      <c r="AF57" s="46"/>
+      <c r="AG57" s="46"/>
+      <c r="AH57" s="46"/>
+      <c r="AI57" s="46"/>
+    </row>
+    <row r="58" spans="9:60" x14ac:dyDescent="0.35">
       <c r="M58" s="28"/>
       <c r="X58" s="28"/>
       <c r="AB58" s="28"/>
-      <c r="AE58" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="AF58" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="AG58" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="AH58" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="AI58" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="59" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="AE58" s="2"/>
+      <c r="AF58" s="1"/>
+      <c r="AG58" s="1"/>
+      <c r="AH58" s="1"/>
+      <c r="AI58" s="1"/>
+    </row>
+    <row r="59" spans="9:60" x14ac:dyDescent="0.35">
       <c r="M59" s="28"/>
       <c r="X59" s="28"/>
       <c r="AB59" s="28"/>
-      <c r="AE59" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="AF59" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="AG59" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="AH59" s="2">
-        <v>0</v>
-      </c>
-      <c r="AI59" s="2">
-        <v>0.499</v>
-      </c>
-      <c r="AJ59" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="60" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="AE59" s="2"/>
+      <c r="AF59" s="2"/>
+      <c r="AG59" s="2"/>
+      <c r="AH59" s="2"/>
+      <c r="AI59" s="2"/>
+      <c r="AJ59" s="2"/>
+    </row>
+    <row r="60" spans="9:60" x14ac:dyDescent="0.35">
       <c r="M60" s="28"/>
       <c r="X60" s="28"/>
       <c r="AB60" s="28"/>
-      <c r="AE60" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="AF60" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="AG60" s="2">
-        <v>1</v>
-      </c>
-      <c r="AH60" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="AI60" s="2">
-        <v>0.999</v>
-      </c>
-    </row>
-    <row r="61" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="AE60" s="2"/>
+      <c r="AF60" s="2"/>
+      <c r="AG60" s="2"/>
+      <c r="AH60" s="2"/>
+      <c r="AI60" s="2"/>
+    </row>
+    <row r="61" spans="9:60" x14ac:dyDescent="0.35">
       <c r="M61" s="28"/>
       <c r="X61" s="28"/>
       <c r="AB61" s="28"/>
     </row>
-    <row r="62" spans="9:36" x14ac:dyDescent="0.25">
+    <row r="62" spans="9:60" x14ac:dyDescent="0.35">
       <c r="M62" s="28"/>
       <c r="X62" s="28"/>
       <c r="AB62" s="28"/>
-      <c r="AE62" s="45" t="s">
-        <v>26</v>
-      </c>
-      <c r="AF62" s="45"/>
-      <c r="AG62" s="45"/>
-      <c r="AH62" s="45"/>
-      <c r="AI62" s="45"/>
-    </row>
-    <row r="63" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="AE62" s="48"/>
+      <c r="AF62" s="48"/>
+      <c r="AG62" s="48"/>
+      <c r="AH62" s="48"/>
+      <c r="AI62" s="48"/>
+    </row>
+    <row r="63" spans="9:60" x14ac:dyDescent="0.35">
       <c r="M63" s="28"/>
       <c r="X63" s="28"/>
       <c r="AB63" s="28"/>
-      <c r="AE63" s="45"/>
-      <c r="AF63" s="45"/>
-      <c r="AG63" s="45"/>
-      <c r="AH63" s="45"/>
-      <c r="AI63" s="45"/>
-    </row>
-    <row r="64" spans="9:36" x14ac:dyDescent="0.25">
+      <c r="AE63" s="48"/>
+      <c r="AF63" s="48"/>
+      <c r="AG63" s="48"/>
+      <c r="AH63" s="48"/>
+      <c r="AI63" s="48"/>
+    </row>
+    <row r="64" spans="9:60" x14ac:dyDescent="0.35">
       <c r="M64" s="28"/>
       <c r="X64" s="28"/>
       <c r="AB64" s="28"/>
     </row>
-    <row r="65" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="65" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M65" s="28"/>
       <c r="X65" s="28"/>
       <c r="AB65" s="28"/>
     </row>
-    <row r="66" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="66" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M66" s="28"/>
       <c r="X66" s="28"/>
       <c r="AB66" s="28"/>
     </row>
-    <row r="67" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="67" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M67" s="28"/>
       <c r="X67" s="28"/>
       <c r="AB67" s="28"/>
     </row>
-    <row r="68" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="68" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M68" s="28"/>
       <c r="X68" s="28"/>
       <c r="AB68" s="28"/>
     </row>
-    <row r="69" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="69" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M69" s="28"/>
       <c r="X69" s="28"/>
       <c r="AB69" s="28"/>
     </row>
-    <row r="70" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="70" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M70" s="28"/>
       <c r="X70" s="28"/>
       <c r="AB70" s="28"/>
     </row>
-    <row r="71" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="71" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M71" s="28"/>
       <c r="X71" s="28"/>
       <c r="AB71" s="28"/>
     </row>
-    <row r="72" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="72" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M72" s="28"/>
       <c r="X72" s="28"/>
       <c r="AB72" s="28"/>
     </row>
-    <row r="73" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="73" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M73" s="28"/>
       <c r="X73" s="28"/>
       <c r="AB73" s="28"/>
     </row>
-    <row r="74" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="74" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M74" s="28"/>
       <c r="X74" s="28"/>
       <c r="AB74" s="28"/>
     </row>
-    <row r="75" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="75" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M75" s="28"/>
       <c r="X75" s="28"/>
       <c r="AB75" s="28"/>
     </row>
-    <row r="76" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="76" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M76" s="28"/>
       <c r="X76" s="28"/>
       <c r="AB76" s="28"/>
     </row>
-    <row r="77" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="77" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M77" s="28"/>
       <c r="X77" s="28"/>
       <c r="AB77" s="28"/>
     </row>
-    <row r="78" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="78" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M78" s="28"/>
       <c r="X78" s="28"/>
       <c r="AB78" s="28"/>
     </row>
-    <row r="79" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="79" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M79" s="28"/>
       <c r="X79" s="28"/>
       <c r="AB79" s="28"/>
     </row>
-    <row r="80" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="80" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M80" s="28"/>
       <c r="X80" s="28"/>
       <c r="AB80" s="28"/>
     </row>
-    <row r="81" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="81" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M81" s="28"/>
       <c r="X81" s="28"/>
       <c r="AB81" s="28"/>
     </row>
-    <row r="82" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="82" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M82" s="28"/>
       <c r="X82" s="28"/>
       <c r="AB82" s="28"/>
     </row>
-    <row r="83" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="83" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M83" s="28"/>
       <c r="X83" s="28"/>
       <c r="AB83" s="28"/>
     </row>
-    <row r="84" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="84" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M84" s="28"/>
       <c r="X84" s="28"/>
       <c r="AB84" s="28"/>
     </row>
-    <row r="85" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="85" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M85" s="28"/>
       <c r="X85" s="28"/>
       <c r="AB85" s="28"/>
     </row>
-    <row r="86" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="86" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M86" s="28"/>
       <c r="X86" s="28"/>
       <c r="AB86" s="28"/>
     </row>
-    <row r="87" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="87" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M87" s="28"/>
       <c r="X87" s="28"/>
       <c r="AB87" s="28"/>
     </row>
-    <row r="88" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="88" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M88" s="28"/>
       <c r="X88" s="28"/>
       <c r="AB88" s="28"/>
     </row>
-    <row r="89" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="89" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M89" s="28"/>
       <c r="AB89" s="28"/>
     </row>
-    <row r="90" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="90" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M90" s="28"/>
       <c r="AB90" s="28"/>
     </row>
-    <row r="91" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="91" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M91" s="28"/>
       <c r="AB91" s="28"/>
     </row>
-    <row r="92" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="92" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M92" s="28"/>
       <c r="AB92" s="28"/>
     </row>
-    <row r="93" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="93" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M93" s="28"/>
       <c r="AB93" s="28"/>
     </row>
-    <row r="94" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="94" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M94" s="28"/>
       <c r="AB94" s="28"/>
     </row>
-    <row r="95" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="95" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M95" s="28"/>
       <c r="AB95" s="28"/>
     </row>
-    <row r="96" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="96" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M96" s="28"/>
       <c r="AB96" s="28"/>
     </row>
-    <row r="97" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="97" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M97" s="28"/>
       <c r="AB97" s="28"/>
     </row>
-    <row r="98" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="98" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M98" s="28"/>
       <c r="AB98" s="28"/>
     </row>
-    <row r="99" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="99" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M99" s="28"/>
       <c r="AB99" s="28"/>
     </row>
-    <row r="100" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="100" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M100" s="28"/>
       <c r="AB100" s="28"/>
     </row>
-    <row r="101" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="101" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M101" s="28"/>
       <c r="AB101" s="28"/>
     </row>
-    <row r="102" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="102" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M102" s="28"/>
       <c r="AB102" s="28"/>
     </row>
-    <row r="103" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="103" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M103" s="28"/>
       <c r="AB103" s="28"/>
     </row>
-    <row r="104" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="104" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M104" s="28"/>
       <c r="AB104" s="28"/>
     </row>
-    <row r="105" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="105" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M105" s="28"/>
       <c r="AB105" s="28"/>
     </row>
-    <row r="106" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="106" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M106" s="28"/>
       <c r="AB106" s="28"/>
     </row>
-    <row r="107" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="107" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M107" s="28"/>
       <c r="AB107" s="28"/>
     </row>
-    <row r="108" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="108" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M108" s="28"/>
       <c r="AB108" s="28"/>
     </row>
-    <row r="109" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="109" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M109" s="28"/>
       <c r="AB109" s="28"/>
     </row>
-    <row r="110" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="110" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M110" s="28"/>
       <c r="AB110" s="28"/>
     </row>
-    <row r="111" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="111" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M111" s="28"/>
       <c r="AB111" s="28"/>
     </row>
-    <row r="112" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="112" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M112" s="28"/>
       <c r="AB112" s="28"/>
     </row>
-    <row r="113" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="113" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M113" s="28"/>
       <c r="AB113" s="28"/>
     </row>
-    <row r="114" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="114" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M114" s="28"/>
       <c r="AB114" s="28"/>
     </row>
-    <row r="115" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="115" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M115" s="28"/>
       <c r="AB115" s="28"/>
     </row>
-    <row r="116" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="116" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M116" s="28"/>
       <c r="AB116" s="28"/>
     </row>
-    <row r="117" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="117" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M117" s="28"/>
       <c r="AB117" s="28"/>
     </row>
-    <row r="118" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="118" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M118" s="28"/>
       <c r="AB118" s="28"/>
     </row>
-    <row r="119" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="119" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M119" s="28"/>
       <c r="AB119" s="28"/>
     </row>
-    <row r="120" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="120" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M120" s="28"/>
       <c r="AB120" s="28"/>
     </row>
-    <row r="121" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="121" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M121" s="28"/>
       <c r="AB121" s="28"/>
     </row>
-    <row r="122" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="122" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M122" s="28"/>
       <c r="AB122" s="28"/>
     </row>
-    <row r="123" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="123" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M123" s="28"/>
       <c r="AB123" s="28"/>
     </row>
-    <row r="124" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="124" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M124" s="28"/>
       <c r="AB124" s="28"/>
     </row>
-    <row r="125" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="125" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M125" s="28"/>
       <c r="AB125" s="28"/>
     </row>
-    <row r="126" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="126" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M126" s="28"/>
       <c r="AB126" s="28"/>
     </row>
-    <row r="127" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="127" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M127" s="28"/>
       <c r="AB127" s="28"/>
     </row>
-    <row r="128" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="128" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M128" s="28"/>
       <c r="AB128" s="28"/>
     </row>
-    <row r="129" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="129" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M129" s="28"/>
       <c r="AB129" s="28"/>
     </row>
-    <row r="130" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="130" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M130" s="28"/>
       <c r="AB130" s="28"/>
     </row>
-    <row r="131" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="131" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M131" s="28"/>
       <c r="AB131" s="28"/>
     </row>
-    <row r="132" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="132" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M132" s="28"/>
       <c r="AB132" s="28"/>
     </row>
-    <row r="133" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="133" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M133" s="28"/>
       <c r="AB133" s="28"/>
     </row>
-    <row r="134" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="134" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M134" s="28"/>
       <c r="AB134" s="28"/>
     </row>
-    <row r="135" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="135" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M135" s="28"/>
       <c r="AB135" s="28"/>
     </row>
-    <row r="136" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="136" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M136" s="28"/>
       <c r="AB136" s="28"/>
     </row>
-    <row r="137" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="137" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M137" s="28"/>
       <c r="AB137" s="28"/>
     </row>
-    <row r="138" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="138" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M138" s="28"/>
       <c r="AB138" s="28"/>
     </row>
-    <row r="139" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="139" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M139" s="28"/>
       <c r="AB139" s="28"/>
     </row>
-    <row r="140" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="140" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M140" s="28"/>
       <c r="AB140" s="28"/>
     </row>
-    <row r="141" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="141" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M141" s="28"/>
       <c r="AB141" s="28"/>
     </row>
-    <row r="142" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="142" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M142" s="28"/>
       <c r="AB142" s="28"/>
     </row>
-    <row r="143" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="143" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M143" s="28"/>
       <c r="AB143" s="28"/>
     </row>
-    <row r="144" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="144" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M144" s="28"/>
       <c r="AB144" s="28"/>
     </row>
-    <row r="145" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="145" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M145" s="28"/>
       <c r="AB145" s="28"/>
     </row>
-    <row r="146" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="146" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M146" s="28"/>
       <c r="AB146" s="28"/>
     </row>
-    <row r="147" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="147" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M147" s="28"/>
       <c r="AB147" s="28"/>
     </row>
-    <row r="148" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="148" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M148" s="28"/>
       <c r="AB148" s="28"/>
     </row>
-    <row r="149" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="149" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M149" s="28"/>
       <c r="AB149" s="28"/>
     </row>
-    <row r="150" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="150" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M150" s="28"/>
       <c r="AB150" s="28"/>
     </row>
-    <row r="151" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="151" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M151" s="28"/>
       <c r="AB151" s="28"/>
     </row>
-    <row r="152" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="152" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M152" s="28"/>
       <c r="AB152" s="28"/>
     </row>
-    <row r="153" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="153" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M153" s="28"/>
       <c r="AB153" s="28"/>
     </row>
-    <row r="154" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="154" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M154" s="28"/>
       <c r="AB154" s="28"/>
     </row>
-    <row r="155" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="155" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M155" s="28"/>
       <c r="AB155" s="28"/>
     </row>
-    <row r="156" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="156" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M156" s="28"/>
       <c r="AB156" s="28"/>
     </row>
-    <row r="157" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="157" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M157" s="28"/>
       <c r="AB157" s="28"/>
     </row>
-    <row r="158" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="158" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M158" s="28"/>
       <c r="AB158" s="28"/>
     </row>
-    <row r="159" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="159" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M159" s="28"/>
       <c r="AB159" s="28"/>
     </row>
-    <row r="160" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="160" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M160" s="28"/>
       <c r="AB160" s="28"/>
     </row>
-    <row r="161" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="161" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M161" s="28"/>
       <c r="AB161" s="28"/>
     </row>
-    <row r="162" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="162" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M162" s="28"/>
       <c r="AB162" s="28"/>
     </row>
-    <row r="163" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="163" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M163" s="28"/>
       <c r="AB163" s="28"/>
     </row>
-    <row r="164" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="164" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M164" s="28"/>
       <c r="AB164" s="28"/>
     </row>
-    <row r="165" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="165" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M165" s="28"/>
       <c r="AB165" s="28"/>
     </row>
-    <row r="166" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="166" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M166" s="28"/>
       <c r="AB166" s="28"/>
     </row>
-    <row r="167" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="167" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M167" s="28"/>
       <c r="AB167" s="28"/>
     </row>
-    <row r="168" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="168" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M168" s="28"/>
       <c r="AB168" s="28"/>
     </row>
-    <row r="169" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="169" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M169" s="28"/>
       <c r="AB169" s="28"/>
     </row>
-    <row r="170" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="170" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M170" s="28"/>
       <c r="AB170" s="28"/>
     </row>
-    <row r="171" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="171" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M171" s="28"/>
       <c r="AB171" s="28"/>
     </row>
-    <row r="172" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="172" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M172" s="28"/>
       <c r="AB172" s="28"/>
     </row>
-    <row r="173" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="173" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M173" s="28"/>
       <c r="AB173" s="28"/>
     </row>
-    <row r="174" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="174" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M174" s="28"/>
       <c r="AB174" s="28"/>
     </row>
-    <row r="175" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="175" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M175" s="28"/>
       <c r="AB175" s="28"/>
     </row>
-    <row r="176" spans="13:28" x14ac:dyDescent="0.25">
+    <row r="176" spans="13:28" x14ac:dyDescent="0.35">
       <c r="M176" s="28"/>
       <c r="AB176" s="28"/>
     </row>
-    <row r="177" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="177" spans="13:13" x14ac:dyDescent="0.35">
       <c r="M177" s="28"/>
     </row>
-    <row r="178" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="178" spans="13:13" x14ac:dyDescent="0.35">
       <c r="M178" s="28"/>
     </row>
-    <row r="179" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="179" spans="13:13" x14ac:dyDescent="0.35">
       <c r="M179" s="28"/>
     </row>
-    <row r="180" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="180" spans="13:13" x14ac:dyDescent="0.35">
       <c r="M180" s="28"/>
     </row>
-    <row r="181" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="181" spans="13:13" x14ac:dyDescent="0.35">
       <c r="M181" s="28"/>
     </row>
-    <row r="182" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="182" spans="13:13" x14ac:dyDescent="0.35">
       <c r="M182" s="28"/>
     </row>
   </sheetData>
-  <mergeCells count="37">
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="AD10:AM10"/>
-    <mergeCell ref="O11:V11"/>
-    <mergeCell ref="AA11:AC11"/>
-    <mergeCell ref="Y11:Z11"/>
+  <mergeCells count="38">
+    <mergeCell ref="J38:BH38"/>
+    <mergeCell ref="AE52:AI52"/>
+    <mergeCell ref="AE57:AI57"/>
+    <mergeCell ref="AE62:AI63"/>
+    <mergeCell ref="BE11:BH11"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="AW11:AZ11"/>
+    <mergeCell ref="BA11:BD11"/>
+    <mergeCell ref="AO10:BD10"/>
+    <mergeCell ref="J9:BD9"/>
+    <mergeCell ref="K2:O2"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="W11:X11"/>
+    <mergeCell ref="Q3:R3"/>
+    <mergeCell ref="Q4:R4"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="Q2:T2"/>
     <mergeCell ref="S3:T3"/>
@@ -4948,23 +6197,13 @@
     <mergeCell ref="B14:F14"/>
     <mergeCell ref="B19:F19"/>
     <mergeCell ref="AO11:AR11"/>
-    <mergeCell ref="AE52:AI52"/>
-    <mergeCell ref="AE57:AI57"/>
-    <mergeCell ref="AE62:AI63"/>
-    <mergeCell ref="BE11:BH11"/>
-    <mergeCell ref="E2:H2"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="AW11:AZ11"/>
-    <mergeCell ref="BA11:BD11"/>
-    <mergeCell ref="AO10:BD10"/>
-    <mergeCell ref="J9:BD9"/>
-    <mergeCell ref="K2:O2"/>
-    <mergeCell ref="L11:N11"/>
-    <mergeCell ref="W11:X11"/>
-    <mergeCell ref="Q3:R3"/>
-    <mergeCell ref="Q4:R4"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="AD10:AM10"/>
+    <mergeCell ref="O11:V11"/>
+    <mergeCell ref="AA11:AC11"/>
+    <mergeCell ref="Y11:Z11"/>
   </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>